<commit_message>
review: sync PRISMA tracker, 90-paper references and publication-lineage audits
Upload 13 pending files from local commits 504eb4c, 598e8e1, 99d81a9 and 589e766.

- Populate the 90-record seed screening log and distinguish candidates from formally included studies.
- Add the Markdown bibliography and BibTeX, CSV and RIS reference exports.
- Add the exact/near-duplicate audit and 16-record publication-lineage verification.
- Preserve preprints and unresolved venue claims without counting versions as separate studies.

All repository file hashes match local checkpoint 589e7668e8afc124933a94307d0f52256ac27fc5. Uploaded via the authenticated GitHub connection because terminal SSH could not reach GitHub.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R76953715105d4881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="Ra4df7c7edb924150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R283f0baa2de94d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R6ed4c31a2a764c72"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R6f67d86b9f054ea9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R20fabfa668464059"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R17e1a3eabb454e1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R4b0de1100bbc4c92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R408c59cf19964d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R7210efa6825a41ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -329,7 +329,7 @@
         <x:color rgb="FF7F6000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -339,7 +339,7 @@
         <x:color rgb="FFC00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -350,7 +350,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -360,7 +360,7 @@
         <x:color rgb="FFC00000"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -549,7 +549,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6b0a161f65fc4f34"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R588affd2d8104e37"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -870,10 +870,9 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="16" t="str">
-        <x:v>Seed papers coded</x:v>
+        <x:v>Candidate seed records</x:v>
       </x:c>
       <x:c r="B6" s="17" t="n">
-        <x:f>COUNTA('Evidence Matrix'!$A$2:$A$91)</x:f>
         <x:v>90</x:v>
       </x:c>
       <x:c r="D6" s="16" t="str">
@@ -885,11 +884,10 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="16" t="str">
-        <x:v>Peer-reviewed</x:v>
+        <x:v>Formal database records imported</x:v>
       </x:c>
       <x:c r="B7" s="17" t="n">
-        <x:f>COUNTIF('Evidence Matrix'!$G$2:$G$91,"Yes")</x:f>
-        <x:v>81</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="16" t="str">
         <x:v>Blind diffusion</x:v>
@@ -900,11 +898,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="16" t="str">
-        <x:v>Preprints / mixed lineage</x:v>
+        <x:v>Duplicates removed</x:v>
       </x:c>
       <x:c r="B8" s="17" t="n">
-        <x:f>COUNTIF('Evidence Matrix'!$G$2:$G$91,"&lt;&gt;Yes")</x:f>
-        <x:v>9</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D8" s="16" t="str">
         <x:v>All-in-one restoration</x:v>
@@ -915,11 +912,10 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="str">
-        <x:v>Closest competitors</x:v>
+        <x:v>Title/abstract screened</x:v>
       </x:c>
       <x:c r="B9" s="17" t="n">
-        <x:f>COUNTIF('Evidence Matrix'!$AB$2:$AB$91,"Yes")</x:f>
-        <x:v>62</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D9" s="18" t="str">
         <x:v>Reliability / UQ</x:v>
@@ -930,38 +926,34 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="16" t="str">
-        <x:v>Joint image/operator</x:v>
+        <x:v>Full texts assessed</x:v>
       </x:c>
       <x:c r="B10" s="17" t="n">
-        <x:f>COUNTIF('Evidence Matrix'!$O$2:$O$91,"Yes")</x:f>
-        <x:v>16</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="16" t="str">
-        <x:v>Any image UQ</x:v>
+        <x:v>Formally included studies</x:v>
       </x:c>
       <x:c r="B11" s="17" t="n">
-        <x:f>COUNTIF('Evidence Matrix'!$P$2:$P$91,"Yes")</x:f>
-        <x:v>21</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="16" t="str">
-        <x:v>Any calibration</x:v>
+        <x:v>Formally excluded studies</x:v>
       </x:c>
       <x:c r="B12" s="17" t="n">
-        <x:f>COUNTIF('Evidence Matrix'!$R$2:$R$91,"Yes")</x:f>
-        <x:v>9</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="18" t="str">
-        <x:v>Any abstention</x:v>
-      </x:c>
-      <x:c r="B13" s="19" t="n">
-        <x:f>COUNTIF('Evidence Matrix'!$X$2:$X$91,"Yes")</x:f>
-        <x:v>3</x:v>
+        <x:v>PRISMA screening</x:v>
+      </x:c>
+      <x:c r="B13" s="19" t="str">
+        <x:v>Not started</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1127,7 +1119,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1dea0ab9ca5e4e10"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R797d5a006f324de9"/>
 </x:worksheet>
 </file>
 
@@ -10099,7 +10091,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd10a9baff94744ae"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c4e6da3c08b48bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10176,11 +10168,21 @@
         <x:v>S001</x:v>
       </x:c>
       <x:c r="B2" s="39"/>
-      <x:c r="C2" s="1" t="str"/>
-      <x:c r="D2" s="1" t="str"/>
-      <x:c r="E2" s="1" t="str"/>
-      <x:c r="F2" s="1" t="str"/>
-      <x:c r="G2" s="1" t="str"/>
+      <x:c r="C2" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P001</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="str">
+        <x:v>Deep Learning for Handling Kernel/Model Uncertainty in Image Deconvolution</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="str">
+        <x:v>https://doi.org/10.1109/CVPR42600.2020.00246</x:v>
+      </x:c>
       <x:c r="H2" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10190,13 +10192,15 @@
       <x:c r="J2" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K2" s="1" t="str"/>
-      <x:c r="L2" s="1" t="str"/>
+      <x:c r="K2" s="1"/>
+      <x:c r="L2" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M2" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N2" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10204,11 +10208,21 @@
         <x:v>S002</x:v>
       </x:c>
       <x:c r="B3" s="39"/>
-      <x:c r="C3" s="1" t="str"/>
-      <x:c r="D3" s="1" t="str"/>
-      <x:c r="E3" s="1" t="str"/>
-      <x:c r="F3" s="1" t="str"/>
-      <x:c r="G3" s="1" t="str"/>
+      <x:c r="C3" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D3" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P002</x:v>
+      </x:c>
+      <x:c r="E3" s="1" t="str">
+        <x:v>NETT: Solving Inverse Problems with Deep Neural Networks</x:v>
+      </x:c>
+      <x:c r="F3" s="1" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G3" s="1" t="str">
+        <x:v>https://doi.org/10.1088/1361-6420/ab6d57</x:v>
+      </x:c>
       <x:c r="H3" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10218,13 +10232,15 @@
       <x:c r="J3" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K3" s="1" t="str"/>
-      <x:c r="L3" s="1" t="str"/>
+      <x:c r="K3" s="1"/>
+      <x:c r="L3" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M3" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N3" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -10232,11 +10248,21 @@
         <x:v>S003</x:v>
       </x:c>
       <x:c r="B4" s="39"/>
-      <x:c r="C4" s="1" t="str"/>
-      <x:c r="D4" s="1" t="str"/>
-      <x:c r="E4" s="1" t="str"/>
-      <x:c r="F4" s="1" t="str"/>
-      <x:c r="G4" s="1" t="str"/>
+      <x:c r="C4" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D4" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P003</x:v>
+      </x:c>
+      <x:c r="E4" s="1" t="str">
+        <x:v>On Instabilities of Deep Learning in Image Reconstruction and the Potential Costs of AI</x:v>
+      </x:c>
+      <x:c r="F4" s="1" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G4" s="1" t="str">
+        <x:v>https://doi.org/10.1073/pnas.1907377117</x:v>
+      </x:c>
       <x:c r="H4" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10246,13 +10272,15 @@
       <x:c r="J4" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K4" s="1" t="str"/>
-      <x:c r="L4" s="1" t="str"/>
+      <x:c r="K4" s="1"/>
+      <x:c r="L4" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M4" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N4" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -10260,11 +10288,21 @@
         <x:v>S004</x:v>
       </x:c>
       <x:c r="B5" s="39"/>
-      <x:c r="C5" s="1" t="str"/>
-      <x:c r="D5" s="1" t="str"/>
-      <x:c r="E5" s="1" t="str"/>
-      <x:c r="F5" s="1" t="str"/>
-      <x:c r="G5" s="1" t="str"/>
+      <x:c r="C5" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P004</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="str">
+        <x:v>Real-World Blur Dataset for Learning and Benchmarking Deblurring Algorithms</x:v>
+      </x:c>
+      <x:c r="F5" s="1" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G5" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content_CVPR_2020/html/Rim_Real-World_Blur_Dataset_for_Learning_and_Benchmarking_Deblurring_Algorithms_CVPR_2020_paper.html</x:v>
+      </x:c>
       <x:c r="H5" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10274,13 +10312,15 @@
       <x:c r="J5" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K5" s="1" t="str"/>
-      <x:c r="L5" s="1" t="str"/>
+      <x:c r="K5" s="1"/>
+      <x:c r="L5" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M5" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N5" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10288,11 +10328,21 @@
         <x:v>S005</x:v>
       </x:c>
       <x:c r="B6" s="39"/>
-      <x:c r="C6" s="1" t="str"/>
-      <x:c r="D6" s="1" t="str"/>
-      <x:c r="E6" s="1" t="str"/>
-      <x:c r="F6" s="1" t="str"/>
-      <x:c r="G6" s="1" t="str"/>
+      <x:c r="C6" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D6" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P005</x:v>
+      </x:c>
+      <x:c r="E6" s="1" t="str">
+        <x:v>Robust Reconstruction With Deep Learning to Handle Model Mismatch in Lensless Imaging</x:v>
+      </x:c>
+      <x:c r="F6" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G6" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TCI.2021.3114542</x:v>
+      </x:c>
       <x:c r="H6" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10302,13 +10352,15 @@
       <x:c r="J6" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K6" s="1" t="str"/>
-      <x:c r="L6" s="1" t="str"/>
+      <x:c r="K6" s="1"/>
+      <x:c r="L6" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M6" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N6" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -10316,11 +10368,21 @@
         <x:v>S006</x:v>
       </x:c>
       <x:c r="B7" s="39"/>
-      <x:c r="C7" s="1" t="str"/>
-      <x:c r="D7" s="1" t="str"/>
-      <x:c r="E7" s="1" t="str"/>
-      <x:c r="F7" s="1" t="str"/>
-      <x:c r="G7" s="1" t="str"/>
+      <x:c r="C7" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D7" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P006</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="str">
+        <x:v>Deep Equilibrium Architectures for Inverse Problems in Imaging</x:v>
+      </x:c>
+      <x:c r="F7" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G7" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TCI.2021.3118944</x:v>
+      </x:c>
       <x:c r="H7" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10330,13 +10392,15 @@
       <x:c r="J7" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K7" s="1" t="str"/>
-      <x:c r="L7" s="1" t="str"/>
+      <x:c r="K7" s="1"/>
+      <x:c r="L7" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M7" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N7" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -10344,11 +10408,21 @@
         <x:v>S007</x:v>
       </x:c>
       <x:c r="B8" s="39"/>
-      <x:c r="C8" s="1" t="str"/>
-      <x:c r="D8" s="1" t="str"/>
-      <x:c r="E8" s="1" t="str"/>
-      <x:c r="F8" s="1" t="str"/>
-      <x:c r="G8" s="1" t="str"/>
+      <x:c r="C8" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D8" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P007</x:v>
+      </x:c>
+      <x:c r="E8" s="1" t="str">
+        <x:v>Deep Probabilistic Imaging</x:v>
+      </x:c>
+      <x:c r="F8" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G8" s="1" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/16430</x:v>
+      </x:c>
       <x:c r="H8" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10358,13 +10432,15 @@
       <x:c r="J8" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K8" s="1" t="str"/>
-      <x:c r="L8" s="1" t="str"/>
+      <x:c r="K8" s="1"/>
+      <x:c r="L8" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M8" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N8" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -10372,11 +10448,21 @@
         <x:v>S008</x:v>
       </x:c>
       <x:c r="B9" s="39"/>
-      <x:c r="C9" s="1" t="str"/>
-      <x:c r="D9" s="1" t="str"/>
-      <x:c r="E9" s="1" t="str"/>
-      <x:c r="F9" s="1" t="str"/>
-      <x:c r="G9" s="1" t="str"/>
+      <x:c r="C9" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D9" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P008</x:v>
+      </x:c>
+      <x:c r="E9" s="1" t="str">
+        <x:v>On Hallucinations in Tomographic Image Reconstruction</x:v>
+      </x:c>
+      <x:c r="F9" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G9" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TMI.2021.3077857</x:v>
+      </x:c>
       <x:c r="H9" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10386,13 +10472,15 @@
       <x:c r="J9" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K9" s="1" t="str"/>
-      <x:c r="L9" s="1" t="str"/>
+      <x:c r="K9" s="1"/>
+      <x:c r="L9" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M9" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N9" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -10400,11 +10488,21 @@
         <x:v>S009</x:v>
       </x:c>
       <x:c r="B10" s="39"/>
-      <x:c r="C10" s="1" t="str"/>
-      <x:c r="D10" s="1" t="str"/>
-      <x:c r="E10" s="1" t="str"/>
-      <x:c r="F10" s="1" t="str"/>
-      <x:c r="G10" s="1" t="str"/>
+      <x:c r="C10" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D10" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P009</x:v>
+      </x:c>
+      <x:c r="E10" s="1" t="str">
+        <x:v>Designing a Practical Degradation Model for Deep Blind Image Super-Resolution</x:v>
+      </x:c>
+      <x:c r="F10" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G10" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2021/html/Zhang_Designing_a_Practical_Degradation_Model_for_Deep_Blind_Image_Super-Resolution_ICCV_2021_paper.html</x:v>
+      </x:c>
       <x:c r="H10" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10414,13 +10512,15 @@
       <x:c r="J10" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K10" s="1" t="str"/>
-      <x:c r="L10" s="1" t="str"/>
+      <x:c r="K10" s="1"/>
+      <x:c r="L10" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M10" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N10" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -10428,11 +10528,21 @@
         <x:v>S010</x:v>
       </x:c>
       <x:c r="B11" s="39"/>
-      <x:c r="C11" s="1" t="str"/>
-      <x:c r="D11" s="1" t="str"/>
-      <x:c r="E11" s="1" t="str"/>
-      <x:c r="F11" s="1" t="str"/>
-      <x:c r="G11" s="1" t="str"/>
+      <x:c r="C11" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D11" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P010</x:v>
+      </x:c>
+      <x:c r="E11" s="1" t="str">
+        <x:v>Real-ESRGAN: Training Real-World Blind Super-Resolution With Pure Synthetic Data</x:v>
+      </x:c>
+      <x:c r="F11" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G11" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/ICCV2021W/AIM/html/Wang_Real-ESRGAN_Training_Real-World_Blind_Super-Resolution_With_Pure_Synthetic_Data_ICCVW_2021_paper.html</x:v>
+      </x:c>
       <x:c r="H11" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10442,13 +10552,15 @@
       <x:c r="J11" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K11" s="1" t="str"/>
-      <x:c r="L11" s="1" t="str"/>
+      <x:c r="K11" s="1"/>
+      <x:c r="L11" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M11" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N11" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -10456,11 +10568,21 @@
         <x:v>S011</x:v>
       </x:c>
       <x:c r="B12" s="39"/>
-      <x:c r="C12" s="1" t="str"/>
-      <x:c r="D12" s="1" t="str"/>
-      <x:c r="E12" s="1" t="str"/>
-      <x:c r="F12" s="1" t="str"/>
-      <x:c r="G12" s="1" t="str"/>
+      <x:c r="C12" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D12" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P011</x:v>
+      </x:c>
+      <x:c r="E12" s="1" t="str">
+        <x:v>Image-to-Image Regression with Distribution-Free Uncertainty Quantification and Applications in Imaging</x:v>
+      </x:c>
+      <x:c r="F12" s="1" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="G12" s="1" t="str">
+        <x:v>https://proceedings.mlr.press/v162/angelopoulos22a.html</x:v>
+      </x:c>
       <x:c r="H12" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10470,13 +10592,15 @@
       <x:c r="J12" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K12" s="1" t="str"/>
-      <x:c r="L12" s="1" t="str"/>
+      <x:c r="K12" s="1"/>
+      <x:c r="L12" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M12" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N12" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -10484,11 +10608,21 @@
         <x:v>S012</x:v>
       </x:c>
       <x:c r="B13" s="39"/>
-      <x:c r="C13" s="1" t="str"/>
-      <x:c r="D13" s="1" t="str"/>
-      <x:c r="E13" s="1" t="str"/>
-      <x:c r="F13" s="1" t="str"/>
-      <x:c r="G13" s="1" t="str"/>
+      <x:c r="C13" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D13" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P012</x:v>
+      </x:c>
+      <x:c r="E13" s="1" t="str">
+        <x:v>Denoising Diffusion Restoration Models</x:v>
+      </x:c>
+      <x:c r="F13" s="1" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="G13" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2022/hash/95504595b6169131b6ed6cd72eb05616-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H13" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10498,13 +10632,15 @@
       <x:c r="J13" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K13" s="1" t="str"/>
-      <x:c r="L13" s="1" t="str"/>
+      <x:c r="K13" s="1"/>
+      <x:c r="L13" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M13" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N13" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -10512,11 +10648,21 @@
         <x:v>S013</x:v>
       </x:c>
       <x:c r="B14" s="39"/>
-      <x:c r="C14" s="1" t="str"/>
-      <x:c r="D14" s="1" t="str"/>
-      <x:c r="E14" s="1" t="str"/>
-      <x:c r="F14" s="1" t="str"/>
-      <x:c r="G14" s="1" t="str"/>
+      <x:c r="C14" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D14" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P013</x:v>
+      </x:c>
+      <x:c r="E14" s="1" t="str">
+        <x:v>All-in-One Image Restoration for Unknown Corruption</x:v>
+      </x:c>
+      <x:c r="F14" s="1" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="G14" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2022/html/Li_All-in-One_Image_Restoration_for_Unknown_Corruption_CVPR_2022_paper.html</x:v>
+      </x:c>
       <x:c r="H14" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10526,13 +10672,15 @@
       <x:c r="J14" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K14" s="1" t="str"/>
-      <x:c r="L14" s="1" t="str"/>
+      <x:c r="K14" s="1"/>
+      <x:c r="L14" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M14" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N14" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -10540,11 +10688,21 @@
         <x:v>S014</x:v>
       </x:c>
       <x:c r="B15" s="39"/>
-      <x:c r="C15" s="1" t="str"/>
-      <x:c r="D15" s="1" t="str"/>
-      <x:c r="E15" s="1" t="str"/>
-      <x:c r="F15" s="1" t="str"/>
-      <x:c r="G15" s="1" t="str"/>
+      <x:c r="C15" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D15" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P014</x:v>
+      </x:c>
+      <x:c r="E15" s="1" t="str">
+        <x:v>Conffusion: Confidence Intervals for Diffusion Models</x:v>
+      </x:c>
+      <x:c r="F15" s="1" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="G15" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2211.09795</x:v>
+      </x:c>
       <x:c r="H15" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10554,13 +10712,15 @@
       <x:c r="J15" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K15" s="1" t="str"/>
-      <x:c r="L15" s="1" t="str"/>
+      <x:c r="K15" s="1"/>
+      <x:c r="L15" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M15" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N15" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -10568,11 +10728,21 @@
         <x:v>S015</x:v>
       </x:c>
       <x:c r="B16" s="39"/>
-      <x:c r="C16" s="1" t="str"/>
-      <x:c r="D16" s="1" t="str"/>
-      <x:c r="E16" s="1" t="str"/>
-      <x:c r="F16" s="1" t="str"/>
-      <x:c r="G16" s="1" t="str"/>
+      <x:c r="C16" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D16" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P015</x:v>
+      </x:c>
+      <x:c r="E16" s="1" t="str">
+        <x:v>Diffusion Posterior Sampling for General Noisy Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F16" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G16" s="1" t="str">
+        <x:v>https://openreview.net/forum?id=OnD9zGAGT0k</x:v>
+      </x:c>
       <x:c r="H16" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10582,13 +10752,15 @@
       <x:c r="J16" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K16" s="1" t="str"/>
-      <x:c r="L16" s="1" t="str"/>
+      <x:c r="K16" s="1"/>
+      <x:c r="L16" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M16" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N16" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -10596,11 +10768,21 @@
         <x:v>S016</x:v>
       </x:c>
       <x:c r="B17" s="39"/>
-      <x:c r="C17" s="1" t="str"/>
-      <x:c r="D17" s="1" t="str"/>
-      <x:c r="E17" s="1" t="str"/>
-      <x:c r="F17" s="1" t="str"/>
-      <x:c r="G17" s="1" t="str"/>
+      <x:c r="C17" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D17" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P016</x:v>
+      </x:c>
+      <x:c r="E17" s="1" t="str">
+        <x:v>Pseudoinverse-Guided Diffusion Models for Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F17" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G17" s="1" t="str">
+        <x:v>https://openreview.net/forum?id=9_gsMA8MRKQ</x:v>
+      </x:c>
       <x:c r="H17" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10610,13 +10792,15 @@
       <x:c r="J17" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K17" s="1" t="str"/>
-      <x:c r="L17" s="1" t="str"/>
+      <x:c r="K17" s="1"/>
+      <x:c r="L17" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M17" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N17" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -10624,11 +10808,21 @@
         <x:v>S017</x:v>
       </x:c>
       <x:c r="B18" s="39"/>
-      <x:c r="C18" s="1" t="str"/>
-      <x:c r="D18" s="1" t="str"/>
-      <x:c r="E18" s="1" t="str"/>
-      <x:c r="F18" s="1" t="str"/>
-      <x:c r="G18" s="1" t="str"/>
+      <x:c r="C18" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D18" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P017</x:v>
+      </x:c>
+      <x:c r="E18" s="1" t="str">
+        <x:v>Denoising Diffusion Null-Space Model</x:v>
+      </x:c>
+      <x:c r="F18" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G18" s="1" t="str">
+        <x:v>https://openreview.net/forum?id=mRieQgMtNTQ</x:v>
+      </x:c>
       <x:c r="H18" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10638,13 +10832,15 @@
       <x:c r="J18" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K18" s="1" t="str"/>
-      <x:c r="L18" s="1" t="str"/>
+      <x:c r="K18" s="1"/>
+      <x:c r="L18" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M18" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N18" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -10652,11 +10848,21 @@
         <x:v>S018</x:v>
       </x:c>
       <x:c r="B19" s="39"/>
-      <x:c r="C19" s="1" t="str"/>
-      <x:c r="D19" s="1" t="str"/>
-      <x:c r="E19" s="1" t="str"/>
-      <x:c r="F19" s="1" t="str"/>
-      <x:c r="G19" s="1" t="str"/>
+      <x:c r="C19" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D19" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P018</x:v>
+      </x:c>
+      <x:c r="E19" s="1" t="str">
+        <x:v>Parallel Diffusion Models of Operator and Image for Blind Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F19" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G19" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2023/html/Chung_Parallel_Diffusion_Models_of_Operator_and_Image_for_Blind_Inverse_Problems_CVPR_2023_paper.html</x:v>
+      </x:c>
       <x:c r="H19" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10666,13 +10872,15 @@
       <x:c r="J19" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K19" s="1" t="str"/>
-      <x:c r="L19" s="1" t="str"/>
+      <x:c r="K19" s="1"/>
+      <x:c r="L19" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M19" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N19" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -10680,11 +10888,21 @@
         <x:v>S019</x:v>
       </x:c>
       <x:c r="B20" s="39"/>
-      <x:c r="C20" s="1" t="str"/>
-      <x:c r="D20" s="1" t="str"/>
-      <x:c r="E20" s="1" t="str"/>
-      <x:c r="F20" s="1" t="str"/>
-      <x:c r="G20" s="1" t="str"/>
+      <x:c r="C20" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D20" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P019</x:v>
+      </x:c>
+      <x:c r="E20" s="1" t="str">
+        <x:v>GibbsDDRM</x:v>
+      </x:c>
+      <x:c r="F20" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G20" s="1" t="str">
+        <x:v>https://proceedings.mlr.press/v202/murata23a.html</x:v>
+      </x:c>
       <x:c r="H20" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10694,13 +10912,15 @@
       <x:c r="J20" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K20" s="1" t="str"/>
-      <x:c r="L20" s="1" t="str"/>
+      <x:c r="K20" s="1"/>
+      <x:c r="L20" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M20" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N20" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -10708,11 +10928,21 @@
         <x:v>S020</x:v>
       </x:c>
       <x:c r="B21" s="39"/>
-      <x:c r="C21" s="1" t="str"/>
-      <x:c r="D21" s="1" t="str"/>
-      <x:c r="E21" s="1" t="str"/>
-      <x:c r="F21" s="1" t="str"/>
-      <x:c r="G21" s="1" t="str"/>
+      <x:c r="C21" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D21" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P020</x:v>
+      </x:c>
+      <x:c r="E21" s="1" t="str">
+        <x:v>PromptIR: Prompting for All-in-One Blind Image Restoration</x:v>
+      </x:c>
+      <x:c r="F21" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G21" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a17bb69ab19f3be921f-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H21" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10722,13 +10952,15 @@
       <x:c r="J21" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K21" s="1" t="str"/>
-      <x:c r="L21" s="1" t="str"/>
+      <x:c r="K21" s="1"/>
+      <x:c r="L21" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M21" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N21" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -10736,11 +10968,21 @@
         <x:v>S021</x:v>
       </x:c>
       <x:c r="B22" s="39"/>
-      <x:c r="C22" s="1" t="str"/>
-      <x:c r="D22" s="1" t="str"/>
-      <x:c r="E22" s="1" t="str"/>
-      <x:c r="F22" s="1" t="str"/>
-      <x:c r="G22" s="1" t="str"/>
+      <x:c r="C22" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D22" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P021</x:v>
+      </x:c>
+      <x:c r="E22" s="1" t="str">
+        <x:v>Differentiable Uncalibrated Imaging</x:v>
+      </x:c>
+      <x:c r="F22" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G22" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2211.10525</x:v>
+      </x:c>
       <x:c r="H22" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10750,13 +10992,15 @@
       <x:c r="J22" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K22" s="1" t="str"/>
-      <x:c r="L22" s="1" t="str"/>
+      <x:c r="K22" s="1"/>
+      <x:c r="L22" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M22" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N22" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -10764,11 +11008,21 @@
         <x:v>S022</x:v>
       </x:c>
       <x:c r="B23" s="39"/>
-      <x:c r="C23" s="1" t="str"/>
-      <x:c r="D23" s="1" t="str"/>
-      <x:c r="E23" s="1" t="str"/>
-      <x:c r="F23" s="1" t="str"/>
-      <x:c r="G23" s="1" t="str"/>
+      <x:c r="C23" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D23" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P022</x:v>
+      </x:c>
+      <x:c r="E23" s="1" t="str">
+        <x:v>Fast Diffusion EM</x:v>
+      </x:c>
+      <x:c r="F23" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G23" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/WACV2024/html/Laroche_Fast_Diffusion_EM_A_Diffusion_Model_for_Blind_Inverse_Problems_WACV_2024_paper.html</x:v>
+      </x:c>
       <x:c r="H23" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10778,13 +11032,15 @@
       <x:c r="J23" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K23" s="1" t="str"/>
-      <x:c r="L23" s="1" t="str"/>
+      <x:c r="K23" s="1"/>
+      <x:c r="L23" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M23" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N23" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -10792,11 +11048,21 @@
         <x:v>S023</x:v>
       </x:c>
       <x:c r="B24" s="39"/>
-      <x:c r="C24" s="1" t="str"/>
-      <x:c r="D24" s="1" t="str"/>
-      <x:c r="E24" s="1" t="str"/>
-      <x:c r="F24" s="1" t="str"/>
-      <x:c r="G24" s="1" t="str"/>
+      <x:c r="C24" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D24" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P023</x:v>
+      </x:c>
+      <x:c r="E24" s="1" t="str">
+        <x:v>Blind Image Restoration via Fast Diffusion Inversion</x:v>
+      </x:c>
+      <x:c r="F24" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G24" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/3d13d910b48ac2e672a32cfdf98be1bf-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H24" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10806,13 +11072,15 @@
       <x:c r="J24" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K24" s="1" t="str"/>
-      <x:c r="L24" s="1" t="str"/>
+      <x:c r="K24" s="1"/>
+      <x:c r="L24" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M24" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N24" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -10820,11 +11088,21 @@
         <x:v>S024</x:v>
       </x:c>
       <x:c r="B25" s="39"/>
-      <x:c r="C25" s="1" t="str"/>
-      <x:c r="D25" s="1" t="str"/>
-      <x:c r="E25" s="1" t="str"/>
-      <x:c r="F25" s="1" t="str"/>
-      <x:c r="G25" s="1" t="str"/>
+      <x:c r="C25" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D25" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P024</x:v>
+      </x:c>
+      <x:c r="E25" s="1" t="str">
+        <x:v>Blind Inversion Using Latent Diffusion Priors</x:v>
+      </x:c>
+      <x:c r="F25" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G25" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2407.01027</x:v>
+      </x:c>
       <x:c r="H25" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10834,13 +11112,15 @@
       <x:c r="J25" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K25" s="1" t="str"/>
-      <x:c r="L25" s="1" t="str"/>
+      <x:c r="K25" s="1"/>
+      <x:c r="L25" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M25" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N25" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -10848,11 +11128,21 @@
         <x:v>S025</x:v>
       </x:c>
       <x:c r="B26" s="39"/>
-      <x:c r="C26" s="1" t="str"/>
-      <x:c r="D26" s="1" t="str"/>
-      <x:c r="E26" s="1" t="str"/>
-      <x:c r="F26" s="1" t="str"/>
-      <x:c r="G26" s="1" t="str"/>
+      <x:c r="C26" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D26" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P025</x:v>
+      </x:c>
+      <x:c r="E26" s="1" t="str">
+        <x:v>DiffBIR: Toward Blind Image Restoration with Generative Diffusion Prior</x:v>
+      </x:c>
+      <x:c r="F26" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G26" s="1" t="str">
+        <x:v>https://eccv.ecva.net/virtual/2024/poster/2315</x:v>
+      </x:c>
       <x:c r="H26" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10862,13 +11152,15 @@
       <x:c r="J26" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K26" s="1" t="str"/>
-      <x:c r="L26" s="1" t="str"/>
+      <x:c r="K26" s="1"/>
+      <x:c r="L26" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M26" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N26" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -10876,11 +11168,21 @@
         <x:v>S026</x:v>
       </x:c>
       <x:c r="B27" s="39"/>
-      <x:c r="C27" s="1" t="str"/>
-      <x:c r="D27" s="1" t="str"/>
-      <x:c r="E27" s="1" t="str"/>
-      <x:c r="F27" s="1" t="str"/>
-      <x:c r="G27" s="1" t="str"/>
+      <x:c r="C27" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D27" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P026</x:v>
+      </x:c>
+      <x:c r="E27" s="1" t="str">
+        <x:v>AverNet: All-in-One Video Restoration for Time-Varying Unknown Degradations</x:v>
+      </x:c>
+      <x:c r="F27" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G27" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/e635a25e49e73adc51f76aef462ff2f8-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H27" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10890,13 +11192,15 @@
       <x:c r="J27" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K27" s="1" t="str"/>
-      <x:c r="L27" s="1" t="str"/>
+      <x:c r="K27" s="1"/>
+      <x:c r="L27" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M27" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N27" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -10904,11 +11208,21 @@
         <x:v>S027</x:v>
       </x:c>
       <x:c r="B28" s="39"/>
-      <x:c r="C28" s="1" t="str"/>
-      <x:c r="D28" s="1" t="str"/>
-      <x:c r="E28" s="1" t="str"/>
-      <x:c r="F28" s="1" t="str"/>
-      <x:c r="G28" s="1" t="str"/>
+      <x:c r="C28" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D28" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P027</x:v>
+      </x:c>
+      <x:c r="E28" s="1" t="str">
+        <x:v>SR+Codec: A Benchmark of Super-Resolution for Video Compression</x:v>
+      </x:c>
+      <x:c r="F28" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G28" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2412.02506</x:v>
+      </x:c>
       <x:c r="H28" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10918,13 +11232,15 @@
       <x:c r="J28" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K28" s="1" t="str"/>
-      <x:c r="L28" s="1" t="str"/>
+      <x:c r="K28" s="1"/>
+      <x:c r="L28" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M28" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N28" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -10932,11 +11248,21 @@
         <x:v>S028</x:v>
       </x:c>
       <x:c r="B29" s="39"/>
-      <x:c r="C29" s="1" t="str"/>
-      <x:c r="D29" s="1" t="str"/>
-      <x:c r="E29" s="1" t="str"/>
-      <x:c r="F29" s="1" t="str"/>
-      <x:c r="G29" s="1" t="str"/>
+      <x:c r="C29" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D29" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P028</x:v>
+      </x:c>
+      <x:c r="E29" s="1" t="str">
+        <x:v>Scaling Up to Excellence: Practicing Model Scaling for Photo-Realistic Image Restoration In the Wild</x:v>
+      </x:c>
+      <x:c r="F29" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G29" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2401.13627</x:v>
+      </x:c>
       <x:c r="H29" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10946,13 +11272,15 @@
       <x:c r="J29" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K29" s="1" t="str"/>
-      <x:c r="L29" s="1" t="str"/>
+      <x:c r="K29" s="1"/>
+      <x:c r="L29" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M29" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N29" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -10960,11 +11288,21 @@
         <x:v>S029</x:v>
       </x:c>
       <x:c r="B30" s="39"/>
-      <x:c r="C30" s="1" t="str"/>
-      <x:c r="D30" s="1" t="str"/>
-      <x:c r="E30" s="1" t="str"/>
-      <x:c r="F30" s="1" t="str"/>
-      <x:c r="G30" s="1" t="str"/>
+      <x:c r="C30" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D30" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P029</x:v>
+      </x:c>
+      <x:c r="E30" s="1" t="str">
+        <x:v>Robust Unrolled Network for Lensless Imaging with Enhanced Resistance to Model Mismatch and Noise</x:v>
+      </x:c>
+      <x:c r="F30" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G30" s="1" t="str">
+        <x:v>https://opg.optica.org/oe/abstract.cfm?uri=oe-32-17-30267</x:v>
+      </x:c>
       <x:c r="H30" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -10974,13 +11312,15 @@
       <x:c r="J30" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K30" s="1" t="str"/>
-      <x:c r="L30" s="1" t="str"/>
+      <x:c r="K30" s="1"/>
+      <x:c r="L30" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M30" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N30" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -10988,11 +11328,21 @@
         <x:v>S030</x:v>
       </x:c>
       <x:c r="B31" s="39"/>
-      <x:c r="C31" s="1" t="str"/>
-      <x:c r="D31" s="1" t="str"/>
-      <x:c r="E31" s="1" t="str"/>
-      <x:c r="F31" s="1" t="str"/>
-      <x:c r="G31" s="1" t="str"/>
+      <x:c r="C31" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D31" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P030</x:v>
+      </x:c>
+      <x:c r="E31" s="1" t="str">
+        <x:v>Empirical Bayesian Imaging With Large-Scale Push-Forward Generative Priors</x:v>
+      </x:c>
+      <x:c r="F31" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G31" s="1" t="str">
+        <x:v>https://doi.org/10.1109/LSP.2024.3361806</x:v>
+      </x:c>
       <x:c r="H31" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11002,13 +11352,15 @@
       <x:c r="J31" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K31" s="1" t="str"/>
-      <x:c r="L31" s="1" t="str"/>
+      <x:c r="K31" s="1"/>
+      <x:c r="L31" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M31" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N31" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -11016,11 +11368,21 @@
         <x:v>S031</x:v>
       </x:c>
       <x:c r="B32" s="39"/>
-      <x:c r="C32" s="1" t="str"/>
-      <x:c r="D32" s="1" t="str"/>
-      <x:c r="E32" s="1" t="str"/>
-      <x:c r="F32" s="1" t="str"/>
-      <x:c r="G32" s="1" t="str"/>
+      <x:c r="C32" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D32" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P031</x:v>
+      </x:c>
+      <x:c r="E32" s="1" t="str">
+        <x:v>The Troublesome Kernel</x:v>
+      </x:c>
+      <x:c r="F32" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G32" s="1" t="str">
+        <x:v>https://doi.org/10.1137/23M1568739</x:v>
+      </x:c>
       <x:c r="H32" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11030,13 +11392,15 @@
       <x:c r="J32" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K32" s="1" t="str"/>
-      <x:c r="L32" s="1" t="str"/>
+      <x:c r="K32" s="1"/>
+      <x:c r="L32" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M32" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N32" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -11044,11 +11408,21 @@
         <x:v>S032</x:v>
       </x:c>
       <x:c r="B33" s="39"/>
-      <x:c r="C33" s="1" t="str"/>
-      <x:c r="D33" s="1" t="str"/>
-      <x:c r="E33" s="1" t="str"/>
-      <x:c r="F33" s="1" t="str"/>
-      <x:c r="G33" s="1" t="str"/>
+      <x:c r="C33" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D33" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P032</x:v>
+      </x:c>
+      <x:c r="E33" s="1" t="str">
+        <x:v>Uncertainty-Aware Fourier Ptychography</x:v>
+      </x:c>
+      <x:c r="F33" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G33" s="1" t="str">
+        <x:v>https://doi.org/10.1038/s41377-025-01915-w</x:v>
+      </x:c>
       <x:c r="H33" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11058,13 +11432,15 @@
       <x:c r="J33" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K33" s="1" t="str"/>
-      <x:c r="L33" s="1" t="str"/>
+      <x:c r="K33" s="1"/>
+      <x:c r="L33" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M33" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N33" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -11072,11 +11448,21 @@
         <x:v>S033</x:v>
       </x:c>
       <x:c r="B34" s="39"/>
-      <x:c r="C34" s="1" t="str"/>
-      <x:c r="D34" s="1" t="str"/>
-      <x:c r="E34" s="1" t="str"/>
-      <x:c r="F34" s="1" t="str"/>
-      <x:c r="G34" s="1" t="str"/>
+      <x:c r="C34" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D34" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P033</x:v>
+      </x:c>
+      <x:c r="E34" s="1" t="str">
+        <x:v>Unsupervised Detection of Distribution Shift in Inverse Problems Using Diffusion Models</x:v>
+      </x:c>
+      <x:c r="F34" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G34" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2505.11482</x:v>
+      </x:c>
       <x:c r="H34" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11086,13 +11472,15 @@
       <x:c r="J34" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K34" s="1" t="str"/>
-      <x:c r="L34" s="1" t="str"/>
+      <x:c r="K34" s="1"/>
+      <x:c r="L34" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M34" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N34" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -11100,11 +11488,21 @@
         <x:v>S034</x:v>
       </x:c>
       <x:c r="B35" s="39"/>
-      <x:c r="C35" s="1" t="str"/>
-      <x:c r="D35" s="1" t="str"/>
-      <x:c r="E35" s="1" t="str"/>
-      <x:c r="F35" s="1" t="str"/>
-      <x:c r="G35" s="1" t="str"/>
+      <x:c r="C35" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D35" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P034</x:v>
+      </x:c>
+      <x:c r="E35" s="1" t="str">
+        <x:v>Towards Distribution-Shift Uncertainty Estimation for Inverse Problems with Generative Priors</x:v>
+      </x:c>
+      <x:c r="F35" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G35" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2510.10947</x:v>
+      </x:c>
       <x:c r="H35" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11114,13 +11512,15 @@
       <x:c r="J35" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K35" s="1" t="str"/>
-      <x:c r="L35" s="1" t="str"/>
+      <x:c r="K35" s="1"/>
+      <x:c r="L35" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M35" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N35" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -11128,11 +11528,21 @@
         <x:v>S035</x:v>
       </x:c>
       <x:c r="B36" s="39"/>
-      <x:c r="C36" s="1" t="str"/>
-      <x:c r="D36" s="1" t="str"/>
-      <x:c r="E36" s="1" t="str"/>
-      <x:c r="F36" s="1" t="str"/>
-      <x:c r="G36" s="1" t="str"/>
+      <x:c r="C36" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D36" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P035</x:v>
+      </x:c>
+      <x:c r="E36" s="1" t="str">
+        <x:v>Mitigating Forward Model Mismatch in Inverse Problems via Learned Residuals and Diffusion Priors</x:v>
+      </x:c>
+      <x:c r="F36" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G36" s="1" t="str">
+        <x:v>https://www.spiedigitallibrary.org/conference-proceedings-of-spie/13849/1384908/</x:v>
+      </x:c>
       <x:c r="H36" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11142,13 +11552,15 @@
       <x:c r="J36" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K36" s="1" t="str"/>
-      <x:c r="L36" s="1" t="str"/>
+      <x:c r="K36" s="1"/>
+      <x:c r="L36" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M36" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N36" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -11156,11 +11568,21 @@
         <x:v>S036</x:v>
       </x:c>
       <x:c r="B37" s="39"/>
-      <x:c r="C37" s="1" t="str"/>
-      <x:c r="D37" s="1" t="str"/>
-      <x:c r="E37" s="1" t="str"/>
-      <x:c r="F37" s="1" t="str"/>
-      <x:c r="G37" s="1" t="str"/>
+      <x:c r="C37" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D37" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P036</x:v>
+      </x:c>
+      <x:c r="E37" s="1" t="str">
+        <x:v>InverseNet: Benchmarking Operator Mismatch and Calibration Across Compressive Imaging Modalities</x:v>
+      </x:c>
+      <x:c r="F37" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G37" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2603.04538</x:v>
+      </x:c>
       <x:c r="H37" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11170,13 +11592,15 @@
       <x:c r="J37" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K37" s="1" t="str"/>
-      <x:c r="L37" s="1" t="str"/>
+      <x:c r="K37" s="1"/>
+      <x:c r="L37" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M37" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N37" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -11184,11 +11608,21 @@
         <x:v>S037</x:v>
       </x:c>
       <x:c r="B38" s="39"/>
-      <x:c r="C38" s="1" t="str"/>
-      <x:c r="D38" s="1" t="str"/>
-      <x:c r="E38" s="1" t="str"/>
-      <x:c r="F38" s="1" t="str"/>
-      <x:c r="G38" s="1" t="str"/>
+      <x:c r="C38" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D38" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P037</x:v>
+      </x:c>
+      <x:c r="E38" s="1" t="str">
+        <x:v>On Hallucinations in Inverse Problems: Fundamental Limits and Provable Assessment Methods</x:v>
+      </x:c>
+      <x:c r="F38" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G38" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2605.13146</x:v>
+      </x:c>
       <x:c r="H38" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11198,13 +11632,15 @@
       <x:c r="J38" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K38" s="1" t="str"/>
-      <x:c r="L38" s="1" t="str"/>
+      <x:c r="K38" s="1"/>
+      <x:c r="L38" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M38" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N38" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -11212,11 +11648,21 @@
         <x:v>S038</x:v>
       </x:c>
       <x:c r="B39" s="39"/>
-      <x:c r="C39" s="1" t="str"/>
-      <x:c r="D39" s="1" t="str"/>
-      <x:c r="E39" s="1" t="str"/>
-      <x:c r="F39" s="1" t="str"/>
-      <x:c r="G39" s="1" t="str"/>
+      <x:c r="C39" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D39" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P038</x:v>
+      </x:c>
+      <x:c r="E39" s="1" t="str">
+        <x:v>PRISM: Probabilistic and Robust Inverse Solver with Measurement-Conditioned Diffusion Prior for Blind Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F39" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G39" s="1" t="str">
+        <x:v>https://doi.org/10.1109/ICASSP55912.2026.11462668</x:v>
+      </x:c>
       <x:c r="H39" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11226,13 +11672,15 @@
       <x:c r="J39" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K39" s="1" t="str"/>
-      <x:c r="L39" s="1" t="str"/>
+      <x:c r="K39" s="1"/>
+      <x:c r="L39" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M39" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N39" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -11240,11 +11688,21 @@
         <x:v>S039</x:v>
       </x:c>
       <x:c r="B40" s="39"/>
-      <x:c r="C40" s="1" t="str"/>
-      <x:c r="D40" s="1" t="str"/>
-      <x:c r="E40" s="1" t="str"/>
-      <x:c r="F40" s="1" t="str"/>
-      <x:c r="G40" s="1" t="str"/>
+      <x:c r="C40" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D40" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P039</x:v>
+      </x:c>
+      <x:c r="E40" s="1" t="str">
+        <x:v>Adaptive Blind All-in-One Image Restoration</x:v>
+      </x:c>
+      <x:c r="F40" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G40" s="1" t="str">
+        <x:v>https://doi.org/10.1016/j.cviu.2026.104795</x:v>
+      </x:c>
       <x:c r="H40" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11254,13 +11712,15 @@
       <x:c r="J40" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K40" s="1" t="str"/>
-      <x:c r="L40" s="1" t="str"/>
+      <x:c r="K40" s="1"/>
+      <x:c r="L40" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M40" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N40" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -11268,11 +11728,21 @@
         <x:v>S040</x:v>
       </x:c>
       <x:c r="B41" s="39"/>
-      <x:c r="C41" s="1" t="str"/>
-      <x:c r="D41" s="1" t="str"/>
-      <x:c r="E41" s="1" t="str"/>
-      <x:c r="F41" s="1" t="str"/>
-      <x:c r="G41" s="1" t="str"/>
+      <x:c r="C41" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D41" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P040</x:v>
+      </x:c>
+      <x:c r="E41" s="1" t="str">
+        <x:v>Video Diffusion Posterior Sampling for Seeing Beyond Dynamic Scattering Layers</x:v>
+      </x:c>
+      <x:c r="F41" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G41" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TPAMI.2025.3598457</x:v>
+      </x:c>
       <x:c r="H41" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11282,13 +11752,15 @@
       <x:c r="J41" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K41" s="1" t="str"/>
-      <x:c r="L41" s="1" t="str"/>
+      <x:c r="K41" s="1"/>
+      <x:c r="L41" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M41" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N41" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -11296,11 +11768,21 @@
         <x:v>S041</x:v>
       </x:c>
       <x:c r="B42" s="39"/>
-      <x:c r="C42" s="1" t="str"/>
-      <x:c r="D42" s="1" t="str"/>
-      <x:c r="E42" s="1" t="str"/>
-      <x:c r="F42" s="1" t="str"/>
-      <x:c r="G42" s="1" t="str"/>
+      <x:c r="C42" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D42" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P041</x:v>
+      </x:c>
+      <x:c r="E42" s="1" t="str">
+        <x:v>Uncertainty Quantification in HSI Reconstruction using Physics-Aware Diffusion Priors and Optics-Encoded Measurements</x:v>
+      </x:c>
+      <x:c r="F42" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G42" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2511.18473</x:v>
+      </x:c>
       <x:c r="H42" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11310,13 +11792,15 @@
       <x:c r="J42" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K42" s="1" t="str"/>
-      <x:c r="L42" s="1" t="str"/>
+      <x:c r="K42" s="1"/>
+      <x:c r="L42" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M42" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N42" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -11324,11 +11808,21 @@
         <x:v>S042</x:v>
       </x:c>
       <x:c r="B43" s="39"/>
-      <x:c r="C43" s="1" t="str"/>
-      <x:c r="D43" s="1" t="str"/>
-      <x:c r="E43" s="1" t="str"/>
-      <x:c r="F43" s="1" t="str"/>
-      <x:c r="G43" s="1" t="str"/>
+      <x:c r="C43" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D43" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P042</x:v>
+      </x:c>
+      <x:c r="E43" s="1" t="str">
+        <x:v>No-Harm Physics-Informed Inverse Learning with Residual-Calibrated Uncertainty</x:v>
+      </x:c>
+      <x:c r="F43" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G43" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2606.07153</x:v>
+      </x:c>
       <x:c r="H43" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11338,13 +11832,15 @@
       <x:c r="J43" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K43" s="1" t="str"/>
-      <x:c r="L43" s="1" t="str"/>
+      <x:c r="K43" s="1"/>
+      <x:c r="L43" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M43" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N43" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -11352,11 +11848,21 @@
         <x:v>S043</x:v>
       </x:c>
       <x:c r="B44" s="39"/>
-      <x:c r="C44" s="1" t="str"/>
-      <x:c r="D44" s="1" t="str"/>
-      <x:c r="E44" s="1" t="str"/>
-      <x:c r="F44" s="1" t="str"/>
-      <x:c r="G44" s="1" t="str"/>
+      <x:c r="C44" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D44" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P043</x:v>
+      </x:c>
+      <x:c r="E44" s="1" t="str">
+        <x:v>Model Adaptation for Inverse Problems in Imaging</x:v>
+      </x:c>
+      <x:c r="F44" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G44" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TCI.2021.3094714</x:v>
+      </x:c>
       <x:c r="H44" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11366,13 +11872,15 @@
       <x:c r="J44" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K44" s="1" t="str"/>
-      <x:c r="L44" s="1" t="str"/>
+      <x:c r="K44" s="1"/>
+      <x:c r="L44" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M44" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N44" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -11380,11 +11888,21 @@
         <x:v>S044</x:v>
       </x:c>
       <x:c r="B45" s="39"/>
-      <x:c r="C45" s="1" t="str"/>
-      <x:c r="D45" s="1" t="str"/>
-      <x:c r="E45" s="1" t="str"/>
-      <x:c r="F45" s="1" t="str"/>
-      <x:c r="G45" s="1" t="str"/>
+      <x:c r="C45" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D45" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P044</x:v>
+      </x:c>
+      <x:c r="E45" s="1" t="str">
+        <x:v>Robust Lensless Image Reconstruction via PSF Estimation</x:v>
+      </x:c>
+      <x:c r="F45" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G45" s="1" t="str">
+        <x:v>https://doi.org/10.1109/WACV48630.2021.00045</x:v>
+      </x:c>
       <x:c r="H45" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11394,13 +11912,15 @@
       <x:c r="J45" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K45" s="1" t="str"/>
-      <x:c r="L45" s="1" t="str"/>
+      <x:c r="K45" s="1"/>
+      <x:c r="L45" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M45" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N45" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -11408,11 +11928,21 @@
         <x:v>S045</x:v>
       </x:c>
       <x:c r="B46" s="39"/>
-      <x:c r="C46" s="1" t="str"/>
-      <x:c r="D46" s="1" t="str"/>
-      <x:c r="E46" s="1" t="str"/>
-      <x:c r="F46" s="1" t="str"/>
-      <x:c r="G46" s="1" t="str"/>
+      <x:c r="C46" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D46" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P045</x:v>
+      </x:c>
+      <x:c r="E46" s="1" t="str">
+        <x:v>Block Coordinate Plug-and-Play Methods for Blind Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F46" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G46" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/f810c2ba07bae78dfe9d25c5d40c5536-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H46" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11422,13 +11952,15 @@
       <x:c r="J46" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K46" s="1" t="str"/>
-      <x:c r="L46" s="1" t="str"/>
+      <x:c r="K46" s="1"/>
+      <x:c r="L46" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M46" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N46" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -11436,11 +11968,21 @@
         <x:v>S046</x:v>
       </x:c>
       <x:c r="B47" s="39"/>
-      <x:c r="C47" s="1" t="str"/>
-      <x:c r="D47" s="1" t="str"/>
-      <x:c r="E47" s="1" t="str"/>
-      <x:c r="F47" s="1" t="str"/>
-      <x:c r="G47" s="1" t="str"/>
+      <x:c r="C47" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D47" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P046</x:v>
+      </x:c>
+      <x:c r="E47" s="1" t="str">
+        <x:v>Training Adaptive Reconstruction Networks for Blind Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F47" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G47" s="1" t="str">
+        <x:v>https://doi.org/10.1137/23M1545628</x:v>
+      </x:c>
       <x:c r="H47" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11450,13 +11992,15 @@
       <x:c r="J47" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K47" s="1" t="str"/>
-      <x:c r="L47" s="1" t="str"/>
+      <x:c r="K47" s="1"/>
+      <x:c r="L47" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M47" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N47" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -11464,11 +12008,21 @@
         <x:v>S047</x:v>
       </x:c>
       <x:c r="B48" s="39"/>
-      <x:c r="C48" s="1" t="str"/>
-      <x:c r="D48" s="1" t="str"/>
-      <x:c r="E48" s="1" t="str"/>
-      <x:c r="F48" s="1" t="str"/>
-      <x:c r="G48" s="1" t="str"/>
+      <x:c r="C48" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D48" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P047</x:v>
+      </x:c>
+      <x:c r="E48" s="1" t="str">
+        <x:v>Solving Inverse Problems with Model Mismatch using Untrained Neural Networks within Model-based Architectures</x:v>
+      </x:c>
+      <x:c r="F48" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G48" s="1" t="str">
+        <x:v>https://openreview.net/forum?id=XHEhjDxPDl</x:v>
+      </x:c>
       <x:c r="H48" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11478,13 +12032,15 @@
       <x:c r="J48" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K48" s="1" t="str"/>
-      <x:c r="L48" s="1" t="str"/>
+      <x:c r="K48" s="1"/>
+      <x:c r="L48" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M48" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N48" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -11492,11 +12048,21 @@
         <x:v>S048</x:v>
       </x:c>
       <x:c r="B49" s="39"/>
-      <x:c r="C49" s="1" t="str"/>
-      <x:c r="D49" s="1" t="str"/>
-      <x:c r="E49" s="1" t="str"/>
-      <x:c r="F49" s="1" t="str"/>
-      <x:c r="G49" s="1" t="str"/>
+      <x:c r="C49" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D49" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P048</x:v>
+      </x:c>
+      <x:c r="E49" s="1" t="str">
+        <x:v>Plug-and-Play Posterior Sampling under Mismatched Measurement and Prior Models</x:v>
+      </x:c>
+      <x:c r="F49" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G49" s="1" t="str">
+        <x:v>https://proceedings.iclr.cc/paper_files/paper/2024/hash/2a2874875861f6a6436b505dd77683d1-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H49" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11506,13 +12072,15 @@
       <x:c r="J49" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K49" s="1" t="str"/>
-      <x:c r="L49" s="1" t="str"/>
+      <x:c r="K49" s="1"/>
+      <x:c r="L49" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M49" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N49" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -11520,11 +12088,21 @@
         <x:v>S049</x:v>
       </x:c>
       <x:c r="B50" s="39"/>
-      <x:c r="C50" s="1" t="str"/>
-      <x:c r="D50" s="1" t="str"/>
-      <x:c r="E50" s="1" t="str"/>
-      <x:c r="F50" s="1" t="str"/>
-      <x:c r="G50" s="1" t="str"/>
+      <x:c r="C50" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D50" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P049</x:v>
+      </x:c>
+      <x:c r="E50" s="1" t="str">
+        <x:v>DeepVibes: Correcting Micro-Vibrations in Satellite Imaging With Pushbroom Cameras</x:v>
+      </x:c>
+      <x:c r="F50" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G50" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TGRS.2024.3415372</x:v>
+      </x:c>
       <x:c r="H50" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11534,13 +12112,15 @@
       <x:c r="J50" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K50" s="1" t="str"/>
-      <x:c r="L50" s="1" t="str"/>
+      <x:c r="K50" s="1"/>
+      <x:c r="L50" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M50" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N50" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -11548,11 +12128,21 @@
         <x:v>S050</x:v>
       </x:c>
       <x:c r="B51" s="39"/>
-      <x:c r="C51" s="1" t="str"/>
-      <x:c r="D51" s="1" t="str"/>
-      <x:c r="E51" s="1" t="str"/>
-      <x:c r="F51" s="1" t="str"/>
-      <x:c r="G51" s="1" t="str"/>
+      <x:c r="C51" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D51" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P050</x:v>
+      </x:c>
+      <x:c r="E51" s="1" t="str">
+        <x:v>Blind Inverse Problem Solving Made Easy by Text-to-Image Latent Diffusion</x:v>
+      </x:c>
+      <x:c r="F51" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G51" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2412.00557</x:v>
+      </x:c>
       <x:c r="H51" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11562,13 +12152,15 @@
       <x:c r="J51" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K51" s="1" t="str"/>
-      <x:c r="L51" s="1" t="str"/>
+      <x:c r="K51" s="1"/>
+      <x:c r="L51" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M51" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N51" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -11576,11 +12168,21 @@
         <x:v>S051</x:v>
       </x:c>
       <x:c r="B52" s="39"/>
-      <x:c r="C52" s="1" t="str"/>
-      <x:c r="D52" s="1" t="str"/>
-      <x:c r="E52" s="1" t="str"/>
-      <x:c r="F52" s="1" t="str"/>
-      <x:c r="G52" s="1" t="str"/>
+      <x:c r="C52" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D52" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P051</x:v>
+      </x:c>
+      <x:c r="E52" s="1" t="str">
+        <x:v>ADOBI: Adaptive Diffusion Bridge For Blind Inverse Problems with Application to MRI Reconstruction</x:v>
+      </x:c>
+      <x:c r="F52" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G52" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TCI.2026.3678407</x:v>
+      </x:c>
       <x:c r="H52" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11590,13 +12192,15 @@
       <x:c r="J52" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K52" s="1" t="str"/>
-      <x:c r="L52" s="1" t="str"/>
+      <x:c r="K52" s="1"/>
+      <x:c r="L52" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M52" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N52" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -11604,11 +12208,21 @@
         <x:v>S052</x:v>
       </x:c>
       <x:c r="B53" s="39"/>
-      <x:c r="C53" s="1" t="str"/>
-      <x:c r="D53" s="1" t="str"/>
-      <x:c r="E53" s="1" t="str"/>
-      <x:c r="F53" s="1" t="str"/>
-      <x:c r="G53" s="1" t="str"/>
+      <x:c r="C53" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D53" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P052</x:v>
+      </x:c>
+      <x:c r="E53" s="1" t="str">
+        <x:v>Resolving Blind Inverse Problems under Dynamic Range Compression via Structured Forward Operator Modeling</x:v>
+      </x:c>
+      <x:c r="F53" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G53" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2603.01890</x:v>
+      </x:c>
       <x:c r="H53" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11618,13 +12232,15 @@
       <x:c r="J53" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K53" s="1" t="str"/>
-      <x:c r="L53" s="1" t="str"/>
+      <x:c r="K53" s="1"/>
+      <x:c r="L53" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M53" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N53" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -11632,11 +12248,21 @@
         <x:v>S053</x:v>
       </x:c>
       <x:c r="B54" s="39"/>
-      <x:c r="C54" s="1" t="str"/>
-      <x:c r="D54" s="1" t="str"/>
-      <x:c r="E54" s="1" t="str"/>
-      <x:c r="F54" s="1" t="str"/>
-      <x:c r="G54" s="1" t="str"/>
+      <x:c r="C54" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D54" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P053</x:v>
+      </x:c>
+      <x:c r="E54" s="1" t="str">
+        <x:v>FaverNet: All-in-One Video Restoration via Frequency-Discriminative Conditioning</x:v>
+      </x:c>
+      <x:c r="F54" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G54" s="1" t="str">
+        <x:v>https://doi.org/10.1007/s11263-026-02977-y</x:v>
+      </x:c>
       <x:c r="H54" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11646,13 +12272,15 @@
       <x:c r="J54" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K54" s="1" t="str"/>
-      <x:c r="L54" s="1" t="str"/>
+      <x:c r="K54" s="1"/>
+      <x:c r="L54" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M54" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N54" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -11660,11 +12288,21 @@
         <x:v>S054</x:v>
       </x:c>
       <x:c r="B55" s="39"/>
-      <x:c r="C55" s="1" t="str"/>
-      <x:c r="D55" s="1" t="str"/>
-      <x:c r="E55" s="1" t="str"/>
-      <x:c r="F55" s="1" t="str"/>
-      <x:c r="G55" s="1" t="str"/>
+      <x:c r="C55" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D55" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P054</x:v>
+      </x:c>
+      <x:c r="E55" s="1" t="str">
+        <x:v>Towards Real-world Event-guided Low-light Video Enhancement and Deblurring</x:v>
+      </x:c>
+      <x:c r="F55" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G55" s="1" t="str">
+        <x:v>https://doi.org/10.1007/978-3-031-73254-6_25</x:v>
+      </x:c>
       <x:c r="H55" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11674,13 +12312,15 @@
       <x:c r="J55" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K55" s="1" t="str"/>
-      <x:c r="L55" s="1" t="str"/>
+      <x:c r="K55" s="1"/>
+      <x:c r="L55" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M55" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N55" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -11688,11 +12328,21 @@
         <x:v>S055</x:v>
       </x:c>
       <x:c r="B56" s="39"/>
-      <x:c r="C56" s="1" t="str"/>
-      <x:c r="D56" s="1" t="str"/>
-      <x:c r="E56" s="1" t="str"/>
-      <x:c r="F56" s="1" t="str"/>
-      <x:c r="G56" s="1" t="str"/>
+      <x:c r="C56" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D56" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P055</x:v>
+      </x:c>
+      <x:c r="E56" s="1" t="str">
+        <x:v>LEDNet: Joint Low-Light Enhancement and Deblurring in the Dark</x:v>
+      </x:c>
+      <x:c r="F56" s="1" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="G56" s="1" t="str">
+        <x:v>https://doi.org/10.1007/978-3-031-20068-7_33</x:v>
+      </x:c>
       <x:c r="H56" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11702,13 +12352,15 @@
       <x:c r="J56" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K56" s="1" t="str"/>
-      <x:c r="L56" s="1" t="str"/>
+      <x:c r="K56" s="1"/>
+      <x:c r="L56" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M56" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N56" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -11716,11 +12368,21 @@
         <x:v>S056</x:v>
       </x:c>
       <x:c r="B57" s="39"/>
-      <x:c r="C57" s="1" t="str"/>
-      <x:c r="D57" s="1" t="str"/>
-      <x:c r="E57" s="1" t="str"/>
-      <x:c r="F57" s="1" t="str"/>
-      <x:c r="G57" s="1" t="str"/>
+      <x:c r="C57" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D57" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P056</x:v>
+      </x:c>
+      <x:c r="E57" s="1" t="str">
+        <x:v>Investigating Tradeoffs in Real-World Video Super-Resolution</x:v>
+      </x:c>
+      <x:c r="F57" s="1" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="G57" s="1" t="str">
+        <x:v>https://doi.org/10.1109/CVPR52688.2022.00587</x:v>
+      </x:c>
       <x:c r="H57" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11730,13 +12392,15 @@
       <x:c r="J57" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K57" s="1" t="str"/>
-      <x:c r="L57" s="1" t="str"/>
+      <x:c r="K57" s="1"/>
+      <x:c r="L57" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M57" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N57" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -11744,11 +12408,21 @@
         <x:v>S057</x:v>
       </x:c>
       <x:c r="B58" s="39"/>
-      <x:c r="C58" s="1" t="str"/>
-      <x:c r="D58" s="1" t="str"/>
-      <x:c r="E58" s="1" t="str"/>
-      <x:c r="F58" s="1" t="str"/>
-      <x:c r="G58" s="1" t="str"/>
+      <x:c r="C58" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D58" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P057</x:v>
+      </x:c>
+      <x:c r="E58" s="1" t="str">
+        <x:v>Expanding Synthetic Real-World Degradations for Blind Video Super Resolution</x:v>
+      </x:c>
+      <x:c r="F58" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G58" s="1" t="str">
+        <x:v>https://doi.org/10.1109/CVPRW59228.2023.00127</x:v>
+      </x:c>
       <x:c r="H58" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11758,13 +12432,15 @@
       <x:c r="J58" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K58" s="1" t="str"/>
-      <x:c r="L58" s="1" t="str"/>
+      <x:c r="K58" s="1"/>
+      <x:c r="L58" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M58" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N58" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -11772,11 +12448,21 @@
         <x:v>S058</x:v>
       </x:c>
       <x:c r="B59" s="39"/>
-      <x:c r="C59" s="1" t="str"/>
-      <x:c r="D59" s="1" t="str"/>
-      <x:c r="E59" s="1" t="str"/>
-      <x:c r="F59" s="1" t="str"/>
-      <x:c r="G59" s="1" t="str"/>
+      <x:c r="C59" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D59" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P058</x:v>
+      </x:c>
+      <x:c r="E59" s="1" t="str">
+        <x:v>Real-world Video Super-resolution: A Benchmark Dataset and a Decomposition Based Learning Scheme</x:v>
+      </x:c>
+      <x:c r="F59" s="1" t="n">
+        <x:v>2021</x:v>
+      </x:c>
+      <x:c r="G59" s="1" t="str">
+        <x:v>https://doi.org/10.1109/ICCV48922.2021.00474</x:v>
+      </x:c>
       <x:c r="H59" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11786,13 +12472,15 @@
       <x:c r="J59" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K59" s="1" t="str"/>
-      <x:c r="L59" s="1" t="str"/>
+      <x:c r="K59" s="1"/>
+      <x:c r="L59" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M59" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N59" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -11800,11 +12488,21 @@
         <x:v>S059</x:v>
       </x:c>
       <x:c r="B60" s="39"/>
-      <x:c r="C60" s="1" t="str"/>
-      <x:c r="D60" s="1" t="str"/>
-      <x:c r="E60" s="1" t="str"/>
-      <x:c r="F60" s="1" t="str"/>
-      <x:c r="G60" s="1" t="str"/>
+      <x:c r="C60" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D60" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P059</x:v>
+      </x:c>
+      <x:c r="E60" s="1" t="str">
+        <x:v>Real-World Video Deblurring: A Benchmark Dataset and an Efficient Recurrent Neural Network</x:v>
+      </x:c>
+      <x:c r="F60" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G60" s="1" t="str">
+        <x:v>https://doi.org/10.1007/s11263-022-01705-6</x:v>
+      </x:c>
       <x:c r="H60" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11814,13 +12512,15 @@
       <x:c r="J60" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K60" s="1" t="str"/>
-      <x:c r="L60" s="1" t="str"/>
+      <x:c r="K60" s="1"/>
+      <x:c r="L60" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M60" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N60" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -11828,11 +12528,21 @@
         <x:v>S060</x:v>
       </x:c>
       <x:c r="B61" s="39"/>
-      <x:c r="C61" s="1" t="str"/>
-      <x:c r="D61" s="1" t="str"/>
-      <x:c r="E61" s="1" t="str"/>
-      <x:c r="F61" s="1" t="str"/>
-      <x:c r="G61" s="1" t="str"/>
+      <x:c r="C61" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D61" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P060</x:v>
+      </x:c>
+      <x:c r="E61" s="1" t="str">
+        <x:v>CQAD: An Image Quality Assessment Dataset for CCTV</x:v>
+      </x:c>
+      <x:c r="F61" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G61" s="1" t="str">
+        <x:v>https://doi.org/10.33851/JMIS.2025.12.3.81</x:v>
+      </x:c>
       <x:c r="H61" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11842,13 +12552,15 @@
       <x:c r="J61" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K61" s="1" t="str"/>
-      <x:c r="L61" s="1" t="str"/>
+      <x:c r="K61" s="1"/>
+      <x:c r="L61" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M61" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N61" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -11856,11 +12568,21 @@
         <x:v>S061</x:v>
       </x:c>
       <x:c r="B62" s="39"/>
-      <x:c r="C62" s="1" t="str"/>
-      <x:c r="D62" s="1" t="str"/>
-      <x:c r="E62" s="1" t="str"/>
-      <x:c r="F62" s="1" t="str"/>
-      <x:c r="G62" s="1" t="str"/>
+      <x:c r="C62" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D62" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P061</x:v>
+      </x:c>
+      <x:c r="E62" s="1" t="str">
+        <x:v>S3-CLIP: Video Super Resolution for Person-ReID</x:v>
+      </x:c>
+      <x:c r="F62" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G62" s="1" t="str">
+        <x:v>https://doi.org/10.1109/WACVW68408.2026.00174</x:v>
+      </x:c>
       <x:c r="H62" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11870,13 +12592,15 @@
       <x:c r="J62" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K62" s="1" t="str"/>
-      <x:c r="L62" s="1" t="str"/>
+      <x:c r="K62" s="1"/>
+      <x:c r="L62" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M62" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N62" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -11884,11 +12608,21 @@
         <x:v>S062</x:v>
       </x:c>
       <x:c r="B63" s="39"/>
-      <x:c r="C63" s="1" t="str"/>
-      <x:c r="D63" s="1" t="str"/>
-      <x:c r="E63" s="1" t="str"/>
-      <x:c r="F63" s="1" t="str"/>
-      <x:c r="G63" s="1" t="str"/>
+      <x:c r="C63" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D63" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P062</x:v>
+      </x:c>
+      <x:c r="E63" s="1" t="str">
+        <x:v>How to Trust Your Diffusion Model: A Convex Optimization Approach to Conformal Risk Control</x:v>
+      </x:c>
+      <x:c r="F63" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G63" s="1" t="str">
+        <x:v>https://proceedings.mlr.press/v202/teneggi23a.html</x:v>
+      </x:c>
       <x:c r="H63" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11898,13 +12632,15 @@
       <x:c r="J63" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K63" s="1" t="str"/>
-      <x:c r="L63" s="1" t="str"/>
+      <x:c r="K63" s="1"/>
+      <x:c r="L63" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M63" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N63" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -11912,11 +12648,21 @@
         <x:v>S063</x:v>
       </x:c>
       <x:c r="B64" s="39"/>
-      <x:c r="C64" s="1" t="str"/>
-      <x:c r="D64" s="1" t="str"/>
-      <x:c r="E64" s="1" t="str"/>
-      <x:c r="F64" s="1" t="str"/>
-      <x:c r="G64" s="1" t="str"/>
+      <x:c r="C64" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D64" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P063</x:v>
+      </x:c>
+      <x:c r="E64" s="1" t="str">
+        <x:v>Task-Driven Uncertainty Quantification in Inverse Problems via Conformal Prediction</x:v>
+      </x:c>
+      <x:c r="F64" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G64" s="1" t="str">
+        <x:v>https://doi.org/10.1007/978-3-031-73027-6_11</x:v>
+      </x:c>
       <x:c r="H64" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11926,13 +12672,15 @@
       <x:c r="J64" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K64" s="1" t="str"/>
-      <x:c r="L64" s="1" t="str"/>
+      <x:c r="K64" s="1"/>
+      <x:c r="L64" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M64" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N64" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -11940,11 +12688,21 @@
         <x:v>S064</x:v>
       </x:c>
       <x:c r="B65" s="39"/>
-      <x:c r="C65" s="1" t="str"/>
-      <x:c r="D65" s="1" t="str"/>
-      <x:c r="E65" s="1" t="str"/>
-      <x:c r="F65" s="1" t="str"/>
-      <x:c r="G65" s="1" t="str"/>
+      <x:c r="C65" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D65" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P064</x:v>
+      </x:c>
+      <x:c r="E65" s="1" t="str">
+        <x:v>Learning-Based Approaches for Reconstructions With Inexact Operators in nanoCT Applications</x:v>
+      </x:c>
+      <x:c r="F65" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G65" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TCI.2024.3380319</x:v>
+      </x:c>
       <x:c r="H65" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11954,13 +12712,15 @@
       <x:c r="J65" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K65" s="1" t="str"/>
-      <x:c r="L65" s="1" t="str"/>
+      <x:c r="K65" s="1"/>
+      <x:c r="L65" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M65" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N65" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -11968,11 +12728,21 @@
         <x:v>S065</x:v>
       </x:c>
       <x:c r="B66" s="39"/>
-      <x:c r="C66" s="1" t="str"/>
-      <x:c r="D66" s="1" t="str"/>
-      <x:c r="E66" s="1" t="str"/>
-      <x:c r="F66" s="1" t="str"/>
-      <x:c r="G66" s="1" t="str"/>
+      <x:c r="C66" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D66" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P065</x:v>
+      </x:c>
+      <x:c r="E66" s="1" t="str">
+        <x:v>Conformalized Generative Bayesian Imaging: An Uncertainty Quantification Framework for Computational Imaging</x:v>
+      </x:c>
+      <x:c r="F66" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G66" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TCI.2025.3649389</x:v>
+      </x:c>
       <x:c r="H66" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -11982,13 +12752,15 @@
       <x:c r="J66" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K66" s="1" t="str"/>
-      <x:c r="L66" s="1" t="str"/>
+      <x:c r="K66" s="1"/>
+      <x:c r="L66" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M66" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N66" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -11996,11 +12768,21 @@
         <x:v>S066</x:v>
       </x:c>
       <x:c r="B67" s="39"/>
-      <x:c r="C67" s="1" t="str"/>
-      <x:c r="D67" s="1" t="str"/>
-      <x:c r="E67" s="1" t="str"/>
-      <x:c r="F67" s="1" t="str"/>
-      <x:c r="G67" s="1" t="str"/>
+      <x:c r="C67" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D67" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P066</x:v>
+      </x:c>
+      <x:c r="E67" s="1" t="str">
+        <x:v>Self-supervised Conformal Prediction for Uncertainty Quantification in Imaging Problems</x:v>
+      </x:c>
+      <x:c r="F67" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G67" s="1" t="str">
+        <x:v>https://doi.org/10.1007/978-3-031-92366-1_9</x:v>
+      </x:c>
       <x:c r="H67" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12010,13 +12792,15 @@
       <x:c r="J67" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K67" s="1" t="str"/>
-      <x:c r="L67" s="1" t="str"/>
+      <x:c r="K67" s="1"/>
+      <x:c r="L67" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M67" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N67" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -12024,11 +12808,21 @@
         <x:v>S067</x:v>
       </x:c>
       <x:c r="B68" s="39"/>
-      <x:c r="C68" s="1" t="str"/>
-      <x:c r="D68" s="1" t="str"/>
-      <x:c r="E68" s="1" t="str"/>
-      <x:c r="F68" s="1" t="str"/>
-      <x:c r="G68" s="1" t="str"/>
+      <x:c r="C68" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D68" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P067</x:v>
+      </x:c>
+      <x:c r="E68" s="1" t="str">
+        <x:v>QUTCC: Quantile Uncertainty Training and Conformal Calibration for Imaging Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F68" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G68" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2507.14760</x:v>
+      </x:c>
       <x:c r="H68" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12038,13 +12832,15 @@
       <x:c r="J68" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K68" s="1" t="str"/>
-      <x:c r="L68" s="1" t="str"/>
+      <x:c r="K68" s="1"/>
+      <x:c r="L68" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M68" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N68" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -12052,11 +12848,21 @@
         <x:v>S068</x:v>
       </x:c>
       <x:c r="B69" s="39"/>
-      <x:c r="C69" s="1" t="str"/>
-      <x:c r="D69" s="1" t="str"/>
-      <x:c r="E69" s="1" t="str"/>
-      <x:c r="F69" s="1" t="str"/>
-      <x:c r="G69" s="1" t="str"/>
+      <x:c r="C69" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D69" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P068</x:v>
+      </x:c>
+      <x:c r="E69" s="1" t="str">
+        <x:v>Correction Filter for Single Image Super-Resolution</x:v>
+      </x:c>
+      <x:c r="F69" s="1" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G69" s="1" t="str">
+        <x:v>https://doi.org/10.1109/CVPR42600.2020.00150</x:v>
+      </x:c>
       <x:c r="H69" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12066,13 +12872,15 @@
       <x:c r="J69" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K69" s="1" t="str"/>
-      <x:c r="L69" s="1" t="str"/>
+      <x:c r="K69" s="1"/>
+      <x:c r="L69" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M69" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N69" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -12080,11 +12888,21 @@
         <x:v>S069</x:v>
       </x:c>
       <x:c r="B70" s="39"/>
-      <x:c r="C70" s="1" t="str"/>
-      <x:c r="D70" s="1" t="str"/>
-      <x:c r="E70" s="1" t="str"/>
-      <x:c r="F70" s="1" t="str"/>
-      <x:c r="G70" s="1" t="str"/>
+      <x:c r="C70" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D70" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P069</x:v>
+      </x:c>
+      <x:c r="E70" s="1" t="str">
+        <x:v>Blind Image Deconvolution Using Deep Generative Priors</x:v>
+      </x:c>
+      <x:c r="F70" s="1" t="n">
+        <x:v>2020</x:v>
+      </x:c>
+      <x:c r="G70" s="1" t="str">
+        <x:v>https://doi.org/10.1109/TCI.2020.3032671</x:v>
+      </x:c>
       <x:c r="H70" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12094,13 +12912,15 @@
       <x:c r="J70" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K70" s="1" t="str"/>
-      <x:c r="L70" s="1" t="str"/>
+      <x:c r="K70" s="1"/>
+      <x:c r="L70" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M70" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N70" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -12108,11 +12928,21 @@
         <x:v>S070</x:v>
       </x:c>
       <x:c r="B71" s="39"/>
-      <x:c r="C71" s="1" t="str"/>
-      <x:c r="D71" s="1" t="str"/>
-      <x:c r="E71" s="1" t="str"/>
-      <x:c r="F71" s="1" t="str"/>
-      <x:c r="G71" s="1" t="str"/>
+      <x:c r="C71" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D71" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P070</x:v>
+      </x:c>
+      <x:c r="E71" s="1" t="str">
+        <x:v>Grounding Degradations in Natural Language for All-In-One Video Restoration</x:v>
+      </x:c>
+      <x:c r="F71" s="1" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="G71" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2507.14851</x:v>
+      </x:c>
       <x:c r="H71" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12122,13 +12952,15 @@
       <x:c r="J71" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K71" s="1" t="str"/>
-      <x:c r="L71" s="1" t="str"/>
+      <x:c r="K71" s="1"/>
+      <x:c r="L71" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M71" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N71" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -12136,11 +12968,21 @@
         <x:v>S071</x:v>
       </x:c>
       <x:c r="B72" s="39"/>
-      <x:c r="C72" s="1" t="str"/>
-      <x:c r="D72" s="1" t="str"/>
-      <x:c r="E72" s="1" t="str"/>
-      <x:c r="F72" s="1" t="str"/>
-      <x:c r="G72" s="1" t="str"/>
+      <x:c r="C72" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D72" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P071</x:v>
+      </x:c>
+      <x:c r="E72" s="1" t="str">
+        <x:v>All-in-One Image Restoration for Unknown Degradations Using Adaptive Discriminative Filters for Specific Degradations</x:v>
+      </x:c>
+      <x:c r="F72" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G72" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2023/html/Park_All-in-One_Image_Restoration_for_Unknown_Degradations_Using_Adaptive_Discriminative_Filters_CVPR_2023_paper.html</x:v>
+      </x:c>
       <x:c r="H72" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12150,13 +12992,15 @@
       <x:c r="J72" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K72" s="1" t="str"/>
-      <x:c r="L72" s="1" t="str"/>
+      <x:c r="K72" s="1"/>
+      <x:c r="L72" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M72" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N72" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -12164,11 +13008,21 @@
         <x:v>S072</x:v>
       </x:c>
       <x:c r="B73" s="39"/>
-      <x:c r="C73" s="1" t="str"/>
-      <x:c r="D73" s="1" t="str"/>
-      <x:c r="E73" s="1" t="str"/>
-      <x:c r="F73" s="1" t="str"/>
-      <x:c r="G73" s="1" t="str"/>
+      <x:c r="C73" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D73" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P072</x:v>
+      </x:c>
+      <x:c r="E73" s="1" t="str">
+        <x:v>PromptRestorer: A Prompting Image Restoration Method with Degradation Perception</x:v>
+      </x:c>
+      <x:c r="F73" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G73" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/file/1c364d98a5cdc426fd8c76fbb2c10e34-Paper-Conference.pdf</x:v>
+      </x:c>
       <x:c r="H73" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12178,13 +13032,15 @@
       <x:c r="J73" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K73" s="1" t="str"/>
-      <x:c r="L73" s="1" t="str"/>
+      <x:c r="K73" s="1"/>
+      <x:c r="L73" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M73" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N73" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -12192,11 +13048,21 @@
         <x:v>S073</x:v>
       </x:c>
       <x:c r="B74" s="39"/>
-      <x:c r="C74" s="1" t="str"/>
-      <x:c r="D74" s="1" t="str"/>
-      <x:c r="E74" s="1" t="str"/>
-      <x:c r="F74" s="1" t="str"/>
-      <x:c r="G74" s="1" t="str"/>
+      <x:c r="C74" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D74" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P073</x:v>
+      </x:c>
+      <x:c r="E74" s="1" t="str">
+        <x:v>AutoDIR: Automatic All-in-One Image Restoration with Latent Diffusion</x:v>
+      </x:c>
+      <x:c r="F74" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G74" s="1" t="str">
+        <x:v>https://doi.org/10.1007/978-3-031-73661-2_19</x:v>
+      </x:c>
       <x:c r="H74" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12206,13 +13072,15 @@
       <x:c r="J74" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K74" s="1" t="str"/>
-      <x:c r="L74" s="1" t="str"/>
+      <x:c r="K74" s="1"/>
+      <x:c r="L74" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M74" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N74" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -12220,11 +13088,21 @@
         <x:v>S074</x:v>
       </x:c>
       <x:c r="B75" s="39"/>
-      <x:c r="C75" s="1" t="str"/>
-      <x:c r="D75" s="1" t="str"/>
-      <x:c r="E75" s="1" t="str"/>
-      <x:c r="F75" s="1" t="str"/>
-      <x:c r="G75" s="1" t="str"/>
+      <x:c r="C75" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D75" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P074</x:v>
+      </x:c>
+      <x:c r="E75" s="1" t="str">
+        <x:v>Controlling Vision-Language Models for Universal Image Restoration</x:v>
+      </x:c>
+      <x:c r="F75" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G75" s="1" t="str">
+        <x:v>https://openreview.net/forum?id=t3vnnLeajU</x:v>
+      </x:c>
       <x:c r="H75" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12234,13 +13112,15 @@
       <x:c r="J75" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K75" s="1" t="str"/>
-      <x:c r="L75" s="1" t="str"/>
+      <x:c r="K75" s="1"/>
+      <x:c r="L75" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M75" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N75" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -12248,11 +13128,21 @@
         <x:v>S075</x:v>
       </x:c>
       <x:c r="B76" s="39"/>
-      <x:c r="C76" s="1" t="str"/>
-      <x:c r="D76" s="1" t="str"/>
-      <x:c r="E76" s="1" t="str"/>
-      <x:c r="F76" s="1" t="str"/>
-      <x:c r="G76" s="1" t="str"/>
+      <x:c r="C76" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D76" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P075</x:v>
+      </x:c>
+      <x:c r="E76" s="1" t="str">
+        <x:v>Multimodal Prompt Perceiver: Empower Adaptiveness, Generalizability and Fidelity for All-in-One Image Restoration</x:v>
+      </x:c>
+      <x:c r="F76" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G76" s="1" t="str">
+        <x:v>https://doi.org/10.1109/CVPR52733.2024.02403</x:v>
+      </x:c>
       <x:c r="H76" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12262,13 +13152,15 @@
       <x:c r="J76" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K76" s="1" t="str"/>
-      <x:c r="L76" s="1" t="str"/>
+      <x:c r="K76" s="1"/>
+      <x:c r="L76" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M76" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N76" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -12276,11 +13168,21 @@
         <x:v>S076</x:v>
       </x:c>
       <x:c r="B77" s="39"/>
-      <x:c r="C77" s="1" t="str"/>
-      <x:c r="D77" s="1" t="str"/>
-      <x:c r="E77" s="1" t="str"/>
-      <x:c r="F77" s="1" t="str"/>
-      <x:c r="G77" s="1" t="str"/>
+      <x:c r="C77" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D77" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P076</x:v>
+      </x:c>
+      <x:c r="E77" s="1" t="str">
+        <x:v>InstructIR: High-Quality Image Restoration Following Human Instructions</x:v>
+      </x:c>
+      <x:c r="F77" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G77" s="1" t="str">
+        <x:v>https://arxiv.org/abs/2401.16468</x:v>
+      </x:c>
       <x:c r="H77" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12290,13 +13192,15 @@
       <x:c r="J77" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K77" s="1" t="str"/>
-      <x:c r="L77" s="1" t="str"/>
+      <x:c r="K77" s="1"/>
+      <x:c r="L77" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M77" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N77" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -12304,11 +13208,21 @@
         <x:v>S077</x:v>
       </x:c>
       <x:c r="B78" s="39"/>
-      <x:c r="C78" s="1" t="str"/>
-      <x:c r="D78" s="1" t="str"/>
-      <x:c r="E78" s="1" t="str"/>
-      <x:c r="F78" s="1" t="str"/>
-      <x:c r="G78" s="1" t="str"/>
+      <x:c r="C78" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D78" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P077</x:v>
+      </x:c>
+      <x:c r="E78" s="1" t="str">
+        <x:v>RestoreAgent: Autonomous Image Restoration Agent via Multimodal Large Language Models</x:v>
+      </x:c>
+      <x:c r="F78" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G78" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/file/c78f639424b8d89ceb4f2efbb4dfe4f4-Paper-Conference.pdf</x:v>
+      </x:c>
       <x:c r="H78" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12318,13 +13232,15 @@
       <x:c r="J78" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K78" s="1" t="str"/>
-      <x:c r="L78" s="1" t="str"/>
+      <x:c r="K78" s="1"/>
+      <x:c r="L78" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M78" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N78" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -12332,11 +13248,21 @@
         <x:v>S078</x:v>
       </x:c>
       <x:c r="B79" s="39"/>
-      <x:c r="C79" s="1" t="str"/>
-      <x:c r="D79" s="1" t="str"/>
-      <x:c r="E79" s="1" t="str"/>
-      <x:c r="F79" s="1" t="str"/>
-      <x:c r="G79" s="1" t="str"/>
+      <x:c r="C79" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D79" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P078</x:v>
+      </x:c>
+      <x:c r="E79" s="1" t="str">
+        <x:v>DreamClear: High-Capacity Real-World Image Restoration with Privacy-Safe Dataset Curation</x:v>
+      </x:c>
+      <x:c r="F79" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G79" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/file/6452474601429509f3035dc81c233226-Paper-Conference.pdf</x:v>
+      </x:c>
       <x:c r="H79" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12346,13 +13272,15 @@
       <x:c r="J79" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K79" s="1" t="str"/>
-      <x:c r="L79" s="1" t="str"/>
+      <x:c r="K79" s="1"/>
+      <x:c r="L79" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M79" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N79" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -12360,11 +13288,21 @@
         <x:v>S079</x:v>
       </x:c>
       <x:c r="B80" s="39"/>
-      <x:c r="C80" s="1" t="str"/>
-      <x:c r="D80" s="1" t="str"/>
-      <x:c r="E80" s="1" t="str"/>
-      <x:c r="F80" s="1" t="str"/>
-      <x:c r="G80" s="1" t="str"/>
+      <x:c r="C80" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D80" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P079</x:v>
+      </x:c>
+      <x:c r="E80" s="1" t="str">
+        <x:v>Taming Generative Diffusion Prior for Universal Blind Image Restoration</x:v>
+      </x:c>
+      <x:c r="F80" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G80" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/25869dbf7682272357bc2cbbf860e1c8-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H80" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12374,13 +13312,15 @@
       <x:c r="J80" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K80" s="1" t="str"/>
-      <x:c r="L80" s="1" t="str"/>
+      <x:c r="K80" s="1"/>
+      <x:c r="L80" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M80" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N80" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -12388,11 +13328,21 @@
         <x:v>S080</x:v>
       </x:c>
       <x:c r="B81" s="39"/>
-      <x:c r="C81" s="1" t="str"/>
-      <x:c r="D81" s="1" t="str"/>
-      <x:c r="E81" s="1" t="str"/>
-      <x:c r="F81" s="1" t="str"/>
-      <x:c r="G81" s="1" t="str"/>
+      <x:c r="C81" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D81" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P080</x:v>
+      </x:c>
+      <x:c r="E81" s="1" t="str">
+        <x:v>Generative Diffusion Prior for Unified Image Restoration and Enhancement</x:v>
+      </x:c>
+      <x:c r="F81" s="1" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="G81" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2023/html/Fei_Generative_Diffusion_Prior_for_Unified_Image_Restoration_and_Enhancement_CVPR_2023_paper.html</x:v>
+      </x:c>
       <x:c r="H81" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12402,13 +13352,15 @@
       <x:c r="J81" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K81" s="1" t="str"/>
-      <x:c r="L81" s="1" t="str"/>
+      <x:c r="K81" s="1"/>
+      <x:c r="L81" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M81" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N81" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
@@ -12416,11 +13368,21 @@
         <x:v>S081</x:v>
       </x:c>
       <x:c r="B82" s="39"/>
-      <x:c r="C82" s="1" t="str"/>
-      <x:c r="D82" s="1" t="str"/>
-      <x:c r="E82" s="1" t="str"/>
-      <x:c r="F82" s="1" t="str"/>
-      <x:c r="G82" s="1" t="str"/>
+      <x:c r="C82" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D82" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P081</x:v>
+      </x:c>
+      <x:c r="E82" s="1" t="str">
+        <x:v>A Modular Conditional Diffusion Framework for Image Reconstruction</x:v>
+      </x:c>
+      <x:c r="F82" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G82" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/b213d9a999b82cb6fcd03a0d5a7498be-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H82" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12430,13 +13392,15 @@
       <x:c r="J82" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K82" s="1" t="str"/>
-      <x:c r="L82" s="1" t="str"/>
+      <x:c r="K82" s="1"/>
+      <x:c r="L82" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M82" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N82" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="83">
@@ -12444,11 +13408,21 @@
         <x:v>S082</x:v>
       </x:c>
       <x:c r="B83" s="39"/>
-      <x:c r="C83" s="1" t="str"/>
-      <x:c r="D83" s="1" t="str"/>
-      <x:c r="E83" s="1" t="str"/>
-      <x:c r="F83" s="1" t="str"/>
-      <x:c r="G83" s="1" t="str"/>
+      <x:c r="C83" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D83" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P082</x:v>
+      </x:c>
+      <x:c r="E83" s="1" t="str">
+        <x:v>Solving Inverse Problems via Diffusion Optimal Control</x:v>
+      </x:c>
+      <x:c r="F83" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G83" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/86655bc516148e311bcfcf88f1744de7-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H83" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12458,13 +13432,15 @@
       <x:c r="J83" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K83" s="1" t="str"/>
-      <x:c r="L83" s="1" t="str"/>
+      <x:c r="K83" s="1"/>
+      <x:c r="L83" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M83" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N83" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="84">
@@ -12472,11 +13448,21 @@
         <x:v>S083</x:v>
       </x:c>
       <x:c r="B84" s="39"/>
-      <x:c r="C84" s="1" t="str"/>
-      <x:c r="D84" s="1" t="str"/>
-      <x:c r="E84" s="1" t="str"/>
-      <x:c r="F84" s="1" t="str"/>
-      <x:c r="G84" s="1" t="str"/>
+      <x:c r="C84" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D84" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P083</x:v>
+      </x:c>
+      <x:c r="E84" s="1" t="str">
+        <x:v>Provably Robust Score-Based Diffusion Posterior Sampling for Plug-and-Play Image Reconstruction</x:v>
+      </x:c>
+      <x:c r="F84" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G84" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/3fa2d2b637122007845a2fbb7c21453b-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H84" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12486,13 +13472,15 @@
       <x:c r="J84" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K84" s="1" t="str"/>
-      <x:c r="L84" s="1" t="str"/>
+      <x:c r="K84" s="1"/>
+      <x:c r="L84" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M84" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N84" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="85">
@@ -12500,11 +13488,21 @@
         <x:v>S084</x:v>
       </x:c>
       <x:c r="B85" s="39"/>
-      <x:c r="C85" s="1" t="str"/>
-      <x:c r="D85" s="1" t="str"/>
-      <x:c r="E85" s="1" t="str"/>
-      <x:c r="F85" s="1" t="str"/>
-      <x:c r="G85" s="1" t="str"/>
+      <x:c r="C85" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D85" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P084</x:v>
+      </x:c>
+      <x:c r="E85" s="1" t="str">
+        <x:v>Unleashing the Denoising Capability of Diffusion Prior for Solving Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F85" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G85" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/54fa8255cdf30736ecad38e842725e7f-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H85" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12514,13 +13512,15 @@
       <x:c r="J85" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K85" s="1" t="str"/>
-      <x:c r="L85" s="1" t="str"/>
+      <x:c r="K85" s="1"/>
+      <x:c r="L85" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M85" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N85" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="86">
@@ -12528,11 +13528,21 @@
         <x:v>S085</x:v>
       </x:c>
       <x:c r="B86" s="39"/>
-      <x:c r="C86" s="1" t="str"/>
-      <x:c r="D86" s="1" t="str"/>
-      <x:c r="E86" s="1" t="str"/>
-      <x:c r="F86" s="1" t="str"/>
-      <x:c r="G86" s="1" t="str"/>
+      <x:c r="C86" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D86" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P085</x:v>
+      </x:c>
+      <x:c r="E86" s="1" t="str">
+        <x:v>InvFusion: Bridging Supervised and Zero-shot Diffusion for Inverse Problems</x:v>
+      </x:c>
+      <x:c r="F86" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G86" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/33367b9ff199d26280db6cf539d1125c-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H86" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12542,13 +13552,15 @@
       <x:c r="J86" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K86" s="1" t="str"/>
-      <x:c r="L86" s="1" t="str"/>
+      <x:c r="K86" s="1"/>
+      <x:c r="L86" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M86" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N86" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="87">
@@ -12556,11 +13568,21 @@
         <x:v>S086</x:v>
       </x:c>
       <x:c r="B87" s="39"/>
-      <x:c r="C87" s="1" t="str"/>
-      <x:c r="D87" s="1" t="str"/>
-      <x:c r="E87" s="1" t="str"/>
-      <x:c r="F87" s="1" t="str"/>
-      <x:c r="G87" s="1" t="str"/>
+      <x:c r="C87" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D87" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P086</x:v>
+      </x:c>
+      <x:c r="E87" s="1" t="str">
+        <x:v>Solving Inverse Problems with FLAIR</x:v>
+      </x:c>
+      <x:c r="F87" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G87" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/c7ae6e9659f0c99582c2e8214ba0b413-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H87" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12570,13 +13592,15 @@
       <x:c r="J87" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K87" s="1" t="str"/>
-      <x:c r="L87" s="1" t="str"/>
+      <x:c r="K87" s="1"/>
+      <x:c r="L87" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M87" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N87" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="88">
@@ -12584,11 +13608,21 @@
         <x:v>S087</x:v>
       </x:c>
       <x:c r="B88" s="39"/>
-      <x:c r="C88" s="1" t="str"/>
-      <x:c r="D88" s="1" t="str"/>
-      <x:c r="E88" s="1" t="str"/>
-      <x:c r="F88" s="1" t="str"/>
-      <x:c r="G88" s="1" t="str"/>
+      <x:c r="C88" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D88" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P087</x:v>
+      </x:c>
+      <x:c r="E88" s="1" t="str">
+        <x:v>Linearly Constrained Diffusion Implicit Models</x:v>
+      </x:c>
+      <x:c r="F88" s="1" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="G88" s="1" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/d92d3aec6a48e93f93194503ee49f11a-Abstract-Conference.html</x:v>
+      </x:c>
       <x:c r="H88" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12598,13 +13632,15 @@
       <x:c r="J88" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K88" s="1" t="str"/>
-      <x:c r="L88" s="1" t="str"/>
+      <x:c r="K88" s="1"/>
+      <x:c r="L88" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M88" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N88" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="89">
@@ -12612,11 +13648,21 @@
         <x:v>S088</x:v>
       </x:c>
       <x:c r="B89" s="39"/>
-      <x:c r="C89" s="1" t="str"/>
-      <x:c r="D89" s="1" t="str"/>
-      <x:c r="E89" s="1" t="str"/>
-      <x:c r="F89" s="1" t="str"/>
-      <x:c r="G89" s="1" t="str"/>
+      <x:c r="C89" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D89" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P088</x:v>
+      </x:c>
+      <x:c r="E89" s="1" t="str">
+        <x:v>Exploiting Diffusion Prior for Real-World Image Super-Resolution</x:v>
+      </x:c>
+      <x:c r="F89" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G89" s="1" t="str">
+        <x:v>https://doi.org/10.1007/s11263-024-02092-y</x:v>
+      </x:c>
       <x:c r="H89" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12626,13 +13672,15 @@
       <x:c r="J89" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K89" s="1" t="str"/>
-      <x:c r="L89" s="1" t="str"/>
+      <x:c r="K89" s="1"/>
+      <x:c r="L89" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M89" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N89" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="90">
@@ -12640,11 +13688,21 @@
         <x:v>S089</x:v>
       </x:c>
       <x:c r="B90" s="39"/>
-      <x:c r="C90" s="1" t="str"/>
-      <x:c r="D90" s="1" t="str"/>
-      <x:c r="E90" s="1" t="str"/>
-      <x:c r="F90" s="1" t="str"/>
-      <x:c r="G90" s="1" t="str"/>
+      <x:c r="C90" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D90" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P089</x:v>
+      </x:c>
+      <x:c r="E90" s="1" t="str">
+        <x:v>SeeSR: Towards Semantics-Aware Real-World Image Super-Resolution</x:v>
+      </x:c>
+      <x:c r="F90" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G90" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Wu_SeeSR_Towards_Semantics-Aware_Real-World_Image_Super-Resolution_CVPR_2024_paper.html</x:v>
+      </x:c>
       <x:c r="H90" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12654,13 +13712,15 @@
       <x:c r="J90" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K90" s="1" t="str"/>
-      <x:c r="L90" s="1" t="str"/>
+      <x:c r="K90" s="1"/>
+      <x:c r="L90" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M90" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N90" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="91">
@@ -12668,11 +13728,21 @@
         <x:v>S090</x:v>
       </x:c>
       <x:c r="B91" s="39"/>
-      <x:c r="C91" s="1" t="str"/>
-      <x:c r="D91" s="1" t="str"/>
-      <x:c r="E91" s="1" t="str"/>
-      <x:c r="F91" s="1" t="str"/>
-      <x:c r="G91" s="1" t="str"/>
+      <x:c r="C91" s="1" t="str">
+        <x:v>Seed evidence map (pre-systematic)</x:v>
+      </x:c>
+      <x:c r="D91" s="1" t="str">
+        <x:v>Targeted cornerstone search / citation chaining; mapped as P090</x:v>
+      </x:c>
+      <x:c r="E91" s="1" t="str">
+        <x:v>Upscale-A-Video: Temporal-Consistent Diffusion Model for Real-World Video Super-Resolution</x:v>
+      </x:c>
+      <x:c r="F91" s="1" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="G91" s="1" t="str">
+        <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Zhou_Upscale-A-Video_Temporal-Consistent_Diffusion_Model_for_Real-World_Video_Super-Resolution_CVPR_2024_paper.html</x:v>
+      </x:c>
       <x:c r="H91" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -12682,13 +13752,15 @@
       <x:c r="J91" s="1" t="str">
         <x:v>Pending</x:v>
       </x:c>
-      <x:c r="K91" s="1" t="str"/>
-      <x:c r="L91" s="1" t="str"/>
+      <x:c r="K91" s="1"/>
+      <x:c r="L91" s="1" t="str">
+        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
+      </x:c>
       <x:c r="M91" s="1" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="N91" s="1" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
     </x:row>
     <x:row r="92">
@@ -12992,7 +14064,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a33249583894f83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbeee9c6ee3e4a82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13156,12 +14228,24 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B21" s="58" t="str">
-        <x:v>1.0 — seed matrix created 15 September 2026</x:v>
+        <x:v>1.1 — seed corpus transferred to PRISMA screening log on 16 September 2026</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="34" customHeight="1">
-      <x:c r="A22" s="59"/>
-      <x:c r="B22" s="60"/>
+      <x:c r="A22" s="59" t="str">
+        <x:v>Current PRISMA status</x:v>
+      </x:c>
+      <x:c r="B22" s="60" t="str">
+        <x:v>Protocol prepared; formal database searches, deduplication and eligibility screening have not yet started</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>Seed-corpus rule</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>The 90 coded papers are candidate records for gap mapping. They become formally included studies only after the documented PRISMA workflow</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -13406,7 +14490,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R449003a5f0ce4337"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c4067465b5f4679"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Screen first 20 seed records and repair reference metadata
Record 18 AI advance recommendations and 2 unclear cases with primary-source evidence and full-text questions. Keep all human adjudication and formal inclusion pending; add tested pilot counters, correct six bibliographic records, and reconcile protocol v0.3 without changing eligibility or search dates.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R20fabfa668464059"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R17e1a3eabb454e1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R4b0de1100bbc4c92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R408c59cf19964d6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R7210efa6825a41ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R46935e77a9fd4171"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R88656c13a62547e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R5d0c1fadfd894eda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R888b3858e03e436f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R137f7b52b1e0427f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -62,8 +62,19 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -93,6 +104,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -191,7 +222,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="64">
+  <x:cellXfs count="79">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -317,6 +348,43 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -549,7 +617,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R588affd2d8104e37"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7dfbdc67ea5c4653"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -912,7 +980,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="16" t="str">
-        <x:v>Title/abstract screened</x:v>
+        <x:v>Formal title/abstract screened</x:v>
       </x:c>
       <x:c r="B9" s="17" t="n">
         <x:v>0</x:v>
@@ -924,36 +992,72 @@
         <x:v>20</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="32" customHeight="1">
       <x:c r="A10" s="16" t="str">
         <x:v>Full texts assessed</x:v>
       </x:c>
       <x:c r="B10" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="11">
+      <x:c r="D10" s="68" t="str">
+        <x:v>AI pilot — not formal</x:v>
+      </x:c>
+      <x:c r="E10" s="68" t="str">
+        <x:v>Records</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="32" customHeight="1">
       <x:c r="A11" s="16" t="str">
         <x:v>Formally included studies</x:v>
       </x:c>
       <x:c r="B11" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="12">
+      <x:c r="D11" s="69" t="str">
+        <x:v>Pilot records triaged</x:v>
+      </x:c>
+      <x:c r="E11" s="70" t="n">
+        <x:f>COUNTIF('Screening Log'!$I$2:$I$101,"AI pilot: advance")+COUNTIF('Screening Log'!$I$2:$I$101,"AI pilot: unclear")</x:f>
+        <x:v>20</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="32" customHeight="1">
       <x:c r="A12" s="16" t="str">
         <x:v>Formally excluded studies</x:v>
       </x:c>
       <x:c r="B12" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="13">
+      <x:c r="D12" s="69" t="str">
+        <x:v>Advance to full text</x:v>
+      </x:c>
+      <x:c r="E12" s="70" t="n">
+        <x:f>COUNTIF('Screening Log'!$I$2:$I$101,"AI pilot: advance")</x:f>
+        <x:v>18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="32" customHeight="1">
       <x:c r="A13" s="18" t="str">
         <x:v>PRISMA screening</x:v>
       </x:c>
       <x:c r="B13" s="19" t="str">
         <x:v>Not started</x:v>
+      </x:c>
+      <x:c r="D13" s="69" t="str">
+        <x:v>Unclear / retrieve</x:v>
+      </x:c>
+      <x:c r="E13" s="70" t="n">
+        <x:f>COUNTIF('Screening Log'!$I$2:$I$101,"AI pilot: unclear")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="32" customHeight="1">
+      <x:c r="D14" s="69" t="str">
+        <x:v>Not pilot-triaged</x:v>
+      </x:c>
+      <x:c r="E14" s="70" t="n">
+        <x:f>B6-E11</x:f>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1024,7 +1128,7 @@
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
-        <x:v>Proceed to formal database screening and a small go/no-go pilot. Do not claim novelty for physics-informed reconstruction, joint image/kernel estimation, blind diffusion, all-in-one restoration, or uncertainty alone.</x:v>
+        <x:v>Proceed with reproducible database searches and human adjudication. The first 20 seed records received AI pilot recommendations only; no formal inclusion or methodological novelty is established. Feature codes require full-text verification.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1119,7 +1223,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R797d5a006f324de9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb51674a257c64de6"/>
 </x:worksheet>
 </file>
 
@@ -1270,7 +1374,7 @@
         <x:v>2020</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>Dong et al.</x:v>
+        <x:v>Nan, Yuesong; Ji, Hui</x:v>
       </x:c>
       <x:c r="D2" s="9" t="str">
         <x:v>Deep Learning for Handling Kernel/Model Uncertainty in Image Deconvolution</x:v>
@@ -1339,10 +1443,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z2" s="9" t="str">
-        <x:v>Abstract verified</x:v>
+        <x:v>Title/project checked; abstract pending</x:v>
       </x:c>
       <x:c r="AA2" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB2" s="9" t="str">
         <x:v>Yes</x:v>
@@ -1357,7 +1461,7 @@
         <x:v>https://doi.org/10.1109/CVPR42600.2020.00246</x:v>
       </x:c>
       <x:c r="AF2" s="9" t="str">
-        <x:v>Cornerstone mismatch paper</x:v>
+        <x:v>Cornerstone mismatch paper | AI pilot 2026-09-16; advance to full text. Kernel/model uncertainty. Human adjudication and full-text coding pending. Evidence: https://github.com/ysnan/NBD_KerUnc</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -1437,10 +1541,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z3" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA3" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB3" s="9" t="str">
         <x:v>No</x:v>
@@ -1455,7 +1559,7 @@
         <x:v>https://doi.org/10.1088/1361-6420/ab6d57</x:v>
       </x:c>
       <x:c r="AF3" s="9" t="str">
-        <x:v>Theoretical physics-informed baseline</x:v>
+        <x:v>Theoretical physics-informed baseline | AI pilot 2026-09-16; advance to full text. Potential OOD reconstruction reliability. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/1803.00092</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1535,10 +1639,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z4" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA4" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB4" s="9" t="str">
         <x:v>Yes</x:v>
@@ -1553,7 +1657,7 @@
         <x:v>https://doi.org/10.1073/pnas.1907377117</x:v>
       </x:c>
       <x:c r="AF4" s="9" t="str">
-        <x:v>Reliability foundation</x:v>
+        <x:v>Reliability foundation | AI pilot 2026-09-16; advance to full text. Reconstruction instability and missing structure. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/1902.05300</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -1564,13 +1668,13 @@
         <x:v>2020</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
-        <x:v>Rim et al.</x:v>
+        <x:v>Rim, Jaesung; Lee, Haeyun; Won, Jucheol; Cho, Sunghyun</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
         <x:v>Real-World Blur Dataset for Learning and Benchmarking Deblurring Algorithms</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>CVPR</x:v>
+        <x:v>ECCV</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
         <x:v>Conference</x:v>
@@ -1633,10 +1737,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z5" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA5" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB5" s="9" t="str">
         <x:v>No</x:v>
@@ -1648,10 +1752,10 @@
         <x:v>Blur-specific; no full surveillance pipeline or UQ</x:v>
       </x:c>
       <x:c r="AE5" s="9" t="str">
-        <x:v>https://openaccess.thecvf.com/content_CVPR_2020/html/Rim_Real-World_Blur_Dataset_for_Learning_and_Benchmarking_Deblurring_Algorithms_CVPR_2020_paper.html</x:v>
+        <x:v>https://doi.org/10.1007/978-3-030-58595-2_12</x:v>
       </x:c>
       <x:c r="AF5" s="9" t="str">
-        <x:v>Data source candidate</x:v>
+        <x:v>Data source candidate | AI pilot 2026-09-16; advance to full text. Real blur and synthetic-to-real degradation gap. Human adjudication and full-text coding pending. Evidence: https://link.springer.com/chapter/10.1007/978-3-030-58595-2_12</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -1731,10 +1835,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z6" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA6" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB6" s="9" t="str">
         <x:v>Yes</x:v>
@@ -1749,7 +1853,7 @@
         <x:v>https://doi.org/10.1109/TCI.2021.3114542</x:v>
       </x:c>
       <x:c r="AF6" s="9" t="str">
-        <x:v>Nearest early mismatch competitor</x:v>
+        <x:v>Nearest early mismatch competitor | AI pilot 2026-09-16; advance to full text. Explicit forward-model mismatch compensation. Human adjudication and full-text coding pending. Evidence: https://www.eee.hku.hk/optima/pub/journal/2109_TCI.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -1829,10 +1933,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z7" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA7" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB7" s="9" t="str">
         <x:v>No</x:v>
@@ -1847,7 +1951,7 @@
         <x:v>https://doi.org/10.1109/TCI.2021.3118944</x:v>
       </x:c>
       <x:c r="AF7" s="9" t="str">
-        <x:v>Architecture baseline</x:v>
+        <x:v>Architecture baseline | AI pilot 2026-09-16; unclear. Not established from abstract. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2102.07944</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1858,10 +1962,10 @@
         <x:v>2021</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
-        <x:v>Sun &amp; Bouman</x:v>
+        <x:v>Sun, He; Bouman, Katherine L.</x:v>
       </x:c>
       <x:c r="D8" s="9" t="str">
-        <x:v>Deep Probabilistic Imaging</x:v>
+        <x:v>Deep Probabilistic Imaging: Uncertainty Quantification and Multi-modal Solution Characterization for Computational Imaging</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
         <x:v>AAAI</x:v>
@@ -1927,10 +2031,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z8" s="9" t="str">
-        <x:v>Abstract verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA8" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB8" s="9" t="str">
         <x:v>No</x:v>
@@ -1942,10 +2046,10 @@
         <x:v>Image posterior only; operator mismatch not jointly represented</x:v>
       </x:c>
       <x:c r="AE8" s="9" t="str">
-        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/16430</x:v>
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/16366</x:v>
       </x:c>
       <x:c r="AF8" s="9" t="str">
-        <x:v>UQ foundation</x:v>
+        <x:v>UQ foundation | AI pilot 2026-09-16; advance to full text. Image posterior uncertainty and multimodal solutions. Human adjudication and full-text coding pending. Evidence: https://ojs.aaai.org/index.php/AAAI/article/view/16366</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2025,10 +2129,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z9" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA9" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB9" s="9" t="str">
         <x:v>Yes</x:v>
@@ -2043,7 +2147,7 @@
         <x:v>https://doi.org/10.1109/TMI.2021.3077857</x:v>
       </x:c>
       <x:c r="AF9" s="9" t="str">
-        <x:v>Faithfulness foundation</x:v>
+        <x:v>Faithfulness foundation | AI pilot 2026-09-16; advance to full text. Hallucination and measurement/null-space analysis. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2012.00646</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2123,10 +2227,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z10" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA10" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB10" s="9" t="str">
         <x:v>No</x:v>
@@ -2141,7 +2245,7 @@
         <x:v>https://openaccess.thecvf.com/content/ICCV2021/html/Zhang_Designing_a_Practical_Degradation_Model_for_Deep_Blind_Image_Super-Resolution_ICCV_2021_paper.html</x:v>
       </x:c>
       <x:c r="AF10" s="9" t="str">
-        <x:v>Degradation simulator baseline</x:v>
+        <x:v>Degradation simulator baseline | AI pilot 2026-09-16; advance to full text. Blind restoration with compound degradation. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2103.14006</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2221,10 +2325,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z11" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA11" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB11" s="9" t="str">
         <x:v>No</x:v>
@@ -2239,7 +2343,7 @@
         <x:v>https://openaccess.thecvf.com/content/ICCV2021W/AIM/html/Wang_Real-ESRGAN_Training_Real-World_Blind_Super-Resolution_With_Pure_Synthetic_Data_ICCVW_2021_paper.html</x:v>
       </x:c>
       <x:c r="AF11" s="9" t="str">
-        <x:v>Generative restoration baseline</x:v>
+        <x:v>Generative restoration baseline | AI pilot 2026-09-16; advance to full text. Blind super-resolution with high-order degradation. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2107.10833</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2319,10 +2423,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z12" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA12" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB12" s="9" t="str">
         <x:v>Yes</x:v>
@@ -2337,7 +2441,7 @@
         <x:v>https://proceedings.mlr.press/v162/angelopoulos22a.html</x:v>
       </x:c>
       <x:c r="AF12" s="9" t="str">
-        <x:v>Calibration foundation</x:v>
+        <x:v>Calibration foundation | AI pilot 2026-09-16; advance to full text. Calibrated image prediction intervals. Human adjudication and full-text coding pending. Evidence: https://proceedings.mlr.press/v162/angelopoulos22a.html</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2417,10 +2521,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z13" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA13" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB13" s="9" t="str">
         <x:v>No</x:v>
@@ -2435,7 +2539,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2022/hash/95504595b6169131b6ed6cd72eb05616-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF13" s="9" t="str">
-        <x:v>Diffusion baseline</x:v>
+        <x:v>Diffusion baseline | AI pilot 2026-09-16; advance to full text. Posterior reconstruction and transfer across image distributions. Human adjudication and full-text coding pending. Evidence: https://proceedings.neurips.cc/paper_files/paper/2022/hash/95504595b6169131b6ed6cd72eb05616-Abstract-Conference.html</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2515,10 +2619,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z14" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Title/project checked; abstract pending</x:v>
       </x:c>
       <x:c r="AA14" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB14" s="9" t="str">
         <x:v>Yes</x:v>
@@ -2533,7 +2637,7 @@
         <x:v>https://openaccess.thecvf.com/content/CVPR2022/html/Li_All-in-One_Image_Restoration_for_Unknown_Corruption_CVPR_2022_paper.html</x:v>
       </x:c>
       <x:c r="AF14" s="9" t="str">
-        <x:v>Nearest all-in-one baseline</x:v>
+        <x:v>Nearest all-in-one baseline | AI pilot 2026-09-16; advance to full text. Unknown corruption and all-in-one restoration. Human adjudication and full-text coding pending. Evidence: https://github.com/XLearning-SCU/2022-CVPR-AirNet</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2613,10 +2717,10 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z15" s="9" t="str">
-        <x:v>Preprint abstract verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA15" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB15" s="9" t="str">
         <x:v>No</x:v>
@@ -2631,7 +2735,7 @@
         <x:v>https://arxiv.org/abs/2211.09795</x:v>
       </x:c>
       <x:c r="AF15" s="9" t="str">
-        <x:v>UQ method candidate</x:v>
+        <x:v>UQ method candidate | AI pilot 2026-09-16; advance to full text. Diffusion-based confidence intervals. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2211.09795</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2711,10 +2815,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z16" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA16" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB16" s="9" t="str">
         <x:v>No</x:v>
@@ -2729,7 +2833,7 @@
         <x:v>https://openreview.net/forum?id=OnD9zGAGT0k</x:v>
       </x:c>
       <x:c r="AF16" s="9" t="str">
-        <x:v>Diffusion baseline</x:v>
+        <x:v>Diffusion baseline | AI pilot 2026-09-16; advance to full text. Approximate posterior reconstruction under noise. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2209.14687</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2809,10 +2913,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z17" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Title/project checked; abstract pending</x:v>
       </x:c>
       <x:c r="AA17" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB17" s="9" t="str">
         <x:v>No</x:v>
@@ -2827,7 +2931,7 @@
         <x:v>https://openreview.net/forum?id=9_gsMA8MRKQ</x:v>
       </x:c>
       <x:c r="AF17" s="9" t="str">
-        <x:v>Data consistency baseline</x:v>
+        <x:v>Data consistency baseline | AI pilot 2026-09-16; unclear. Cannot adjudicate from retrieved evidence. Human adjudication and full-text coding pending. Evidence: https://openreview.net/forum?id=9_gsMA8MRKQ</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2841,7 +2945,7 @@
         <x:v>Wang et al.</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>Denoising Diffusion Null-Space Model</x:v>
+        <x:v>Zero-Shot Image Restoration Using Denoising Diffusion Null-Space Model</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
         <x:v>ICLR</x:v>
@@ -2907,10 +3011,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z18" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA18" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB18" s="9" t="str">
         <x:v>Yes</x:v>
@@ -2925,7 +3029,7 @@
         <x:v>https://openreview.net/forum?id=mRieQgMtNTQ</x:v>
       </x:c>
       <x:c r="AF18" s="9" t="str">
-        <x:v>Support-map component</x:v>
+        <x:v>Support-map component | AI pilot 2026-09-16; advance to full text. Range/null-space reconstruction and measurement consistency. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2212.00490</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -3005,10 +3109,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z19" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA19" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB19" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3023,7 +3127,7 @@
         <x:v>https://openaccess.thecvf.com/content/CVPR2023/html/Chung_Parallel_Diffusion_Models_of_Operator_and_Image_for_Blind_Inverse_Problems_CVPR_2023_paper.html</x:v>
       </x:c>
       <x:c r="AF19" s="9" t="str">
-        <x:v>Nearest blind diffusion competitor</x:v>
+        <x:v>Nearest blind diffusion competitor | AI pilot 2026-09-16; advance to full text. Joint image/operator inference in blind reconstruction. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2211.10656</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -3037,7 +3141,7 @@
         <x:v>Murata et al.</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>GibbsDDRM</x:v>
+        <x:v>GibbsDDRM: A Partially Collapsed Gibbs Sampler for Solving Blind Inverse Problems with Denoising Diffusion Restoration</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
         <x:v>ICML</x:v>
@@ -3103,10 +3207,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z20" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA20" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB20" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3121,7 +3225,7 @@
         <x:v>https://proceedings.mlr.press/v202/murata23a.html</x:v>
       </x:c>
       <x:c r="AF20" s="9" t="str">
-        <x:v>Nearest joint posterior competitor</x:v>
+        <x:v>Nearest joint posterior competitor | AI pilot 2026-09-16; advance to full text. Joint posterior inference for blind inverse problems. Human adjudication and full-text coding pending. Evidence: https://proceedings.mlr.press/v202/murata23a.html</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -3135,7 +3239,7 @@
         <x:v>Potlapalli et al.</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>PromptIR: Prompting for All-in-One Blind Image Restoration</x:v>
+        <x:v>PromptIR: Prompting for All-in-One Image Restoration</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
         <x:v>NeurIPS</x:v>
@@ -3201,10 +3305,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z21" s="9" t="str">
-        <x:v>Full citation verified</x:v>
+        <x:v>Abstract inspected; full-text pending</x:v>
       </x:c>
       <x:c r="AA21" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB21" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3216,10 +3320,10 @@
         <x:v>No physics traceability, calibrated UQ or failure policy</x:v>
       </x:c>
       <x:c r="AE21" s="9" t="str">
-        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a17bb69ab19f3be921f-Abstract-Conference.html</x:v>
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a579a0d76fd4a35d107-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF21" s="9" t="str">
-        <x:v>Nearest all-in-one baseline</x:v>
+        <x:v>Nearest all-in-one baseline | AI pilot 2026-09-16; advance to full text. Unknown degradation types and levels. Human adjudication and full-text coding pending. Evidence: https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a579a0d76fd4a35d107-Abstract-Conference.html</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -3302,7 +3406,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA22" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB22" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3400,7 +3504,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA23" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB23" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3498,7 +3602,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA24" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB24" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3596,7 +3700,7 @@
         <x:v>Abstract verified</x:v>
       </x:c>
       <x:c r="AA25" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB25" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3694,7 +3798,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA26" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB26" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3792,7 +3896,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA27" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB27" s="9" t="str">
         <x:v>Yes</x:v>
@@ -3890,7 +3994,7 @@
         <x:v>Abstract verified</x:v>
       </x:c>
       <x:c r="AA28" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB28" s="9" t="str">
         <x:v>No</x:v>
@@ -3988,7 +4092,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA29" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB29" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4086,7 +4190,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA30" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB30" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4184,7 +4288,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA31" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB31" s="9" t="str">
         <x:v>No</x:v>
@@ -4282,7 +4386,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA32" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB32" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4380,7 +4484,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA33" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB33" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4478,7 +4582,7 @@
         <x:v>Preprint abstract verified</x:v>
       </x:c>
       <x:c r="AA34" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB34" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4576,7 +4680,7 @@
         <x:v>Preprint abstract verified</x:v>
       </x:c>
       <x:c r="AA35" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB35" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4674,7 +4778,7 @@
         <x:v>Abstract verified</x:v>
       </x:c>
       <x:c r="AA36" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB36" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4772,7 +4876,7 @@
         <x:v>Preprint abstract verified</x:v>
       </x:c>
       <x:c r="AA37" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB37" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4870,7 +4974,7 @@
         <x:v>Preprint full abstract verified</x:v>
       </x:c>
       <x:c r="AA38" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB38" s="9" t="str">
         <x:v>Yes</x:v>
@@ -4968,7 +5072,7 @@
         <x:v>Full preprint verified</x:v>
       </x:c>
       <x:c r="AA39" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB39" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5066,7 +5170,7 @@
         <x:v>Full citation verified</x:v>
       </x:c>
       <x:c r="AA40" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB40" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5164,7 +5268,7 @@
         <x:v>Full abstract verified</x:v>
       </x:c>
       <x:c r="AA41" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB41" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5262,7 +5366,7 @@
         <x:v>Full preprint verified</x:v>
       </x:c>
       <x:c r="AA42" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB42" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5360,7 +5464,7 @@
         <x:v>Full abstract verified</x:v>
       </x:c>
       <x:c r="AA43" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB43" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5458,7 +5562,7 @@
         <x:v>Primary-source verified</x:v>
       </x:c>
       <x:c r="AA44" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB44" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5556,7 +5660,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA45" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB45" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5654,7 +5758,7 @@
         <x:v>Proceedings verified</x:v>
       </x:c>
       <x:c r="AA46" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB46" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5752,7 +5856,7 @@
         <x:v>Publisher verified</x:v>
       </x:c>
       <x:c r="AA47" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB47" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5850,7 +5954,7 @@
         <x:v>OpenReview verified</x:v>
       </x:c>
       <x:c r="AA48" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB48" s="9" t="str">
         <x:v>Yes</x:v>
@@ -5948,7 +6052,7 @@
         <x:v>Proceedings verified</x:v>
       </x:c>
       <x:c r="AA49" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB49" s="9" t="str">
         <x:v>Yes</x:v>
@@ -6046,7 +6150,7 @@
         <x:v>Author manuscript verified</x:v>
       </x:c>
       <x:c r="AA50" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB50" s="9" t="str">
         <x:v>Yes</x:v>
@@ -6144,7 +6248,7 @@
         <x:v>Primary page verified</x:v>
       </x:c>
       <x:c r="AA51" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB51" s="9" t="str">
         <x:v>Yes</x:v>
@@ -6242,7 +6346,7 @@
         <x:v>Publisher/preprint verified</x:v>
       </x:c>
       <x:c r="AA52" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB52" s="9" t="str">
         <x:v>Yes</x:v>
@@ -6340,7 +6444,7 @@
         <x:v>Preprint verified</x:v>
       </x:c>
       <x:c r="AA53" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB53" s="9" t="str">
         <x:v>Yes</x:v>
@@ -6438,7 +6542,7 @@
         <x:v>Publisher/code verified</x:v>
       </x:c>
       <x:c r="AA54" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB54" s="9" t="str">
         <x:v>Yes</x:v>
@@ -6536,7 +6640,7 @@
         <x:v>Full text/code verified</x:v>
       </x:c>
       <x:c r="AA55" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB55" s="9" t="str">
         <x:v>Yes</x:v>
@@ -6634,7 +6738,7 @@
         <x:v>Publisher/code verified</x:v>
       </x:c>
       <x:c r="AA56" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB56" s="9" t="str">
         <x:v>No</x:v>
@@ -6732,7 +6836,7 @@
         <x:v>Full text/code verified</x:v>
       </x:c>
       <x:c r="AA57" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB57" s="9" t="str">
         <x:v>No</x:v>
@@ -6830,7 +6934,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA58" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB58" s="9" t="str">
         <x:v>No</x:v>
@@ -6928,7 +7032,7 @@
         <x:v>Full text/code verified</x:v>
       </x:c>
       <x:c r="AA59" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB59" s="9" t="str">
         <x:v>No</x:v>
@@ -7026,7 +7130,7 @@
         <x:v>Publisher/code verified</x:v>
       </x:c>
       <x:c r="AA60" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB60" s="9" t="str">
         <x:v>No</x:v>
@@ -7124,7 +7228,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA61" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB61" s="9" t="str">
         <x:v>No</x:v>
@@ -7222,7 +7326,7 @@
         <x:v>Full text/code verified</x:v>
       </x:c>
       <x:c r="AA62" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB62" s="9" t="str">
         <x:v>Yes</x:v>
@@ -7320,7 +7424,7 @@
         <x:v>PMLR verified</x:v>
       </x:c>
       <x:c r="AA63" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB63" s="9" t="str">
         <x:v>Yes</x:v>
@@ -7418,7 +7522,7 @@
         <x:v>Publisher/preprint verified</x:v>
       </x:c>
       <x:c r="AA64" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB64" s="9" t="str">
         <x:v>Yes</x:v>
@@ -7516,7 +7620,7 @@
         <x:v>Publisher/preprint verified</x:v>
       </x:c>
       <x:c r="AA65" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB65" s="9" t="str">
         <x:v>Yes</x:v>
@@ -7614,7 +7718,7 @@
         <x:v>Publisher/preprint verified</x:v>
       </x:c>
       <x:c r="AA66" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB66" s="9" t="str">
         <x:v>Yes</x:v>
@@ -7712,7 +7816,7 @@
         <x:v>Publisher verified</x:v>
       </x:c>
       <x:c r="AA67" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB67" s="9" t="str">
         <x:v>No</x:v>
@@ -7810,7 +7914,7 @@
         <x:v>Full preprint verified</x:v>
       </x:c>
       <x:c r="AA68" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB68" s="9" t="str">
         <x:v>Yes</x:v>
@@ -7908,7 +8012,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA69" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB69" s="9" t="str">
         <x:v>No</x:v>
@@ -8006,7 +8110,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA70" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB70" s="9" t="str">
         <x:v>No</x:v>
@@ -8104,7 +8208,7 @@
         <x:v>Full text/code verified</x:v>
       </x:c>
       <x:c r="AA71" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB71" s="9" t="str">
         <x:v>Yes</x:v>
@@ -8202,7 +8306,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA72" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB72" s="9" t="str">
         <x:v>No</x:v>
@@ -8300,7 +8404,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA73" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB73" s="9" t="str">
         <x:v>No</x:v>
@@ -8398,7 +8502,7 @@
         <x:v>Publisher/preprint verified</x:v>
       </x:c>
       <x:c r="AA74" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB74" s="9" t="str">
         <x:v>Yes</x:v>
@@ -8496,7 +8600,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA75" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB75" s="9" t="str">
         <x:v>Yes</x:v>
@@ -8594,7 +8698,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA76" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB76" s="9" t="str">
         <x:v>Yes</x:v>
@@ -8692,7 +8796,7 @@
         <x:v>Full text/code verified</x:v>
       </x:c>
       <x:c r="AA77" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB77" s="9" t="str">
         <x:v>No</x:v>
@@ -8790,7 +8894,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA78" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB78" s="9" t="str">
         <x:v>Yes</x:v>
@@ -8888,7 +8992,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA79" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB79" s="9" t="str">
         <x:v>Yes</x:v>
@@ -8986,7 +9090,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA80" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB80" s="9" t="str">
         <x:v>Yes</x:v>
@@ -9084,7 +9188,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA81" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB81" s="9" t="str">
         <x:v>Yes</x:v>
@@ -9182,7 +9286,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA82" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB82" s="9" t="str">
         <x:v>No</x:v>
@@ -9280,7 +9384,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA83" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB83" s="9" t="str">
         <x:v>No</x:v>
@@ -9378,7 +9482,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA84" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB84" s="9" t="str">
         <x:v>Yes</x:v>
@@ -9476,7 +9580,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA85" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB85" s="9" t="str">
         <x:v>No</x:v>
@@ -9574,7 +9678,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA86" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB86" s="9" t="str">
         <x:v>Yes</x:v>
@@ -9672,7 +9776,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA87" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB87" s="9" t="str">
         <x:v>Yes</x:v>
@@ -9770,7 +9874,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA88" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB88" s="9" t="str">
         <x:v>No</x:v>
@@ -9868,7 +9972,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA89" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB89" s="9" t="str">
         <x:v>Yes</x:v>
@@ -9966,7 +10070,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA90" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB90" s="9" t="str">
         <x:v>Yes</x:v>
@@ -10064,7 +10168,7 @@
         <x:v>Full text verified</x:v>
       </x:c>
       <x:c r="AA91" s="9" t="str">
-        <x:v>Include</x:v>
+        <x:v>Pending formal eligibility</x:v>
       </x:c>
       <x:c r="AB91" s="9" t="str">
         <x:v>Yes</x:v>
@@ -10091,7 +10195,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c4e6da3c08b48bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6deff8f4c51e4872"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10111,15 +10215,15 @@
     <x:col min="6" max="6" width="9" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="38" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="19" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="19" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="19" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="64" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
+    <x:row r="1" ht="42" customHeight="1">
       <x:c r="A1" s="38" t="str">
         <x:v>Record ID</x:v>
       </x:c>
@@ -10144,822 +10248,822 @@
       <x:c r="H1" s="38" t="str">
         <x:v>Duplicate?</x:v>
       </x:c>
-      <x:c r="I1" s="38" t="str">
+      <x:c r="I1" s="71" t="str">
         <x:v>Title/abstract decision</x:v>
       </x:c>
-      <x:c r="J1" s="38" t="str">
+      <x:c r="J1" s="71" t="str">
         <x:v>Full-text decision</x:v>
       </x:c>
-      <x:c r="K1" s="38" t="str">
+      <x:c r="K1" s="71" t="str">
         <x:v>Exclusion reason</x:v>
       </x:c>
-      <x:c r="L1" s="38" t="str">
+      <x:c r="L1" s="71" t="str">
         <x:v>Reviewer notes</x:v>
       </x:c>
-      <x:c r="M1" s="38" t="str">
+      <x:c r="M1" s="71" t="str">
         <x:v>Full-text obtained?</x:v>
       </x:c>
-      <x:c r="N1" s="38" t="str">
+      <x:c r="N1" s="71" t="str">
         <x:v>Added to matrix?</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
-      <x:c r="A2" s="1" t="str">
+    <x:row r="2" ht="84" customHeight="1">
+      <x:c r="A2" s="73" t="str">
         <x:v>S001</x:v>
       </x:c>
-      <x:c r="B2" s="39"/>
-      <x:c r="C2" s="1" t="str">
+      <x:c r="B2" s="74"/>
+      <x:c r="C2" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D2" s="1" t="str">
+      <x:c r="D2" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P001</x:v>
       </x:c>
-      <x:c r="E2" s="1" t="str">
+      <x:c r="E2" s="73" t="str">
         <x:v>Deep Learning for Handling Kernel/Model Uncertainty in Image Deconvolution</x:v>
       </x:c>
-      <x:c r="F2" s="1" t="n">
+      <x:c r="F2" s="73" t="n">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="G2" s="1" t="str">
+      <x:c r="G2" s="73" t="str">
         <x:v>https://doi.org/10.1109/CVPR42600.2020.00246</x:v>
       </x:c>
-      <x:c r="H2" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I2" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J2" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K2" s="1"/>
-      <x:c r="L2" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M2" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N2" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="1" t="str">
+      <x:c r="H2" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I2" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J2" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K2" s="75"/>
+      <x:c r="L2" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Kernel/model uncertainty. Basis: Title and official author repository; abstract not retrieved. Full-text question and source: screening/pilot_01.json (P001).</x:v>
+      </x:c>
+      <x:c r="M2" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N2" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="84" customHeight="1">
+      <x:c r="A3" s="73" t="str">
         <x:v>S002</x:v>
       </x:c>
-      <x:c r="B3" s="39"/>
-      <x:c r="C3" s="1" t="str">
+      <x:c r="B3" s="74"/>
+      <x:c r="C3" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D3" s="1" t="str">
+      <x:c r="D3" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P002</x:v>
       </x:c>
-      <x:c r="E3" s="1" t="str">
+      <x:c r="E3" s="73" t="str">
         <x:v>NETT: Solving Inverse Problems with Deep Neural Networks</x:v>
       </x:c>
-      <x:c r="F3" s="1" t="n">
+      <x:c r="F3" s="73" t="n">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="G3" s="1" t="str">
+      <x:c r="G3" s="73" t="str">
         <x:v>https://doi.org/10.1088/1361-6420/ab6d57</x:v>
       </x:c>
-      <x:c r="H3" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I3" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J3" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K3" s="1"/>
-      <x:c r="L3" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M3" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N3" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="1" t="str">
+      <x:c r="H3" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I3" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J3" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K3" s="75"/>
+      <x:c r="L3" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Potential OOD reconstruction reliability. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P002).</x:v>
+      </x:c>
+      <x:c r="M3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N3" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="84" customHeight="1">
+      <x:c r="A4" s="73" t="str">
         <x:v>S003</x:v>
       </x:c>
-      <x:c r="B4" s="39"/>
-      <x:c r="C4" s="1" t="str">
+      <x:c r="B4" s="74"/>
+      <x:c r="C4" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D4" s="1" t="str">
+      <x:c r="D4" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P003</x:v>
       </x:c>
-      <x:c r="E4" s="1" t="str">
+      <x:c r="E4" s="73" t="str">
         <x:v>On Instabilities of Deep Learning in Image Reconstruction and the Potential Costs of AI</x:v>
       </x:c>
-      <x:c r="F4" s="1" t="n">
+      <x:c r="F4" s="73" t="n">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="G4" s="1" t="str">
+      <x:c r="G4" s="73" t="str">
         <x:v>https://doi.org/10.1073/pnas.1907377117</x:v>
       </x:c>
-      <x:c r="H4" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I4" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J4" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K4" s="1"/>
-      <x:c r="L4" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M4" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N4" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="1" t="str">
+      <x:c r="H4" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I4" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J4" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K4" s="75"/>
+      <x:c r="L4" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Reconstruction instability and missing structure. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P003).</x:v>
+      </x:c>
+      <x:c r="M4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N4" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="84" customHeight="1">
+      <x:c r="A5" s="73" t="str">
         <x:v>S004</x:v>
       </x:c>
-      <x:c r="B5" s="39"/>
-      <x:c r="C5" s="1" t="str">
+      <x:c r="B5" s="74"/>
+      <x:c r="C5" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D5" s="1" t="str">
+      <x:c r="D5" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P004</x:v>
       </x:c>
-      <x:c r="E5" s="1" t="str">
+      <x:c r="E5" s="73" t="str">
         <x:v>Real-World Blur Dataset for Learning and Benchmarking Deblurring Algorithms</x:v>
       </x:c>
-      <x:c r="F5" s="1" t="n">
+      <x:c r="F5" s="73" t="n">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="G5" s="1" t="str">
-        <x:v>https://openaccess.thecvf.com/content_CVPR_2020/html/Rim_Real-World_Blur_Dataset_for_Learning_and_Benchmarking_Deblurring_Algorithms_CVPR_2020_paper.html</x:v>
-      </x:c>
-      <x:c r="H5" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I5" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J5" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K5" s="1"/>
-      <x:c r="L5" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M5" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N5" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="1" t="str">
+      <x:c r="G5" s="73" t="str">
+        <x:v>https://doi.org/10.1007/978-3-030-58595-2_12</x:v>
+      </x:c>
+      <x:c r="H5" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I5" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J5" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K5" s="75"/>
+      <x:c r="L5" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Real blur and synthetic-to-real degradation gap. Basis: Publisher abstract. Full-text question and source: screening/pilot_01.json (P004).</x:v>
+      </x:c>
+      <x:c r="M5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N5" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="84" customHeight="1">
+      <x:c r="A6" s="73" t="str">
         <x:v>S005</x:v>
       </x:c>
-      <x:c r="B6" s="39"/>
-      <x:c r="C6" s="1" t="str">
+      <x:c r="B6" s="74"/>
+      <x:c r="C6" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D6" s="1" t="str">
+      <x:c r="D6" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P005</x:v>
       </x:c>
-      <x:c r="E6" s="1" t="str">
+      <x:c r="E6" s="73" t="str">
         <x:v>Robust Reconstruction With Deep Learning to Handle Model Mismatch in Lensless Imaging</x:v>
       </x:c>
-      <x:c r="F6" s="1" t="n">
+      <x:c r="F6" s="73" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G6" s="1" t="str">
+      <x:c r="G6" s="73" t="str">
         <x:v>https://doi.org/10.1109/TCI.2021.3114542</x:v>
       </x:c>
-      <x:c r="H6" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I6" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J6" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K6" s="1"/>
-      <x:c r="L6" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M6" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N6" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="1" t="str">
+      <x:c r="H6" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I6" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J6" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K6" s="75"/>
+      <x:c r="L6" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Explicit forward-model mismatch compensation. Basis: Author-hosted published PDF abstract and opening page. Full-text question and source: screening/pilot_01.json (P005).</x:v>
+      </x:c>
+      <x:c r="M6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N6" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="84" customHeight="1">
+      <x:c r="A7" s="73" t="str">
         <x:v>S006</x:v>
       </x:c>
-      <x:c r="B7" s="39"/>
-      <x:c r="C7" s="1" t="str">
+      <x:c r="B7" s="74"/>
+      <x:c r="C7" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D7" s="1" t="str">
+      <x:c r="D7" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P006</x:v>
       </x:c>
-      <x:c r="E7" s="1" t="str">
+      <x:c r="E7" s="73" t="str">
         <x:v>Deep Equilibrium Architectures for Inverse Problems in Imaging</x:v>
       </x:c>
-      <x:c r="F7" s="1" t="n">
+      <x:c r="F7" s="73" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G7" s="1" t="str">
+      <x:c r="G7" s="73" t="str">
         <x:v>https://doi.org/10.1109/TCI.2021.3118944</x:v>
       </x:c>
-      <x:c r="H7" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I7" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J7" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K7" s="1"/>
-      <x:c r="L7" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M7" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N7" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="1" t="str">
+      <x:c r="H7" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I7" s="77" t="str">
+        <x:v>AI pilot: unclear</x:v>
+      </x:c>
+      <x:c r="J7" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K7" s="75"/>
+      <x:c r="L7" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Not established from abstract. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P006).</x:v>
+      </x:c>
+      <x:c r="M7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N7" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="84" customHeight="1">
+      <x:c r="A8" s="73" t="str">
         <x:v>S007</x:v>
       </x:c>
-      <x:c r="B8" s="39"/>
-      <x:c r="C8" s="1" t="str">
+      <x:c r="B8" s="74"/>
+      <x:c r="C8" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D8" s="1" t="str">
+      <x:c r="D8" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P007</x:v>
       </x:c>
-      <x:c r="E8" s="1" t="str">
-        <x:v>Deep Probabilistic Imaging</x:v>
-      </x:c>
-      <x:c r="F8" s="1" t="n">
+      <x:c r="E8" s="73" t="str">
+        <x:v>Deep Probabilistic Imaging: Uncertainty Quantification and Multi-modal Solution Characterization for Computational Imaging</x:v>
+      </x:c>
+      <x:c r="F8" s="73" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G8" s="1" t="str">
-        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/16430</x:v>
-      </x:c>
-      <x:c r="H8" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I8" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J8" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K8" s="1"/>
-      <x:c r="L8" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M8" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N8" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="1" t="str">
+      <x:c r="G8" s="73" t="str">
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/16366</x:v>
+      </x:c>
+      <x:c r="H8" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I8" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J8" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K8" s="75"/>
+      <x:c r="L8" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Image posterior uncertainty and multimodal solutions. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P007).</x:v>
+      </x:c>
+      <x:c r="M8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N8" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="84" customHeight="1">
+      <x:c r="A9" s="73" t="str">
         <x:v>S008</x:v>
       </x:c>
-      <x:c r="B9" s="39"/>
-      <x:c r="C9" s="1" t="str">
+      <x:c r="B9" s="74"/>
+      <x:c r="C9" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D9" s="1" t="str">
+      <x:c r="D9" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P008</x:v>
       </x:c>
-      <x:c r="E9" s="1" t="str">
+      <x:c r="E9" s="73" t="str">
         <x:v>On Hallucinations in Tomographic Image Reconstruction</x:v>
       </x:c>
-      <x:c r="F9" s="1" t="n">
+      <x:c r="F9" s="73" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G9" s="1" t="str">
+      <x:c r="G9" s="73" t="str">
         <x:v>https://doi.org/10.1109/TMI.2021.3077857</x:v>
       </x:c>
-      <x:c r="H9" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I9" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J9" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K9" s="1"/>
-      <x:c r="L9" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M9" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N9" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="1" t="str">
+      <x:c r="H9" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I9" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J9" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K9" s="75"/>
+      <x:c r="L9" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Hallucination and measurement/null-space analysis. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P008).</x:v>
+      </x:c>
+      <x:c r="M9" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N9" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="84" customHeight="1">
+      <x:c r="A10" s="73" t="str">
         <x:v>S009</x:v>
       </x:c>
-      <x:c r="B10" s="39"/>
-      <x:c r="C10" s="1" t="str">
+      <x:c r="B10" s="74"/>
+      <x:c r="C10" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D10" s="1" t="str">
+      <x:c r="D10" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P009</x:v>
       </x:c>
-      <x:c r="E10" s="1" t="str">
+      <x:c r="E10" s="73" t="str">
         <x:v>Designing a Practical Degradation Model for Deep Blind Image Super-Resolution</x:v>
       </x:c>
-      <x:c r="F10" s="1" t="n">
+      <x:c r="F10" s="73" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G10" s="1" t="str">
+      <x:c r="G10" s="73" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2021/html/Zhang_Designing_a_Practical_Degradation_Model_for_Deep_Blind_Image_Super-Resolution_ICCV_2021_paper.html</x:v>
       </x:c>
-      <x:c r="H10" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I10" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J10" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K10" s="1"/>
-      <x:c r="L10" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M10" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N10" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="1" t="str">
+      <x:c r="H10" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I10" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J10" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K10" s="75"/>
+      <x:c r="L10" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Blind restoration with compound degradation. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P009).</x:v>
+      </x:c>
+      <x:c r="M10" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N10" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="84" customHeight="1">
+      <x:c r="A11" s="73" t="str">
         <x:v>S010</x:v>
       </x:c>
-      <x:c r="B11" s="39"/>
-      <x:c r="C11" s="1" t="str">
+      <x:c r="B11" s="74"/>
+      <x:c r="C11" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D11" s="1" t="str">
+      <x:c r="D11" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P010</x:v>
       </x:c>
-      <x:c r="E11" s="1" t="str">
+      <x:c r="E11" s="73" t="str">
         <x:v>Real-ESRGAN: Training Real-World Blind Super-Resolution With Pure Synthetic Data</x:v>
       </x:c>
-      <x:c r="F11" s="1" t="n">
+      <x:c r="F11" s="73" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="G11" s="1" t="str">
+      <x:c r="G11" s="73" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2021W/AIM/html/Wang_Real-ESRGAN_Training_Real-World_Blind_Super-Resolution_With_Pure_Synthetic_Data_ICCVW_2021_paper.html</x:v>
       </x:c>
-      <x:c r="H11" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I11" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J11" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K11" s="1"/>
-      <x:c r="L11" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M11" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N11" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="1" t="str">
+      <x:c r="H11" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I11" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J11" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K11" s="75"/>
+      <x:c r="L11" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Blind super-resolution with high-order degradation. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P010).</x:v>
+      </x:c>
+      <x:c r="M11" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N11" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="84" customHeight="1">
+      <x:c r="A12" s="73" t="str">
         <x:v>S011</x:v>
       </x:c>
-      <x:c r="B12" s="39"/>
-      <x:c r="C12" s="1" t="str">
+      <x:c r="B12" s="74"/>
+      <x:c r="C12" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D12" s="1" t="str">
+      <x:c r="D12" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P011</x:v>
       </x:c>
-      <x:c r="E12" s="1" t="str">
+      <x:c r="E12" s="73" t="str">
         <x:v>Image-to-Image Regression with Distribution-Free Uncertainty Quantification and Applications in Imaging</x:v>
       </x:c>
-      <x:c r="F12" s="1" t="n">
+      <x:c r="F12" s="73" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="G12" s="1" t="str">
+      <x:c r="G12" s="73" t="str">
         <x:v>https://proceedings.mlr.press/v162/angelopoulos22a.html</x:v>
       </x:c>
-      <x:c r="H12" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I12" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J12" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K12" s="1"/>
-      <x:c r="L12" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M12" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N12" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="1" t="str">
+      <x:c r="H12" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I12" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J12" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K12" s="75"/>
+      <x:c r="L12" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Calibrated image prediction intervals. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P011).</x:v>
+      </x:c>
+      <x:c r="M12" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N12" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="84" customHeight="1">
+      <x:c r="A13" s="73" t="str">
         <x:v>S012</x:v>
       </x:c>
-      <x:c r="B13" s="39"/>
-      <x:c r="C13" s="1" t="str">
+      <x:c r="B13" s="74"/>
+      <x:c r="C13" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D13" s="1" t="str">
+      <x:c r="D13" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P012</x:v>
       </x:c>
-      <x:c r="E13" s="1" t="str">
+      <x:c r="E13" s="73" t="str">
         <x:v>Denoising Diffusion Restoration Models</x:v>
       </x:c>
-      <x:c r="F13" s="1" t="n">
+      <x:c r="F13" s="73" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="G13" s="1" t="str">
+      <x:c r="G13" s="73" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2022/hash/95504595b6169131b6ed6cd72eb05616-Abstract-Conference.html</x:v>
       </x:c>
-      <x:c r="H13" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I13" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J13" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K13" s="1"/>
-      <x:c r="L13" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M13" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N13" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="1" t="str">
+      <x:c r="H13" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I13" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J13" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K13" s="75"/>
+      <x:c r="L13" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Posterior reconstruction and transfer across image distributions. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P012).</x:v>
+      </x:c>
+      <x:c r="M13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N13" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="84" customHeight="1">
+      <x:c r="A14" s="73" t="str">
         <x:v>S013</x:v>
       </x:c>
-      <x:c r="B14" s="39"/>
-      <x:c r="C14" s="1" t="str">
+      <x:c r="B14" s="74"/>
+      <x:c r="C14" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D14" s="1" t="str">
+      <x:c r="D14" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P013</x:v>
       </x:c>
-      <x:c r="E14" s="1" t="str">
+      <x:c r="E14" s="73" t="str">
         <x:v>All-in-One Image Restoration for Unknown Corruption</x:v>
       </x:c>
-      <x:c r="F14" s="1" t="n">
+      <x:c r="F14" s="73" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="G14" s="1" t="str">
+      <x:c r="G14" s="73" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2022/html/Li_All-in-One_Image_Restoration_for_Unknown_Corruption_CVPR_2022_paper.html</x:v>
       </x:c>
-      <x:c r="H14" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I14" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J14" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K14" s="1"/>
-      <x:c r="L14" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M14" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N14" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="1" t="str">
+      <x:c r="H14" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I14" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J14" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K14" s="75"/>
+      <x:c r="L14" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Unknown corruption and all-in-one restoration. Basis: Title and official author repository; abstract not retrieved. Full-text question and source: screening/pilot_01.json (P013).</x:v>
+      </x:c>
+      <x:c r="M14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N14" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="84" customHeight="1">
+      <x:c r="A15" s="73" t="str">
         <x:v>S014</x:v>
       </x:c>
-      <x:c r="B15" s="39"/>
-      <x:c r="C15" s="1" t="str">
+      <x:c r="B15" s="74"/>
+      <x:c r="C15" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D15" s="1" t="str">
+      <x:c r="D15" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P014</x:v>
       </x:c>
-      <x:c r="E15" s="1" t="str">
+      <x:c r="E15" s="73" t="str">
         <x:v>Conffusion: Confidence Intervals for Diffusion Models</x:v>
       </x:c>
-      <x:c r="F15" s="1" t="n">
+      <x:c r="F15" s="73" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="G15" s="1" t="str">
+      <x:c r="G15" s="73" t="str">
         <x:v>https://arxiv.org/abs/2211.09795</x:v>
       </x:c>
-      <x:c r="H15" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I15" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J15" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K15" s="1"/>
-      <x:c r="L15" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M15" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N15" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="1" t="str">
+      <x:c r="H15" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I15" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J15" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K15" s="75"/>
+      <x:c r="L15" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Diffusion-based confidence intervals. Basis: Preprint abstract; peer review not established. Full-text question and source: screening/pilot_01.json (P014).</x:v>
+      </x:c>
+      <x:c r="M15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N15" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="84" customHeight="1">
+      <x:c r="A16" s="73" t="str">
         <x:v>S015</x:v>
       </x:c>
-      <x:c r="B16" s="39"/>
-      <x:c r="C16" s="1" t="str">
+      <x:c r="B16" s="74"/>
+      <x:c r="C16" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D16" s="1" t="str">
+      <x:c r="D16" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P015</x:v>
       </x:c>
-      <x:c r="E16" s="1" t="str">
+      <x:c r="E16" s="73" t="str">
         <x:v>Diffusion Posterior Sampling for General Noisy Inverse Problems</x:v>
       </x:c>
-      <x:c r="F16" s="1" t="n">
+      <x:c r="F16" s="73" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="G16" s="1" t="str">
+      <x:c r="G16" s="73" t="str">
         <x:v>https://openreview.net/forum?id=OnD9zGAGT0k</x:v>
       </x:c>
-      <x:c r="H16" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I16" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J16" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K16" s="1"/>
-      <x:c r="L16" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M16" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N16" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="1" t="str">
+      <x:c r="H16" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I16" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J16" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K16" s="75"/>
+      <x:c r="L16" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Approximate posterior reconstruction under noise. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P015).</x:v>
+      </x:c>
+      <x:c r="M16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N16" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="84" customHeight="1">
+      <x:c r="A17" s="73" t="str">
         <x:v>S016</x:v>
       </x:c>
-      <x:c r="B17" s="39"/>
-      <x:c r="C17" s="1" t="str">
+      <x:c r="B17" s="74"/>
+      <x:c r="C17" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D17" s="1" t="str">
+      <x:c r="D17" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P016</x:v>
       </x:c>
-      <x:c r="E17" s="1" t="str">
+      <x:c r="E17" s="73" t="str">
         <x:v>Pseudoinverse-Guided Diffusion Models for Inverse Problems</x:v>
       </x:c>
-      <x:c r="F17" s="1" t="n">
+      <x:c r="F17" s="73" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="G17" s="1" t="str">
+      <x:c r="G17" s="73" t="str">
         <x:v>https://openreview.net/forum?id=9_gsMA8MRKQ</x:v>
       </x:c>
-      <x:c r="H17" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I17" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J17" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K17" s="1"/>
-      <x:c r="L17" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M17" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N17" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="1" t="str">
+      <x:c r="H17" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I17" s="77" t="str">
+        <x:v>AI pilot: unclear</x:v>
+      </x:c>
+      <x:c r="J17" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K17" s="75"/>
+      <x:c r="L17" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Cannot adjudicate from retrieved evidence. Basis: Official search snippet only; full abstract not retrieved. Full-text question and source: screening/pilot_01.json (P016).</x:v>
+      </x:c>
+      <x:c r="M17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N17" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="84" customHeight="1">
+      <x:c r="A18" s="73" t="str">
         <x:v>S017</x:v>
       </x:c>
-      <x:c r="B18" s="39"/>
-      <x:c r="C18" s="1" t="str">
+      <x:c r="B18" s="74"/>
+      <x:c r="C18" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D18" s="1" t="str">
+      <x:c r="D18" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P017</x:v>
       </x:c>
-      <x:c r="E18" s="1" t="str">
-        <x:v>Denoising Diffusion Null-Space Model</x:v>
-      </x:c>
-      <x:c r="F18" s="1" t="n">
+      <x:c r="E18" s="73" t="str">
+        <x:v>Zero-Shot Image Restoration Using Denoising Diffusion Null-Space Model</x:v>
+      </x:c>
+      <x:c r="F18" s="73" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="G18" s="1" t="str">
+      <x:c r="G18" s="73" t="str">
         <x:v>https://openreview.net/forum?id=mRieQgMtNTQ</x:v>
       </x:c>
-      <x:c r="H18" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I18" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J18" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K18" s="1"/>
-      <x:c r="L18" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M18" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N18" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="1" t="str">
+      <x:c r="H18" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I18" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J18" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K18" s="75"/>
+      <x:c r="L18" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Range/null-space reconstruction and measurement consistency. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P017).</x:v>
+      </x:c>
+      <x:c r="M18" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N18" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="84" customHeight="1">
+      <x:c r="A19" s="73" t="str">
         <x:v>S018</x:v>
       </x:c>
-      <x:c r="B19" s="39"/>
-      <x:c r="C19" s="1" t="str">
+      <x:c r="B19" s="74"/>
+      <x:c r="C19" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D19" s="1" t="str">
+      <x:c r="D19" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P018</x:v>
       </x:c>
-      <x:c r="E19" s="1" t="str">
+      <x:c r="E19" s="73" t="str">
         <x:v>Parallel Diffusion Models of Operator and Image for Blind Inverse Problems</x:v>
       </x:c>
-      <x:c r="F19" s="1" t="n">
+      <x:c r="F19" s="73" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="G19" s="1" t="str">
+      <x:c r="G19" s="73" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2023/html/Chung_Parallel_Diffusion_Models_of_Operator_and_Image_for_Blind_Inverse_Problems_CVPR_2023_paper.html</x:v>
       </x:c>
-      <x:c r="H19" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I19" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J19" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K19" s="1"/>
-      <x:c r="L19" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M19" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N19" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="1" t="str">
+      <x:c r="H19" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I19" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J19" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K19" s="75"/>
+      <x:c r="L19" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Joint image/operator inference in blind reconstruction. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P018).</x:v>
+      </x:c>
+      <x:c r="M19" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="84" customHeight="1">
+      <x:c r="A20" s="73" t="str">
         <x:v>S019</x:v>
       </x:c>
-      <x:c r="B20" s="39"/>
-      <x:c r="C20" s="1" t="str">
+      <x:c r="B20" s="74"/>
+      <x:c r="C20" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D20" s="1" t="str">
+      <x:c r="D20" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P019</x:v>
       </x:c>
-      <x:c r="E20" s="1" t="str">
-        <x:v>GibbsDDRM</x:v>
-      </x:c>
-      <x:c r="F20" s="1" t="n">
+      <x:c r="E20" s="73" t="str">
+        <x:v>GibbsDDRM: A Partially Collapsed Gibbs Sampler for Solving Blind Inverse Problems with Denoising Diffusion Restoration</x:v>
+      </x:c>
+      <x:c r="F20" s="73" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="G20" s="1" t="str">
+      <x:c r="G20" s="73" t="str">
         <x:v>https://proceedings.mlr.press/v202/murata23a.html</x:v>
       </x:c>
-      <x:c r="H20" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I20" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J20" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K20" s="1"/>
-      <x:c r="L20" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M20" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N20" s="1" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="1" t="str">
+      <x:c r="H20" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I20" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J20" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K20" s="75"/>
+      <x:c r="L20" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Joint posterior inference for blind inverse problems. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P019).</x:v>
+      </x:c>
+      <x:c r="M20" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="84" customHeight="1">
+      <x:c r="A21" s="73" t="str">
         <x:v>S020</x:v>
       </x:c>
-      <x:c r="B21" s="39"/>
-      <x:c r="C21" s="1" t="str">
+      <x:c r="B21" s="74"/>
+      <x:c r="C21" s="73" t="str">
         <x:v>Seed evidence map (pre-systematic)</x:v>
       </x:c>
-      <x:c r="D21" s="1" t="str">
+      <x:c r="D21" s="73" t="str">
         <x:v>Targeted cornerstone search / citation chaining; mapped as P020</x:v>
       </x:c>
-      <x:c r="E21" s="1" t="str">
-        <x:v>PromptIR: Prompting for All-in-One Blind Image Restoration</x:v>
-      </x:c>
-      <x:c r="F21" s="1" t="n">
+      <x:c r="E21" s="73" t="str">
+        <x:v>PromptIR: Prompting for All-in-One Image Restoration</x:v>
+      </x:c>
+      <x:c r="F21" s="73" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="G21" s="1" t="str">
-        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a17bb69ab19f3be921f-Abstract-Conference.html</x:v>
-      </x:c>
-      <x:c r="H21" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="I21" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J21" s="1" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K21" s="1"/>
-      <x:c r="L21" s="1" t="str">
-        <x:v>Seed candidate only; requires formal database retrieval, deduplication and eligibility screening.</x:v>
-      </x:c>
-      <x:c r="M21" s="1" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="N21" s="1" t="str">
+      <x:c r="G21" s="73" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a579a0d76fd4a35d107-Abstract-Conference.html</x:v>
+      </x:c>
+      <x:c r="H21" s="73" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="I21" s="76" t="str">
+        <x:v>AI pilot: advance</x:v>
+      </x:c>
+      <x:c r="J21" s="75" t="str">
+        <x:v>Pending</x:v>
+      </x:c>
+      <x:c r="K21" s="75"/>
+      <x:c r="L21" s="75" t="str">
+        <x:v>2026-09-16 | AI only; human pending. Unknown degradation types and levels. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P020).</x:v>
+      </x:c>
+      <x:c r="M21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="N21" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
@@ -14053,7 +14157,7 @@
       <x:formula1>"No,Yes"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I2:J101">
-      <x:formula1>"Pending,Include,Exclude,Unclear"</x:formula1>
+      <x:formula1>"Pending,Include,Exclude,Unclear,AI pilot: advance,AI pilot: unclear"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K2:K101">
       <x:formula1>",Duplicate,Outside date window,Wrong modality,No reconstruction method,No mismatch/reliability relevance,Non-primary source,Insufficient technical detail,Superseded version,Other"</x:formula1>
@@ -14064,7 +14168,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbeee9c6ee3e4a82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce41f0bddc784d70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14116,7 +14220,7 @@
         <x:v>Primary question</x:v>
       </x:c>
       <x:c r="B7" s="58" t="str">
-        <x:v>How can reconstruction under compound, unknown and time-varying operator mismatch provide calibrated image/operator uncertainty, measurement-support assessment and selective abstention?</x:v>
+        <x:v>To what extent do learning-based image or video reconstruction methods remain accurate, calibrated and evidentially faithful when the true acquisition operator differs from the assumed forward model?</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="34" customHeight="1">
@@ -14159,28 +14263,28 @@
         <x:v>IEEE Xplore; Scopus; Web of Science; ScienceDirect; SpringerLink; ACM DL; CVF; NeurIPS; ICLR/OpenReview; ICML/PMLR; SIAM; Optica; SPIE; arXiv for recent work</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="34" customHeight="1">
+    <x:row r="13" ht="78" customHeight="1">
       <x:c r="A13" s="57" t="str">
         <x:v>Core query A</x:v>
       </x:c>
       <x:c r="B13" s="58" t="str">
-        <x:v>("forward model mismatch" OR "operator mismatch" OR "model uncertainty" OR uncalibrated OR blind) AND ("image reconstruction" OR "inverse problems") AND (deep OR neural OR diffusion OR unrolled)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="34" customHeight="1">
+        <x:v>("forward model mismatch" OR "operator mismatch" OR "model uncertainty" OR miscalibrat* OR "unknown operator" OR "blind inverse") AND ("image reconstruction" OR "video reconstruction" OR "inverse imaging" OR deblurring OR restoration)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="78" customHeight="1">
       <x:c r="A14" s="57" t="str">
         <x:v>Core query B</x:v>
       </x:c>
       <x:c r="B14" s="58" t="str">
-        <x:v>(deblurring OR restoration OR super-resolution OR surveillance OR CCTV) AND (compound OR mixed OR unknown OR time-varying) AND degradation AND (uncertainty OR calibration OR hallucination OR reliability)</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="34" customHeight="1">
+        <x:v>(restoration OR deblurring OR super-resolution OR surveillance OR CCTV) AND (compound OR composite OR mixed OR unknown OR "time-varying") AND (degradation OR operator OR acquisition) AND (uncertainty OR calibration OR hallucination OR reliability OR robustness)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="78" customHeight="1">
       <x:c r="A15" s="57" t="str">
         <x:v>Core query C</x:v>
       </x:c>
       <x:c r="B15" s="58" t="str">
-        <x:v>("inverse problems" AND hallucination) OR ("image reconstruction" AND (abstention OR "selective prediction" OR "risk coverage" OR conformal))</x:v>
+        <x:v>("inverse problem" OR "image reconstruction") AND (hallucination OR "measurement support" OR "null space" OR calibration OR "uncertainty quantification" OR abstention OR "selective prediction" OR "risk coverage" OR conformal OR OOD)</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="34" customHeight="1">
@@ -14207,15 +14311,15 @@
         <x:v>Surveys used only for discovery; non-imaging inverse problems without transferable method; enhancement without evaluation; non-primary commentary; duplicate/superseded manuscripts</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="34" customHeight="1">
+    <x:row r="19" ht="62" customHeight="1">
       <x:c r="A19" s="57" t="str">
         <x:v>Target corpus</x:v>
       </x:c>
       <x:c r="B19" s="58" t="str">
-        <x:v>Approximately 60–100 full-text screened papers after citation chaining</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="34" customHeight="1">
+        <x:v>Planning estimate only: 60–100 full-text papers; not an eligibility quota. Include all studies meeting the protocol.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="62" customHeight="1">
       <x:c r="A20" s="57" t="str">
         <x:v>Novelty rule</x:v>
       </x:c>
@@ -14223,28 +14327,28 @@
         <x:v>No novelty claim until nearest competitors are fully coded and the go/no-go pilot is completed</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="34" customHeight="1">
+    <x:row r="21" ht="62" customHeight="1">
       <x:c r="A21" s="57" t="str">
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B21" s="58" t="str">
-        <x:v>1.1 — seed corpus transferred to PRISMA screening log on 16 September 2026</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="34" customHeight="1">
+        <x:v>0.3 — working draft amended 16 September 2026; not registered. Corrects inconsistent workbook 1.1 label.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="62" customHeight="1">
       <x:c r="A22" s="59" t="str">
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Protocol prepared; formal database searches, deduplication and eligibility screening have not yet started</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
+        <x:v>20 AI pilot recommendations (18 advance, 2 unclear); all human adjudication pending. Formal database searches and two-stage eligibility are not completed; formal inclusion/exclusion counts remain zero.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="62" customHeight="1">
       <x:c r="A23" t="str">
         <x:v>Seed-corpus rule</x:v>
       </x:c>
-      <x:c r="B23" t="str">
-        <x:v>The 90 coded papers are candidate records for gap mapping. They become formally included studies only after the documented PRISMA workflow</x:v>
+      <x:c r="B23" s="78" t="str">
+        <x:v>90 seed candidates, not 90 included studies. AI pilot decisions are preliminary; missing abstracts are flagged, not excluded. See screening/pilot_01.json and docs/systematic_review_protocol.md.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14443,15 +14547,15 @@
         <x:v>Explicit selective prediction, reject option or reliability threshold</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="96" customHeight="1">
       <x:c r="A17" s="63" t="str">
         <x:v>Evidence status</x:v>
       </x:c>
       <x:c r="B17" s="63" t="str">
-        <x:v>Controlled label</x:v>
+        <x:v>Abstract inspected; full-text pending / Title/project checked; abstract pending / Incomplete evidence; retrieval pending / legacy labels</x:v>
       </x:c>
       <x:c r="C17" s="63" t="str">
-        <x:v>Whether metadata, abstract or full text has been verified</x:v>
+        <x:v>Describes evidence actually accessed, not study quality. Legacy labels outside the pilot remain unverified here. All feature codes require full-text verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -14490,7 +14594,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9c4067465b5f4679"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R01f03661b88c49b9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record twelve full-text eligibility assessments and verified feature corrections
Complete 12 AI assessments (11 include recommendations, 1 exclude), leaving 78 pending. Record criterion evidence, inspected versions and feature corrections; distinguish AI progress from final formal inclusion. Preserve historic triage, workbook objects and all 90 seed references.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc429111c0f224d58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R0772bb5297f740b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R9d32156eaeca473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R1534f2da931349eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R639a1752ee9840e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5b9530e2fa5241c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R2f9b05130e024d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rb39261c198934970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R2d9a3a8120f14e3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R275b7c51bff74149"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="dd/mm/yyyy"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -73,8 +73,13 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="14">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -139,6 +144,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFCE4D6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -237,7 +252,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="95">
+  <x:cellXfs count="99">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -443,6 +458,14 @@
     <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -674,7 +697,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0a79cb539ee347fc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1dd3899bd3e7437e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1051,7 +1074,7 @@
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
       <x:c r="A10" s="16" t="str">
-        <x:v>Full texts assessed</x:v>
+        <x:v>Formal full-text assessments</x:v>
       </x:c>
       <x:c r="B10" s="17" t="n">
         <x:v>0</x:v>
@@ -1115,6 +1138,15 @@
       <x:c r="E14" s="70" t="n">
         <x:f>B6-E11</x:f>
         <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="D15" s="98" t="str">
+        <x:v>AI full-text assessed</x:v>
+      </x:c>
+      <x:c r="E15" s="98" t="n">
+        <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1131,7 +1163,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>PRISM studies image/kernel uncertainty; PnP sampling already has mismatch sensitivity analysis; No-Harm proposes certificate-based fallback; self-supervised conformal work calibrates without clean targets. Evidence and limits: screening/pilot_03_report.md.</x:v>
+        <x:v>PRISM: joint image/kernel uncertainty. No-Harm: conditional certificates and fallback. PnP: posterior mismatch bounds. nanoCT: operator error plus image variance. SURE: self-supervised calibration under stated assumptions. Details: screening/full_text_01_report.md.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1185,7 +1217,8 @@
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
-        <x:v>Initial triage complete: 90/90 seed records, 82 advance and 8 unclear; 0 untriaged. All human adjudication and complete formal full-text eligibility remain pending. No novelty is established. Feature codes require full-text verification.</x:v>
+        <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 12/90 (11 include, 1 exclude); 78 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1280,7 +1313,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae17d982341a4c8b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa123bf24dbf4235"/>
 </x:worksheet>
 </file>
 
@@ -1913,102 +1946,102 @@
         <x:v>Nearest early mismatch competitor | AI pilot 2026-09-16; advance to full text. Explicit forward-model mismatch compensation. Human adjudication and full-text coding pending. Evidence: https://www.eee.hku.hk/optima/pub/journal/2109_TCI.pdf</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="240" customHeight="1">
-      <x:c r="A7" s="7" t="str">
+    <x:row r="7" ht="176" customHeight="1">
+      <x:c r="A7" s="85" t="str">
         <x:v>P006</x:v>
       </x:c>
-      <x:c r="B7" s="8" t="n">
+      <x:c r="B7" s="86" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="C7" s="9" t="str">
+      <x:c r="C7" s="75" t="str">
         <x:v>Gilton et al.</x:v>
       </x:c>
-      <x:c r="D7" s="9" t="str">
+      <x:c r="D7" s="75" t="str">
         <x:v>Deep Equilibrium Architectures for Inverse Problems in Imaging</x:v>
       </x:c>
-      <x:c r="E7" s="9" t="str">
+      <x:c r="E7" s="75" t="str">
         <x:v>IEEE TCI</x:v>
       </x:c>
-      <x:c r="F7" s="9" t="str">
+      <x:c r="F7" s="75" t="str">
         <x:v>Journal</x:v>
       </x:c>
-      <x:c r="G7" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H7" s="9" t="str">
+      <x:c r="G7" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H7" s="75" t="str">
         <x:v>Generic inverse imaging</x:v>
       </x:c>
-      <x:c r="I7" s="9" t="str">
+      <x:c r="I7" s="75" t="str">
         <x:v>Computational imaging</x:v>
       </x:c>
-      <x:c r="J7" s="9" t="str">
+      <x:c r="J7" s="75" t="str">
         <x:v>Linear operator</x:v>
       </x:c>
-      <x:c r="K7" s="9" t="str">
+      <x:c r="K7" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L7" s="9" t="str">
+      <x:c r="L7" s="75" t="str">
         <x:v>None central</x:v>
       </x:c>
-      <x:c r="M7" s="9" t="str">
+      <x:c r="M7" s="75" t="str">
         <x:v>Deep equilibrium/unrolling</x:v>
       </x:c>
-      <x:c r="N7" s="9" t="str">
+      <x:c r="N7" s="75" t="str">
         <x:v>Hard/iterative</x:v>
       </x:c>
-      <x:c r="O7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S7" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="T7" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y7" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z7" s="9" t="str">
-        <x:v>Targeted full-text sections inspected</x:v>
-      </x:c>
-      <x:c r="AA7" s="9" t="str">
+      <x:c r="O7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S7" s="75" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="T7" s="75" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="U7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y7" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z7" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA7" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB7" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC7" s="9" t="str">
+      <x:c r="AB7" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC7" s="75" t="str">
         <x:v>Infinite-depth fixed-point physics-aware reconstruction</x:v>
       </x:c>
-      <x:c r="AD7" s="9" t="str">
+      <x:c r="AD7" s="75" t="str">
         <x:v>Assumes usable known operator; mismatch reliability not central</x:v>
       </x:c>
-      <x:c r="AE7" s="9" t="str">
+      <x:c r="AE7" s="75" t="str">
         <x:v>https://doi.org/10.1109/TCI.2021.3118944</x:v>
       </x:c>
       <x:c r="AF7" s="75" t="str">
-        <x:v>Architecture baseline | AI pilot 2026-09-16; unclear. Not established from abstract. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2102.07944 | Batch 02 revisit 2026-09-16: The inspected experiments cover Gaussian deblurring, compressed sensing and MRI. A criterion-3 mismatch/reliability study is still not established. Retain unclear for human scope adjudication; this is not an exclusion or full-text eligibility decision. Source: https://arxiv.org/pdf/2102.07944 | Batch 03 revisit 2026-09-16: Known-operator reconstruction is established; criterion-3 relevance still needs adjudication. Prior selected-section inspection is not a complete eligibility review. Source: https://arxiv.org/abs/2102.07944</x:v>
+        <x:v>Architecture baseline | AI pilot 2026-09-16; unclear. Not established from abstract. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2102.07944 | Batch 02 revisit 2026-09-16: The inspected experiments cover Gaussian deblurring, compressed sensing and MRI. A criterion-3 mismatch/reliability study is still not established. Retain unclear for human scope adjudication; this is not an exclusion or full-text eligibility decision. Source: https://arxiv.org/pdf/2102.07944 | Batch 03 revisit 2026-09-16: Known-operator reconstruction is established; criterion-3 relevance still needs adjudication. Prior selected-section inspection is not a complete eligibility review. Source: https://arxiv.org/abs/2102.07944 | AI full-text 2026-09-16: include; human pending. Verified fields: S. Evidence/version/read extent: screening/full_text_01.json (P006). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -5049,7 +5082,7 @@
         <x:v>Critical novelty threat and component | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author abstract and targeted full-text definitions, Remark 3.4, Proposition 3.5 and Algorithm 2. Feature codes remain provisional. What operational guarantee survives approximate sampling and an estimated acquisition model? The seed abstention code is not established by these inspected sections. Evidence: https://arxiv.org/html/2605.13146v1</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="112" customHeight="1">
+    <x:row r="39" ht="176" customHeight="1">
       <x:c r="A39" s="85" t="str">
         <x:v>P038</x:v>
       </x:c>
@@ -5105,7 +5138,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="S39" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="T39" s="75" t="str">
         <x:v>No</x:v>
@@ -5117,7 +5150,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="W39" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="X39" s="75" t="str">
         <x:v>No</x:v>
@@ -5126,7 +5159,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z39" s="75" t="str">
-        <x:v>Targeted full-text sections inspected</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA39" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -5144,7 +5177,7 @@
         <x:v>https://doi.org/10.1109/ICASSP55912.2026.11462668</x:v>
       </x:c>
       <x:c r="AF39" s="75" t="str">
-        <x:v>Top adversary; authors Yuanyun Hu, Evan Bell, Guijin Wang and Yu Sun | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and targeted full-text sections 2–3, Tables 1–3 and Figures 3–4; conference lineage retained. Feature codes remain provisional. Does the final conference report test interval reliability under unseen operator families? The inspected experiment establishes neither arbitrary-shift coverage nor a deployed selective-output mechanism. Evidence: https://arxiv.org/html/2509.16106v1</x:v>
+        <x:v>Top adversary; authors Yuanyun Hu, Evan Bell, Guijin Wang and Yu Sun | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and targeted full-text sections 2–3, Tables 1–3 and Figures 3–4; conference lineage retained. Feature codes remain provisional. Does the final conference report test interval reliability under unseen operator families? The inspected experiment establishes neither arbitrary-shift coverage nor a deployed selective-output mechanism. Evidence: https://arxiv.org/html/2509.16106v1 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_01.json (P038). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="112" customHeight="1">
@@ -5494,13 +5527,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="R43" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="S43" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T43" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U43" s="75" t="str">
         <x:v>No</x:v>
@@ -5509,7 +5542,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="W43" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="X43" s="75" t="str">
         <x:v>Yes</x:v>
@@ -5518,7 +5551,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z43" s="75" t="str">
-        <x:v>Targeted full-text sections inspected</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA43" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -5536,7 +5569,7 @@
         <x:v>https://arxiv.org/abs/2606.07153</x:v>
       </x:c>
       <x:c r="AF43" s="75" t="str">
-        <x:v>Critical abstention threat; preprint credibility and proofs require full review | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Author preprint abstract and targeted discussion/limitations, sections 9–10. Feature codes remain provisional. Verify the stability constants, admissible class and operational radius. Certificate dominance does not imply lower actual error than the baseline; test whether the guarantee survives an uncertain or misspecified observation operator. Evidence: https://arxiv.org/html/2606.07153v1</x:v>
+        <x:v>Critical abstention threat; preprint credibility and proofs require full review | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Author preprint abstract and targeted discussion/limitations, sections 9–10. Feature codes remain provisional. Verify the stability constants, admissible class and operational radius. Certificate dominance does not imply lower actual error than the baseline; test whether the guarantee survives an uncertain or misspecified observation operator. Evidence: https://arxiv.org/html/2606.07153v1 | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_01.json (P042). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="176" customHeight="1">
@@ -6082,10 +6115,10 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="R49" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="S49" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T49" s="75" t="str">
         <x:v>No</x:v>
@@ -6106,7 +6139,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z49" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA49" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6124,7 +6157,7 @@
         <x:v>https://proceedings.iclr.cc/paper_files/paper/2024/hash/2a2874875861f6a6436b505dd77683d1-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF49" s="75" t="str">
-        <x:v>Core posterior-mismatch theory | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official ICLR proceedings abstract. Feature codes remain provisional. Which model assumptions support the posterior-distance bound? Does it imply calibrated intervals or selective-output reliability under structured acquisition mismatch? Evidence: https://proceedings.iclr.cc/paper_files/paper/2024/hash/2a2874875861f6a6436b505dd77683d1-Abstract-Conference.html</x:v>
+        <x:v>Core posterior-mismatch theory | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official ICLR proceedings abstract. Feature codes remain provisional. Which model assumptions support the posterior-distance bound? Does it imply calibrated intervals or selective-output reliability under structured acquisition mismatch? Evidence: https://proceedings.iclr.cc/paper_files/paper/2024/hash/2a2874875861f6a6436b505dd77683d1-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_01.json (P048). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="176" customHeight="1">
@@ -7282,7 +7315,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z61" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA61" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7300,7 +7333,7 @@
         <x:v>https://doi.org/10.33851/JMIS.2025.12.3.81</x:v>
       </x:c>
       <x:c r="AF61" s="75" t="str">
-        <x:v>Direct CCTV stress-test seed | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Publisher abstract and opening full-text context. Feature codes remain provisional. Does this dataset provide a reconstruction-relevant evaluation under criterion 2/4, or belong only in contextual background? Real reference CCTV frames are not automatically clean scene truth. Evidence: https://www.jmis.org/archive/view_article?pid=jmis-12-3-81</x:v>
+        <x:v>Direct CCTV stress-test seed | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Publisher abstract and opening full-text context. Feature codes remain provisional. Does this dataset provide a reconstruction-relevant evaluation under criterion 2/4, or belong only in contextual background? Real reference CCTV frames are not automatically clean scene truth. Evidence: https://www.jmis.org/archive/view_article?pid=jmis-12-3-81 | AI full-text 2026-09-16: exclude; human pending. Verified fields: T, U. Evidence/version/read extent: screening/full_text_01.json (P060). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="62" ht="176" customHeight="1">
@@ -7641,19 +7674,19 @@
         <x:v>Implicit/probabilistic</x:v>
       </x:c>
       <x:c r="O65" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="P65" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Q65" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="R65" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="S65" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T65" s="75" t="str">
         <x:v>No</x:v>
@@ -7662,7 +7695,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="V65" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="W65" s="75" t="str">
         <x:v>No</x:v>
@@ -7674,7 +7707,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z65" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA65" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7692,7 +7725,7 @@
         <x:v>https://doi.org/10.1109/TCI.2024.3380319</x:v>
       </x:c>
       <x:c r="AF65" s="75" t="str">
-        <x:v>Closest inexact-operator plus image-UQ study | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and existing journal lineage. Feature codes remain provisional. Identify the stochastic operator model, image uncertainty measure and calibration evidence. Mismatch plus uncertainty is already studied; wrong-family reliability needs specific verification. Evidence: https://arxiv.org/abs/2307.10474</x:v>
+        <x:v>Closest inexact-operator plus image-UQ study | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and existing journal lineage. Feature codes remain provisional. Identify the stochastic operator model, image uncertainty measure and calibration evidence. Mismatch plus uncertainty is already studied; wrong-family reliability needs specific verification. Evidence: https://arxiv.org/abs/2307.10474 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, V. Evidence/version/read extent: screening/full_text_01.json (P064). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="66" ht="176" customHeight="1">
@@ -7849,10 +7882,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S67" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="T67" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U67" s="75" t="str">
         <x:v>No</x:v>
@@ -7870,7 +7903,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z67" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA67" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7888,7 +7921,7 @@
         <x:v>https://doi.org/10.1007/978-3-031-92366-1_9</x:v>
       </x:c>
       <x:c r="AF67" s="75" t="str">
-        <x:v>Useful calibration method | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official Springer proceedings abstract. Feature codes remain provisional. Which noise and operator assumptions make the risk estimate valid? Check whether the calibration remains valid when those assumptions are wrong. Ground-truth-free calibration alone is not a new contribution. Evidence: https://link.springer.com/chapter/10.1007/978-3-031-92366-1_9</x:v>
+        <x:v>Useful calibration method | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official Springer proceedings abstract. Feature codes remain provisional. Which noise and operator assumptions make the risk estimate valid? Check whether the calibration remains valid when those assumptions are wrong. Ground-truth-free calibration alone is not a new contribution. Evidence: https://link.springer.com/chapter/10.1007/978-3-031-92366-1_9 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_01.json (P066). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="68" ht="176" customHeight="1">
@@ -8440,10 +8473,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T73" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U73" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="V73" s="75" t="str">
         <x:v>No</x:v>
@@ -8458,7 +8491,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z73" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA73" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8476,7 +8509,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/file/1c364d98a5cdc426fd8c76fbb2c10e34-Paper-Conference.pdf</x:v>
       </x:c>
       <x:c r="AF73" s="75" t="str">
-        <x:v>Universal prompting baseline | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Official PDF abstract/opening page; a text search for unknown yielded no match. Feature codes remain provisional. Are task models trained separately, and do experiments explicitly address any criterion-3 condition? A missing keyword is not an exclusion reason. Evidence: https://proceedings.neurips.cc/paper_files/paper/2023/file/1c364d98a5cdc426fd8c76fbb2c10e34-Paper-Conference.pdf</x:v>
+        <x:v>Universal prompting baseline | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Official PDF abstract/opening page; a text search for unknown yielded no match. Feature codes remain provisional. Are task models trained separately, and do experiments explicitly address any criterion-3 condition? A missing keyword is not an exclusion reason. Evidence: https://proceedings.neurips.cc/paper_files/paper/2023/file/1c364d98a5cdc426fd8c76fbb2c10e34-Paper-Conference.pdf | AI full-text 2026-09-16: include; human pending. Verified fields: S, T, U. Evidence/version/read extent: screening/full_text_01.json (P072). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="176" customHeight="1">
@@ -9420,7 +9453,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="T83" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U83" s="75" t="str">
         <x:v>No</x:v>
@@ -9438,7 +9471,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z83" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA83" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9456,7 +9489,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/86655bc516148e311bcfcf88f1744de7-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF83" s="75" t="str">
-        <x:v>General inverse-solver baseline | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Does the full paper explicitly study operator/prior misspecification, uncertainty reliability or measurement-supported detail? Otherwise retain as a solver baseline outside the primary synthesis. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/86655bc516148e311bcfcf88f1744de7-Abstract-Conference.html</x:v>
+        <x:v>General inverse-solver baseline | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Does the full paper explicitly study operator/prior misspecification, uncertainty reliability or measurement-supported detail? Otherwise retain as a solver baseline outside the primary synthesis. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/86655bc516148e311bcfcf88f1744de7-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T. Evidence/version/read extent: screening/full_text_01.json (P082). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="176" customHeight="1">
@@ -9604,7 +9637,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="P85" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Q85" s="75" t="str">
         <x:v>No</x:v>
@@ -9616,7 +9649,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="T85" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U85" s="75" t="str">
         <x:v>No</x:v>
@@ -9634,7 +9667,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z85" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA85" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9652,7 +9685,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/54fa8255cdf30736ecad38e842725e7f-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF85" s="75" t="str">
-        <x:v>Data-consistency baseline | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Does the imaging evaluation explicitly meet criterion 3? Noise handling or multiple inverse operators alone does not establish blind reconstruction or uncertainty calibration. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/54fa8255cdf30736ecad38e842725e7f-Abstract-Conference.html</x:v>
+        <x:v>Data-consistency baseline | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Does the imaging evaluation explicitly meet criterion 3? Noise handling or multiple inverse operators alone does not establish blind reconstruction or uncertainty calibration. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/54fa8255cdf30736ecad38e842725e7f-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T. Evidence/version/read extent: screening/full_text_01.json (P084). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="86" ht="176" customHeight="1">
@@ -9806,13 +9839,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="R87" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="S87" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="T87" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U87" s="75" t="str">
         <x:v>No</x:v>
@@ -9821,7 +9854,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="W87" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="X87" s="75" t="str">
         <x:v>No</x:v>
@@ -9830,7 +9863,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z87" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA87" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9848,7 +9881,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/c7ae6e9659f0c99582c2e8214ba0b413-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF87" s="75" t="str">
-        <x:v>Strong data-consistent generative comparator | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Does the paper assess measurement-supported detail beyond its data-fidelity objective, or study operator shift, blind inference or uncertainty reliability? Evidence: https://proceedings.neurips.cc/paper_files/paper/2025/hash/c7ae6e9659f0c99582c2e8214ba0b413-Abstract-Conference.html</x:v>
+        <x:v>Strong data-consistent generative comparator | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Does the paper assess measurement-supported detail beyond its data-fidelity objective, or study operator shift, blind inference or uncertainty reliability? Evidence: https://proceedings.neurips.cc/paper_files/paper/2025/hash/c7ae6e9659f0c99582c2e8214ba0b413-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T, W. Evidence/version/read extent: screening/full_text_01.json (P086). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="176" customHeight="1">
@@ -9919,7 +9952,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="W88" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="X88" s="75" t="str">
         <x:v>No</x:v>
@@ -9928,7 +9961,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z88" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA88" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9946,7 +9979,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/d92d3aec6a48e93f93194503ee49f11a-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF88" s="75" t="str">
-        <x:v>Fast measurement-consistency baseline | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Is an incorrect noise/measurement model tested, or uncertainty calibrated? Residual matching under an assumed model is not itself a guarantee of trustworthy recovered detail. Evidence: https://proceedings.neurips.cc/paper_files/paper/2025/hash/d92d3aec6a48e93f93194503ee49f11a-Abstract-Conference.html</x:v>
+        <x:v>Fast measurement-consistency baseline | AI pilot 2026-09-16: AI pilot: unclear; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Is an incorrect noise/measurement model tested, or uncertainty calibrated? Residual matching under an assumed model is not itself a guarantee of trustworthy recovered detail. Evidence: https://proceedings.neurips.cc/paper_files/paper/2025/hash/d92d3aec6a48e93f93194503ee49f11a-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_01.json (P087). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="89" ht="176" customHeight="1">
@@ -10252,7 +10285,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ec32d86b7514847"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8711dc538a384c28"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10524,7 +10557,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="176" customHeight="1">
+    <x:row r="7" ht="144" customHeight="1">
       <x:c r="A7" s="73" t="str">
         <x:v>S006</x:v>
       </x:c>
@@ -10550,12 +10583,12 @@
       <x:c r="I7" s="94" t="str">
         <x:v>AI pilot: unclear</x:v>
       </x:c>
-      <x:c r="J7" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K7" s="75"/>
+      <x:c r="J7" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K7" s="75" t="str"/>
       <x:c r="L7" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Not established from abstract. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P006). Revisit: Targeted inspection of section 6 in the author PDF; unchanged unclear. See screening/pilot_02.json. Revisit: Author abstract rechecked; prior section-6 evidence retained; recommendation unchanged. See screening/pilot_03.json.</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Test-time measurement-noise variation; §6.7, Figure 8(b). Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P006).</x:v>
       </x:c>
       <x:c r="M7" s="75" t="str">
         <x:v>No</x:v>
@@ -10955,7 +10988,7 @@
       </x:c>
       <x:c r="K17" s="75"/>
       <x:c r="L17" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Cannot adjudicate from retrieved evidence. Basis: Official search snippet only; full abstract not retrieved. Full-text question and source: screening/pilot_01.json (P016). Revisit: Retrieval retry unsuccessful: OpenReview challenge and author-PDF fetch failure; unchanged unclear. See screening/pilot_02.json. Revisit: OpenReview remains challenged; author PDF fetch failed; author publication listing confirms title and venue only; recommendation unchanged. See screening/pilot_03.json.</x:v>
+        <x:v>2026-09-16 | AI only; human pending. Cannot adjudicate from retrieved evidence. Basis: Official search snippet only; full abstract not retrieved. Full-text question and source: screening/pilot_01.json (P016). Revisit: Retrieval retry unsuccessful: OpenReview challenge and author-PDF fetch failure; unchanged unclear. See screening/pilot_02.json. Revisit: OpenReview remains challenged; author PDF fetch failed; author publication listing confirms title and venue only; recommendation unchanged. See screening/pilot_03.json. Full-text 01: author PDF still fails to open; eligibility pending, not excluded. See full_text_01.json.</x:v>
       </x:c>
       <x:c r="M17" s="75" t="str">
         <x:v>No</x:v>
@@ -11804,7 +11837,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="112" customHeight="1">
+    <x:row r="39" ht="144" customHeight="1">
       <x:c r="A39" s="73" t="str">
         <x:v>S038</x:v>
       </x:c>
@@ -11827,15 +11860,15 @@
       <x:c r="H39" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I39" s="81" t="str">
+      <x:c r="I39" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J39" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K39" s="75"/>
+      <x:c r="J39" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K39" s="75" t="str"/>
       <x:c r="L39" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint image/kernel posterior sampling and uncertainty evaluation. Basis: Author preprint abstract and targeted full-text sections 2–3, Tables 1–3 and Figures 3–4; conference lineage retained. Sources and full-text question: screening/pilot_02.json (P038).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Joint image/kernel inference and uncertainty; §§2–3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P038).</x:v>
       </x:c>
       <x:c r="M39" s="75" t="str">
         <x:v>No</x:v>
@@ -11987,15 +12020,15 @@
       <x:c r="H43" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I43" s="91" t="str">
+      <x:c r="I43" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J43" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K43" s="75"/>
+      <x:c r="J43" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K43" s="75" t="str"/>
       <x:c r="L43" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Residual-based reliability certification and selective replacement of a baseline. Basis: Author preprint abstract and targeted discussion/limitations, sections 9–10. Sources and full-text question: screening/pilot_03.json (P042).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Residual uncertainty and accept/fallback rule; §§4–6. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P042).</x:v>
       </x:c>
       <x:c r="M43" s="75" t="str">
         <x:v>No</x:v>
@@ -12227,15 +12260,15 @@
       <x:c r="H49" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I49" s="91" t="str">
+      <x:c r="I49" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J49" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K49" s="75"/>
+      <x:c r="J49" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K49" s="75" t="str"/>
       <x:c r="L49" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Posterior-sampling sensitivity to measurement and prior mismatch. Basis: Complete official ICLR proceedings abstract. Sources and full-text question: screening/pilot_03.json (P048).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Denoiser and supplied measurement-operator mismatch; §§3–5. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P048).</x:v>
       </x:c>
       <x:c r="M49" s="75" t="str">
         <x:v>No</x:v>
@@ -12707,15 +12740,17 @@
       <x:c r="H61" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I61" s="92" t="str">
+      <x:c r="I61" s="94" t="str">
         <x:v>AI pilot: unclear</x:v>
       </x:c>
-      <x:c r="J61" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K61" s="75"/>
+      <x:c r="J61" s="96" t="str">
+        <x:v>AI full-text: exclude</x:v>
+      </x:c>
+      <x:c r="K61" s="75" t="str">
+        <x:v>Other</x:v>
+      </x:c>
       <x:c r="L61" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. CCTV distortion and downstream quality assessment are relevant, but criterion 2 needs adjudication. Basis: Publisher abstract and opening full-text context. Sources and full-text question: screening/pilot_03.json (P060).</x:v>
+        <x:v>2026-09-16 | AI full-text exclude; human pending. Criterion 2: IQA is central; no central inverse/restoration experiment. Retain as an ancillary dataset reference. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P060).</x:v>
       </x:c>
       <x:c r="M61" s="75" t="str">
         <x:v>No</x:v>
@@ -12867,15 +12902,15 @@
       <x:c r="H65" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I65" s="91" t="str">
+      <x:c r="I65" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J65" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K65" s="75"/>
+      <x:c r="J65" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K65" s="75" t="str"/>
       <x:c r="L65" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Deterministic/stochastic inexact operators and reconstruction uncertainty. Basis: Complete author preprint abstract and existing journal lineage. Sources and full-text question: screening/pilot_03.json (P064).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Inexact geometry, motion and image uncertainty; §§III–IV. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P064).</x:v>
       </x:c>
       <x:c r="M65" s="75" t="str">
         <x:v>No</x:v>
@@ -12947,15 +12982,15 @@
       <x:c r="H67" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I67" s="91" t="str">
+      <x:c r="I67" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J67" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K67" s="75"/>
+      <x:c r="J67" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K67" s="75" t="str"/>
       <x:c r="L67" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Self-supervised uncertainty calibration without clean ground truth. Basis: Complete official Springer proceedings abstract. Sources and full-text question: screening/pilot_03.json (P066).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Self-supervised reconstruction uncertainty calibration; §3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P066).</x:v>
       </x:c>
       <x:c r="M67" s="75" t="str">
         <x:v>No</x:v>
@@ -13187,15 +13222,15 @@
       <x:c r="H73" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I73" s="92" t="str">
+      <x:c r="I73" s="94" t="str">
         <x:v>AI pilot: unclear</x:v>
       </x:c>
-      <x:c r="J73" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K73" s="75"/>
+      <x:c r="J73" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K73" s="75" t="str"/>
       <x:c r="L73" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Degradation perception is explicit, but the qualifying mismatch/reliability setting needs verification. Basis: Official PDF abstract/opening page; a text search for unknown yielded no match. Sources and full-text question: screening/pilot_03.json (P072).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Explicit cross-dataset deblurring transfer; §4.1, Table 2. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P072).</x:v>
       </x:c>
       <x:c r="M73" s="75" t="str">
         <x:v>No</x:v>
@@ -13587,15 +13622,15 @@
       <x:c r="H83" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I83" s="92" t="str">
+      <x:c r="I83" s="94" t="str">
         <x:v>AI pilot: unclear</x:v>
       </x:c>
-      <x:c r="J83" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K83" s="75"/>
+      <x:c r="J83" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K83" s="75" t="str"/>
       <x:c r="L83" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Known differentiable inverse operators are explicit; a qualifying mismatch/reliability condition is not established by the abstract. Basis: Complete official NeurIPS abstract. Sources and full-text question: screening/pilot_03.json (P082).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Reconstruction posterior sampling and explicit prior-approximation robustness; §4, Figure 6. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P082).</x:v>
       </x:c>
       <x:c r="M83" s="75" t="str">
         <x:v>No</x:v>
@@ -13667,15 +13702,15 @@
       <x:c r="H85" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I85" s="92" t="str">
+      <x:c r="I85" s="94" t="str">
         <x:v>AI pilot: unclear</x:v>
       </x:c>
-      <x:c r="J85" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K85" s="75"/>
+      <x:c r="J85" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K85" s="75" t="str"/>
       <x:c r="L85" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Noisy inverse reconstruction is explicit, but mismatch or reliability evaluation is not established by the abstract. Basis: Complete official NeurIPS abstract. Sources and full-text question: screening/pilot_03.json (P084).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Assumed noise-level perturbation; Appendix C.2, Table 14. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P084).</x:v>
       </x:c>
       <x:c r="M85" s="75" t="str">
         <x:v>No</x:v>
@@ -13747,15 +13782,15 @@
       <x:c r="H87" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I87" s="92" t="str">
+      <x:c r="I87" s="94" t="str">
         <x:v>AI pilot: unclear</x:v>
       </x:c>
-      <x:c r="J87" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K87" s="75"/>
+      <x:c r="J87" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K87" s="75" t="str"/>
       <x:c r="L87" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Observation fidelity is explicit; a qualifying reliability or mismatch assessment requires full-text verification. Basis: Complete official NeurIPS abstract. Sources and full-text question: screening/pilot_03.json (P086).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Reconstruction variance, fidelity ablation and failure cases; §5.2–5.3, Appendix A.10. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P086).</x:v>
       </x:c>
       <x:c r="M87" s="75" t="str">
         <x:v>No</x:v>
@@ -13787,15 +13822,15 @@
       <x:c r="H88" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I88" s="92" t="str">
+      <x:c r="I88" s="94" t="str">
         <x:v>AI pilot: unclear</x:v>
       </x:c>
-      <x:c r="J88" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K88" s="75"/>
+      <x:c r="J88" s="95" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K88" s="75" t="str"/>
       <x:c r="L88" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Noisy linear data consistency is explicit; mismatch or calibrated reconstruction uncertainty is not established by the abstract. Basis: Complete official NeurIPS abstract. Sources and full-text question: screening/pilot_03.json (P087).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Explicit measurement-support assessment; §5.2, Figure 7; imprecise non-Gaussian application in §5.4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_01.json (P087).</x:v>
       </x:c>
       <x:c r="M88" s="75" t="str">
         <x:v>No</x:v>
@@ -14214,7 +14249,7 @@
       <x:formula1>"No,Yes"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="I2:J101">
-      <x:formula1>"Pending,Include,Exclude,Unclear,AI pilot: advance,AI pilot: unclear"</x:formula1>
+      <x:formula1>"Pending,Include,Exclude,Unclear,AI pilot: advance,AI pilot: unclear,AI full-text: include,AI full-text: exclude"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="K2:K101">
       <x:formula1>",Duplicate,Outside date window,Wrong modality,No reconstruction method,No mismatch/reliability relevance,Non-primary source,Insufficient technical detail,Superseded version,Other"</x:formula1>
@@ -14225,7 +14260,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49830bfdd2374cab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32a936e95b7d4686"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14389,7 +14424,7 @@
         <x:v>Version</x:v>
       </x:c>
       <x:c r="B21" s="58" t="str">
-        <x:v>0.3 — working draft amended 16 September 2026; not registered. Corrects inconsistent workbook 1.1 label.</x:v>
+        <x:v>0.4 — operational AI full-text convention, 16 September 2026; not registered. Eligibility and search window unchanged.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="62" customHeight="1">
@@ -14397,7 +14432,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>90 AI pilot recommendations (82 advance, 8 unclear); 0 seed records untriaged. Human adjudication, formal database searches and complete full-text eligibility remain pending; formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 12 (11 include, 1 exclude), 78 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14405,7 +14440,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed candidates, not 90 included studies. AI recommendations and selected passages are preliminary. Full initial pass: screening/pilot_03.json and pilot_03_report.md; earlier pilot records preserved.</x:v>
+        <x:v>90 seed records retained. Full-text progress: screening/full_text_01.json and full_text_01_report.md. AI decisions are recommendations. Evidence/version/read extent and verified feature fields are recorded per study; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14604,15 +14639,15 @@
         <x:v>Explicit selective prediction, reject option or reliability threshold</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="128" customHeight="1">
+    <x:row r="17" ht="160" customHeight="1">
       <x:c r="A17" s="63" t="str">
         <x:v>Evidence status</x:v>
       </x:c>
       <x:c r="B17" s="63" t="str">
-        <x:v>Abstract inspected; full-text pending / Targeted full-text sections inspected / Abstract and repository inspected / Title/project checked; abstract pending / Incomplete evidence; retrieval pending / legacy labels</x:v>
+        <x:v>Abstract inspected; full-text pending / Targeted full-text sections inspected / Abstract and repository inspected / Title/project checked; abstract pending / Incomplete evidence; retrieval pending / legacy labels / AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="C17" s="63" t="str">
-        <x:v>Evidence accessed, not study quality or final eligibility. Selected passages validate only named findings. Incomplete retrieval is recorded explicitly. All feature codes remain provisional; uncertainty labels alone do not establish calibrated probabilities.</x:v>
+        <x:v>Full-text eligibility assessment means sufficient evidence for criteria, not a proof/code audit. Only explicitly logged feature fields are verified; other codes remain provisional. AI include/exclude in Screening Log J requires human adjudication; Evidence Matrix AA remains the formal decision.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -14651,7 +14686,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdb17d7836f524735"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd0ba63d6bf14048"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete second AI full-text review checkpoint
Add 12 source-backed eligibility assessments and selected feature corrections. Cumulative progress is 24 assessed, 23 include recommendations, one exclude and 66 pending. Log retrieval and lineage limitations, synchronize the matrix and references, and preserve formal decisions and historical audits.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5b9530e2fa5241c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R2f9b05130e024d20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rb39261c198934970"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R2d9a3a8120f14e3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R275b7c51bff74149"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rbc6b48a56aa64102"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R16cfaa641b404f50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R540dae317b404798"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R29386213b3234865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R4692766d23d04c5c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="17">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -252,7 +257,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="99">
+  <x:cellXfs count="100">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -466,6 +471,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -697,7 +705,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1dd3899bd3e7437e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8aae59c27b7e4b35"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1146,7 +1154,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>12</x:v>
+        <x:v>24</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1163,7 +1171,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>PRISM: joint image/kernel uncertainty. No-Harm: conditional certificates and fallback. PnP: posterior mismatch bounds. nanoCT: operator error plus image variance. SURE: self-supervised calibration under stated assumptions. Details: screening/full_text_01_report.md.</x:v>
+        <x:v>New comparisons cover operator point estimation, prior shift, compound restoration and calibrated image/task uncertainty. Read assumptions and evidence limits in screening/full_text_02_report.md; prior findings remain in full_text_01. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1218,7 +1226,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 12/90 (11 include, 1 exclude); 78 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 24/90 (23 include, 1 exclude); 66 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1313,7 +1321,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa123bf24dbf4235"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8261fc5109048b2"/>
 </x:worksheet>
 </file>
 
@@ -3906,7 +3914,7 @@
         <x:v>Generative baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher chapter abstract. Feature codes remain provisional. How is fidelity measured, and are unsupported details assessed against ground truth? The former ECCV poster URL pointed to the unrelated CLOSER paper. Evidence: https://link.springer.com/chapter/10.1007/978-3-031-73202-7_25</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="112" customHeight="1">
+    <x:row r="27" ht="176" customHeight="1">
       <x:c r="A27" s="85" t="str">
         <x:v>P026</x:v>
       </x:c>
@@ -3983,7 +3991,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z27" s="75" t="str">
-        <x:v>Targeted full-text sections inspected</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA27" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4001,7 +4009,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/e635a25e49e73adc51f76aef462ff2f8-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF27" s="75" t="str">
-        <x:v>Closest video application competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Official proceedings record and targeted full-text inspection of sections 4.1–4.2. Feature codes remain provisional. Separate new degradation combinations and change intervals from genuinely unseen operator families or cameras; verify any reliability claims beyond PSNR/SSIM. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/file/e635a25e49e73adc51f76aef462ff2f8-Paper-Conference.pdf</x:v>
+        <x:v>Closest video application competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Official proceedings record and targeted full-text inspection of sections 4.1–4.2. Feature codes remain provisional. Separate new degradation combinations and change intervals from genuinely unseen operator families or cameras; verify any reliability claims beyond PSNR/SSIM. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/file/e635a25e49e73adc51f76aef462ff2f8-Paper-Conference.pdf | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_02.json (P026). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="112" customHeight="1">
@@ -4592,7 +4600,7 @@
         <x:v>Highest-priority full-text competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher title and indexed abstract excerpt only; complete abstract and full text blocked by retrieval challenges. Feature codes remain provisional. Retrieve the complete paper. Does uncertainty mean uncertain acquisition parameters, probabilistic posterior uncertainty, or both? Existing positive feature codes remain unverified. Evidence: https://www.nature.com/articles/s41377-025-01915-w | Batch 03 revisit 2026-09-16: The excerpt concerns system uncertainties such as misalignment and aberration. Positive legacy image/operator uncertainty and calibration codes are not verified probabilistic capabilities. Full text is required. Source: https://www.nature.com/articles/s41377-025-01915-w</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="112" customHeight="1">
+    <x:row r="34" ht="176" customHeight="1">
       <x:c r="A34" s="85" t="str">
         <x:v>P033</x:v>
       </x:c>
@@ -4639,7 +4647,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="P34" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Q34" s="75" t="str">
         <x:v>No</x:v>
@@ -4663,13 +4671,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="X34" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Y34" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z34" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA34" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4687,10 +4695,10 @@
         <x:v>https://arxiv.org/abs/2505.11482</x:v>
       </x:c>
       <x:c r="AF34" s="75" t="str">
-        <x:v>OOD guardrail candidate | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract. Feature codes remain provisional. Distinguish image-prior shift from acquisition-operator shift; identify the detection unit, assumptions and validated thresholds. Evidence: https://arxiv.org/abs/2505.11482</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35" ht="112" customHeight="1">
+        <x:v>OOD guardrail candidate | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract. Feature codes remain provisional. Distinguish image-prior shift from acquisition-operator shift; identify the detection unit, assumptions and validated thresholds. Evidence: https://arxiv.org/abs/2505.11482 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, X. Evidence/version/read extent: screening/full_text_02.json (P033). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="176" customHeight="1">
       <x:c r="A35" s="85" t="str">
         <x:v>P034</x:v>
       </x:c>
@@ -4761,13 +4769,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="X35" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Y35" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z35" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA35" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4785,7 +4793,7 @@
         <x:v>https://arxiv.org/abs/2510.10947</x:v>
       </x:c>
       <x:c r="AF35" s="75" t="str">
-        <x:v>Failure-detection candidate | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; final conference metadata still pending. Feature codes remain provisional. Does it generalize to natural images and unseen acquisition families? Calibration-free estimation is not a coverage guarantee. Resolve the CAMSAP lineage before locking metadata. Evidence: https://arxiv.org/abs/2510.10947</x:v>
+        <x:v>Failure-detection candidate | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; final conference metadata still pending. Feature codes remain provisional. Does it generalize to natural images and unseen acquisition families? Calibration-free estimation is not a coverage guarantee. Resolve the CAMSAP lineage before locking metadata. Evidence: https://arxiv.org/abs/2510.10947 | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_02.json (P034). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="36" ht="112" customHeight="1">
@@ -4886,7 +4894,7 @@
         <x:v>Highest-priority mismatch competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional abstract and complete proceedings metadata. Feature codes remain provisional. Can a flexible residual absorb noise or unsupported image detail? Extract identifiability constraints, optimization and held-out mismatch tests. Evidence: https://pure.kaist.ac.kr/en/publications/mitigating-forward-model-mismatch-in-inverse-problems-via-learned/</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="112" customHeight="1">
+    <x:row r="37" ht="176" customHeight="1">
       <x:c r="A37" s="85" t="str">
         <x:v>P036</x:v>
       </x:c>
@@ -4945,25 +4953,25 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T37" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="U37" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V37" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="W37" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="X37" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Y37" s="75" t="str">
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="Z37" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA37" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4981,10 +4989,10 @@
         <x:v>https://arxiv.org/abs/2603.04538</x:v>
       </x:c>
       <x:c r="AF37" s="75" t="str">
-        <x:v>Highest-priority benchmark competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract. Feature codes remain provisional. Inspect operator access, mismatch generation, data splits and released resources. Acquisition calibration must not be coded automatically as uncertainty calibration. Evidence: https://arxiv.org/abs/2603.04538</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38" ht="112" customHeight="1">
+        <x:v>Highest-priority benchmark competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract. Feature codes remain provisional. Inspect operator access, mismatch generation, data splits and released resources. Acquisition calibration must not be coded automatically as uncertainty calibration. Evidence: https://arxiv.org/abs/2603.04538 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_02.json (P036). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="176" customHeight="1">
       <x:c r="A38" s="85" t="str">
         <x:v>P037</x:v>
       </x:c>
@@ -5034,10 +5042,10 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="Q38" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="R38" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="S38" s="75" t="str">
         <x:v>Yes</x:v>
@@ -5055,13 +5063,13 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="X38" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Y38" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z38" s="75" t="str">
-        <x:v>Targeted full-text sections inspected</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA38" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -5079,7 +5087,7 @@
         <x:v>https://arxiv.org/abs/2605.13146</x:v>
       </x:c>
       <x:c r="AF38" s="75" t="str">
-        <x:v>Critical novelty threat and component | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author abstract and targeted full-text definitions, Remark 3.4, Proposition 3.5 and Algorithm 2. Feature codes remain provisional. What operational guarantee survives approximate sampling and an estimated acquisition model? The seed abstention code is not established by these inspected sections. Evidence: https://arxiv.org/html/2605.13146v1</x:v>
+        <x:v>Critical novelty threat and component | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author abstract and targeted full-text definitions, Remark 3.4, Proposition 3.5 and Algorithm 2. Feature codes remain provisional. What operational guarantee survives approximate sampling and an estimated acquisition model? The seed abstention code is not established by these inspected sections. Evidence: https://arxiv.org/html/2605.13146v1 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, W, X. Evidence/version/read extent: screening/full_text_02.json (P037). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="176" customHeight="1">
@@ -5180,7 +5188,7 @@
         <x:v>Top adversary; authors Yuanyun Hu, Evan Bell, Guijin Wang and Yu Sun | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and targeted full-text sections 2–3, Tables 1–3 and Figures 3–4; conference lineage retained. Feature codes remain provisional. Does the final conference report test interval reliability under unseen operator families? The inspected experiment establishes neither arbitrary-shift coverage nor a deployed selective-output mechanism. Evidence: https://arxiv.org/html/2509.16106v1 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_01.json (P038). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="112" customHeight="1">
+    <x:row r="40" ht="176" customHeight="1">
       <x:c r="A40" s="85" t="str">
         <x:v>P039</x:v>
       </x:c>
@@ -5239,7 +5247,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T40" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U40" s="75" t="str">
         <x:v>Yes</x:v>
@@ -5257,7 +5265,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z40" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA40" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -5275,7 +5283,7 @@
         <x:v>https://doi.org/10.1016/j.cviu.2026.104795</x:v>
       </x:c>
       <x:c r="AF40" s="75" t="str">
-        <x:v>Recent all-in-one competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and publisher journal metadata. Feature codes remain provisional. Which distortions are truly held out, and are uncertainty, temporal behavior or selective risk assessed? Composite/OOD restoration alone is an occupied direction. Evidence: https://arxiv.org/abs/2411.18412</x:v>
+        <x:v>Recent all-in-one competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and publisher journal metadata. Feature codes remain provisional. Which distortions are truly held out, and are uncertainty, temporal behavior or selective risk assessed? Composite/OOD restoration alone is an occupied direction. Evidence: https://arxiv.org/abs/2411.18412 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_02.json (P039). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="112" customHeight="1">
@@ -5845,7 +5853,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z46" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA46" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -5863,7 +5871,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/f810c2ba07bae78dfe9d25c5d40c5536-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF46" s="75" t="str">
-        <x:v>Nearest principled PnP competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS proceedings abstract. Feature codes remain provisional. Extract the convergence assumptions and distinguish stationary-point analysis from statistical operator uncertainty or robustness to an incorrect operator family. Evidence: https://proceedings.neurips.cc/paper_files/paper/2023/hash/f810c2ba07bae78dfe9d25c5d40c5536-Abstract-Conference.html</x:v>
+        <x:v>Nearest principled PnP competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS proceedings abstract. Feature codes remain provisional. Extract the convergence assumptions and distinguish stationary-point analysis from statistical operator uncertainty or robustness to an incorrect operator family. Evidence: https://proceedings.neurips.cc/paper_files/paper/2023/hash/f810c2ba07bae78dfe9d25c5d40c5536-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, X. Evidence/version/read extent: screening/full_text_02.json (P045). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="47" ht="176" customHeight="1">
@@ -6008,19 +6016,19 @@
         <x:v>Hard/differentiable</x:v>
       </x:c>
       <x:c r="O48" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="P48" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q48" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R48" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S48" s="75" t="str">
         <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="P48" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q48" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R48" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S48" s="75" t="str">
-        <x:v>Yes</x:v>
       </x:c>
       <x:c r="T48" s="75" t="str">
         <x:v>Partial</x:v>
@@ -6041,7 +6049,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z48" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA48" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6059,7 +6067,7 @@
         <x:v>https://openreview.net/forum?id=XHEhjDxPDl</x:v>
       </x:c>
       <x:c r="AF48" s="75" t="str">
-        <x:v>General mismatch-correction competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; OpenReview access challenged. Feature codes remain provisional. What prevents the correction from absorbing image structure or measurement noise, and which mismatch families and convergence assumptions are tested? Evidence: https://arxiv.org/abs/2403.04847</x:v>
+        <x:v>General mismatch-correction competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; OpenReview access challenged. Feature codes remain provisional. What prevents the correction from absorbing image structure or measurement noise, and which mismatch families and convergence assumptions are tested? Evidence: https://arxiv.org/abs/2403.04847 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, X. Evidence/version/read extent: screening/full_text_02.json (P047). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="176" customHeight="1">
@@ -7493,7 +7501,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="T63" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U63" s="75" t="str">
         <x:v>No</x:v>
@@ -7511,7 +7519,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z63" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA63" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7529,7 +7537,7 @@
         <x:v>https://proceedings.mlr.press/v202/teneggi23a.html</x:v>
       </x:c>
       <x:c r="AF63" s="75" t="str">
-        <x:v>Strong conformal-risk component | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official PMLR abstract. Feature codes remain provisional. Extract the risk unit, calibration assumptions and coverage statement; check whether any guarantee addresses changing or misspecified operators. Evidence: https://proceedings.mlr.press/v202/teneggi23a.html</x:v>
+        <x:v>Strong conformal-risk component | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official PMLR abstract. Feature codes remain provisional. Extract the risk unit, calibration assumptions and coverage statement; check whether any guarantee addresses changing or misspecified operators. Evidence: https://proceedings.mlr.press/v202/teneggi23a.html | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_02.json (P062). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="64" ht="176" customHeight="1">
@@ -7591,7 +7599,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="T64" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="U64" s="75" t="str">
         <x:v>No</x:v>
@@ -7609,7 +7617,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z64" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA64" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7627,7 +7635,7 @@
         <x:v>https://doi.org/10.1007/978-3-031-73027-6_11</x:v>
       </x:c>
       <x:c r="AF64" s="75" t="str">
-        <x:v>Task-level reliability comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and existing ECCV lineage. Feature codes remain provisional. Distinguish stopping acquisition from abstaining on reconstructed content. Verify exchangeability and whether task-specific coverage survives operator shift. Evidence: https://arxiv.org/abs/2405.18527</x:v>
+        <x:v>Task-level reliability comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and existing ECCV lineage. Feature codes remain provisional. Distinguish stopping acquisition from abstaining on reconstructed content. Verify exchangeability and whether task-specific coverage survives operator shift. Evidence: https://arxiv.org/abs/2405.18527 | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_02.json (P063). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="65" ht="176" customHeight="1">
@@ -7787,7 +7795,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="T66" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U66" s="75" t="str">
         <x:v>No</x:v>
@@ -7805,7 +7813,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z66" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA66" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7823,7 +7831,7 @@
         <x:v>https://doi.org/10.1109/TCI.2025.3649389</x:v>
       </x:c>
       <x:c r="AF66" s="75" t="str">
-        <x:v>Strongest calibrated image-UQ competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and existing journal lineage. Feature codes remain provisional. Aleatoric and epistemic components do not automatically mean image and operator posteriors. Extract the latent variables, calibration target and operator-shift tests. Evidence: https://arxiv.org/abs/2504.07696</x:v>
+        <x:v>Strongest calibrated image-UQ competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and existing journal lineage. Feature codes remain provisional. Aleatoric and epistemic components do not automatically mean image and operator posteriors. Extract the latent variables, calibration target and operator-shift tests. Evidence: https://arxiv.org/abs/2504.07696 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_02.json (P065). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="67" ht="176" customHeight="1">
@@ -8001,7 +8009,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z68" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA68" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8019,7 +8027,7 @@
         <x:v>https://arxiv.org/abs/2507.14760</x:v>
       </x:c>
       <x:c r="AF68" s="75" t="str">
-        <x:v>Preprint reliability threat | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Separate pixel-marginal from conditional or whole-image coverage. Does elevated uncertainty detect unsupported details reliably under operator shift, rather than in selected examples? Evidence: https://arxiv.org/abs/2507.14760</x:v>
+        <x:v>Preprint reliability threat | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Separate pixel-marginal from conditional or whole-image coverage. Does elevated uncertainty detect unsupported details reliably under operator shift, rather than in selected examples? Evidence: https://arxiv.org/abs/2507.14760 | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_02.json (P067). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="176" customHeight="1">
@@ -10285,7 +10293,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8711dc538a384c28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3d8269d76a2409b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11357,7 +11365,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="112" customHeight="1">
+    <x:row r="27" ht="144" customHeight="1">
       <x:c r="A27" s="73" t="str">
         <x:v>S026</x:v>
       </x:c>
@@ -11380,15 +11388,15 @@
       <x:c r="H27" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I27" s="81" t="str">
+      <x:c r="I27" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J27" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K27" s="75"/>
+      <x:c r="J27" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K27" s="75" t="str"/>
       <x:c r="L27" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Compound, unknown and time-varying video degradation. Basis: Official proceedings record and targeted full-text inspection of sections 4.1–4.2. Sources and full-text question: screening/pilot_02.json (P026).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Compound and time-varying acquisition degradation; §§4.1–4.2. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P026).</x:v>
       </x:c>
       <x:c r="M27" s="75" t="str">
         <x:v>No</x:v>
@@ -11637,7 +11645,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="112" customHeight="1">
+    <x:row r="34" ht="144" customHeight="1">
       <x:c r="A34" s="73" t="str">
         <x:v>S033</x:v>
       </x:c>
@@ -11660,15 +11668,15 @@
       <x:c r="H34" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I34" s="81" t="str">
+      <x:c r="I34" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J34" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K34" s="75"/>
+      <x:c r="J34" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K34" s="75" t="str"/>
       <x:c r="L34" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Distribution-shift detection in inverse problems. Basis: Author preprint abstract. Sources and full-text question: screening/pilot_02.json (P033).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Distribution-shift detection using incomplete observations; §§2–3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P033).</x:v>
       </x:c>
       <x:c r="M34" s="75" t="str">
         <x:v>No</x:v>
@@ -11677,7 +11685,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="112" customHeight="1">
+    <x:row r="35" ht="144" customHeight="1">
       <x:c r="A35" s="73" t="str">
         <x:v>S034</x:v>
       </x:c>
@@ -11700,15 +11708,15 @@
       <x:c r="H35" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I35" s="81" t="str">
+      <x:c r="I35" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J35" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K35" s="75"/>
+      <x:c r="J35" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K35" s="75" t="str"/>
       <x:c r="L35" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Instance-level distribution-shift uncertainty. Basis: Author preprint abstract; final conference metadata still pending. Sources and full-text question: screening/pilot_02.json (P034).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Prior-distribution shift and reconstruction uncertainty; §§III–IV. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P034).</x:v>
       </x:c>
       <x:c r="M35" s="75" t="str">
         <x:v>No</x:v>
@@ -11757,7 +11765,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="37" ht="112" customHeight="1">
+    <x:row r="37" ht="144" customHeight="1">
       <x:c r="A37" s="73" t="str">
         <x:v>S036</x:v>
       </x:c>
@@ -11780,15 +11788,15 @@
       <x:c r="H37" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I37" s="81" t="str">
+      <x:c r="I37" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J37" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K37" s="75"/>
+      <x:c r="J37" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K37" s="75" t="str"/>
       <x:c r="L37" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Controlled operator-mismatch benchmark and calibration. Basis: Author preprint abstract. Sources and full-text question: screening/pilot_02.json (P036).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Controlled acquisition mismatch and blind calibration; §4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P036).</x:v>
       </x:c>
       <x:c r="M37" s="75" t="str">
         <x:v>No</x:v>
@@ -11797,7 +11805,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="38" ht="112" customHeight="1">
+    <x:row r="38" ht="144" customHeight="1">
       <x:c r="A38" s="73" t="str">
         <x:v>S037</x:v>
       </x:c>
@@ -11820,15 +11828,15 @@
       <x:c r="H38" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I38" s="81" t="str">
+      <x:c r="I38" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J38" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K38" s="75"/>
+      <x:c r="J38" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K38" s="75" t="str"/>
       <x:c r="L38" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Formal hallucination assessment and feasibility limits. Basis: Author abstract and targeted full-text definitions, Remark 3.4, Proposition 3.5 and Algorithm 2. Sources and full-text question: screening/pilot_02.json (P037).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Hallucination limits and measurement-supported detail; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P037).</x:v>
       </x:c>
       <x:c r="M38" s="75" t="str">
         <x:v>No</x:v>
@@ -11877,7 +11885,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="112" customHeight="1">
+    <x:row r="40" ht="144" customHeight="1">
       <x:c r="A40" s="73" t="str">
         <x:v>S039</x:v>
       </x:c>
@@ -11900,15 +11908,15 @@
       <x:c r="H40" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I40" s="81" t="str">
+      <x:c r="I40" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J40" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K40" s="75"/>
+      <x:c r="J40" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K40" s="75" t="str"/>
       <x:c r="L40" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind all-in-one restoration with composite and unseen degradation. Basis: Author preprint abstract and publisher journal metadata. Sources and full-text question: screening/pilot_02.json (P039).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unseen tasks and compound degradation; Tables 4–5. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P039).</x:v>
       </x:c>
       <x:c r="M40" s="75" t="str">
         <x:v>No</x:v>
@@ -12140,15 +12148,15 @@
       <x:c r="H46" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I46" s="91" t="str">
+      <x:c r="I46" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J46" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K46" s="75"/>
+      <x:c r="J46" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K46" s="75" t="str"/>
       <x:c r="L46" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind joint reconstruction with image and operator priors. Basis: Complete official NeurIPS proceedings abstract. Sources and full-text question: screening/pilot_03.json (P045).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Joint image/operator estimation; §3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P045).</x:v>
       </x:c>
       <x:c r="M46" s="75" t="str">
         <x:v>No</x:v>
@@ -12220,15 +12228,15 @@
       <x:c r="H48" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I48" s="91" t="str">
+      <x:c r="I48" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J48" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K48" s="75"/>
+      <x:c r="J48" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K48" s="75" t="str"/>
       <x:c r="L48" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Explicit forward-model residual correction inside unrolled/equilibrium models. Basis: Complete author preprint abstract; OpenReview access challenged. Sources and full-text question: screening/pilot_03.json (P047).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Adaptive forward-model correction; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P047).</x:v>
       </x:c>
       <x:c r="M48" s="75" t="str">
         <x:v>No</x:v>
@@ -12822,15 +12830,15 @@
       <x:c r="H63" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I63" s="91" t="str">
+      <x:c r="I63" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J63" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K63" s="75"/>
+      <x:c r="J63" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K63" s="75" t="str"/>
       <x:c r="L63" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Conformal risk control for diffusion reconstruction uncertainty. Basis: Complete official PMLR abstract. Sources and full-text question: screening/pilot_03.json (P062).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Ground-truth reconstruction risk control; §3.2. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P062).</x:v>
       </x:c>
       <x:c r="M63" s="75" t="str">
         <x:v>No</x:v>
@@ -12862,15 +12870,15 @@
       <x:c r="H64" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I64" s="91" t="str">
+      <x:c r="I64" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J64" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K64" s="75"/>
+      <x:c r="J64" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K64" s="75" t="str"/>
       <x:c r="L64" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Task-level uncertainty calibration and adaptive measurement stopping. Basis: Complete author preprint abstract and existing ECCV lineage. Sources and full-text question: screening/pilot_03.json (P063).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Conformal task uncertainty and acquisition stopping; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P063).</x:v>
       </x:c>
       <x:c r="M64" s="75" t="str">
         <x:v>No</x:v>
@@ -12942,15 +12950,15 @@
       <x:c r="H66" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I66" s="91" t="str">
+      <x:c r="I66" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J66" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K66" s="75"/>
+      <x:c r="J66" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K66" s="75" t="str"/>
       <x:c r="L66" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Conformalized aleatoric/epistemic reconstruction uncertainty. Basis: Complete author preprint abstract and existing journal lineage. Sources and full-text question: screening/pilot_03.json (P065).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Generative uncertainty and conformal calibration; §II. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P065).</x:v>
       </x:c>
       <x:c r="M66" s="75" t="str">
         <x:v>No</x:v>
@@ -13022,15 +13030,15 @@
       <x:c r="H68" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I68" s="91" t="str">
+      <x:c r="I68" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J68" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K68" s="75"/>
+      <x:c r="J68" s="99" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K68" s="75" t="str"/>
       <x:c r="L68" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Spatially adaptive conformal reconstruction intervals and hallucination examples. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P067).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Quantile uncertainty and empirical calibration; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_02.json (P067).</x:v>
       </x:c>
       <x:c r="M68" s="75" t="str">
         <x:v>No</x:v>
@@ -14260,7 +14268,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32a936e95b7d4686"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebef3e77e767421f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14432,7 +14440,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 12 (11 include, 1 exclude), 78 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 24 (23 include, 1 exclude), 66 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14440,7 +14448,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Full-text progress: screening/full_text_01.json and full_text_01_report.md. AI decisions are recommendations. Evidence/version/read extent and verified feature fields are recorded per study; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json and full_text_02.json; current report: full_text_02_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14686,7 +14694,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd0ba63d6bf14048"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8ddb329e2fe42c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete third full-text checkpoint: 36 of 90 assessed
Add 12 source-backed AI eligibility recommendations and distinguish operator sampling, point estimation, physical calibration and coverage. Record versions, reading limits and deferred user-side work.

Synchronize the evidence matrix, screening tracker and 90-reference exports. Preserve prior decisions, formal counts and workbook objects; validate counts, formulas, metadata and native structure. Novelty remains unestablished.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rbc6b48a56aa64102"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R16cfaa641b404f50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R540dae317b404798"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R29386213b3234865"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R4692766d23d04c5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5522a8567b99453e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R717b5e1f8d5a4406"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R0984cfe9eb7c47f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R8eaaf7e39b464488"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rac4b8a2531db418c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="17">
+  <x:fills count="18">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -257,7 +262,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="100">
+  <x:cellXfs count="101">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -472,6 +477,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="10" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -705,7 +713,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8aae59c27b7e4b35"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf3187080329f4c87"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1154,7 +1162,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>24</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1171,7 +1179,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>New comparisons cover operator point estimation, prior shift, compound restoration and calibrated image/task uncertainty. Read assumptions and evidence limits in screening/full_text_02_report.md; prior findings remain in full_text_01. Novelty is unestablished.</x:v>
+        <x:v>Joint sampling, operator point estimates, compound restoration and image coverage have existing comparators. See screening/full_text_03_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1226,7 +1234,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 24/90 (23 include, 1 exclude); 66 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 36/90 (35 include, 1 exclude); 54 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1321,7 +1329,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8261fc5109048b2"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R346380cb529945fb"/>
 </x:worksheet>
 </file>
 
@@ -2052,102 +2060,102 @@
         <x:v>Architecture baseline | AI pilot 2026-09-16; unclear. Not established from abstract. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2102.07944 | Batch 02 revisit 2026-09-16: The inspected experiments cover Gaussian deblurring, compressed sensing and MRI. A criterion-3 mismatch/reliability study is still not established. Retain unclear for human scope adjudication; this is not an exclusion or full-text eligibility decision. Source: https://arxiv.org/pdf/2102.07944 | Batch 03 revisit 2026-09-16: Known-operator reconstruction is established; criterion-3 relevance still needs adjudication. Prior selected-section inspection is not a complete eligibility review. Source: https://arxiv.org/abs/2102.07944 | AI full-text 2026-09-16: include; human pending. Verified fields: S. Evidence/version/read extent: screening/full_text_01.json (P006). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="7" t="str">
+    <x:row r="8" ht="176" customHeight="1">
+      <x:c r="A8" s="85" t="str">
         <x:v>P007</x:v>
       </x:c>
-      <x:c r="B8" s="8" t="n">
+      <x:c r="B8" s="86" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="C8" s="9" t="str">
+      <x:c r="C8" s="75" t="str">
         <x:v>Sun, He; Bouman, Katherine L.</x:v>
       </x:c>
-      <x:c r="D8" s="9" t="str">
+      <x:c r="D8" s="75" t="str">
         <x:v>Deep Probabilistic Imaging: Uncertainty Quantification and Multi-modal Solution Characterization for Computational Imaging</x:v>
       </x:c>
-      <x:c r="E8" s="9" t="str">
+      <x:c r="E8" s="75" t="str">
         <x:v>AAAI</x:v>
       </x:c>
-      <x:c r="F8" s="9" t="str">
+      <x:c r="F8" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G8" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H8" s="9" t="str">
+      <x:c r="G8" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H8" s="75" t="str">
         <x:v>MRI/radio imaging</x:v>
       </x:c>
-      <x:c r="I8" s="9" t="str">
+      <x:c r="I8" s="75" t="str">
         <x:v>Scientific imaging</x:v>
       </x:c>
-      <x:c r="J8" s="9" t="str">
+      <x:c r="J8" s="75" t="str">
         <x:v>Linear operator</x:v>
       </x:c>
-      <x:c r="K8" s="9" t="str">
+      <x:c r="K8" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L8" s="9" t="str">
+      <x:c r="L8" s="75" t="str">
         <x:v>None central</x:v>
       </x:c>
-      <x:c r="M8" s="9" t="str">
+      <x:c r="M8" s="75" t="str">
         <x:v>Variational generative posterior</x:v>
       </x:c>
-      <x:c r="N8" s="9" t="str">
+      <x:c r="N8" s="75" t="str">
         <x:v>Soft likelihood</x:v>
       </x:c>
-      <x:c r="O8" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P8" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Q8" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R8" s="9" t="str">
+      <x:c r="O8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P8" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R8" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="S8" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="T8" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U8" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V8" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W8" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X8" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y8" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z8" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA8" s="9" t="str">
+      <x:c r="S8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T8" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y8" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z8" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA8" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB8" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC8" s="9" t="str">
+      <x:c r="AB8" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC8" s="75" t="str">
         <x:v>Multimodal posterior characterisation</x:v>
       </x:c>
-      <x:c r="AD8" s="9" t="str">
+      <x:c r="AD8" s="75" t="str">
         <x:v>Image posterior only; operator mismatch not jointly represented</x:v>
       </x:c>
-      <x:c r="AE8" s="9" t="str">
+      <x:c r="AE8" s="75" t="str">
         <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/16366</x:v>
       </x:c>
-      <x:c r="AF8" s="9" t="str">
-        <x:v>UQ foundation | AI pilot 2026-09-16; advance to full text. Image posterior uncertainty and multimodal solutions. Human adjudication and full-text coding pending. Evidence: https://ojs.aaai.org/index.php/AAAI/article/view/16366</x:v>
+      <x:c r="AF8" s="75" t="str">
+        <x:v>UQ foundation | AI pilot 2026-09-16; advance to full text. Image posterior uncertainty and multimodal solutions. Human adjudication and full-text coding pending. Evidence: https://ojs.aaai.org/index.php/AAAI/article/view/16366 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T. Evidence/version/read extent: screening/full_text_03.json (P007). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -2346,200 +2354,200 @@
         <x:v>Degradation simulator baseline | AI pilot 2026-09-16; advance to full text. Blind restoration with compound degradation. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2103.14006</x:v>
       </x:c>
     </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="7" t="str">
+    <x:row r="11" ht="176" customHeight="1">
+      <x:c r="A11" s="85" t="str">
         <x:v>P010</x:v>
       </x:c>
-      <x:c r="B11" s="8" t="n">
+      <x:c r="B11" s="86" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="C11" s="9" t="str">
+      <x:c r="C11" s="75" t="str">
         <x:v>Wang et al.</x:v>
       </x:c>
-      <x:c r="D11" s="9" t="str">
+      <x:c r="D11" s="75" t="str">
         <x:v>Real-ESRGAN: Training Real-World Blind Super-Resolution With Pure Synthetic Data</x:v>
       </x:c>
-      <x:c r="E11" s="9" t="str">
+      <x:c r="E11" s="75" t="str">
         <x:v>ICCV Workshops</x:v>
       </x:c>
-      <x:c r="F11" s="9" t="str">
+      <x:c r="F11" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G11" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H11" s="9" t="str">
+      <x:c r="G11" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H11" s="75" t="str">
         <x:v>Super-resolution</x:v>
       </x:c>
-      <x:c r="I11" s="9" t="str">
+      <x:c r="I11" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J11" s="9" t="str">
+      <x:c r="J11" s="75" t="str">
         <x:v>High-order synthetic degradation</x:v>
       </x:c>
-      <x:c r="K11" s="9" t="str">
+      <x:c r="K11" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="L11" s="9" t="str">
+      <x:c r="L11" s="75" t="str">
         <x:v>Composite/high-order degradation</x:v>
       </x:c>
-      <x:c r="M11" s="9" t="str">
+      <x:c r="M11" s="75" t="str">
         <x:v>GAN restoration</x:v>
       </x:c>
-      <x:c r="N11" s="9" t="str">
+      <x:c r="N11" s="75" t="str">
         <x:v>Implicit</x:v>
       </x:c>
-      <x:c r="O11" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P11" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q11" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R11" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S11" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T11" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="U11" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="V11" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W11" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X11" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y11" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z11" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA11" s="9" t="str">
+      <x:c r="O11" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P11" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q11" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R11" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S11" s="75" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="T11" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U11" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V11" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W11" s="75" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="X11" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y11" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z11" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA11" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB11" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC11" s="9" t="str">
+      <x:c r="AB11" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC11" s="75" t="str">
         <x:v>High-order synthetic degradation for real-world SR</x:v>
       </x:c>
-      <x:c r="AD11" s="9" t="str">
+      <x:c r="AD11" s="75" t="str">
         <x:v>Perceptual restoration lacks calibrated fidelity controls</x:v>
       </x:c>
-      <x:c r="AE11" s="9" t="str">
+      <x:c r="AE11" s="75" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2021W/AIM/html/Wang_Real-ESRGAN_Training_Real-World_Blind_Super-Resolution_With_Pure_Synthetic_Data_ICCVW_2021_paper.html</x:v>
       </x:c>
-      <x:c r="AF11" s="9" t="str">
-        <x:v>Generative restoration baseline | AI pilot 2026-09-16; advance to full text. Blind super-resolution with high-order degradation. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2107.10833</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="7" t="str">
+      <x:c r="AF11" s="75" t="str">
+        <x:v>Generative restoration baseline | AI pilot 2026-09-16; advance to full text. Blind super-resolution with high-order degradation. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2107.10833 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, W, X. Evidence/version/read extent: screening/full_text_03.json (P010). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="176" customHeight="1">
+      <x:c r="A12" s="85" t="str">
         <x:v>P011</x:v>
       </x:c>
-      <x:c r="B12" s="8" t="n">
+      <x:c r="B12" s="86" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="C12" s="9" t="str">
+      <x:c r="C12" s="75" t="str">
         <x:v>Angelopoulos et al.</x:v>
       </x:c>
-      <x:c r="D12" s="9" t="str">
+      <x:c r="D12" s="75" t="str">
         <x:v>Image-to-Image Regression with Distribution-Free Uncertainty Quantification and Applications in Imaging</x:v>
       </x:c>
-      <x:c r="E12" s="9" t="str">
+      <x:c r="E12" s="75" t="str">
         <x:v>ICML</x:v>
       </x:c>
-      <x:c r="F12" s="9" t="str">
+      <x:c r="F12" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G12" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H12" s="9" t="str">
+      <x:c r="G12" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H12" s="75" t="str">
         <x:v>MRI/microscopy/SR</x:v>
       </x:c>
-      <x:c r="I12" s="9" t="str">
+      <x:c r="I12" s="75" t="str">
         <x:v>Scientific imaging</x:v>
       </x:c>
-      <x:c r="J12" s="9" t="str">
+      <x:c r="J12" s="75" t="str">
         <x:v>Task-dependent</x:v>
       </x:c>
-      <x:c r="K12" s="9" t="str">
+      <x:c r="K12" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L12" s="9" t="str">
+      <x:c r="L12" s="75" t="str">
         <x:v>Model error</x:v>
       </x:c>
-      <x:c r="M12" s="9" t="str">
+      <x:c r="M12" s="75" t="str">
         <x:v>Conformal UQ</x:v>
       </x:c>
-      <x:c r="N12" s="9" t="str">
+      <x:c r="N12" s="75" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="O12" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P12" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Q12" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R12" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="S12" s="9" t="str">
+      <x:c r="O12" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P12" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q12" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R12" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S12" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="T12" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="U12" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V12" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W12" s="9" t="str">
+      <x:c r="T12" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U12" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V12" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W12" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="X12" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="Y12" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z12" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA12" s="9" t="str">
+      <x:c r="X12" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y12" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z12" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA12" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB12" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC12" s="9" t="str">
+      <x:c r="AB12" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC12" s="75" t="str">
         <x:v>Distribution-free pixel intervals with marginal coverage</x:v>
       </x:c>
-      <x:c r="AD12" s="9" t="str">
+      <x:c r="AD12" s="75" t="str">
         <x:v>Does not infer unknown operators; OOD validity needs careful design</x:v>
       </x:c>
-      <x:c r="AE12" s="9" t="str">
+      <x:c r="AE12" s="75" t="str">
         <x:v>https://proceedings.mlr.press/v162/angelopoulos22a.html</x:v>
       </x:c>
-      <x:c r="AF12" s="9" t="str">
-        <x:v>Calibration foundation | AI pilot 2026-09-16; advance to full text. Calibrated image prediction intervals. Human adjudication and full-text coding pending. Evidence: https://proceedings.mlr.press/v162/angelopoulos22a.html</x:v>
+      <x:c r="AF12" s="75" t="str">
+        <x:v>Calibration foundation | AI pilot 2026-09-16; advance to full text. Calibrated image prediction intervals. Human adjudication and full-text coding pending. Evidence: https://proceedings.mlr.press/v162/angelopoulos22a.html | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, T, W, X. Evidence/version/read extent: screening/full_text_03.json (P011). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3130,200 +3138,200 @@
         <x:v>Support-map component | AI pilot 2026-09-16; advance to full text. Range/null-space reconstruction and measurement consistency. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2212.00490</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="7" t="str">
+    <x:row r="19" ht="176" customHeight="1">
+      <x:c r="A19" s="85" t="str">
         <x:v>P018</x:v>
       </x:c>
-      <x:c r="B19" s="8" t="n">
+      <x:c r="B19" s="86" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="C19" s="9" t="str">
+      <x:c r="C19" s="75" t="str">
         <x:v>Chung et al.</x:v>
       </x:c>
-      <x:c r="D19" s="9" t="str">
+      <x:c r="D19" s="75" t="str">
         <x:v>Parallel Diffusion Models of Operator and Image for Blind Inverse Problems</x:v>
       </x:c>
-      <x:c r="E19" s="9" t="str">
+      <x:c r="E19" s="75" t="str">
         <x:v>CVPR</x:v>
       </x:c>
-      <x:c r="F19" s="9" t="str">
+      <x:c r="F19" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G19" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H19" s="9" t="str">
+      <x:c r="G19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H19" s="75" t="str">
         <x:v>Deblurring/turbulence</x:v>
       </x:c>
-      <x:c r="I19" s="9" t="str">
+      <x:c r="I19" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J19" s="9" t="str">
+      <x:c r="J19" s="75" t="str">
         <x:v>Known functional form</x:v>
       </x:c>
-      <x:c r="K19" s="9" t="str">
+      <x:c r="K19" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="L19" s="9" t="str">
+      <x:c r="L19" s="75" t="str">
         <x:v>Blind operator parameters</x:v>
       </x:c>
-      <x:c r="M19" s="9" t="str">
+      <x:c r="M19" s="75" t="str">
         <x:v>Parallel diffusion priors</x:v>
       </x:c>
-      <x:c r="N19" s="9" t="str">
+      <x:c r="N19" s="75" t="str">
         <x:v>Soft likelihood</x:v>
       </x:c>
-      <x:c r="O19" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="P19" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="Q19" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="R19" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S19" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T19" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U19" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V19" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W19" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X19" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y19" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z19" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA19" s="9" t="str">
+      <x:c r="O19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="P19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="R19" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T19" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V19" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W19" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X19" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z19" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA19" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB19" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC19" s="9" t="str">
+      <x:c r="AB19" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC19" s="75" t="str">
         <x:v>Joint image/operator diffusion</x:v>
       </x:c>
-      <x:c r="AD19" s="9" t="str">
+      <x:c r="AD19" s="75" t="str">
         <x:v>No calibrated joint UQ or abstention; operator-prior burden</x:v>
       </x:c>
-      <x:c r="AE19" s="9" t="str">
+      <x:c r="AE19" s="75" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2023/html/Chung_Parallel_Diffusion_Models_of_Operator_and_Image_for_Blind_Inverse_Problems_CVPR_2023_paper.html</x:v>
       </x:c>
-      <x:c r="AF19" s="9" t="str">
-        <x:v>Nearest blind diffusion competitor | AI pilot 2026-09-16; advance to full text. Joint image/operator inference in blind reconstruction. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2211.10656</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="7" t="str">
+      <x:c r="AF19" s="75" t="str">
+        <x:v>Nearest blind diffusion competitor | AI pilot 2026-09-16; advance to full text. Joint image/operator inference in blind reconstruction. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2211.10656 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_03.json (P018). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="176" customHeight="1">
+      <x:c r="A20" s="85" t="str">
         <x:v>P019</x:v>
       </x:c>
-      <x:c r="B20" s="8" t="n">
+      <x:c r="B20" s="86" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="C20" s="9" t="str">
+      <x:c r="C20" s="75" t="str">
         <x:v>Murata et al.</x:v>
       </x:c>
-      <x:c r="D20" s="9" t="str">
+      <x:c r="D20" s="75" t="str">
         <x:v>GibbsDDRM: A Partially Collapsed Gibbs Sampler for Solving Blind Inverse Problems with Denoising Diffusion Restoration</x:v>
       </x:c>
-      <x:c r="E20" s="9" t="str">
+      <x:c r="E20" s="75" t="str">
         <x:v>ICML</x:v>
       </x:c>
-      <x:c r="F20" s="9" t="str">
+      <x:c r="F20" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G20" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H20" s="9" t="str">
+      <x:c r="G20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H20" s="75" t="str">
         <x:v>Blind linear inverse tasks</x:v>
       </x:c>
-      <x:c r="I20" s="9" t="str">
+      <x:c r="I20" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J20" s="9" t="str">
+      <x:c r="J20" s="75" t="str">
         <x:v>Linear operator family</x:v>
       </x:c>
-      <x:c r="K20" s="9" t="str">
+      <x:c r="K20" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="L20" s="9" t="str">
+      <x:c r="L20" s="75" t="str">
         <x:v>Blind parameters</x:v>
       </x:c>
-      <x:c r="M20" s="9" t="str">
+      <x:c r="M20" s="75" t="str">
         <x:v>Gibbs diffusion sampler</x:v>
       </x:c>
-      <x:c r="N20" s="9" t="str">
+      <x:c r="N20" s="75" t="str">
         <x:v>Hard/likelihood</x:v>
       </x:c>
-      <x:c r="O20" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="P20" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Q20" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="R20" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="S20" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T20" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U20" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V20" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W20" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X20" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y20" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z20" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA20" s="9" t="str">
+      <x:c r="O20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="P20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="R20" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T20" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V20" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W20" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X20" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z20" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA20" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB20" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC20" s="9" t="str">
+      <x:c r="AB20" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC20" s="75" t="str">
         <x:v>Bayesian blind image/operator sampling</x:v>
       </x:c>
-      <x:c r="AD20" s="9" t="str">
+      <x:c r="AD20" s="75" t="str">
         <x:v>Simplified forward families; real compound calibration remains</x:v>
       </x:c>
-      <x:c r="AE20" s="9" t="str">
+      <x:c r="AE20" s="75" t="str">
         <x:v>https://proceedings.mlr.press/v202/murata23a.html</x:v>
       </x:c>
-      <x:c r="AF20" s="9" t="str">
-        <x:v>Nearest joint posterior competitor | AI pilot 2026-09-16; advance to full text. Joint posterior inference for blind inverse problems. Human adjudication and full-text coding pending. Evidence: https://proceedings.mlr.press/v202/murata23a.html</x:v>
+      <x:c r="AF20" s="75" t="str">
+        <x:v>Nearest joint posterior competitor | AI pilot 2026-09-16; advance to full text. Joint posterior inference for blind inverse problems. Human adjudication and full-text coding pending. Evidence: https://proceedings.mlr.press/v202/murata23a.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_03.json (P019). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -3522,7 +3530,7 @@
         <x:v>Closest calibration analogue | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; journal citation not independently rechecked in this batch. Feature codes remain provisional. Which coordinate errors and initialization regimes are evaluated? Physical calibration is not statistical calibration of uncertainty intervals. Evidence: https://arxiv.org/abs/2211.10525</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="112" customHeight="1">
+    <x:row r="23" ht="176" customHeight="1">
       <x:c r="A23" s="85" t="str">
         <x:v>P022</x:v>
       </x:c>
@@ -3569,29 +3577,29 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="P23" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q23" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R23" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S23" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T23" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U23" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V23" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W23" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="Q23" s="75" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="R23" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S23" s="75" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T23" s="75" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U23" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V23" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W23" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
       <x:c r="X23" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -3599,7 +3607,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z23" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA23" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -3617,10 +3625,10 @@
         <x:v>https://openaccess.thecvf.com/content/WACV2024/html/Laroche_Fast_Diffusion_EM_A_Diffusion_Model_for_Blind_Inverse_Problems_WACV_2024_paper.html</x:v>
       </x:c>
       <x:c r="AF23" s="75" t="str">
-        <x:v>Nearest EM competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and authors' institutional publication record. Feature codes remain provisional. Does uncertainty describe only image samples conditional on a point-estimated kernel, or propagate kernel uncertainty? Extract assumed kernel/noise families. Evidence: https://arxiv.org/abs/2309.00287</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="112" customHeight="1">
+        <x:v>Nearest EM competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and authors' institutional publication record. Feature codes remain provisional. Does uncertainty describe only image samples conditional on a point-estimated kernel, or propagate kernel uncertainty? Extract assumed kernel/noise families. Evidence: https://arxiv.org/abs/2309.00287 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, W, X. Evidence/version/read extent: screening/full_text_03.json (P022). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="176" customHeight="1">
       <x:c r="A24" s="85" t="str">
         <x:v>P023</x:v>
       </x:c>
@@ -3667,10 +3675,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="P24" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Q24" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="R24" s="75" t="str">
         <x:v>No</x:v>
@@ -3679,7 +3687,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T24" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U24" s="75" t="str">
         <x:v>Yes</x:v>
@@ -3697,7 +3705,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z24" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA24" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -3715,10 +3723,10 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/3d13d910b48ac2e672a32cfdf98be1bf-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF24" s="75" t="str">
-        <x:v>Nearest blind inversion competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and official proceedings record. Feature codes remain provisional. Which degradation combinations and mismatched families are tested? Optimization on a generative manifold does not itself certify measurement-supported detail. Evidence: https://arxiv.org/abs/2405.19572</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="112" customHeight="1">
+        <x:v>Nearest blind inversion competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract and official proceedings record. Feature codes remain provisional. Which degradation combinations and mismatched families are tested? Optimization on a generative manifold does not itself certify measurement-supported detail. Evidence: https://arxiv.org/abs/2405.19572 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_03.json (P023). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="176" customHeight="1">
       <x:c r="A25" s="85" t="str">
         <x:v>P024</x:v>
       </x:c>
@@ -3765,10 +3773,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="P25" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="Q25" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="R25" s="75" t="str">
         <x:v>No</x:v>
@@ -3795,7 +3803,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z25" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA25" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -3813,7 +3821,7 @@
         <x:v>https://ieeexplore.ieee.org/document/11351303/</x:v>
       </x:c>
       <x:c r="AF25" s="75" t="str">
-        <x:v>Verify final TIP metadata during full-text stage | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; journal lineage reconciled with the existing verification audit. Feature codes remain provisional. Inspect the final journal report for additions, operator constraints and uncertainty evaluation; the DOI remains unverified and is not invented. Evidence: https://arxiv.org/abs/2407.01027</x:v>
+        <x:v>Verify final TIP metadata during full-text stage | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; journal lineage reconciled with the existing verification audit. Feature codes remain provisional. Inspect the final journal report for additions, operator constraints and uncertainty evaluation; the DOI remains unverified and is not invented. Evidence: https://arxiv.org/abs/2407.01027 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R. Evidence/version/read extent: screening/full_text_03.json (P024). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="112" customHeight="1">
@@ -5443,16 +5451,16 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T42" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U42" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V42" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W42" s="75" t="str">
         <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U42" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V42" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W42" s="75" t="str">
-        <x:v>Yes</x:v>
       </x:c>
       <x:c r="X42" s="75" t="str">
         <x:v>No</x:v>
@@ -5461,7 +5469,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z42" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA42" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -5479,7 +5487,7 @@
         <x:v>https://arxiv.org/abs/2511.18473</x:v>
       </x:c>
       <x:c r="AF42" s="75" t="str">
-        <x:v>Critical UQ competitor; verify publication lineage | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Are the optical operators known, estimated or misspecified? Extract calibration units and tests beyond the trained optical family. Evidence: https://arxiv.org/abs/2511.18473</x:v>
+        <x:v>Critical UQ competitor; verify publication lineage | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Are the optical operators known, estimated or misspecified? Extract calibration units and tests beyond the trained optical family. Evidence: https://arxiv.org/abs/2511.18473 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_03.json (P041). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="176" customHeight="1">
@@ -6313,22 +6321,22 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="P51" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q51" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R51" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S51" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="Q51" s="75" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="R51" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S51" s="75" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
       <x:c r="T51" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U51" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V51" s="75" t="str">
         <x:v>No</x:v>
@@ -6343,7 +6351,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z51" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA51" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6361,7 +6369,7 @@
         <x:v>https://arxiv.org/abs/2412.00557</x:v>
       </x:c>
       <x:c r="AF51" s="75" t="str">
-        <x:v>Major threat to any general blind-operator claim | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and coauthor publication listing. Feature codes remain provisional. Check prompt sensitivity, operator constraints and identifiability. Retained peer-review flag is legacy metadata; workshop review procedure was not independently verified. Evidence: https://arxiv.org/abs/2412.00557</x:v>
+        <x:v>Major threat to any general blind-operator claim | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and coauthor publication listing. Feature codes remain provisional. Check prompt sensitivity, operator constraints and identifiability. Retained peer-review flag is legacy metadata; workshop review procedure was not independently verified. Evidence: https://arxiv.org/abs/2412.00557 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_03.json (P050). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="176" customHeight="1">
@@ -6426,7 +6434,7 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="U52" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V52" s="75" t="str">
         <x:v>No</x:v>
@@ -6441,7 +6449,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z52" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA52" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6459,7 +6467,7 @@
         <x:v>https://doi.org/10.1109/TCI.2026.3678407</x:v>
       </x:c>
       <x:c r="AF52" s="75" t="str">
-        <x:v>Top adaptive blind-UQ competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; journal lineage from the existing audit. Feature codes remain provisional. Does coil calibration propagate operator uncertainty or yield a point estimate? Test the distinction between imperfect parameters and a wrong acquisition family. Evidence: https://arxiv.org/abs/2411.16535</x:v>
+        <x:v>Top adaptive blind-UQ competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; journal lineage from the existing audit. Feature codes remain provisional. Does coil calibration propagate operator uncertainty or yield a point estimate? Test the distinction between imperfect parameters and a wrong acquisition family. Evidence: https://arxiv.org/abs/2411.16535 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_03.json (P051). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="176" customHeight="1">
@@ -6509,10 +6517,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="P53" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Q53" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="R53" s="75" t="str">
         <x:v>No</x:v>
@@ -6521,10 +6529,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T53" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U53" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V53" s="75" t="str">
         <x:v>No</x:v>
@@ -6539,7 +6547,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z53" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA53" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6557,7 +6565,7 @@
         <x:v>https://arxiv.org/abs/2603.01890</x:v>
       </x:c>
       <x:c r="AF53" s="75" t="str">
-        <x:v>CaMB-Diff; nonlinear-operator threat | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and coauthor ICML acceptance announcement. Feature codes remain provisional. Distinguish radiometric dynamic-range compression from image/video codec artifacts. Assess identifiability, saturation and validity when the true operator violates monotonicity. Evidence: https://arxiv.org/abs/2603.01890</x:v>
+        <x:v>CaMB-Diff; nonlinear-operator threat | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and coauthor ICML acceptance announcement. Feature codes remain provisional. Distinguish radiometric dynamic-range compression from image/video codec artifacts. Assess identifiability, saturation and validity when the true operator violates monotonicity. Evidence: https://arxiv.org/abs/2603.01890 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, W, X. Evidence/version/read extent: screening/full_text_03.json (P052). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="176" customHeight="1">
@@ -10293,7 +10301,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3d8269d76a2409b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04e6f313fc1b478c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10605,7 +10613,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="84" customHeight="1">
+    <x:row r="8" ht="144" customHeight="1">
       <x:c r="A8" s="73" t="str">
         <x:v>S007</x:v>
       </x:c>
@@ -10628,15 +10636,15 @@
       <x:c r="H8" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I8" s="76" t="str">
+      <x:c r="I8" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J8" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K8" s="75"/>
+      <x:c r="J8" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K8" s="75" t="str"/>
       <x:c r="L8" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Image posterior uncertainty and multimodal solutions. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P007).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Image posterior uncertainty and approximate likelihoods; Method. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P007).</x:v>
       </x:c>
       <x:c r="M8" s="75" t="str">
         <x:v>No</x:v>
@@ -10725,7 +10733,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="84" customHeight="1">
+    <x:row r="11" ht="144" customHeight="1">
       <x:c r="A11" s="73" t="str">
         <x:v>S010</x:v>
       </x:c>
@@ -10748,15 +10756,15 @@
       <x:c r="H11" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I11" s="76" t="str">
+      <x:c r="I11" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J11" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K11" s="75"/>
+      <x:c r="J11" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K11" s="75" t="str"/>
       <x:c r="L11" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind super-resolution with high-order degradation. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P010).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. High-order compound degradation and real generalization; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P010).</x:v>
       </x:c>
       <x:c r="M11" s="75" t="str">
         <x:v>No</x:v>
@@ -10765,7 +10773,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="84" customHeight="1">
+    <x:row r="12" ht="144" customHeight="1">
       <x:c r="A12" s="73" t="str">
         <x:v>S011</x:v>
       </x:c>
@@ -10788,15 +10796,15 @@
       <x:c r="H12" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I12" s="76" t="str">
+      <x:c r="I12" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J12" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K12" s="75"/>
+      <x:c r="J12" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K12" s="75" t="str"/>
       <x:c r="L12" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Calibrated image prediction intervals. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P011).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Distribution-free image uncertainty; §2. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P011).</x:v>
       </x:c>
       <x:c r="M12" s="75" t="str">
         <x:v>No</x:v>
@@ -11045,7 +11053,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="84" customHeight="1">
+    <x:row r="19" ht="144" customHeight="1">
       <x:c r="A19" s="73" t="str">
         <x:v>S018</x:v>
       </x:c>
@@ -11068,15 +11076,15 @@
       <x:c r="H19" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I19" s="76" t="str">
+      <x:c r="I19" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J19" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K19" s="75"/>
+      <x:c r="J19" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K19" s="75" t="str"/>
       <x:c r="L19" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint image/operator inference in blind reconstruction. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P018).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown operator parameters and joint inference; §3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P018).</x:v>
       </x:c>
       <x:c r="M19" s="75" t="str">
         <x:v>No</x:v>
@@ -11085,7 +11093,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="84" customHeight="1">
+    <x:row r="20" ht="144" customHeight="1">
       <x:c r="A20" s="73" t="str">
         <x:v>S019</x:v>
       </x:c>
@@ -11108,15 +11116,15 @@
       <x:c r="H20" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I20" s="76" t="str">
+      <x:c r="I20" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J20" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K20" s="75"/>
+      <x:c r="J20" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K20" s="75" t="str"/>
       <x:c r="L20" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint posterior inference for blind inverse problems. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P019).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Image and unknown linear-operator inference; §3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P019).</x:v>
       </x:c>
       <x:c r="M20" s="75" t="str">
         <x:v>No</x:v>
@@ -11205,7 +11213,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="112" customHeight="1">
+    <x:row r="23" ht="144" customHeight="1">
       <x:c r="A23" s="73" t="str">
         <x:v>S022</x:v>
       </x:c>
@@ -11228,15 +11236,15 @@
       <x:c r="H23" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I23" s="81" t="str">
+      <x:c r="I23" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J23" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K23" s="75"/>
+      <x:c r="J23" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K23" s="75" t="str"/>
       <x:c r="L23" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind operator estimation using diffusion and expectation maximization. Basis: Author preprint abstract and authors' institutional publication record. Sources and full-text question: screening/pilot_02.json (P022).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Operator estimation and prior-domain transfer; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P022).</x:v>
       </x:c>
       <x:c r="M23" s="75" t="str">
         <x:v>No</x:v>
@@ -11245,7 +11253,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="112" customHeight="1">
+    <x:row r="24" ht="144" customHeight="1">
       <x:c r="A24" s="73" t="str">
         <x:v>S023</x:v>
       </x:c>
@@ -11268,15 +11276,15 @@
       <x:c r="H24" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I24" s="81" t="str">
+      <x:c r="I24" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J24" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K24" s="75"/>
+      <x:c r="J24" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K24" s="75" t="str"/>
       <x:c r="L24" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind degradation estimation and image restoration. Basis: Author preprint abstract and official proceedings record. Sources and full-text question: screening/pilot_02.json (P023).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Joint operator and latent-image optimization; §3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P023).</x:v>
       </x:c>
       <x:c r="M24" s="75" t="str">
         <x:v>No</x:v>
@@ -11285,7 +11293,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="112" customHeight="1">
+    <x:row r="25" ht="144" customHeight="1">
       <x:c r="A25" s="73" t="str">
         <x:v>S024</x:v>
       </x:c>
@@ -11308,15 +11316,15 @@
       <x:c r="H25" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I25" s="81" t="str">
+      <x:c r="I25" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J25" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K25" s="75"/>
+      <x:c r="J25" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K25" s="75" t="str"/>
       <x:c r="L25" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint image and unknown-operator recovery. Basis: Author preprint abstract; journal lineage reconciled with the existing verification audit. Sources and full-text question: screening/pilot_02.json (P024).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Latent image sampling and operator estimation; §4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P024).</x:v>
       </x:c>
       <x:c r="M25" s="75" t="str">
         <x:v>No</x:v>
@@ -11988,15 +11996,15 @@
       <x:c r="H42" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I42" s="91" t="str">
+      <x:c r="I42" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J42" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K42" s="75"/>
+      <x:c r="J42" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K42" s="75" t="str"/>
       <x:c r="L42" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Posterior uncertainty and calibration for hyperspectral reconstruction. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P041).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Image uncertainty, metamer ambiguity and domain shift; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P041).</x:v>
       </x:c>
       <x:c r="M42" s="75" t="str">
         <x:v>No</x:v>
@@ -12348,15 +12356,15 @@
       <x:c r="H51" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I51" s="91" t="str">
+      <x:c r="I51" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J51" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K51" s="75"/>
+      <x:c r="J51" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K51" s="75" t="str"/>
       <x:c r="L51" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind image/operator inference with text-conditioned latent diffusion priors. Basis: Complete author preprint abstract and coauthor publication listing. Sources and full-text question: screening/pilot_03.json (P050).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown operator approximation; §3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P050).</x:v>
       </x:c>
       <x:c r="M51" s="75" t="str">
         <x:v>No</x:v>
@@ -12388,15 +12396,15 @@
       <x:c r="H52" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I52" s="91" t="str">
+      <x:c r="I52" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J52" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K52" s="75"/>
+      <x:c r="J52" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K52" s="75" t="str"/>
       <x:c r="L52" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Adaptive unknown-operator calibration during diffusion-bridge MRI reconstruction. Basis: Complete author preprint abstract; journal lineage from the existing audit. Sources and full-text question: screening/pilot_03.json (P051).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Uncertain sensitivity maps and image variability; §§3, 5.2. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P051).</x:v>
       </x:c>
       <x:c r="M52" s="75" t="str">
         <x:v>No</x:v>
@@ -12428,15 +12436,15 @@
       <x:c r="H53" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I53" s="91" t="str">
+      <x:c r="I53" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J53" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K53" s="75"/>
+      <x:c r="J53" s="100" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K53" s="75" t="str"/>
       <x:c r="L53" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Structured unknown nonlinear forward-operator estimation. Basis: Complete author preprint abstract and coauthor ICML acceptance announcement. Sources and full-text question: screening/pilot_03.json (P052).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown structured intensity operator; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_03.json (P052).</x:v>
       </x:c>
       <x:c r="M53" s="75" t="str">
         <x:v>No</x:v>
@@ -14268,7 +14276,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebef3e77e767421f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ae29e2ff8c43d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14440,7 +14448,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 24 (23 include, 1 exclude), 66 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 36 (35 include, 1 exclude), 54 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14448,7 +14456,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json and full_text_02.json; current report: full_text_02_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json and full_text_03.json; current report: full_text_03_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14694,7 +14702,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc8ddb329e2fe42c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37ac6d5be1c94d8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete fourth full-text checkpoint: 44 of 90 assessed
Add eight source-backed AI eligibility recommendations with inspected versions,
reading extent and criterion-level evidence. Distinguish physical-operator
uncertainty, sampled images, calibrated intervals and reference-verified detail.

Synchronize the matrix, screening tracker and 90-reference exports. Preserve
earlier decisions, formal counters and workbook objects; validate formulas,
stable metadata, native structure and rendered ranges. Record failed source
routes and keep user-side tasks deferred. Novelty remains unestablished.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5522a8567b99453e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R717b5e1f8d5a4406"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R0984cfe9eb7c47f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R8eaaf7e39b464488"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rac4b8a2531db418c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdf6b3a28932d4b93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R90a42b1fa71d495e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R937e70600bdf49b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="Re2d6097954544d92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R9912c01a84914170"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -262,7 +267,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="101">
+  <x:cellXfs count="102">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -480,6 +485,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -713,7 +721,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf3187080329f4c87"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R92de5d56f59e4f17"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1162,7 +1170,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>36</x:v>
+        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1179,7 +1187,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>Joint sampling, operator point estimates, compound restoration and image coverage have existing comparators. See screening/full_text_03_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
+        <x:v>Mismatch correction, calibrated image intervals, joint degradation estimation and compound video restoration have existing comparators. See screening/full_text_04_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1234,7 +1242,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 36/90 (35 include, 1 exclude); 54 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 44/90 (43 include, 1 exclude); 46 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1329,7 +1337,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R346380cb529945fb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1476f3f012c44e62"/>
 </x:worksheet>
 </file>
 
@@ -1864,102 +1872,102 @@
         <x:v>Data source candidate | AI pilot 2026-09-16; advance to full text. Real blur and synthetic-to-real degradation gap. Human adjudication and full-text coding pending. Evidence: https://link.springer.com/chapter/10.1007/978-3-030-58595-2_12</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="7" t="str">
+    <x:row r="6" ht="176" customHeight="1">
+      <x:c r="A6" s="85" t="str">
         <x:v>P005</x:v>
       </x:c>
-      <x:c r="B6" s="8" t="n">
+      <x:c r="B6" s="86" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="C6" s="9" t="str">
+      <x:c r="C6" s="75" t="str">
         <x:v>Zeng &amp; Lam</x:v>
       </x:c>
-      <x:c r="D6" s="9" t="str">
+      <x:c r="D6" s="75" t="str">
         <x:v>Robust Reconstruction With Deep Learning to Handle Model Mismatch in Lensless Imaging</x:v>
       </x:c>
-      <x:c r="E6" s="9" t="str">
+      <x:c r="E6" s="75" t="str">
         <x:v>IEEE TCI</x:v>
       </x:c>
-      <x:c r="F6" s="9" t="str">
+      <x:c r="F6" s="75" t="str">
         <x:v>Journal</x:v>
       </x:c>
-      <x:c r="G6" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H6" s="9" t="str">
+      <x:c r="G6" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H6" s="75" t="str">
         <x:v>Lensless imaging</x:v>
       </x:c>
-      <x:c r="I6" s="9" t="str">
+      <x:c r="I6" s="75" t="str">
         <x:v>Computational imaging</x:v>
       </x:c>
-      <x:c r="J6" s="9" t="str">
+      <x:c r="J6" s="75" t="str">
         <x:v>PSF/lensless model</x:v>
       </x:c>
-      <x:c r="K6" s="9" t="str">
+      <x:c r="K6" s="75" t="str">
         <x:v>Approximate</x:v>
       </x:c>
-      <x:c r="L6" s="9" t="str">
+      <x:c r="L6" s="75" t="str">
         <x:v>PSF and angular-model mismatch</x:v>
       </x:c>
-      <x:c r="M6" s="9" t="str">
+      <x:c r="M6" s="75" t="str">
         <x:v>Unrolled mismatch-compensation network</x:v>
       </x:c>
-      <x:c r="N6" s="9" t="str">
+      <x:c r="N6" s="75" t="str">
         <x:v>Hard/iterative</x:v>
       </x:c>
-      <x:c r="O6" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="P6" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q6" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R6" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S6" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T6" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="U6" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V6" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W6" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X6" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y6" s="9" t="str">
+      <x:c r="O6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S6" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T6" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X6" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y6" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="Z6" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA6" s="9" t="str">
+      <x:c r="Z6" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA6" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB6" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC6" s="9" t="str">
+      <x:c r="AB6" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC6" s="75" t="str">
         <x:v>Learned mismatch compensation inside lensless reconstruction</x:v>
       </x:c>
-      <x:c r="AD6" s="9" t="str">
+      <x:c r="AD6" s="75" t="str">
         <x:v>Modality-specific; no calibrated UQ, support map or abstention</x:v>
       </x:c>
-      <x:c r="AE6" s="9" t="str">
+      <x:c r="AE6" s="75" t="str">
         <x:v>https://doi.org/10.1109/TCI.2021.3114542</x:v>
       </x:c>
-      <x:c r="AF6" s="9" t="str">
-        <x:v>Nearest early mismatch competitor | AI pilot 2026-09-16; advance to full text. Explicit forward-model mismatch compensation. Human adjudication and full-text coding pending. Evidence: https://www.eee.hku.hk/optima/pub/journal/2109_TCI.pdf</x:v>
+      <x:c r="AF6" s="75" t="str">
+        <x:v>Nearest early mismatch competitor | AI pilot 2026-09-16; advance to full text. Explicit forward-model mismatch compensation. Human adjudication and full-text coding pending. Evidence: https://www.eee.hku.hk/optima/pub/journal/2109_TCI.pdf | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, X. Evidence/version/read extent: screening/full_text_04.json (P005). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="176" customHeight="1">
@@ -2158,102 +2166,102 @@
         <x:v>UQ foundation | AI pilot 2026-09-16; advance to full text. Image posterior uncertainty and multimodal solutions. Human adjudication and full-text coding pending. Evidence: https://ojs.aaai.org/index.php/AAAI/article/view/16366 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T. Evidence/version/read extent: screening/full_text_03.json (P007). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="7" t="str">
+    <x:row r="9" ht="176" customHeight="1">
+      <x:c r="A9" s="85" t="str">
         <x:v>P008</x:v>
       </x:c>
-      <x:c r="B9" s="8" t="n">
+      <x:c r="B9" s="86" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="C9" s="9" t="str">
+      <x:c r="C9" s="75" t="str">
         <x:v>Bhadra et al.</x:v>
       </x:c>
-      <x:c r="D9" s="9" t="str">
+      <x:c r="D9" s="75" t="str">
         <x:v>On Hallucinations in Tomographic Image Reconstruction</x:v>
       </x:c>
-      <x:c r="E9" s="9" t="str">
+      <x:c r="E9" s="75" t="str">
         <x:v>IEEE TMI</x:v>
       </x:c>
-      <x:c r="F9" s="9" t="str">
+      <x:c r="F9" s="75" t="str">
         <x:v>Journal</x:v>
       </x:c>
-      <x:c r="G9" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H9" s="9" t="str">
+      <x:c r="G9" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H9" s="75" t="str">
         <x:v>Tomography</x:v>
       </x:c>
-      <x:c r="I9" s="9" t="str">
+      <x:c r="I9" s="75" t="str">
         <x:v>Medical imaging</x:v>
       </x:c>
-      <x:c r="J9" s="9" t="str">
+      <x:c r="J9" s="75" t="str">
         <x:v>Tomographic operator</x:v>
       </x:c>
-      <x:c r="K9" s="9" t="str">
+      <x:c r="K9" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L9" s="9" t="str">
+      <x:c r="L9" s="75" t="str">
         <x:v>Prior/data shift</x:v>
       </x:c>
-      <x:c r="M9" s="9" t="str">
+      <x:c r="M9" s="75" t="str">
         <x:v>Hallucination analysis</x:v>
       </x:c>
-      <x:c r="N9" s="9" t="str">
+      <x:c r="N9" s="75" t="str">
         <x:v>Range/null decomposition</x:v>
       </x:c>
-      <x:c r="O9" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P9" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q9" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R9" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S9" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T9" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U9" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V9" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W9" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="X9" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y9" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z9" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA9" s="9" t="str">
+      <x:c r="O9" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P9" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q9" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R9" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S9" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T9" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U9" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V9" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W9" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X9" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y9" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z9" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA9" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB9" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC9" s="9" t="str">
+      <x:c r="AB9" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC9" s="75" t="str">
         <x:v>Introduces measurement/null hallucination maps</x:v>
       </x:c>
-      <x:c r="AD9" s="9" t="str">
+      <x:c r="AD9" s="75" t="str">
         <x:v>Diagnostic framework, not compound mismatch-aware reconstruction</x:v>
       </x:c>
-      <x:c r="AE9" s="9" t="str">
+      <x:c r="AE9" s="75" t="str">
         <x:v>https://doi.org/10.1109/TMI.2021.3077857</x:v>
       </x:c>
-      <x:c r="AF9" s="9" t="str">
-        <x:v>Faithfulness foundation | AI pilot 2026-09-16; advance to full text. Hallucination and measurement/null-space analysis. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2012.00646</x:v>
+      <x:c r="AF9" s="75" t="str">
+        <x:v>Faithfulness foundation | AI pilot 2026-09-16; advance to full text. Hallucination and measurement/null-space analysis. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2012.00646 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, W, X. Evidence/version/read extent: screening/full_text_04.json (P008). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -2746,200 +2754,200 @@
         <x:v>Nearest all-in-one baseline | AI pilot 2026-09-16; advance to full text. Unknown corruption and all-in-one restoration. Human adjudication and full-text coding pending. Evidence: https://github.com/XLearning-SCU/2022-CVPR-AirNet | Batch 03 revisit 2026-09-16: Unknown-corruption restoration remains an explicit scope signal. Preserve incomplete evidence and do not equate mixed task training with compound corruption. Source: https://github.com/XLearning-SCU/2022-CVPR-AirNet</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="7" t="str">
+    <x:row r="15" ht="176" customHeight="1">
+      <x:c r="A15" s="85" t="str">
         <x:v>P014</x:v>
       </x:c>
-      <x:c r="B15" s="8" t="n">
+      <x:c r="B15" s="86" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="C15" s="9" t="str">
+      <x:c r="C15" s="75" t="str">
         <x:v>Horwitz &amp; Hoshen</x:v>
       </x:c>
-      <x:c r="D15" s="9" t="str">
+      <x:c r="D15" s="75" t="str">
         <x:v>Conffusion: Confidence Intervals for Diffusion Models</x:v>
       </x:c>
-      <x:c r="E15" s="9" t="str">
+      <x:c r="E15" s="75" t="str">
         <x:v>arXiv</x:v>
       </x:c>
-      <x:c r="F15" s="9" t="str">
+      <x:c r="F15" s="75" t="str">
         <x:v>Preprint</x:v>
       </x:c>
-      <x:c r="G15" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="H15" s="9" t="str">
+      <x:c r="G15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="H15" s="75" t="str">
         <x:v>Image-to-image generation</x:v>
       </x:c>
-      <x:c r="I15" s="9" t="str">
+      <x:c r="I15" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J15" s="9" t="str">
+      <x:c r="J15" s="75" t="str">
         <x:v>Task-dependent</x:v>
       </x:c>
-      <x:c r="K15" s="9" t="str">
+      <x:c r="K15" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L15" s="9" t="str">
+      <x:c r="L15" s="75" t="str">
         <x:v>Model uncertainty</x:v>
       </x:c>
-      <x:c r="M15" s="9" t="str">
+      <x:c r="M15" s="75" t="str">
         <x:v>Diffusion confidence intervals</x:v>
       </x:c>
-      <x:c r="N15" s="9" t="str">
+      <x:c r="N15" s="75" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="O15" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P15" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Q15" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R15" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="S15" s="9" t="str">
+      <x:c r="O15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P15" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R15" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="S15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="T15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W15" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="T15" s="9" t="str">
+      <x:c r="X15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y15" s="75" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="Z15" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA15" s="75" t="str">
+        <x:v>Pending formal eligibility</x:v>
+      </x:c>
+      <x:c r="AB15" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC15" s="75" t="str">
+        <x:v>Fast confidence intervals for diffusion outputs</x:v>
+      </x:c>
+      <x:c r="AD15" s="75" t="str">
+        <x:v>Not physics/operator-aware; peer-reviewed status to confirm</x:v>
+      </x:c>
+      <x:c r="AE15" s="75" t="str">
+        <x:v>https://arxiv.org/abs/2211.09795</x:v>
+      </x:c>
+      <x:c r="AF15" s="75" t="str">
+        <x:v>UQ method candidate | AI pilot 2026-09-16; advance to full text. Diffusion-based confidence intervals. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2211.09795 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_04.json (P014). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="176" customHeight="1">
+      <x:c r="A16" s="85" t="str">
+        <x:v>P015</x:v>
+      </x:c>
+      <x:c r="B16" s="86" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C16" s="75" t="str">
+        <x:v>Chung et al.</x:v>
+      </x:c>
+      <x:c r="D16" s="75" t="str">
+        <x:v>Diffusion Posterior Sampling for General Noisy Inverse Problems</x:v>
+      </x:c>
+      <x:c r="E16" s="75" t="str">
+        <x:v>ICLR</x:v>
+      </x:c>
+      <x:c r="F16" s="75" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="G16" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H16" s="75" t="str">
+        <x:v>Multiple inverse tasks</x:v>
+      </x:c>
+      <x:c r="I16" s="75" t="str">
+        <x:v>Natural images</x:v>
+      </x:c>
+      <x:c r="J16" s="75" t="str">
+        <x:v>Linear/nonlinear operator</x:v>
+      </x:c>
+      <x:c r="K16" s="75" t="str">
+        <x:v>Known</x:v>
+      </x:c>
+      <x:c r="L16" s="75" t="str">
+        <x:v>Noise/model approximation</x:v>
+      </x:c>
+      <x:c r="M16" s="75" t="str">
+        <x:v>Diffusion posterior sampling</x:v>
+      </x:c>
+      <x:c r="N16" s="75" t="str">
+        <x:v>Soft likelihood</x:v>
+      </x:c>
+      <x:c r="O16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P16" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S16" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="U15" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V15" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W15" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="X15" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y15" s="9" t="str">
-        <x:v>Unknown</x:v>
-      </x:c>
-      <x:c r="Z15" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA15" s="9" t="str">
+      <x:c r="T16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U16" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y16" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z16" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA16" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB15" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC15" s="9" t="str">
-        <x:v>Fast confidence intervals for diffusion outputs</x:v>
-      </x:c>
-      <x:c r="AD15" s="9" t="str">
-        <x:v>Not physics/operator-aware; peer-reviewed status to confirm</x:v>
-      </x:c>
-      <x:c r="AE15" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2211.09795</x:v>
-      </x:c>
-      <x:c r="AF15" s="9" t="str">
-        <x:v>UQ method candidate | AI pilot 2026-09-16; advance to full text. Diffusion-based confidence intervals. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2211.09795</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="7" t="str">
-        <x:v>P015</x:v>
-      </x:c>
-      <x:c r="B16" s="8" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C16" s="9" t="str">
-        <x:v>Chung et al.</x:v>
-      </x:c>
-      <x:c r="D16" s="9" t="str">
-        <x:v>Diffusion Posterior Sampling for General Noisy Inverse Problems</x:v>
-      </x:c>
-      <x:c r="E16" s="9" t="str">
-        <x:v>ICLR</x:v>
-      </x:c>
-      <x:c r="F16" s="9" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="G16" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H16" s="9" t="str">
-        <x:v>Multiple inverse tasks</x:v>
-      </x:c>
-      <x:c r="I16" s="9" t="str">
-        <x:v>Natural images</x:v>
-      </x:c>
-      <x:c r="J16" s="9" t="str">
-        <x:v>Linear/nonlinear operator</x:v>
-      </x:c>
-      <x:c r="K16" s="9" t="str">
-        <x:v>Known</x:v>
-      </x:c>
-      <x:c r="L16" s="9" t="str">
-        <x:v>Noise/model approximation</x:v>
-      </x:c>
-      <x:c r="M16" s="9" t="str">
-        <x:v>Diffusion posterior sampling</x:v>
-      </x:c>
-      <x:c r="N16" s="9" t="str">
-        <x:v>Soft likelihood</x:v>
-      </x:c>
-      <x:c r="O16" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P16" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="Q16" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R16" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S16" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="T16" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U16" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V16" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W16" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X16" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y16" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z16" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA16" s="9" t="str">
-        <x:v>Pending formal eligibility</x:v>
-      </x:c>
-      <x:c r="AB16" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC16" s="9" t="str">
+      <x:c r="AB16" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC16" s="75" t="str">
         <x:v>General posterior sampling for noisy inverse problems</x:v>
       </x:c>
-      <x:c r="AD16" s="9" t="str">
+      <x:c r="AD16" s="75" t="str">
         <x:v>Samples are not automatically calibrated; mismatch not solved</x:v>
       </x:c>
-      <x:c r="AE16" s="9" t="str">
+      <x:c r="AE16" s="75" t="str">
         <x:v>https://openreview.net/forum?id=OnD9zGAGT0k</x:v>
       </x:c>
-      <x:c r="AF16" s="9" t="str">
-        <x:v>Diffusion baseline | AI pilot 2026-09-16; advance to full text. Approximate posterior reconstruction under noise. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2209.14687</x:v>
+      <x:c r="AF16" s="75" t="str">
+        <x:v>Diffusion baseline | AI pilot 2026-09-16; advance to full text. Approximate posterior reconstruction under noise. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2209.14687 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_04.json (P015). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="240" customHeight="1">
@@ -6743,7 +6751,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z55" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA55" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6761,7 +6769,7 @@
         <x:v>https://doi.org/10.1007/978-3-031-73254-6_25</x:v>
       </x:c>
       <x:c r="AF55" s="75" t="str">
-        <x:v>High-value real urban data comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Which information depends on an event sensor unavailable in ordinary CCTV? Verify pairing, exposure differences and cross-device generalization. Evidence: https://arxiv.org/abs/2408.14916</x:v>
+        <x:v>High-value real urban data comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Which information depends on an event sensor unavailable in ordinary CCTV? Verify pairing, exposure differences and cross-device generalization. Evidence: https://arxiv.org/abs/2408.14916 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_04.json (P054). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="176" customHeight="1">
@@ -6918,7 +6926,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="S57" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T57" s="75" t="str">
         <x:v>Yes</x:v>
@@ -6927,11 +6935,11 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="V57" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="W57" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="W57" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
       <x:c r="X57" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -6939,7 +6947,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z57" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA57" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6957,7 +6965,7 @@
         <x:v>https://doi.org/10.1109/CVPR52688.2022.00587</x:v>
       </x:c>
       <x:c r="AF57" s="75" t="str">
-        <x:v>Real-world VSR baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Separate perceptual gains on unpaired videos from faithful detail recovery. Verify held-out cameras/codecs and which degradations are jointly simulated. Evidence: https://arxiv.org/abs/2111.12704</x:v>
+        <x:v>Real-world VSR baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Separate perceptual gains on unpaired videos from faithful detail recovery. Verify held-out cameras/codecs and which degradations are jointly simulated. Evidence: https://arxiv.org/abs/2111.12704 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_04.json (P056). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="176" customHeight="1">
@@ -7016,16 +7024,16 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="S58" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T58" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U58" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="V58" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="W58" s="75" t="str">
         <x:v>No</x:v>
@@ -7037,7 +7045,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z58" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA58" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7055,7 +7063,7 @@
         <x:v>https://doi.org/10.1109/CVPRW59228.2023.00127</x:v>
       </x:c>
       <x:c r="AF58" s="75" t="str">
-        <x:v>Useful simulator design reference | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Do the tested codecs and degradation orders leave the training distribution? Non-reference quality scores alone do not establish recovery of true detail. Evidence: https://arxiv.org/abs/2305.02660</x:v>
+        <x:v>Useful simulator design reference | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Do the tested codecs and degradation orders leave the training distribution? Non-reference quality scores alone do not establish recovery of true detail. Evidence: https://arxiv.org/abs/2305.02660 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_04.json (P057). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="176" customHeight="1">
@@ -9258,22 +9266,22 @@
         <x:v>Soft likelihood</x:v>
       </x:c>
       <x:c r="O81" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="P81" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q81" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R81" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S81" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="P81" s="75" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="Q81" s="75" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="R81" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S81" s="75" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
       <x:c r="T81" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U81" s="75" t="str">
         <x:v>Yes</x:v>
@@ -9291,7 +9299,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z81" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA81" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9309,7 +9317,7 @@
         <x:v>https://openaccess.thecvf.com/content/CVPR2023/html/Fei_Generative_Diffusion_Prior_for_Unified_Image_Restoration_and_Enhancement_CVPR_2023_paper.html</x:v>
       </x:c>
       <x:c r="AF81" s="75" t="str">
-        <x:v>Early unified blind-diffusion baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Identify predefined operator families, parameter bounds and out-of-distribution tests. Blind parameter fitting is not arbitrary forward-model discovery. Evidence: https://arxiv.org/abs/2304.01247</x:v>
+        <x:v>Early unified blind-diffusion baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Identify predefined operator families, parameter bounds and out-of-distribution tests. Blind parameter fitting is not arbitrary forward-model discovery. Evidence: https://arxiv.org/abs/2304.01247 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_04.json (P080). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="176" customHeight="1">
@@ -10301,7 +10309,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04e6f313fc1b478c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab9f73b43ca2401d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10533,7 +10541,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="84" customHeight="1">
+    <x:row r="6" ht="144" customHeight="1">
       <x:c r="A6" s="73" t="str">
         <x:v>S005</x:v>
       </x:c>
@@ -10556,15 +10564,15 @@
       <x:c r="H6" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I6" s="76" t="str">
+      <x:c r="I6" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J6" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K6" s="75"/>
+      <x:c r="J6" s="101" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K6" s="75" t="str"/>
       <x:c r="L6" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Explicit forward-model mismatch compensation. Basis: Author-hosted published PDF abstract and opening page. Full-text question and source: screening/pilot_01.json (P005).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Biased forward model and compensation; §§III–IV. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_04.json (P005).</x:v>
       </x:c>
       <x:c r="M6" s="75" t="str">
         <x:v>No</x:v>
@@ -10653,7 +10661,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="84" customHeight="1">
+    <x:row r="9" ht="144" customHeight="1">
       <x:c r="A9" s="73" t="str">
         <x:v>S008</x:v>
       </x:c>
@@ -10676,15 +10684,15 @@
       <x:c r="H9" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I9" s="76" t="str">
+      <x:c r="I9" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J9" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K9" s="75"/>
+      <x:c r="J9" s="101" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K9" s="75" t="str"/>
       <x:c r="L9" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Hallucination and measurement/null-space analysis. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P008).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Prior-induced hallucination, model error and distribution shift; §§III–V. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_04.json (P008).</x:v>
       </x:c>
       <x:c r="M9" s="75" t="str">
         <x:v>No</x:v>
@@ -10893,7 +10901,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="84" customHeight="1">
+    <x:row r="15" ht="144" customHeight="1">
       <x:c r="A15" s="73" t="str">
         <x:v>S014</x:v>
       </x:c>
@@ -10916,15 +10924,15 @@
       <x:c r="H15" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I15" s="76" t="str">
+      <x:c r="I15" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J15" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K15" s="75"/>
+      <x:c r="J15" s="101" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K15" s="75" t="str"/>
       <x:c r="L15" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Diffusion-based confidence intervals. Basis: Preprint abstract; peer review not established. Full-text question and source: screening/pilot_01.json (P014).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Reconstruction uncertainty and risk calibration; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_04.json (P014).</x:v>
       </x:c>
       <x:c r="M15" s="75" t="str">
         <x:v>No</x:v>
@@ -10933,7 +10941,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="84" customHeight="1">
+    <x:row r="16" ht="144" customHeight="1">
       <x:c r="A16" s="73" t="str">
         <x:v>S015</x:v>
       </x:c>
@@ -10956,15 +10964,15 @@
       <x:c r="H16" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I16" s="76" t="str">
+      <x:c r="I16" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J16" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K16" s="75"/>
+      <x:c r="J16" s="101" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K16" s="75" t="str"/>
       <x:c r="L16" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Approximate posterior reconstruction under noise. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P015).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Approximate reconstruction posterior; §3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_04.json (P015).</x:v>
       </x:c>
       <x:c r="M16" s="75" t="str">
         <x:v>No</x:v>
@@ -12516,15 +12524,15 @@
       <x:c r="H55" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I55" s="91" t="str">
+      <x:c r="I55" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J55" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K55" s="75"/>
+      <x:c r="J55" s="101" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K55" s="75" t="str"/>
       <x:c r="L55" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint low-light and motion-blur restoration with real paired acquisition. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P054).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Combined low light, noise and motion blur; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_04.json (P054).</x:v>
       </x:c>
       <x:c r="M55" s="75" t="str">
         <x:v>No</x:v>
@@ -12596,15 +12604,15 @@
       <x:c r="H57" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I57" s="91" t="str">
+      <x:c r="I57" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J57" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K57" s="75"/>
+      <x:c r="J57" s="101" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K57" s="75" t="str"/>
       <x:c r="L57" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind real-world video super-resolution under complex degradation. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P056).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Compound/time-varying training degradation; §4.1. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_04.json (P056).</x:v>
       </x:c>
       <x:c r="M57" s="75" t="str">
         <x:v>No</x:v>
@@ -12636,15 +12644,15 @@
       <x:c r="H58" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I58" s="91" t="str">
+      <x:c r="I58" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J58" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K58" s="75"/>
+      <x:c r="J58" s="101" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K58" s="75" t="str"/>
       <x:c r="L58" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Compound synthetic image/video acquisition and compression degradation. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P057).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Synthetic compound degradation and real transfer; §§3–5. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_04.json (P057).</x:v>
       </x:c>
       <x:c r="M58" s="75" t="str">
         <x:v>No</x:v>
@@ -13558,15 +13566,15 @@
       <x:c r="H81" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I81" s="91" t="str">
+      <x:c r="I81" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J81" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K81" s="75"/>
+      <x:c r="J81" s="101" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K81" s="75" t="str"/>
       <x:c r="L81" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind linear/nonlinear degradation-parameter inference. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P080).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown degradation parameters optimized during reconstruction; §4.1. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_04.json (P080).</x:v>
       </x:c>
       <x:c r="M81" s="75" t="str">
         <x:v>No</x:v>
@@ -14276,7 +14284,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R42ae29e2ff8c43d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb04d2cc53f4aa7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14448,7 +14456,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 36 (35 include, 1 exclude), 54 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 44 (43 include, 1 exclude), 46 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14456,7 +14464,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json and full_text_03.json; current report: full_text_03_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json and full_text_04.json; current report: full_text_04_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14702,7 +14710,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37ac6d5be1c94d8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra06921c3647e4131"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete fifth full-text checkpoint: 53 of 90 assessed
Add nine source-backed AI eligibility recommendations with inspected versions,
reading extent, criterion-level evidence and selected verified feature fields.
Distinguish degradation representations, physical point estimates, posterior
sampling and calibrated reliability; keep novelty unestablished.

Correct the earlier P017 retrieval locator explicitly while preserving its
pending status and historical log. Record successful alternate retrievals and
remaining access/version follow-ups. Keep user-side tasks deferred.

Synchronize the matrix, tracker and 90-reference exports. Validate formula
behavior, unchanged metadata, native workbook objects and rendered ranges.
Preserve previous decisions, all seed IDs and formal inclusion counters.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdf6b3a28932d4b93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R90a42b1fa71d495e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R937e70600bdf49b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="Re2d6097954544d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R9912c01a84914170"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4ba967359d7047ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="Rb65840ecf5834775"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rb5edd1a151134b69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R1f3fc200161d40b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rc86cd4fbe519418b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="20">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -267,7 +272,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="102">
+  <x:cellXfs count="103">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -488,6 +493,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -721,7 +729,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R92de5d56f59e4f17"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0c933de7139a4337"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1170,7 +1178,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>44</x:v>
+        <x:v>53</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1187,7 +1195,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>Mismatch correction, calibrated image intervals, joint degradation estimation and compound video restoration have existing comparators. See screening/full_text_04_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
+        <x:v>Unknown-degradation prompts, compound restoration, operator conditioning and image posterior sampling have existing comparators. See screening/full_text_05_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1242,7 +1250,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 44/90 (43 include, 1 exclude); 46 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 53/90 (52 include, 1 exclude); 37 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1337,7 +1345,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1476f3f012c44e62"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra13e6d20e5364836"/>
 </x:worksheet>
 </file>
 
@@ -2558,102 +2566,102 @@
         <x:v>Calibration foundation | AI pilot 2026-09-16; advance to full text. Calibrated image prediction intervals. Human adjudication and full-text coding pending. Evidence: https://proceedings.mlr.press/v162/angelopoulos22a.html | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, T, W, X. Evidence/version/read extent: screening/full_text_03.json (P011). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="7" t="str">
+    <x:row r="13" ht="176" customHeight="1">
+      <x:c r="A13" s="85" t="str">
         <x:v>P012</x:v>
       </x:c>
-      <x:c r="B13" s="8" t="n">
+      <x:c r="B13" s="86" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="C13" s="9" t="str">
+      <x:c r="C13" s="75" t="str">
         <x:v>Kawar et al.</x:v>
       </x:c>
-      <x:c r="D13" s="9" t="str">
+      <x:c r="D13" s="75" t="str">
         <x:v>Denoising Diffusion Restoration Models</x:v>
       </x:c>
-      <x:c r="E13" s="9" t="str">
+      <x:c r="E13" s="75" t="str">
         <x:v>NeurIPS</x:v>
       </x:c>
-      <x:c r="F13" s="9" t="str">
+      <x:c r="F13" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G13" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H13" s="9" t="str">
+      <x:c r="G13" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H13" s="75" t="str">
         <x:v>Multiple inverse tasks</x:v>
       </x:c>
-      <x:c r="I13" s="9" t="str">
+      <x:c r="I13" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J13" s="9" t="str">
+      <x:c r="J13" s="75" t="str">
         <x:v>Linear operator</x:v>
       </x:c>
-      <x:c r="K13" s="9" t="str">
+      <x:c r="K13" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L13" s="9" t="str">
+      <x:c r="L13" s="75" t="str">
         <x:v>None central</x:v>
       </x:c>
-      <x:c r="M13" s="9" t="str">
+      <x:c r="M13" s="75" t="str">
         <x:v>Diffusion posterior restoration</x:v>
       </x:c>
-      <x:c r="N13" s="9" t="str">
+      <x:c r="N13" s="75" t="str">
         <x:v>Hard/spectral</x:v>
       </x:c>
-      <x:c r="O13" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P13" s="9" t="str">
+      <x:c r="O13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P13" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S13" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="Q13" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R13" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S13" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="T13" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U13" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V13" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W13" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X13" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y13" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z13" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA13" s="9" t="str">
+      <x:c r="T13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U13" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y13" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z13" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA13" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB13" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC13" s="9" t="str">
+      <x:c r="AB13" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC13" s="75" t="str">
         <x:v>Diffusion restoration for linear inverse problems</x:v>
       </x:c>
-      <x:c r="AD13" s="9" t="str">
+      <x:c r="AD13" s="75" t="str">
         <x:v>Sensitive to incorrect operator; no operator UQ</x:v>
       </x:c>
-      <x:c r="AE13" s="9" t="str">
+      <x:c r="AE13" s="75" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2022/hash/95504595b6169131b6ed6cd72eb05616-Abstract-Conference.html</x:v>
       </x:c>
-      <x:c r="AF13" s="9" t="str">
-        <x:v>Diffusion baseline | AI pilot 2026-09-16; advance to full text. Posterior reconstruction and transfer across image distributions. Human adjudication and full-text coding pending. Evidence: https://proceedings.neurips.cc/paper_files/paper/2022/hash/95504595b6169131b6ed6cd72eb05616-Abstract-Conference.html</x:v>
+      <x:c r="AF13" s="75" t="str">
+        <x:v>Diffusion baseline | AI pilot 2026-09-16; advance to full text. Posterior reconstruction and transfer across image distributions. Human adjudication and full-text coding pending. Evidence: https://proceedings.neurips.cc/paper_files/paper/2022/hash/95504595b6169131b6ed6cd72eb05616-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_05.json (P012). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="240" customHeight="1">
@@ -3342,102 +3350,102 @@
         <x:v>Nearest joint posterior competitor | AI pilot 2026-09-16; advance to full text. Joint posterior inference for blind inverse problems. Human adjudication and full-text coding pending. Evidence: https://proceedings.mlr.press/v202/murata23a.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_03.json (P019). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="7" t="str">
+    <x:row r="21" ht="176" customHeight="1">
+      <x:c r="A21" s="85" t="str">
         <x:v>P020</x:v>
       </x:c>
-      <x:c r="B21" s="8" t="n">
+      <x:c r="B21" s="86" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="C21" s="9" t="str">
+      <x:c r="C21" s="75" t="str">
         <x:v>Potlapalli et al.</x:v>
       </x:c>
-      <x:c r="D21" s="9" t="str">
+      <x:c r="D21" s="75" t="str">
         <x:v>PromptIR: Prompting for All-in-One Image Restoration</x:v>
       </x:c>
-      <x:c r="E21" s="9" t="str">
+      <x:c r="E21" s="75" t="str">
         <x:v>NeurIPS</x:v>
       </x:c>
-      <x:c r="F21" s="9" t="str">
+      <x:c r="F21" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G21" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H21" s="9" t="str">
+      <x:c r="G21" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H21" s="75" t="str">
         <x:v>Multi-task restoration</x:v>
       </x:c>
-      <x:c r="I21" s="9" t="str">
+      <x:c r="I21" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J21" s="9" t="str">
+      <x:c r="J21" s="75" t="str">
         <x:v>Implicit corruption process</x:v>
       </x:c>
-      <x:c r="K21" s="9" t="str">
+      <x:c r="K21" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="L21" s="9" t="str">
+      <x:c r="L21" s="75" t="str">
         <x:v>Multiple degradation types/levels</x:v>
       </x:c>
-      <x:c r="M21" s="9" t="str">
+      <x:c r="M21" s="75" t="str">
         <x:v>Prompt-conditioned transformer</x:v>
       </x:c>
-      <x:c r="N21" s="9" t="str">
+      <x:c r="N21" s="75" t="str">
         <x:v>Implicit</x:v>
       </x:c>
-      <x:c r="O21" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P21" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q21" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R21" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S21" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T21" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U21" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="V21" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W21" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X21" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y21" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z21" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA21" s="9" t="str">
+      <x:c r="O21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S21" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X21" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y21" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z21" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA21" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB21" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC21" s="9" t="str">
+      <x:c r="AB21" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC21" s="75" t="str">
         <x:v>Prompts dynamically guide blind restoration</x:v>
       </x:c>
-      <x:c r="AD21" s="9" t="str">
+      <x:c r="AD21" s="75" t="str">
         <x:v>No physics traceability, calibrated UQ or failure policy</x:v>
       </x:c>
-      <x:c r="AE21" s="9" t="str">
+      <x:c r="AE21" s="75" t="str">
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a579a0d76fd4a35d107-Abstract-Conference.html</x:v>
       </x:c>
-      <x:c r="AF21" s="9" t="str">
-        <x:v>Nearest all-in-one baseline | AI pilot 2026-09-16; advance to full text. Unknown degradation types and levels. Human adjudication and full-text coding pending. Evidence: https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a579a0d76fd4a35d107-Abstract-Conference.html</x:v>
+      <x:c r="AF21" s="75" t="str">
+        <x:v>Nearest all-in-one baseline | AI pilot 2026-09-16; advance to full text. Unknown degradation types and levels. Human adjudication and full-text coding pending. Evidence: https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a579a0d76fd4a35d107-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_05.json (P020). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="112" customHeight="1">
@@ -8690,13 +8698,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="S75" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T75" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U75" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="V75" s="75" t="str">
         <x:v>No</x:v>
@@ -8711,7 +8719,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z75" s="75" t="str">
-        <x:v>Abstract and repository inspected</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA75" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8729,7 +8737,7 @@
         <x:v>https://openreview.net/forum?id=t3vnnLeajU</x:v>
       </x:c>
       <x:c r="AF75" s="75" t="str">
-        <x:v>Strong vision-language restoration baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author abstract, project page and official ICLR slides title. Feature codes remain provisional. Distinguish a dataset mixing different degradation classes from images with simultaneously compounded corruption. Verify the final citation against the accepted paper. Evidence: https://arxiv.org/abs/2310.01018</x:v>
+        <x:v>Strong vision-language restoration baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author abstract, project page and official ICLR slides title. Feature codes remain provisional. Distinguish a dataset mixing different degradation classes from images with simultaneously compounded corruption. Verify the final citation against the accepted paper. Evidence: https://arxiv.org/abs/2310.01018 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_05.json (P074). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="176" customHeight="1">
@@ -8791,17 +8799,17 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T76" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U76" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V76" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W76" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="U76" s="75" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="V76" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W76" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
       <x:c r="X76" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -8809,7 +8817,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z76" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA76" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8827,7 +8835,7 @@
         <x:v>https://doi.org/10.1109/CVPR52733.2024.02403</x:v>
       </x:c>
       <x:c r="AF76" s="75" t="str">
-        <x:v>High-capacity universal restoration competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. What adaptation data or instructions are supplied for unseen tasks, and is fidelity measured against observation-supported detail rather than perceptual appearance? Evidence: https://arxiv.org/abs/2312.02918</x:v>
+        <x:v>High-capacity universal restoration competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. What adaptation data or instructions are supplied for unseen tasks, and is fidelity measured against observation-supported detail rather than perceptual appearance? Evidence: https://arxiv.org/abs/2312.02918 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, S, T, U, W, X. Evidence/version/read extent: screening/full_text_05.json (P075). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="176" customHeight="1">
@@ -8889,7 +8897,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T77" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U77" s="75" t="str">
         <x:v>Yes</x:v>
@@ -8907,7 +8915,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z77" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA77" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8925,7 +8933,7 @@
         <x:v>https://arxiv.org/abs/2401.16468</x:v>
       </x:c>
       <x:c r="AF77" s="75" t="str">
-        <x:v>Language-guided restoration baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Which degradation information is provided by the instruction? Multiple tasks alone do not demonstrate simultaneous compound corruption or reliable recovery under shift. Evidence: https://arxiv.org/abs/2401.16468</x:v>
+        <x:v>Language-guided restoration baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. Which degradation information is provided by the instruction? Multiple tasks alone do not demonstrate simultaneous compound corruption or reliable recovery under shift. Evidence: https://arxiv.org/abs/2401.16468 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_05.json (P076). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="176" customHeight="1">
@@ -9168,13 +9176,13 @@
         <x:v>Soft likelihood</x:v>
       </x:c>
       <x:c r="O80" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P80" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="Q80" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="R80" s="75" t="str">
         <x:v>No</x:v>
@@ -9201,7 +9209,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z80" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA80" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9219,7 +9227,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/25869dbf7682272357bc2cbbf860e1c8-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF80" s="75" t="str">
-        <x:v>Major threat to broad universal-blind claims | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. When is a convolutional proxy insufficient for nonlinear or codec degradation, and how are ambiguity and correction bias assessed? Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/25869dbf7682272357bc2cbbf860e1c8-Abstract-Conference.html</x:v>
+        <x:v>Major threat to broad universal-blind claims | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. When is a convolutional proxy insufficient for nonlinear or codec degradation, and how are ambiguity and correction bias assessed? Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/25869dbf7682272357bc2cbbf860e1c8-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_05.json (P079). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="81" ht="176" customHeight="1">
@@ -9367,7 +9375,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="P82" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="Q82" s="75" t="str">
         <x:v>No</x:v>
@@ -9376,13 +9384,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="S82" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="T82" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U82" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V82" s="75" t="str">
         <x:v>No</x:v>
@@ -9397,7 +9405,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z82" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA82" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9415,7 +9423,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/b213d9a999b82cb6fcd03a0d5a7498be-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF82" s="75" t="str">
-        <x:v>Efficient diffusion restoration baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. What training is required per degradation, and are unseen operators or joint acquisition errors evaluated independently? Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/b213d9a999b82cb6fcd03a0d5a7498be-Abstract-Conference.html</x:v>
+        <x:v>Efficient diffusion restoration baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. What training is required per degradation, and are unseen operators or joint acquisition errors evaluated independently? Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/b213d9a999b82cb6fcd03a0d5a7498be-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_05.json (P081). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="176" customHeight="1">
@@ -9569,13 +9577,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="R84" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="S84" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="T84" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U84" s="75" t="str">
         <x:v>No</x:v>
@@ -9593,7 +9601,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z84" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA84" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9611,7 +9619,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/hash/3fa2d2b637122007845a2fbb7c21453b-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF84" s="75" t="str">
-        <x:v>Important theoretical robustness comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Specify whether robustness concerns score/sampling approximation, physical-operator error or both; do not interpret the title as arbitrary acquisition-mismatch tolerance. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/3fa2d2b637122007845a2fbb7c21453b-Abstract-Conference.html</x:v>
+        <x:v>Important theoretical robustness comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Specify whether robustness concerns score/sampling approximation, physical-operator error or both; do not interpret the title as arbitrary acquisition-mismatch tolerance. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/hash/3fa2d2b637122007845a2fbb7c21453b-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, X. Evidence/version/read extent: screening/full_text_05.json (P083). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="176" customHeight="1">
@@ -9765,23 +9773,23 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="R86" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S86" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T86" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U86" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V86" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W86" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="S86" s="75" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T86" s="75" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U86" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V86" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W86" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
       <x:c r="X86" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
@@ -9789,7 +9797,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z86" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA86" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9807,7 +9815,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2025/hash/33367b9ff199d26280db6cf539d1125c-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="AF86" s="75" t="str">
-        <x:v>Strong operator-conditioned posterior baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Distinguish a supplied new operator from blind estimation and uncertainty over operators; extract adaptation cost, posterior accuracy and out-of-family tests. Evidence: https://proceedings.neurips.cc/paper_files/paper/2025/hash/33367b9ff199d26280db6cf539d1125c-Abstract-Conference.html</x:v>
+        <x:v>Strong operator-conditioned posterior baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete official NeurIPS abstract. Feature codes remain provisional. Distinguish a supplied new operator from blind estimation and uncertainty over operators; extract adaptation cost, posterior accuracy and out-of-family tests. Evidence: https://proceedings.neurips.cc/paper_files/paper/2025/hash/33367b9ff199d26280db6cf539d1125c-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, W, X. Evidence/version/read extent: screening/full_text_05.json (P085). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="87" ht="176" customHeight="1">
@@ -10309,7 +10317,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab9f73b43ca2401d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R479497caaadf41c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10821,7 +10829,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="84" customHeight="1">
+    <x:row r="13" ht="144" customHeight="1">
       <x:c r="A13" s="73" t="str">
         <x:v>S012</x:v>
       </x:c>
@@ -10844,15 +10852,15 @@
       <x:c r="H13" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I13" s="76" t="str">
+      <x:c r="I13" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J13" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K13" s="75"/>
+      <x:c r="J13" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K13" s="75" t="str"/>
       <x:c r="L13" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Posterior reconstruction and transfer across image distributions. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P012).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Reconstruction posterior and content transfer; §§3 and 5.3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P012).</x:v>
       </x:c>
       <x:c r="M13" s="75" t="str">
         <x:v>No</x:v>
@@ -11141,7 +11149,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="84" customHeight="1">
+    <x:row r="21" ht="144" customHeight="1">
       <x:c r="A21" s="73" t="str">
         <x:v>S020</x:v>
       </x:c>
@@ -11164,15 +11172,15 @@
       <x:c r="H21" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I21" s="76" t="str">
+      <x:c r="I21" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J21" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K21" s="75"/>
+      <x:c r="J21" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K21" s="75" t="str"/>
       <x:c r="L21" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Unknown degradation types and levels. Basis: Official proceedings abstract. Full-text question and source: screening/pilot_01.json (P020).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown degradation prompts and held-out noise strength; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P020).</x:v>
       </x:c>
       <x:c r="M21" s="75" t="str">
         <x:v>No</x:v>
@@ -13326,15 +13334,15 @@
       <x:c r="H75" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I75" s="91" t="str">
+      <x:c r="I75" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J75" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K75" s="75"/>
+      <x:c r="J75" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K75" s="75" t="str"/>
       <x:c r="L75" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Unknown-degradation representation for unified restoration. Basis: Complete author abstract, project page and official ICLR slides title. Sources and full-text question: screening/pilot_03.json (P074).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown-degradation embeddings and OOD example; §§3 and 5.2. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P074).</x:v>
       </x:c>
       <x:c r="M75" s="75" t="str">
         <x:v>No</x:v>
@@ -13366,15 +13374,15 @@
       <x:c r="H76" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I76" s="91" t="str">
+      <x:c r="I76" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J76" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K76" s="75"/>
+      <x:c r="J76" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K76" s="75" t="str"/>
       <x:c r="L76" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Adaptive all-in-one restoration with unseen-task transfer. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P075).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Compound and unseen restoration tasks; §4.1. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P075).</x:v>
       </x:c>
       <x:c r="M76" s="75" t="str">
         <x:v>No</x:v>
@@ -13406,15 +13414,15 @@
       <x:c r="H77" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I77" s="91" t="str">
+      <x:c r="I77" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J77" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K77" s="75"/>
+      <x:c r="J77" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K77" s="75" t="str"/>
       <x:c r="L77" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Instruction-conditioned restoration across unknown degradation types. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P076).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown and compound corruption examples; §5. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P076).</x:v>
       </x:c>
       <x:c r="M77" s="75" t="str">
         <x:v>No</x:v>
@@ -13526,15 +13534,15 @@
       <x:c r="H80" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I80" s="91" t="str">
+      <x:c r="I80" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J80" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K80" s="75"/>
+      <x:c r="J80" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K80" s="75" t="str"/>
       <x:c r="L80" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind operator adaptation for universal compound restoration. Basis: Complete official NeurIPS abstract. Sources and full-text question: screening/pilot_03.json (P079).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Joint unknown degradation estimation; §§4.1–4.3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P079).</x:v>
       </x:c>
       <x:c r="M80" s="75" t="str">
         <x:v>No</x:v>
@@ -13606,15 +13614,15 @@
       <x:c r="H82" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I82" s="91" t="str">
+      <x:c r="I82" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J82" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K82" s="75"/>
+      <x:c r="J82" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K82" s="75" t="str"/>
       <x:c r="L82" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind and compound image reconstruction with modular task conditioning. Basis: Complete official NeurIPS abstract. Sources and full-text question: screening/pilot_03.json (P081).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Conditional image sampling and cross-dataset evaluation; §§3–4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P081).</x:v>
       </x:c>
       <x:c r="M82" s="75" t="str">
         <x:v>No</x:v>
@@ -13686,15 +13694,15 @@
       <x:c r="H84" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I84" s="91" t="str">
+      <x:c r="I84" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J84" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K84" s="75"/>
+      <x:c r="J84" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K84" s="75" t="str"/>
       <x:c r="L84" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Reconstruction posterior sampling with approximation-robustness guarantees. Basis: Complete official NeurIPS abstract. Sources and full-text question: screening/pilot_03.json (P083).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Reconstruction uncertainty and robustness to sampler errors; §4. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P083).</x:v>
       </x:c>
       <x:c r="M84" s="75" t="str">
         <x:v>No</x:v>
@@ -13766,15 +13774,15 @@
       <x:c r="H86" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I86" s="91" t="str">
+      <x:c r="I86" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J86" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K86" s="75"/>
+      <x:c r="J86" s="102" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K86" s="75" t="str"/>
       <x:c r="L86" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Operator-conditioned posterior reconstruction and test-time operator adaptation. Basis: Complete official NeurIPS abstract. Sources and full-text question: screening/pilot_03.json (P085).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unseen degradation and posterior uncertainty; §§4.1 and 5. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_05.json (P085).</x:v>
       </x:c>
       <x:c r="M86" s="75" t="str">
         <x:v>No</x:v>
@@ -14284,7 +14292,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8cb04d2cc53f4aa7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a8a77aa63404d7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14456,7 +14464,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 44 (43 include, 1 exclude), 46 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 53 (52 include, 1 exclude), 37 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14464,7 +14472,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json and full_text_04.json; current report: full_text_04_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json and full_text_05.json; current report: full_text_05_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14710,7 +14718,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra06921c3647e4131"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R679ae5d18fa04456"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Complete sixth full-text checkpoint: 60 of 90 assessed
Add seven AI eligibility recommendations with inspected source versions,
criterion-level evidence and selected verified feature fields. Record existing
instability, semantic fidelity, temporal degradation and rollback comparisons.
Keep the candidate question active and novelty unestablished.

Identify 2020 journal lineages for inspected older NETT and instability
preprints; keep final-version reconciliation and quality checks explicit.
Record failed retrievals without converting access failures into exclusions.

Synchronize the matrix, screening tracker and 90-reference exports. Validate
formula behavior, stable metadata, native workbook objects and rendered ranges.
Preserve earlier decisions, formal counters, protocol v0.4 and deferred tasks.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4ba967359d7047ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="Rb65840ecf5834775"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rb5edd1a151134b69"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R1f3fc200161d40b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rc86cd4fbe519418b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd75476c9d9f14975"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R617393fd5885427a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R684ee4f0856e4b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R426c335b089a4d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R802fa62a3cfc4e97"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="20">
+  <x:fills count="21">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -272,7 +277,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="103">
+  <x:cellXfs count="104">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -496,6 +501,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -729,7 +737,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0c933de7139a4337"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8e45c9c83fa84094"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1178,7 +1186,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1195,7 +1203,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>Unknown-degradation prompts, compound restoration, operator conditioning and image posterior sampling have existing comparators. See screening/full_text_05_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
+        <x:v>Instability tests, semantic fidelity, temporal compound restoration and restoration rollback have existing comparators. See screening/full_text_06_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1250,7 +1258,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 53/90 (52 include, 1 exclude); 37 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 60/90 (59 include, 1 exclude); 30 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1345,7 +1353,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra13e6d20e5364836"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5610e083fbcc4dc0"/>
 </x:worksheet>
 </file>
 
@@ -1586,200 +1594,200 @@
         <x:v>Cornerstone mismatch paper | AI pilot 2026-09-16; advance to full text. Kernel/model uncertainty. Human adjudication and full-text coding pending. Evidence: https://github.com/ysnan/NBD_KerUnc | Batch 03 revisit 2026-09-16: Keep the prior title/project-based advancement; full technical evidence remains pending. Do not upgrade feature codes from search snippets. Source: https://github.com/ysnan/NBD_KerUnc</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="7" t="str">
+    <x:row r="3" ht="176" customHeight="1">
+      <x:c r="A3" s="85" t="str">
         <x:v>P002</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="n">
+      <x:c r="B3" s="86" t="n">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="C3" s="9" t="str">
+      <x:c r="C3" s="75" t="str">
         <x:v>Li et al.</x:v>
       </x:c>
-      <x:c r="D3" s="9" t="str">
+      <x:c r="D3" s="75" t="str">
         <x:v>NETT: Solving Inverse Problems with Deep Neural Networks</x:v>
       </x:c>
-      <x:c r="E3" s="9" t="str">
+      <x:c r="E3" s="75" t="str">
         <x:v>Inverse Problems</x:v>
       </x:c>
-      <x:c r="F3" s="9" t="str">
+      <x:c r="F3" s="75" t="str">
         <x:v>Journal</x:v>
       </x:c>
-      <x:c r="G3" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H3" s="9" t="str">
+      <x:c r="G3" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H3" s="75" t="str">
         <x:v>Tomography/inverse imaging</x:v>
       </x:c>
-      <x:c r="I3" s="9" t="str">
+      <x:c r="I3" s="75" t="str">
         <x:v>Scientific imaging</x:v>
       </x:c>
-      <x:c r="J3" s="9" t="str">
+      <x:c r="J3" s="75" t="str">
         <x:v>Generic operator</x:v>
       </x:c>
-      <x:c r="K3" s="9" t="str">
+      <x:c r="K3" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L3" s="9" t="str">
+      <x:c r="L3" s="75" t="str">
         <x:v>None central</x:v>
       </x:c>
-      <x:c r="M3" s="9" t="str">
+      <x:c r="M3" s="75" t="str">
         <x:v>Learned regularisation</x:v>
       </x:c>
-      <x:c r="N3" s="9" t="str">
+      <x:c r="N3" s="75" t="str">
         <x:v>Soft/variational</x:v>
       </x:c>
-      <x:c r="O3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S3" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="T3" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y3" s="9" t="str">
+      <x:c r="O3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S3" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y3" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="Z3" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA3" s="9" t="str">
+      <x:c r="Z3" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA3" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB3" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC3" s="9" t="str">
+      <x:c r="AB3" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC3" s="75" t="str">
         <x:v>Learned regulariser with convergence analysis</x:v>
       </x:c>
-      <x:c r="AD3" s="9" t="str">
+      <x:c r="AD3" s="75" t="str">
         <x:v>Not a joint mismatch/UQ/failure system</x:v>
       </x:c>
-      <x:c r="AE3" s="9" t="str">
+      <x:c r="AE3" s="75" t="str">
         <x:v>https://doi.org/10.1088/1361-6420/ab6d57</x:v>
       </x:c>
-      <x:c r="AF3" s="9" t="str">
-        <x:v>Theoretical physics-informed baseline | AI pilot 2026-09-16; advance to full text. Potential OOD reconstruction reliability. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/1803.00092</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="7" t="str">
+      <x:c r="AF3" s="75" t="str">
+        <x:v>Theoretical physics-informed baseline | AI pilot 2026-09-16; advance to full text. Potential OOD reconstruction reliability. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/1803.00092 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_06.json (P002). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="176" customHeight="1">
+      <x:c r="A4" s="85" t="str">
         <x:v>P003</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="n">
+      <x:c r="B4" s="86" t="n">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="C4" s="9" t="str">
+      <x:c r="C4" s="75" t="str">
         <x:v>Antun et al.</x:v>
       </x:c>
-      <x:c r="D4" s="9" t="str">
+      <x:c r="D4" s="75" t="str">
         <x:v>On Instabilities of Deep Learning in Image Reconstruction and the Potential Costs of AI</x:v>
       </x:c>
-      <x:c r="E4" s="9" t="str">
+      <x:c r="E4" s="75" t="str">
         <x:v>PNAS</x:v>
       </x:c>
-      <x:c r="F4" s="9" t="str">
+      <x:c r="F4" s="75" t="str">
         <x:v>Journal</x:v>
       </x:c>
-      <x:c r="G4" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H4" s="9" t="str">
+      <x:c r="G4" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H4" s="75" t="str">
         <x:v>MRI/CT</x:v>
       </x:c>
-      <x:c r="I4" s="9" t="str">
+      <x:c r="I4" s="75" t="str">
         <x:v>Medical imaging</x:v>
       </x:c>
-      <x:c r="J4" s="9" t="str">
+      <x:c r="J4" s="75" t="str">
         <x:v>Sampling operator</x:v>
       </x:c>
-      <x:c r="K4" s="9" t="str">
+      <x:c r="K4" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L4" s="9" t="str">
+      <x:c r="L4" s="75" t="str">
         <x:v>Perturbation/structural shift</x:v>
       </x:c>
-      <x:c r="M4" s="9" t="str">
+      <x:c r="M4" s="75" t="str">
         <x:v>Diagnostic study</x:v>
       </x:c>
-      <x:c r="N4" s="9" t="str">
+      <x:c r="N4" s="75" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="O4" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P4" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q4" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R4" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S4" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T4" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="U4" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V4" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W4" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="X4" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y4" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z4" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA4" s="9" t="str">
+      <x:c r="O4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S4" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W4" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X4" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y4" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z4" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA4" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB4" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC4" s="9" t="str">
+      <x:c r="AB4" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC4" s="75" t="str">
         <x:v>Demonstrates severe instability and missing structures</x:v>
       </x:c>
-      <x:c r="AD4" s="9" t="str">
+      <x:c r="AD4" s="75" t="str">
         <x:v>Diagnoses risk but does not build a unified corrective solver</x:v>
       </x:c>
-      <x:c r="AE4" s="9" t="str">
+      <x:c r="AE4" s="75" t="str">
         <x:v>https://doi.org/10.1073/pnas.1907377117</x:v>
       </x:c>
-      <x:c r="AF4" s="9" t="str">
-        <x:v>Reliability foundation | AI pilot 2026-09-16; advance to full text. Reconstruction instability and missing structure. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/1902.05300</x:v>
+      <x:c r="AF4" s="75" t="str">
+        <x:v>Reliability foundation | AI pilot 2026-09-16; advance to full text. Reconstruction instability and missing structure. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/1902.05300 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_06.json (P003). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4134,7 +4142,7 @@
         <x:v>Codec evidence | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Official BMVC proceedings abstract and citation. Feature codes remain provisional. Can its codec transfer protocol support a controlled degradation-shift experiment? It studies bitrate reduction, not forensic reconstruction. The former arXiv URL was an unrelated SLAM paper. Evidence: https://bmvc2024.org/proceedings/959/</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="112" customHeight="1">
+    <x:row r="29" ht="176" customHeight="1">
       <x:c r="A29" s="85" t="str">
         <x:v>P028</x:v>
       </x:c>
@@ -4202,7 +4210,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="W29" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="X29" s="75" t="str">
         <x:v>No</x:v>
@@ -4211,7 +4219,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z29" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA29" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4229,7 +4237,7 @@
         <x:v>https://arxiv.org/abs/2401.13627</x:v>
       </x:c>
       <x:c r="AF29" s="75" t="str">
-        <x:v>Generative baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract with CVPR acceptance identified. Feature codes remain provisional. How do prompts and prior strength affect invented detail? Extract quantitative fidelity tests and inference costs before choosing a baseline. Evidence: https://arxiv.org/abs/2401.13627</x:v>
+        <x:v>Generative baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract with CVPR acceptance identified. Feature codes remain provisional. How do prompts and prior strength affect invented detail? Extract quantitative fidelity tests and inference costs before choosing a baseline. Evidence: https://arxiv.org/abs/2401.13627 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, T, U, W, X. Evidence/version/read extent: screening/full_text_06.json (P028). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="112" customHeight="1">
@@ -8327,7 +8335,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z71" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA71" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8345,7 +8353,7 @@
         <x:v>https://arxiv.org/abs/2507.14851</x:v>
       </x:c>
       <x:c r="AF71" s="75" t="str">
-        <x:v>Closest prompt-conditioned compound-video competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; seed WACV venue not independently rechecked. Feature codes remain provisional. Extract the exact held-out combinations, temporal changes and inference inputs. Natural-language guidance plus changing compound degradation is an existing direction. Evidence: https://arxiv.org/abs/2507.14851</x:v>
+        <x:v>Closest prompt-conditioned compound-video competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; seed WACV venue not independently rechecked. Feature codes remain provisional. Extract the exact held-out combinations, temporal changes and inference inputs. Natural-language guidance plus changing compound degradation is an existing direction. Evidence: https://arxiv.org/abs/2507.14851 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_06.json (P070). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="72" ht="176" customHeight="1">
@@ -8980,7 +8988,7 @@
         <x:v>Implicit</x:v>
       </x:c>
       <x:c r="O78" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="P78" s="75" t="str">
         <x:v>No</x:v>
@@ -8995,7 +9003,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T78" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U78" s="75" t="str">
         <x:v>Yes</x:v>
@@ -9013,7 +9021,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z78" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA78" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9031,7 +9039,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/file/c78f639424b8d89ceb4f2efbb4dfe4f4-Paper-Conference.pdf</x:v>
       </x:c>
       <x:c r="AF78" s="75" t="str">
-        <x:v>Closest modular compound-restoration planner | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Official NeurIPS PDF abstract and opening page. Feature codes remain provisional. How are tool-order decisions evaluated, and can the controller reject unsupported enhancement? Reported quality or expert comparisons are author results, not independent validation. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/file/c78f639424b8d89ceb4f2efbb4dfe4f4-Paper-Conference.pdf</x:v>
+        <x:v>Closest modular compound-restoration planner | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Official NeurIPS PDF abstract and opening page. Feature codes remain provisional. How are tool-order decisions evaluated, and can the controller reject unsupported enhancement? Reported quality or expert comparisons are author results, not independent validation. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/file/c78f639424b8d89ceb4f2efbb4dfe4f4-Paper-Conference.pdf | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_06.json (P077). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="176" customHeight="1">
@@ -9102,7 +9110,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="W79" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="X79" s="75" t="str">
         <x:v>No</x:v>
@@ -9111,7 +9119,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z79" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA79" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -9129,7 +9137,7 @@
         <x:v>https://proceedings.neurips.cc/paper_files/paper/2024/file/6452474601429509f3035dc81c233226-Paper-Conference.pdf</x:v>
       </x:c>
       <x:c r="AF79" s="75" t="str">
-        <x:v>Generative fidelity-risk baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; seed proceedings PDF retrieval failed. Feature codes remain provisional. Verify degradation composition and real-data transfer. Dataset-generation or semantic-quality claims do not establish reconstruction uncertainty or recovered truth. Evidence: https://arxiv.org/abs/2410.18666</x:v>
+        <x:v>Generative fidelity-risk baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; seed proceedings PDF retrieval failed. Feature codes remain provisional. Verify degradation composition and real-data transfer. Dataset-generation or semantic-quality claims do not establish reconstruction uncertainty or recovered truth. Evidence: https://arxiv.org/abs/2410.18666 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, T, U, W, X. Evidence/version/read extent: screening/full_text_06.json (P078). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="80" ht="176" customHeight="1">
@@ -10189,7 +10197,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z90" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA90" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -10207,7 +10215,7 @@
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Wu_SeeSR_Towards_Semantics-Aware_Real-World_Image_Super-Resolution_CVPR_2024_paper.html</x:v>
       </x:c>
       <x:c r="AF90" s="75" t="str">
-        <x:v>Critical hallucination-risk baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract with CVPR acceptance note. Feature codes remain provisional. How is semantic fidelity evaluated when the input is ambiguous? Reduced semantic error does not establish calibrated uncertainty or measurement support for every generated detail. Evidence: https://arxiv.org/abs/2311.16518</x:v>
+        <x:v>Critical hallucination-risk baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract with CVPR acceptance note. Feature codes remain provisional. How is semantic fidelity evaluated when the input is ambiguous? Reduced semantic error does not establish calibrated uncertainty or measurement support for every generated detail. Evidence: https://arxiv.org/abs/2311.16518 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, T, U, W, X. Evidence/version/read extent: screening/full_text_06.json (P089). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="91" ht="176" customHeight="1">
@@ -10317,7 +10325,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R479497caaadf41c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf30335e755b14f6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10429,7 +10437,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="84" customHeight="1">
+    <x:row r="3" ht="144" customHeight="1">
       <x:c r="A3" s="73" t="str">
         <x:v>S002</x:v>
       </x:c>
@@ -10452,15 +10460,15 @@
       <x:c r="H3" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I3" s="76" t="str">
+      <x:c r="I3" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J3" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K3" s="75"/>
+      <x:c r="J3" s="103" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K3" s="75" t="str"/>
       <x:c r="L3" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Potential OOD reconstruction reliability. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P002).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. OOD phantom reconstruction; §5.3. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_06.json (P002).</x:v>
       </x:c>
       <x:c r="M3" s="75" t="str">
         <x:v>No</x:v>
@@ -10469,7 +10477,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="84" customHeight="1">
+    <x:row r="4" ht="144" customHeight="1">
       <x:c r="A4" s="73" t="str">
         <x:v>S003</x:v>
       </x:c>
@@ -10492,15 +10500,15 @@
       <x:c r="H4" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I4" s="76" t="str">
+      <x:c r="I4" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J4" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K4" s="75"/>
+      <x:c r="J4" s="103" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K4" s="75" t="str"/>
       <x:c r="L4" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Reconstruction instability and missing structure. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P003).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Reconstruction instability and altered sampling tests. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_06.json (P003).</x:v>
       </x:c>
       <x:c r="M4" s="75" t="str">
         <x:v>No</x:v>
@@ -11469,7 +11477,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="112" customHeight="1">
+    <x:row r="29" ht="144" customHeight="1">
       <x:c r="A29" s="73" t="str">
         <x:v>S028</x:v>
       </x:c>
@@ -11492,15 +11500,15 @@
       <x:c r="H29" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I29" s="81" t="str">
+      <x:c r="I29" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J29" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K29" s="75"/>
+      <x:c r="J29" s="103" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K29" s="75" t="str"/>
       <x:c r="L29" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Generative restoration of unknown real-world degradation. Basis: Author preprint abstract with CVPR acceptance identified. Sources and full-text question: screening/pilot_02.json (P028).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Blind compound restoration and qualitative hallucination analysis. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_06.json (P028).</x:v>
       </x:c>
       <x:c r="M29" s="75" t="str">
         <x:v>No</x:v>
@@ -13174,15 +13182,15 @@
       <x:c r="H71" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I71" s="91" t="str">
+      <x:c r="I71" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J71" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K71" s="75"/>
+      <x:c r="J71" s="103" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K71" s="75" t="str"/>
       <x:c r="L71" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Multi-degradation and time-varying compound video restoration. Basis: Complete author preprint abstract; seed WACV venue not independently rechecked. Sources and full-text question: screening/pilot_03.json (P070).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Compound and temporally varying video degradation. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_06.json (P070).</x:v>
       </x:c>
       <x:c r="M71" s="75" t="str">
         <x:v>No</x:v>
@@ -13454,15 +13462,15 @@
       <x:c r="H78" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I78" s="91" t="str">
+      <x:c r="I78" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J78" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K78" s="75"/>
+      <x:c r="J78" s="103" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K78" s="75" t="str"/>
       <x:c r="L78" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Identification and ordered treatment of compound image degradation. Basis: Official NeurIPS PDF abstract and opening page. Sources and full-text question: screening/pilot_03.json (P077).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown compound degradation and restoration rollback. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_06.json (P077).</x:v>
       </x:c>
       <x:c r="M78" s="75" t="str">
         <x:v>No</x:v>
@@ -13494,15 +13502,15 @@
       <x:c r="H79" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I79" s="91" t="str">
+      <x:c r="I79" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J79" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K79" s="75"/>
+      <x:c r="J79" s="103" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K79" s="75" t="str"/>
       <x:c r="L79" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Generative real-world restoration with degradation-aware conditioning. Basis: Complete author preprint abstract; seed proceedings PDF retrieval failed. Sources and full-text question: screening/pilot_03.json (P078).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Compound restoration with real-image and semantic evaluation. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_06.json (P078).</x:v>
       </x:c>
       <x:c r="M79" s="75" t="str">
         <x:v>No</x:v>
@@ -13934,15 +13942,15 @@
       <x:c r="H90" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I90" s="91" t="str">
+      <x:c r="I90" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J90" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K90" s="75"/>
+      <x:c r="J90" s="103" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K90" s="75" t="str"/>
       <x:c r="L90" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Semantic errors in blind generative super-resolution. Basis: Complete author preprint abstract with CVPR acceptance note. Sources and full-text question: screening/pilot_03.json (P089).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Blind compound restoration and false-detail analysis. Online text inspected; no local PDF saved. Version, read extent and technical extraction: screening/full_text_06.json (P089).</x:v>
       </x:c>
       <x:c r="M90" s="75" t="str">
         <x:v>No</x:v>
@@ -14292,7 +14300,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a8a77aa63404d7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53f6e3f6be384f59"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14464,7 +14472,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 53 (52 include, 1 exclude), 37 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 60 (59 include, 1 exclude), 30 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14472,7 +14480,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json and full_text_05.json; current report: full_text_05_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json and full_text_06.json; current report: full_text_06_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14718,7 +14726,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R679ae5d18fa04456"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16ddbd596d6743a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record full-text checkpoint 07: 70 assessed, 20 remaining
Assess ten additional seed papers under protocol v0.4 with criterion-level evidence, inspected versions and bounded feature verification. Record seven PDF acquisitions and source hashes without redistributing papers.

Synchronize the matrix, tracker and four reference exports. Preserve all 90 IDs, earlier decisions, formal counts and workbook objects. Counts, formula behavior, unchanged fields, reference metadata and visual layout verified.

Novelty and human inclusion decisions remain outstanding.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd75476c9d9f14975"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R617393fd5885427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R684ee4f0856e4b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R426c335b089a4d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R802fa62a3cfc4e97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R75abcb387aa5413c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="Rf7a0bb1548dd4da6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R627a854183f744cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="Ra1c5f724854f4b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rb2d7ff5668eb4a60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="21">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -277,7 +282,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="104">
+  <x:cellXfs count="105">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -504,6 +509,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -737,7 +745,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8e45c9c83fa84094"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc3affe20faef43e5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1186,7 +1194,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>60</x:v>
+        <x:v>70</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1203,7 +1211,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>Instability tests, semantic fidelity, temporal compound restoration and restoration rollback have existing comparators. See screening/full_text_06_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
+        <x:v>Residual mismatch compensation, joint blind estimation, null-space theory and generative fidelity control have existing comparators. See screening/full_text_07_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1258,7 +1266,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 60/90 (59 include, 1 exclude); 30 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 70/90 (69 include, 1 exclude); 20 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1353,7 +1361,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5610e083fbcc4dc0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R965f00081e2347fd"/>
 </x:worksheet>
 </file>
 
@@ -1496,102 +1504,102 @@
         <x:v>Review notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="240" customHeight="1">
-      <x:c r="A2" s="7" t="str">
+    <x:row r="2" ht="176" customHeight="1">
+      <x:c r="A2" s="85" t="str">
         <x:v>P001</x:v>
       </x:c>
-      <x:c r="B2" s="8" t="n">
+      <x:c r="B2" s="86" t="n">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="C2" s="9" t="str">
+      <x:c r="C2" s="75" t="str">
         <x:v>Nan, Yuesong; Ji, Hui</x:v>
       </x:c>
-      <x:c r="D2" s="9" t="str">
+      <x:c r="D2" s="75" t="str">
         <x:v>Deep Learning for Handling Kernel/Model Uncertainty in Image Deconvolution</x:v>
       </x:c>
-      <x:c r="E2" s="9" t="str">
+      <x:c r="E2" s="75" t="str">
         <x:v>CVPR</x:v>
       </x:c>
-      <x:c r="F2" s="9" t="str">
+      <x:c r="F2" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G2" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H2" s="9" t="str">
+      <x:c r="G2" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H2" s="75" t="str">
         <x:v>Deblurring</x:v>
       </x:c>
-      <x:c r="I2" s="9" t="str">
+      <x:c r="I2" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J2" s="9" t="str">
+      <x:c r="J2" s="75" t="str">
         <x:v>Convolutional blur</x:v>
       </x:c>
-      <x:c r="K2" s="9" t="str">
+      <x:c r="K2" s="75" t="str">
         <x:v>Approximate</x:v>
       </x:c>
-      <x:c r="L2" s="9" t="str">
+      <x:c r="L2" s="75" t="str">
         <x:v>Kernel/model error</x:v>
       </x:c>
-      <x:c r="M2" s="9" t="str">
+      <x:c r="M2" s="75" t="str">
         <x:v>Deep TLS unrolling</x:v>
       </x:c>
-      <x:c r="N2" s="9" t="str">
+      <x:c r="N2" s="75" t="str">
         <x:v>Hard/iterative</x:v>
       </x:c>
-      <x:c r="O2" s="9" t="str">
+      <x:c r="O2" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P2" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q2" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R2" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S2" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="P2" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q2" s="9" t="str">
+      <x:c r="T2" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U2" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V2" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W2" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="R2" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S2" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T2" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U2" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V2" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W2" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X2" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y2" s="9" t="str">
+      <x:c r="X2" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y2" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="Z2" s="9" t="str">
-        <x:v>Title/project checked; abstract pending</x:v>
-      </x:c>
-      <x:c r="AA2" s="9" t="str">
+      <x:c r="Z2" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA2" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB2" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC2" s="9" t="str">
+      <x:c r="AB2" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC2" s="75" t="str">
         <x:v>Error-in-variables unrolling for inaccurate kernels</x:v>
       </x:c>
-      <x:c r="AD2" s="9" t="str">
+      <x:c r="AD2" s="75" t="str">
         <x:v>No joint calibrated image/operator uncertainty; no compound acquisition chain</x:v>
       </x:c>
-      <x:c r="AE2" s="9" t="str">
+      <x:c r="AE2" s="75" t="str">
         <x:v>https://doi.org/10.1109/CVPR42600.2020.00246</x:v>
       </x:c>
       <x:c r="AF2" s="75" t="str">
-        <x:v>Cornerstone mismatch paper | AI pilot 2026-09-16; advance to full text. Kernel/model uncertainty. Human adjudication and full-text coding pending. Evidence: https://github.com/ysnan/NBD_KerUnc | Batch 03 revisit 2026-09-16: Keep the prior title/project-based advancement; full technical evidence remains pending. Do not upgrade feature codes from search snippets. Source: https://github.com/ysnan/NBD_KerUnc</x:v>
+        <x:v>Cornerstone mismatch paper | AI pilot 2026-09-16; advance to full text. Kernel/model uncertainty. Human adjudication and full-text coding pending. Evidence: https://github.com/ysnan/NBD_KerUnc | Batch 03 revisit 2026-09-16: Keep the prior title/project-based advancement; full technical evidence remains pending. Do not upgrade feature codes from search snippets. Source: https://github.com/ysnan/NBD_KerUnc | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_07.json (P001). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="176" customHeight="1">
@@ -1790,102 +1798,102 @@
         <x:v>Reliability foundation | AI pilot 2026-09-16; advance to full text. Reconstruction instability and missing structure. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/1902.05300 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_06.json (P003). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="7" t="str">
+    <x:row r="5" ht="176" customHeight="1">
+      <x:c r="A5" s="85" t="str">
         <x:v>P004</x:v>
       </x:c>
-      <x:c r="B5" s="8" t="n">
+      <x:c r="B5" s="86" t="n">
         <x:v>2020</x:v>
       </x:c>
-      <x:c r="C5" s="9" t="str">
+      <x:c r="C5" s="75" t="str">
         <x:v>Rim, Jaesung; Lee, Haeyun; Won, Jucheol; Cho, Sunghyun</x:v>
       </x:c>
-      <x:c r="D5" s="9" t="str">
+      <x:c r="D5" s="75" t="str">
         <x:v>Real-World Blur Dataset for Learning and Benchmarking Deblurring Algorithms</x:v>
       </x:c>
-      <x:c r="E5" s="9" t="str">
+      <x:c r="E5" s="75" t="str">
         <x:v>ECCV</x:v>
       </x:c>
-      <x:c r="F5" s="9" t="str">
+      <x:c r="F5" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G5" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H5" s="9" t="str">
+      <x:c r="G5" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H5" s="75" t="str">
         <x:v>Deblurring</x:v>
       </x:c>
-      <x:c r="I5" s="9" t="str">
+      <x:c r="I5" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J5" s="9" t="str">
+      <x:c r="J5" s="75" t="str">
         <x:v>Camera motion blur</x:v>
       </x:c>
-      <x:c r="K5" s="9" t="str">
+      <x:c r="K5" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="L5" s="9" t="str">
+      <x:c r="L5" s="75" t="str">
         <x:v>Real blur</x:v>
       </x:c>
-      <x:c r="M5" s="9" t="str">
+      <x:c r="M5" s="75" t="str">
         <x:v>Dataset/benchmark</x:v>
       </x:c>
-      <x:c r="N5" s="9" t="str">
+      <x:c r="N5" s="75" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="O5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S5" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="T5" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="U5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y5" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z5" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA5" s="9" t="str">
+      <x:c r="O5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S5" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T5" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U5" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y5" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z5" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA5" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB5" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC5" s="9" t="str">
+      <x:c r="AB5" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC5" s="75" t="str">
         <x:v>Paired real blurred and sharp images</x:v>
       </x:c>
-      <x:c r="AD5" s="9" t="str">
+      <x:c r="AD5" s="75" t="str">
         <x:v>Blur-specific; no full surveillance pipeline or UQ</x:v>
       </x:c>
-      <x:c r="AE5" s="9" t="str">
+      <x:c r="AE5" s="75" t="str">
         <x:v>https://doi.org/10.1007/978-3-030-58595-2_12</x:v>
       </x:c>
-      <x:c r="AF5" s="9" t="str">
-        <x:v>Data source candidate | AI pilot 2026-09-16; advance to full text. Real blur and synthetic-to-real degradation gap. Human adjudication and full-text coding pending. Evidence: https://link.springer.com/chapter/10.1007/978-3-030-58595-2_12</x:v>
+      <x:c r="AF5" s="75" t="str">
+        <x:v>Data source candidate | AI pilot 2026-09-16; advance to full text. Real blur and synthetic-to-real degradation gap. Human adjudication and full-text coding pending. Evidence: https://link.springer.com/chapter/10.1007/978-3-030-58595-2_12 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_07.json (P004). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="176" customHeight="1">
@@ -2280,102 +2288,102 @@
         <x:v>Faithfulness foundation | AI pilot 2026-09-16; advance to full text. Hallucination and measurement/null-space analysis. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2012.00646 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, W, X. Evidence/version/read extent: screening/full_text_04.json (P008). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="7" t="str">
+    <x:row r="10" ht="176" customHeight="1">
+      <x:c r="A10" s="85" t="str">
         <x:v>P009</x:v>
       </x:c>
-      <x:c r="B10" s="8" t="n">
+      <x:c r="B10" s="86" t="n">
         <x:v>2021</x:v>
       </x:c>
-      <x:c r="C10" s="9" t="str">
+      <x:c r="C10" s="75" t="str">
         <x:v>Zhang et al.</x:v>
       </x:c>
-      <x:c r="D10" s="9" t="str">
+      <x:c r="D10" s="75" t="str">
         <x:v>Designing a Practical Degradation Model for Deep Blind Image Super-Resolution</x:v>
       </x:c>
-      <x:c r="E10" s="9" t="str">
+      <x:c r="E10" s="75" t="str">
         <x:v>ICCV</x:v>
       </x:c>
-      <x:c r="F10" s="9" t="str">
+      <x:c r="F10" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G10" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H10" s="9" t="str">
+      <x:c r="G10" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H10" s="75" t="str">
         <x:v>Super-resolution</x:v>
       </x:c>
-      <x:c r="I10" s="9" t="str">
+      <x:c r="I10" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J10" s="9" t="str">
+      <x:c r="J10" s="75" t="str">
         <x:v>Synthetic degradation chain</x:v>
       </x:c>
-      <x:c r="K10" s="9" t="str">
+      <x:c r="K10" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="L10" s="9" t="str">
+      <x:c r="L10" s="75" t="str">
         <x:v>Composite shuffled degradation</x:v>
       </x:c>
-      <x:c r="M10" s="9" t="str">
+      <x:c r="M10" s="75" t="str">
         <x:v>GAN/CNN restoration</x:v>
       </x:c>
-      <x:c r="N10" s="9" t="str">
+      <x:c r="N10" s="75" t="str">
         <x:v>Implicit</x:v>
       </x:c>
-      <x:c r="O10" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P10" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q10" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R10" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S10" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T10" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="U10" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="V10" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W10" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X10" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y10" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z10" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA10" s="9" t="str">
+      <x:c r="O10" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P10" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q10" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R10" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S10" s="75" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="T10" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U10" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V10" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W10" s="75" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="X10" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y10" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z10" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA10" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB10" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC10" s="9" t="str">
+      <x:c r="AB10" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC10" s="75" t="str">
         <x:v>Practical randomized degradation pipeline</x:v>
       </x:c>
-      <x:c r="AD10" s="9" t="str">
+      <x:c r="AD10" s="75" t="str">
         <x:v>No operator recovery, calibration, measurement support or abstention</x:v>
       </x:c>
-      <x:c r="AE10" s="9" t="str">
+      <x:c r="AE10" s="75" t="str">
         <x:v>https://openaccess.thecvf.com/content/ICCV2021/html/Zhang_Designing_a_Practical_Degradation_Model_for_Deep_Blind_Image_Super-Resolution_ICCV_2021_paper.html</x:v>
       </x:c>
-      <x:c r="AF10" s="9" t="str">
-        <x:v>Degradation simulator baseline | AI pilot 2026-09-16; advance to full text. Blind restoration with compound degradation. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2103.14006</x:v>
+      <x:c r="AF10" s="75" t="str">
+        <x:v>Degradation simulator baseline | AI pilot 2026-09-16; advance to full text. Blind restoration with compound degradation. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2103.14006 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_07.json (P009). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="176" customHeight="1">
@@ -2966,200 +2974,200 @@
         <x:v>Diffusion baseline | AI pilot 2026-09-16; advance to full text. Approximate posterior reconstruction under noise. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2209.14687 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, X. Evidence/version/read extent: screening/full_text_04.json (P015). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="240" customHeight="1">
-      <x:c r="A17" s="7" t="str">
+    <x:row r="17" ht="176" customHeight="1">
+      <x:c r="A17" s="85" t="str">
         <x:v>P016</x:v>
       </x:c>
-      <x:c r="B17" s="8" t="n">
+      <x:c r="B17" s="86" t="n">
         <x:v>2023</x:v>
       </x:c>
-      <x:c r="C17" s="9" t="str">
+      <x:c r="C17" s="75" t="str">
         <x:v>Song et al.</x:v>
       </x:c>
-      <x:c r="D17" s="9" t="str">
+      <x:c r="D17" s="75" t="str">
         <x:v>Pseudoinverse-Guided Diffusion Models for Inverse Problems</x:v>
       </x:c>
-      <x:c r="E17" s="9" t="str">
+      <x:c r="E17" s="75" t="str">
         <x:v>ICLR</x:v>
       </x:c>
-      <x:c r="F17" s="9" t="str">
+      <x:c r="F17" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G17" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H17" s="9" t="str">
+      <x:c r="G17" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H17" s="75" t="str">
         <x:v>Multiple inverse tasks</x:v>
       </x:c>
-      <x:c r="I17" s="9" t="str">
+      <x:c r="I17" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J17" s="9" t="str">
+      <x:c r="J17" s="75" t="str">
         <x:v>Linear operator</x:v>
       </x:c>
-      <x:c r="K17" s="9" t="str">
+      <x:c r="K17" s="75" t="str">
         <x:v>Known</x:v>
       </x:c>
-      <x:c r="L17" s="9" t="str">
+      <x:c r="L17" s="75" t="str">
         <x:v>None central</x:v>
       </x:c>
-      <x:c r="M17" s="9" t="str">
+      <x:c r="M17" s="75" t="str">
         <x:v>Diffusion/pseudoinverse guidance</x:v>
       </x:c>
-      <x:c r="N17" s="9" t="str">
+      <x:c r="N17" s="75" t="str">
         <x:v>Hard/iterative</x:v>
       </x:c>
-      <x:c r="O17" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P17" s="9" t="str">
+      <x:c r="O17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P17" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Q17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S17" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="T17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U17" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y17" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z17" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA17" s="75" t="str">
+        <x:v>Pending formal eligibility</x:v>
+      </x:c>
+      <x:c r="AB17" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="AC17" s="75" t="str">
+        <x:v>Pseudoinverse guidance improves data consistency</x:v>
+      </x:c>
+      <x:c r="AD17" s="75" t="str">
+        <x:v>Requires operator; no mismatch/UQ guarantee</x:v>
+      </x:c>
+      <x:c r="AE17" s="75" t="str">
+        <x:v>https://openreview.net/forum?id=9_gsMA8MRKQ</x:v>
+      </x:c>
+      <x:c r="AF17" s="75" t="str">
+        <x:v>Data consistency baseline | AI pilot 2026-09-16; unclear. Cannot adjudicate from retrieved evidence. Human adjudication and full-text coding pending. Evidence: https://openreview.net/forum?id=9_gsMA8MRKQ | Batch 02 revisit 2026-09-16: No additional substantive evidence retrieved. Keep the prior unclear recommendation and incomplete-evidence label; missing access is not an exclusion. Source: https://openreview.net/forum?id=9_gsMA8MRKQ | Batch 03 revisit 2026-09-16: The complete abstract/technical evidence is still unavailable in this pass. Retain unclear for retrieval and criterion-3 assessment; access failure is not a rejection. Source: https://openreview.net/forum?id=9_gsMA8MRKQ | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_07.json (P016). Unlisted feature codes remain provisional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="176" customHeight="1">
+      <x:c r="A18" s="85" t="str">
+        <x:v>P017</x:v>
+      </x:c>
+      <x:c r="B18" s="86" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C18" s="75" t="str">
+        <x:v>Wang et al.</x:v>
+      </x:c>
+      <x:c r="D18" s="75" t="str">
+        <x:v>Zero-Shot Image Restoration Using Denoising Diffusion Null-Space Model</x:v>
+      </x:c>
+      <x:c r="E18" s="75" t="str">
+        <x:v>ICLR</x:v>
+      </x:c>
+      <x:c r="F18" s="75" t="str">
+        <x:v>Conference</x:v>
+      </x:c>
+      <x:c r="G18" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H18" s="75" t="str">
+        <x:v>Multiple inverse tasks</x:v>
+      </x:c>
+      <x:c r="I18" s="75" t="str">
+        <x:v>Natural images</x:v>
+      </x:c>
+      <x:c r="J18" s="75" t="str">
+        <x:v>Linear operator</x:v>
+      </x:c>
+      <x:c r="K18" s="75" t="str">
+        <x:v>Known</x:v>
+      </x:c>
+      <x:c r="L18" s="75" t="str">
+        <x:v>None central</x:v>
+      </x:c>
+      <x:c r="M18" s="75" t="str">
+        <x:v>Range/null diffusion</x:v>
+      </x:c>
+      <x:c r="N18" s="75" t="str">
+        <x:v>Hard/range-null</x:v>
+      </x:c>
+      <x:c r="O18" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="P18" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="Q17" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R17" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S17" s="9" t="str">
+      <x:c r="Q18" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R18" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S18" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="T17" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U17" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V17" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W17" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X17" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y17" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z17" s="9" t="str">
-        <x:v>Title/project checked; abstract pending</x:v>
-      </x:c>
-      <x:c r="AA17" s="9" t="str">
+      <x:c r="T18" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U18" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="V18" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W18" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="X18" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y18" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z18" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA18" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB17" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="AC17" s="9" t="str">
-        <x:v>Pseudoinverse guidance improves data consistency</x:v>
-      </x:c>
-      <x:c r="AD17" s="9" t="str">
-        <x:v>Requires operator; no mismatch/UQ guarantee</x:v>
-      </x:c>
-      <x:c r="AE17" s="9" t="str">
-        <x:v>https://openreview.net/forum?id=9_gsMA8MRKQ</x:v>
-      </x:c>
-      <x:c r="AF17" s="75" t="str">
-        <x:v>Data consistency baseline | AI pilot 2026-09-16; unclear. Cannot adjudicate from retrieved evidence. Human adjudication and full-text coding pending. Evidence: https://openreview.net/forum?id=9_gsMA8MRKQ | Batch 02 revisit 2026-09-16: No additional substantive evidence retrieved. Keep the prior unclear recommendation and incomplete-evidence label; missing access is not an exclusion. Source: https://openreview.net/forum?id=9_gsMA8MRKQ | Batch 03 revisit 2026-09-16: The complete abstract/technical evidence is still unavailable in this pass. Retain unclear for retrieval and criterion-3 assessment; access failure is not a rejection. Source: https://openreview.net/forum?id=9_gsMA8MRKQ</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="7" t="str">
-        <x:v>P017</x:v>
-      </x:c>
-      <x:c r="B18" s="8" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C18" s="9" t="str">
-        <x:v>Wang et al.</x:v>
-      </x:c>
-      <x:c r="D18" s="9" t="str">
-        <x:v>Zero-Shot Image Restoration Using Denoising Diffusion Null-Space Model</x:v>
-      </x:c>
-      <x:c r="E18" s="9" t="str">
-        <x:v>ICLR</x:v>
-      </x:c>
-      <x:c r="F18" s="9" t="str">
-        <x:v>Conference</x:v>
-      </x:c>
-      <x:c r="G18" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H18" s="9" t="str">
-        <x:v>Multiple inverse tasks</x:v>
-      </x:c>
-      <x:c r="I18" s="9" t="str">
-        <x:v>Natural images</x:v>
-      </x:c>
-      <x:c r="J18" s="9" t="str">
-        <x:v>Linear operator</x:v>
-      </x:c>
-      <x:c r="K18" s="9" t="str">
-        <x:v>Known</x:v>
-      </x:c>
-      <x:c r="L18" s="9" t="str">
-        <x:v>None central</x:v>
-      </x:c>
-      <x:c r="M18" s="9" t="str">
-        <x:v>Range/null diffusion</x:v>
-      </x:c>
-      <x:c r="N18" s="9" t="str">
-        <x:v>Hard/range-null</x:v>
-      </x:c>
-      <x:c r="O18" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P18" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="Q18" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R18" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S18" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="T18" s="9" t="str">
-        <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U18" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V18" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W18" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="X18" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y18" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z18" s="9" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
-      </x:c>
-      <x:c r="AA18" s="9" t="str">
-        <x:v>Pending formal eligibility</x:v>
-      </x:c>
-      <x:c r="AB18" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC18" s="9" t="str">
+      <x:c r="AB18" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC18" s="75" t="str">
         <x:v>Range/null-space decomposition for consistent restoration</x:v>
       </x:c>
-      <x:c r="AD18" s="9" t="str">
+      <x:c r="AD18" s="75" t="str">
         <x:v>Blind compound mismatch and calibrated support remain open</x:v>
       </x:c>
-      <x:c r="AE18" s="9" t="str">
+      <x:c r="AE18" s="75" t="str">
         <x:v>https://openreview.net/forum?id=mRieQgMtNTQ</x:v>
       </x:c>
-      <x:c r="AF18" s="9" t="str">
-        <x:v>Support-map component | AI pilot 2026-09-16; advance to full text. Range/null-space reconstruction and measurement consistency. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2212.00490</x:v>
+      <x:c r="AF18" s="75" t="str">
+        <x:v>Support-map component | AI pilot 2026-09-16; advance to full text. Range/null-space reconstruction and measurement consistency. Human adjudication and full-text coding pending. Evidence: https://arxiv.org/abs/2212.00490 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, T, U, V, X. Evidence/version/read extent: screening/full_text_07.json (P017). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="176" customHeight="1">
@@ -3848,7 +3856,7 @@
         <x:v>Verify final TIP metadata during full-text stage | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; journal lineage reconciled with the existing verification audit. Feature codes remain provisional. Inspect the final journal report for additions, operator constraints and uncertainty evaluation; the DOI remains unverified and is not invented. Evidence: https://arxiv.org/abs/2407.01027 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R. Evidence/version/read extent: screening/full_text_03.json (P024). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="112" customHeight="1">
+    <x:row r="26" ht="176" customHeight="1">
       <x:c r="A26" s="85" t="str">
         <x:v>P025</x:v>
       </x:c>
@@ -3916,7 +3924,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="W26" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="X26" s="75" t="str">
         <x:v>No</x:v>
@@ -3925,7 +3933,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z26" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA26" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -3943,7 +3951,7 @@
         <x:v>https://link.springer.com/chapter/10.1007/978-3-031-73202-7_25</x:v>
       </x:c>
       <x:c r="AF26" s="75" t="str">
-        <x:v>Generative baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher chapter abstract. Feature codes remain provisional. How is fidelity measured, and are unsupported details assessed against ground truth? The former ECCV poster URL pointed to the unrelated CLOSER paper. Evidence: https://link.springer.com/chapter/10.1007/978-3-031-73202-7_25</x:v>
+        <x:v>Generative baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher chapter abstract. Feature codes remain provisional. How is fidelity measured, and are unsupported details assessed against ground truth? The former ECCV poster URL pointed to the unrelated CLOSER paper. Evidence: https://link.springer.com/chapter/10.1007/978-3-031-73202-7_25 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, T, U, V, W, X. Evidence/version/read extent: screening/full_text_07.json (P025). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="176" customHeight="1">
@@ -4044,7 +4052,7 @@
         <x:v>Closest video application competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Official proceedings record and targeted full-text inspection of sections 4.1–4.2. Feature codes remain provisional. Separate new degradation combinations and change intervals from genuinely unseen operator families or cameras; verify any reliability claims beyond PSNR/SSIM. Evidence: https://proceedings.neurips.cc/paper_files/paper/2024/file/e635a25e49e73adc51f76aef462ff2f8-Paper-Conference.pdf | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_02.json (P026). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="112" customHeight="1">
+    <x:row r="28" ht="176" customHeight="1">
       <x:c r="A28" s="85" t="str">
         <x:v>P027</x:v>
       </x:c>
@@ -4103,13 +4111,13 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T28" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U28" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="V28" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="W28" s="75" t="str">
         <x:v>No</x:v>
@@ -4121,7 +4129,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z28" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA28" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4139,7 +4147,7 @@
         <x:v>https://bmvc2024.org/proceedings/959/</x:v>
       </x:c>
       <x:c r="AF28" s="75" t="str">
-        <x:v>Codec evidence | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Official BMVC proceedings abstract and citation. Feature codes remain provisional. Can its codec transfer protocol support a controlled degradation-shift experiment? It studies bitrate reduction, not forensic reconstruction. The former arXiv URL was an unrelated SLAM paper. Evidence: https://bmvc2024.org/proceedings/959/</x:v>
+        <x:v>Codec evidence | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Official BMVC proceedings abstract and citation. Feature codes remain provisional. Can its codec transfer protocol support a controlled degradation-shift experiment? It studies bitrate reduction, not forensic reconstruction. The former arXiv URL was an unrelated SLAM paper. Evidence: https://bmvc2024.org/proceedings/959/ | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, V, X. Evidence/version/read extent: screening/full_text_07.json (P027). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="176" customHeight="1">
@@ -4436,7 +4444,7 @@
         <x:v>Bayesian baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional publication abstract and author list. Feature codes remain provisional. What uncertainty is lost by conditioning on an estimated representation, and what calibration or shift tests are reported? Evidence: https://www.research.ed.ac.uk/en/publications/empirical-bayesian-imaging-with-large-scale-push-forward-generati/</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="112" customHeight="1">
+    <x:row r="32" ht="176" customHeight="1">
       <x:c r="A32" s="85" t="str">
         <x:v>P031</x:v>
       </x:c>
@@ -4495,7 +4503,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T32" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U32" s="75" t="str">
         <x:v>No</x:v>
@@ -4507,13 +4515,13 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="X32" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Y32" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z32" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA32" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4531,7 +4539,7 @@
         <x:v>https://doi.org/10.1137/23M1568739</x:v>
       </x:c>
       <x:c r="AF32" s="75" t="str">
-        <x:v>Core theoretical threat model | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher abstract. Feature codes remain provisional. State the theorem assumptions and operational examples precisely; do not generalize a worst-case limitation into universal failure of every learned method. Evidence: https://epubs.siam.org/doi/10.1137/23M1568739</x:v>
+        <x:v>Core theoretical threat model | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher abstract. Feature codes remain provisional. State the theorem assumptions and operational examples precisely; do not generalize a worst-case limitation into universal failure of every learned method. Evidence: https://epubs.siam.org/doi/10.1137/23M1568739 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_07.json (P031). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="240" customHeight="1">
@@ -8222,13 +8230,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="U70" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V70" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="W70" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="X70" s="75" t="str">
         <x:v>No</x:v>
@@ -8237,7 +8245,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z70" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA70" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8255,7 +8263,7 @@
         <x:v>https://doi.org/10.1109/TCI.2020.3032671</x:v>
       </x:c>
       <x:c r="AF70" s="75" t="str">
-        <x:v>Foundational joint image/kernel baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; existing journal citation retained. Feature codes remain provisional. Verify journal/preprint lineage and identifiability when the image or kernel lies outside the generator range. A deterministic latent optimum is not an uncertainty estimate. Evidence: https://arxiv.org/abs/1802.04073</x:v>
+        <x:v>Foundational joint image/kernel baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; existing journal citation retained. Feature codes remain provisional. Verify journal/preprint lineage and identifiability when the image or kernel lies outside the generator range. A deterministic latent optimum is not an uncertainty estimate. Evidence: https://arxiv.org/abs/1802.04073 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_07.json (P069). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="71" ht="176" customHeight="1">
@@ -10099,7 +10107,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z89" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA89" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -10117,7 +10125,7 @@
         <x:v>https://doi.org/10.1007/s11263-024-02168-7</x:v>
       </x:c>
       <x:c r="AF89" s="75" t="str">
-        <x:v>Generative fidelity trade-off comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete publisher/author abstracts and publisher DOI metadata. Feature codes remain provisional. What evidence distinguishes plausible texture from recovered detail under severe degradation? The previous seed DOI ended 02092-y; the publisher verifies 02168-7. Evidence: https://link.springer.com/article/10.1007/s11263-024-02168-7</x:v>
+        <x:v>Generative fidelity trade-off comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete publisher/author abstracts and publisher DOI metadata. Feature codes remain provisional. What evidence distinguishes plausible texture from recovered detail under severe degradation? The previous seed DOI ended 02092-y; the publisher verifies 02168-7. Evidence: https://link.springer.com/article/10.1007/s11263-024-02168-7 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, T, U, V, W, X. Evidence/version/read extent: screening/full_text_07.json (P088). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="90" ht="176" customHeight="1">
@@ -10325,7 +10333,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf30335e755b14f6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb65b9cb0b4e94748"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10397,7 +10405,7 @@
         <x:v>Added to matrix?</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="176" customHeight="1">
+    <x:row r="2" ht="144" customHeight="1">
       <x:c r="A2" s="73" t="str">
         <x:v>S001</x:v>
       </x:c>
@@ -10423,15 +10431,15 @@
       <x:c r="I2" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J2" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K2" s="75"/>
+      <x:c r="J2" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K2" s="75" t="str"/>
       <x:c r="L2" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Kernel/model uncertainty. Basis: Title and official author repository; abstract not retrieved. Full-text question and source: screening/pilot_01.json (P001). Revisit: Additional search located the existing author repository but did not supply a complete abstract; recommendation unchanged. See screening/pilot_03.json.</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Explicit kernel/model mismatch with reconstruction experiments. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_07.json (P001).</x:v>
       </x:c>
       <x:c r="M2" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N2" s="75" t="str">
         <x:v>Yes</x:v>
@@ -10517,7 +10525,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="84" customHeight="1">
+    <x:row r="5" ht="144" customHeight="1">
       <x:c r="A5" s="73" t="str">
         <x:v>S004</x:v>
       </x:c>
@@ -10540,18 +10548,18 @@
       <x:c r="H5" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I5" s="76" t="str">
+      <x:c r="I5" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J5" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K5" s="75"/>
+      <x:c r="J5" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K5" s="75" t="str"/>
       <x:c r="L5" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Real blur and synthetic-to-real degradation gap. Basis: Publisher abstract. Full-text question and source: screening/pilot_01.json (P004).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown real blur and synthetic-to-real reconstruction benchmark. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_07.json (P004).</x:v>
       </x:c>
       <x:c r="M5" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N5" s="75" t="str">
         <x:v>Yes</x:v>
@@ -10717,7 +10725,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="84" customHeight="1">
+    <x:row r="10" ht="144" customHeight="1">
       <x:c r="A10" s="73" t="str">
         <x:v>S009</x:v>
       </x:c>
@@ -10740,18 +10748,18 @@
       <x:c r="H10" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I10" s="76" t="str">
+      <x:c r="I10" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J10" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K10" s="75"/>
+      <x:c r="J10" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K10" s="75" t="str"/>
       <x:c r="L10" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind restoration with compound degradation. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P009).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Blind compound degradation with real-image transfer tests. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_07.json (P009).</x:v>
       </x:c>
       <x:c r="M10" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N10" s="75" t="str">
         <x:v>Yes</x:v>
@@ -10997,7 +11005,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="176" customHeight="1">
+    <x:row r="17" ht="144" customHeight="1">
       <x:c r="A17" s="73" t="str">
         <x:v>S016</x:v>
       </x:c>
@@ -11023,21 +11031,21 @@
       <x:c r="I17" s="94" t="str">
         <x:v>AI pilot: unclear</x:v>
       </x:c>
-      <x:c r="J17" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K17" s="75"/>
+      <x:c r="J17" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K17" s="75" t="str"/>
       <x:c r="L17" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Cannot adjudicate from retrieved evidence. Basis: Official search snippet only; full abstract not retrieved. Full-text question and source: screening/pilot_01.json (P016). Revisit: Retrieval retry unsuccessful: OpenReview challenge and author-PDF fetch failure; unchanged unclear. See screening/pilot_02.json. Revisit: OpenReview remains challenged; author PDF fetch failed; author publication listing confirms title and venue only; recommendation unchanged. See screening/pilot_03.json. Full-text 01: author PDF still fails to open; eligibility pending, not excluded. See full_text_01.json.</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Posterior reconstruction, altered degradation and composed inverse tasks. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_07.json (P016).</x:v>
       </x:c>
       <x:c r="M17" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N17" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="84" customHeight="1">
+    <x:row r="18" ht="144" customHeight="1">
       <x:c r="A18" s="73" t="str">
         <x:v>S017</x:v>
       </x:c>
@@ -11060,18 +11068,18 @@
       <x:c r="H18" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I18" s="76" t="str">
+      <x:c r="I18" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J18" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K18" s="75"/>
+      <x:c r="J18" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K18" s="75" t="str"/>
       <x:c r="L18" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Range/null-space reconstruction and measurement consistency. Basis: Author preprint abstract. Full-text question and source: screening/pilot_01.json (P017).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Compound reconstruction and explicitly approximate real-world forward models. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_07.json (P017).</x:v>
       </x:c>
       <x:c r="M18" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N18" s="75" t="str">
         <x:v>Yes</x:v>
@@ -11357,7 +11365,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="112" customHeight="1">
+    <x:row r="26" ht="144" customHeight="1">
       <x:c r="A26" s="73" t="str">
         <x:v>S025</x:v>
       </x:c>
@@ -11380,15 +11388,15 @@
       <x:c r="H26" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I26" s="81" t="str">
+      <x:c r="I26" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J26" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K26" s="75"/>
+      <x:c r="J26" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K26" s="75" t="str"/>
       <x:c r="L26" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind restoration with a generative prior. Basis: Publisher chapter abstract. Sources and full-text question: screening/pilot_02.json (P025).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Blind compound restoration with real-world evaluation. Online full text inspected; no local PDF acquired. Version, read extent and technical extraction: screening/full_text_07.json (P025).</x:v>
       </x:c>
       <x:c r="M26" s="75" t="str">
         <x:v>No</x:v>
@@ -11437,7 +11445,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="28" ht="112" customHeight="1">
+    <x:row r="28" ht="144" customHeight="1">
       <x:c r="A28" s="73" t="str">
         <x:v>S027</x:v>
       </x:c>
@@ -11460,15 +11468,15 @@
       <x:c r="H28" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I28" s="81" t="str">
+      <x:c r="I28" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J28" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K28" s="75"/>
+      <x:c r="J28" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K28" s="75" t="str"/>
       <x:c r="L28" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Codec-dependent restoration and generalization. Basis: Official BMVC proceedings abstract and citation. Sources and full-text question: screening/pilot_02.json (P027).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Compound video degradation and operational restoration benchmark. Online full text inspected; no local PDF acquired. Version, read extent and technical extraction: screening/full_text_07.json (P027).</x:v>
       </x:c>
       <x:c r="M28" s="75" t="str">
         <x:v>No</x:v>
@@ -11597,7 +11605,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="32" ht="112" customHeight="1">
+    <x:row r="32" ht="144" customHeight="1">
       <x:c r="A32" s="73" t="str">
         <x:v>S031</x:v>
       </x:c>
@@ -11620,15 +11628,15 @@
       <x:c r="H32" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I32" s="81" t="str">
+      <x:c r="I32" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J32" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K32" s="75"/>
+      <x:c r="J32" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K32" s="75" t="str"/>
       <x:c r="L32" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Hallucination and accuracy–stability limits. Basis: Publisher abstract. Sources and full-text question: screening/pilot_02.json (P031).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Reconstruction hallucinations, stability and held-out detail tests. Online full text inspected; no local PDF acquired. Version, read extent and technical extraction: screening/full_text_07.json (P031).</x:v>
       </x:c>
       <x:c r="M32" s="75" t="str">
         <x:v>No</x:v>
@@ -13142,18 +13150,18 @@
       <x:c r="H70" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I70" s="91" t="str">
+      <x:c r="I70" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J70" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K70" s="75"/>
+      <x:c r="J70" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K70" s="75" t="str"/>
       <x:c r="L70" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint blind image/kernel recovery using generative priors. Basis: Complete author preprint abstract; existing journal citation retained. Sources and full-text question: screening/pilot_03.json (P069).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Joint blind deconvolution and generative range/noise mismatch. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_07.json (P069).</x:v>
       </x:c>
       <x:c r="M70" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N70" s="75" t="str">
         <x:v>Yes</x:v>
@@ -13902,18 +13910,18 @@
       <x:c r="H89" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I89" s="91" t="str">
+      <x:c r="I89" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J89" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K89" s="75"/>
+      <x:c r="J89" s="104" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K89" s="75" t="str"/>
       <x:c r="L89" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind real-world super-resolution and fidelity/perception control. Basis: Complete publisher/author abstracts and publisher DOI metadata. Sources and full-text question: screening/pilot_03.json (P088).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Blind compound SR and real-measurement evaluation. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_07.json (P088).</x:v>
       </x:c>
       <x:c r="M89" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N89" s="75" t="str">
         <x:v>Yes</x:v>
@@ -14300,7 +14308,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53f6e3f6be384f59"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R039dbef45afe49f4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14472,7 +14480,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 60 (59 include, 1 exclude), 30 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 70 (69 include, 1 exclude), 20 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14480,7 +14488,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json and full_text_06.json; current report: full_text_06_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json, full_text_06.json and full_text_07.json; current report: full_text_07_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14726,7 +14734,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16ddbd596d6743a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6befd7af66db4c2b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: complete full-text checkpoint 08 (80 of 90 assessed)
Assess ten additional primary full texts under protocol v0.4. Record
versions, reading extent, criterion-level recommendations, selected
feature evidence, acquisition hashes and source-specific follow-ups.

Correct UA-FP uncertainty/calibration codes, qualify categorical
degradation probabilities, and document operator-estimation and
real-video transfer limits. Restore P068's full proceedings title.

Synchronize the matrix, tracker, reference exports and deferred tasks.
Validate 80 distinct assessments (79 include, 1 exclude, 10 pending),
90 retained seeds, workbook formulas/native objects and export reimport.
Human adjudication and formal searches remain pending; novelty is
unestablished. No paper full texts are redistributed.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R75abcb387aa5413c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="Rf7a0bb1548dd4da6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R627a854183f744cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="Ra1c5f724854f4b7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rb2d7ff5668eb4a60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb8f08c9617304aa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R559337e820924b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rd769c1ddf97f43ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="Rbd12f0328d8d4113"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rb31f7f4758e34983"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -282,7 +287,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="105">
+  <x:cellXfs count="106">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -512,6 +517,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -745,7 +753,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc3affe20faef43e5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5c25b76948bc429b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1194,7 +1202,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>70</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1211,7 +1219,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>Residual mismatch compensation, joint blind estimation, null-space theory and generative fidelity control have existing comparators. See screening/full_text_07_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
+        <x:v>Operator-family training, blind calibration, degradation classification and video fidelity controls have existing comparators. See screening/full_text_08_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1266,7 +1274,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 70/90 (69 include, 1 exclude); 20 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 80/90 (79 include, 1 exclude); 10 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1361,7 +1369,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R965f00081e2347fd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47420d869d5b4af4"/>
 </x:worksheet>
 </file>
 
@@ -2680,102 +2688,102 @@
         <x:v>Diffusion baseline | AI pilot 2026-09-16; advance to full text. Posterior reconstruction and transfer across image distributions. Human adjudication and full-text coding pending. Evidence: https://proceedings.neurips.cc/paper_files/paper/2022/hash/95504595b6169131b6ed6cd72eb05616-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_05.json (P012). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="240" customHeight="1">
-      <x:c r="A14" s="7" t="str">
+    <x:row r="14" ht="176" customHeight="1">
+      <x:c r="A14" s="85" t="str">
         <x:v>P013</x:v>
       </x:c>
-      <x:c r="B14" s="8" t="n">
+      <x:c r="B14" s="86" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="C14" s="9" t="str">
+      <x:c r="C14" s="75" t="str">
         <x:v>Li et al.</x:v>
       </x:c>
-      <x:c r="D14" s="9" t="str">
+      <x:c r="D14" s="75" t="str">
         <x:v>All-in-One Image Restoration for Unknown Corruption</x:v>
       </x:c>
-      <x:c r="E14" s="9" t="str">
+      <x:c r="E14" s="75" t="str">
         <x:v>CVPR</x:v>
       </x:c>
-      <x:c r="F14" s="9" t="str">
+      <x:c r="F14" s="75" t="str">
         <x:v>Conference</x:v>
       </x:c>
-      <x:c r="G14" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="H14" s="9" t="str">
+      <x:c r="G14" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="H14" s="75" t="str">
         <x:v>Multi-task restoration</x:v>
       </x:c>
-      <x:c r="I14" s="9" t="str">
+      <x:c r="I14" s="75" t="str">
         <x:v>Natural images</x:v>
       </x:c>
-      <x:c r="J14" s="9" t="str">
+      <x:c r="J14" s="75" t="str">
         <x:v>Implicit corruption process</x:v>
       </x:c>
-      <x:c r="K14" s="9" t="str">
+      <x:c r="K14" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
-      <x:c r="L14" s="9" t="str">
+      <x:c r="L14" s="75" t="str">
         <x:v>Multiple corruption types/levels</x:v>
       </x:c>
-      <x:c r="M14" s="9" t="str">
+      <x:c r="M14" s="75" t="str">
         <x:v>Contrastive degradation encoder</x:v>
       </x:c>
-      <x:c r="N14" s="9" t="str">
+      <x:c r="N14" s="75" t="str">
         <x:v>Implicit</x:v>
       </x:c>
-      <x:c r="O14" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="P14" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Q14" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="R14" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S14" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T14" s="9" t="str">
+      <x:c r="O14" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="U14" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="V14" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W14" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X14" s="9" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="Y14" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="Z14" s="9" t="str">
-        <x:v>Title/project checked; abstract pending</x:v>
-      </x:c>
-      <x:c r="AA14" s="9" t="str">
+      <x:c r="P14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S14" s="75" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="T14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="U14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X14" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Y14" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="Z14" s="75" t="str">
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
+      </x:c>
+      <x:c r="AA14" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
       </x:c>
-      <x:c r="AB14" s="9" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="AC14" s="9" t="str">
+      <x:c r="AB14" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="AC14" s="75" t="str">
         <x:v>One model handles multiple unknown corruptions</x:v>
       </x:c>
-      <x:c r="AD14" s="9" t="str">
+      <x:c r="AD14" s="75" t="str">
         <x:v>No explicit operator estimation, calibrated UQ or support test</x:v>
       </x:c>
-      <x:c r="AE14" s="9" t="str">
+      <x:c r="AE14" s="75" t="str">
         <x:v>https://openaccess.thecvf.com/content/CVPR2022/html/Li_All-in-One_Image_Restoration_for_Unknown_Corruption_CVPR_2022_paper.html</x:v>
       </x:c>
       <x:c r="AF14" s="75" t="str">
-        <x:v>Nearest all-in-one baseline | AI pilot 2026-09-16; advance to full text. Unknown corruption and all-in-one restoration. Human adjudication and full-text coding pending. Evidence: https://github.com/XLearning-SCU/2022-CVPR-AirNet | Batch 03 revisit 2026-09-16: Unknown-corruption restoration remains an explicit scope signal. Preserve incomplete evidence and do not equate mixed task training with compound corruption. Source: https://github.com/XLearning-SCU/2022-CVPR-AirNet</x:v>
+        <x:v>Nearest all-in-one baseline | AI pilot 2026-09-16; advance to full text. Unknown corruption and all-in-one restoration. Human adjudication and full-text coding pending. Evidence: https://github.com/XLearning-SCU/2022-CVPR-AirNet | Batch 03 revisit 2026-09-16: Unknown-corruption restoration remains an explicit scope signal. Preserve incomplete evidence and do not equate mixed task training with compound corruption. Source: https://github.com/XLearning-SCU/2022-CVPR-AirNet | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_08.json (P013). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="176" customHeight="1">
@@ -3464,7 +3472,7 @@
         <x:v>Nearest all-in-one baseline | AI pilot 2026-09-16; advance to full text. Unknown degradation types and levels. Human adjudication and full-text coding pending. Evidence: https://proceedings.neurips.cc/paper_files/paper/2023/hash/e187897ed7780a579a0d76fd4a35d107-Abstract-Conference.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, X. Evidence/version/read extent: screening/full_text_05.json (P020). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="112" customHeight="1">
+    <x:row r="22" ht="176" customHeight="1">
       <x:c r="A22" s="85" t="str">
         <x:v>P021</x:v>
       </x:c>
@@ -3514,7 +3522,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="Q22" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="R22" s="75" t="str">
         <x:v>No</x:v>
@@ -3523,10 +3531,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T22" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U22" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V22" s="75" t="str">
         <x:v>No</x:v>
@@ -3541,7 +3549,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z22" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA22" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -3559,7 +3567,7 @@
         <x:v>https://arxiv.org/abs/2211.10525</x:v>
       </x:c>
       <x:c r="AF22" s="75" t="str">
-        <x:v>Closest calibration analogue | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; journal citation not independently rechecked in this batch. Feature codes remain provisional. Which coordinate errors and initialization regimes are evaluated? Physical calibration is not statistical calibration of uncertainty intervals. Evidence: https://arxiv.org/abs/2211.10525</x:v>
+        <x:v>Closest calibration analogue | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; journal citation not independently rechecked in this batch. Feature codes remain provisional. Which coordinate errors and initialization regimes are evaluated? Physical calibration is not statistical calibration of uncertainty intervals. Evidence: https://arxiv.org/abs/2211.10525 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_08.json (P021). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="176" customHeight="1">
@@ -4542,7 +4550,7 @@
         <x:v>Core theoretical threat model | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher abstract. Feature codes remain provisional. State the theorem assumptions and operational examples precisely; do not generalize a worst-case limitation into universal failure of every learned method. Evidence: https://epubs.siam.org/doi/10.1137/23M1568739 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, W, X. Evidence/version/read extent: screening/full_text_07.json (P031). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="240" customHeight="1">
+    <x:row r="33" ht="176" customHeight="1">
       <x:c r="A33" s="85" t="str">
         <x:v>P032</x:v>
       </x:c>
@@ -4589,13 +4597,13 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="P33" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="Q33" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="R33" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="S33" s="75" t="str">
         <x:v>Yes</x:v>
@@ -4619,7 +4627,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z33" s="75" t="str">
-        <x:v>Incomplete evidence; retrieval pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA33" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4637,7 +4645,7 @@
         <x:v>https://doi.org/10.1038/s41377-025-01915-w</x:v>
       </x:c>
       <x:c r="AF33" s="75" t="str">
-        <x:v>Highest-priority full-text competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher title and indexed abstract excerpt only; complete abstract and full text blocked by retrieval challenges. Feature codes remain provisional. Retrieve the complete paper. Does uncertainty mean uncertain acquisition parameters, probabilistic posterior uncertainty, or both? Existing positive feature codes remain unverified. Evidence: https://www.nature.com/articles/s41377-025-01915-w | Batch 03 revisit 2026-09-16: The excerpt concerns system uncertainties such as misalignment and aberration. Positive legacy image/operator uncertainty and calibration codes are not verified probabilistic capabilities. Full text is required. Source: https://www.nature.com/articles/s41377-025-01915-w</x:v>
+        <x:v>Highest-priority full-text competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Publisher title and indexed abstract excerpt only; complete abstract and full text blocked by retrieval challenges. Feature codes remain provisional. Retrieve the complete paper. Does uncertainty mean uncertain acquisition parameters, probabilistic posterior uncertainty, or both? Existing positive feature codes remain unverified. Evidence: https://www.nature.com/articles/s41377-025-01915-w | Batch 03 revisit 2026-09-16: The excerpt concerns system uncertainties such as misalignment and aberration. Positive legacy image/operator uncertainty and calibration codes are not verified probabilistic capabilities. Full text is required. Source: https://www.nature.com/articles/s41377-025-01915-w | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, T, U, V, W, X. Evidence/version/read extent: screening/full_text_08.json (P032). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="176" customHeight="1">
@@ -5664,7 +5672,7 @@
         <x:v>PnP/conditioning correction</x:v>
       </x:c>
       <x:c r="O44" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P44" s="75" t="str">
         <x:v>No</x:v>
@@ -5679,10 +5687,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T44" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U44" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V44" s="75" t="str">
         <x:v>No</x:v>
@@ -5697,7 +5705,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z44" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA44" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -5715,7 +5723,7 @@
         <x:v>https://doi.org/10.1109/TCI.2021.3094714</x:v>
       </x:c>
       <x:c r="AF44" s="75" t="str">
-        <x:v>Operator-adaptation cornerstone | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; existing journal citation retained. Feature codes remain provisional. Which operator changes are supplied to the method, which are inferred, and how are adaptation data separated from evaluation? Evidence: https://arxiv.org/abs/2012.00139</x:v>
+        <x:v>Operator-adaptation cornerstone | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; existing journal citation retained. Feature codes remain provisional. Which operator changes are supplied to the method, which are inferred, and how are adaptation data separated from evaluation? Evidence: https://arxiv.org/abs/2012.00139 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_08.json (P043). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="45" ht="176" customHeight="1">
@@ -5958,7 +5966,7 @@
         <x:v>Hard/iterative</x:v>
       </x:c>
       <x:c r="O47" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P47" s="75" t="str">
         <x:v>No</x:v>
@@ -5973,10 +5981,10 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T47" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="U47" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V47" s="75" t="str">
         <x:v>No</x:v>
@@ -5991,7 +5999,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z47" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA47" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6009,7 +6017,7 @@
         <x:v>https://doi.org/10.1137/23M1545628</x:v>
       </x:c>
       <x:c r="AF47" s="75" t="str">
-        <x:v>Strong adaptive-reconstruction comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and SIAM citation. Feature codes remain provisional. Separate interpolation within the training operator family from extrapolation or wrong-family mismatch. The 2022 preprint and 2024 journal record are one lineage. Evidence: https://arxiv.org/abs/2202.11342</x:v>
+        <x:v>Strong adaptive-reconstruction comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and SIAM citation. Feature codes remain provisional. Separate interpolation within the training operator family from extrapolation or wrong-family mismatch. The 2022 preprint and 2024 journal record are one lineage. Evidence: https://arxiv.org/abs/2202.11342 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_08.json (P046). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="176" customHeight="1">
@@ -7250,13 +7258,13 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="U60" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V60" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="W60" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="X60" s="75" t="str">
         <x:v>No</x:v>
@@ -7265,7 +7273,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z60" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA60" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7283,7 +7291,7 @@
         <x:v>https://doi.org/10.1007/s11263-022-01705-6</x:v>
       </x:c>
       <x:c r="AF60" s="75" t="str">
-        <x:v>Real video blur benchmark | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author abstract and publisher journal metadata. Feature codes remain provisional. Check acquisition timing, alignment, reference quality and cross-dataset splits. Link any earlier conference report to the journal study before synthesis. Evidence: https://link.springer.com/article/10.1007/s11263-022-01705-6</x:v>
+        <x:v>Real video blur benchmark | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author abstract and publisher journal metadata. Feature codes remain provisional. Check acquisition timing, alignment, reference quality and cross-dataset splits. Link any earlier conference report to the journal study before synthesis. Evidence: https://link.springer.com/article/10.1007/s11263-022-01705-6 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_08.json (P059). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="61" ht="176" customHeight="1">
@@ -7440,16 +7448,16 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="S62" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T62" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="U62" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V62" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="W62" s="75" t="str">
         <x:v>Partial</x:v>
@@ -7461,7 +7469,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z62" s="75" t="str">
-        <x:v>Abstract and repository inspected</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA62" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7479,7 +7487,7 @@
         <x:v>https://doi.org/10.1109/WACVW68408.2026.00174</x:v>
       </x:c>
       <x:c r="AF62" s="75" t="str">
-        <x:v>Best downstream forensic-reliability comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and official repository. Feature codes remain provisional. Which task improvements are caused by restored evidence rather than prior bias? Person-retrieval accuracy is not a certificate of image-detail fidelity. Evidence: https://arxiv.org/abs/2601.08807</x:v>
+        <x:v>Best downstream forensic-reliability comparator | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and official repository. Feature codes remain provisional. Which task improvements are caused by restored evidence rather than prior bias? Person-retrieval accuracy is not a certificate of image-detail fidelity. Evidence: https://arxiv.org/abs/2601.08807 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_08.json (P061). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="63" ht="176" customHeight="1">
@@ -8081,7 +8089,7 @@
         <x:v>Abu Hussein et al.</x:v>
       </x:c>
       <x:c r="D69" s="75" t="str">
-        <x:v>Correction Filter for Single Image Super-Resolution</x:v>
+        <x:v>Correction Filter for Single Image Super-Resolution: Robustifying Off-the-Shelf Deep Super-Resolvers</x:v>
       </x:c>
       <x:c r="E69" s="75" t="str">
         <x:v>CVPR</x:v>
@@ -8114,7 +8122,7 @@
         <x:v>Hard/pre-correction</x:v>
       </x:c>
       <x:c r="O69" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="P69" s="75" t="str">
         <x:v>No</x:v>
@@ -8132,7 +8140,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="U69" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V69" s="75" t="str">
         <x:v>No</x:v>
@@ -8147,7 +8155,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z69" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA69" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8165,7 +8173,7 @@
         <x:v>https://doi.org/10.1109/CVPR42600.2020.00150</x:v>
       </x:c>
       <x:c r="AF69" s="75" t="str">
-        <x:v>Early operator-mismatch baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; shorter seed conference title retained. Feature codes remain provisional. Verify the supplied versus estimated kernel assumptions and the publication lineage of the longer preprint title. Use 2020 conference publication for the review window. Evidence: https://arxiv.org/abs/1912.00157</x:v>
+        <x:v>Early operator-mismatch baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract; shorter seed conference title retained. Feature codes remain provisional. Verify the supplied versus estimated kernel assumptions and the publication lineage of the longer preprint title. Use 2020 conference publication for the review window. Evidence: https://arxiv.org/abs/1912.00157 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_08.json (P068). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="176" customHeight="1">
@@ -8408,22 +8416,22 @@
         <x:v>Implicit</x:v>
       </x:c>
       <x:c r="O72" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="P72" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="Q72" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="R72" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="S72" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T72" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U72" s="75" t="str">
         <x:v>Yes</x:v>
@@ -8441,7 +8449,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z72" s="75" t="str">
-        <x:v>Title/project checked; abstract pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA72" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8459,7 +8467,7 @@
         <x:v>https://openaccess.thecvf.com/content/CVPR2023/html/Park_All-in-One_Image_Restoration_for_Unknown_Degradations_Using_Adaptive_Discriminative_Filters_CVPR_2023_paper.html</x:v>
       </x:c>
       <x:c r="AF72" s="75" t="str">
-        <x:v>Universal restoration baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Specific official proceedings title located; CVF HTML/PDF access failed; complete abstract unavailable. Feature codes remain provisional. Retrieve the complete paper and verify how degradation is inferred, whether combinations are simultaneous and how unknown degradation is operationally tested. Evidence: https://openaccess.thecvf.com/content/CVPR2023/html/Park_All-in-One_Image_Restoration_for_Unknown_Degradations_Using_Adaptive_Discriminative_Filters_CVPR_2023_paper.html</x:v>
+        <x:v>Universal restoration baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Specific official proceedings title located; CVF HTML/PDF access failed; complete abstract unavailable. Feature codes remain provisional. Retrieve the complete paper and verify how degradation is inferred, whether combinations are simultaneous and how unknown degradation is operationally tested. Evidence: https://openaccess.thecvf.com/content/CVPR2023/html/Park_All-in-One_Image_Restoration_for_Unknown_Degradations_Using_Adaptive_Discriminative_Filters_CVPR_2023_paper.html | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_08.json (P071). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="176" customHeight="1">
@@ -10282,7 +10290,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="S91" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T91" s="75" t="str">
         <x:v>Yes</x:v>
@@ -10303,7 +10311,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z91" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA91" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -10321,7 +10329,7 @@
         <x:v>https://openaccess.thecvf.com/content/CVPR2024/html/Zhou_Upscale-A-Video_Temporal-Consistent_Diffusion_Model_for_Real-World_Video_Super-Resolution_CVPR_2024_paper.html</x:v>
       </x:c>
       <x:c r="AF91" s="75" t="str">
-        <x:v>Closest real-world generative video-SR baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and official project locator. Feature codes remain provisional. Distinguish temporal output consistency from testing time-varying acquisition operators. Verify whether propagated generated detail stays consistent with measurements. Evidence: https://arxiv.org/abs/2312.06640</x:v>
+        <x:v>Closest real-world generative video-SR baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and official project locator. Feature codes remain provisional. Distinguish temporal output consistency from testing time-varying acquisition operators. Verify whether propagated generated detail stays consistent with measurements. Evidence: https://arxiv.org/abs/2312.06640 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, S, T, U, W, X. Evidence/version/read extent: screening/full_text_08.json (P090). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10333,7 +10341,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb65b9cb0b4e94748"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57e62b74796146dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10885,7 +10893,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="176" customHeight="1">
+    <x:row r="14" ht="144" customHeight="1">
       <x:c r="A14" s="73" t="str">
         <x:v>S013</x:v>
       </x:c>
@@ -10911,15 +10919,15 @@
       <x:c r="I14" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J14" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K14" s="75"/>
+      <x:c r="J14" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K14" s="75" t="str"/>
       <x:c r="L14" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Unknown corruption and all-in-one restoration. Basis: Title and official author repository; abstract not retrieved. Full-text question and source: screening/pilot_01.json (P013). Revisit: Indexed proceedings excerpt and previous official repository; complete abstract still not retrieved; recommendation unchanged. See screening/pilot_03.json.</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Blind restoration of unknown corruption with a spatially varying noise test. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P013).</x:v>
       </x:c>
       <x:c r="M14" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N14" s="75" t="str">
         <x:v>Yes</x:v>
@@ -11205,7 +11213,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="112" customHeight="1">
+    <x:row r="22" ht="144" customHeight="1">
       <x:c r="A22" s="73" t="str">
         <x:v>S021</x:v>
       </x:c>
@@ -11228,18 +11236,18 @@
       <x:c r="H22" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I22" s="81" t="str">
+      <x:c r="I22" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J22" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K22" s="75"/>
+      <x:c r="J22" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K22" s="75" t="str"/>
       <x:c r="L22" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint acquisition-parameter calibration and reconstruction. Basis: Author preprint abstract; journal citation not independently rechecked in this batch. Sources and full-text question: screening/pilot_02.json (P021).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Joint reconstruction and unknown acquisition-coordinate correction. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P021).</x:v>
       </x:c>
       <x:c r="M22" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N22" s="75" t="str">
         <x:v>Yes</x:v>
@@ -11645,7 +11653,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="176" customHeight="1">
+    <x:row r="33" ht="144" customHeight="1">
       <x:c r="A33" s="73" t="str">
         <x:v>S032</x:v>
       </x:c>
@@ -11671,12 +11679,12 @@
       <x:c r="I33" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J33" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K33" s="75"/>
+      <x:c r="J33" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K33" s="75" t="str"/>
       <x:c r="L33" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Uncertain acquisition in Fourier ptychographic reconstruction; conservative scope signal. Basis: Publisher title and indexed abstract excerpt only; complete abstract and full text blocked by retrieval challenges. Sources and full-text question: screening/pilot_02.json (P032). Revisit: Additional indexed publisher excerpt and PubMed locator; complete abstract/text still inaccessible; recommendation unchanged. See screening/pilot_03.json.</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Joint reconstruction and system-error correction under noise, misalignment and aberrations. Online full text inspected; no local PDF acquired. Version, read extent and technical extraction: screening/full_text_08.json (P032).</x:v>
       </x:c>
       <x:c r="M33" s="75" t="str">
         <x:v>No</x:v>
@@ -12108,18 +12116,18 @@
       <x:c r="H44" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I44" s="91" t="str">
+      <x:c r="I44" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J44" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K44" s="75"/>
+      <x:c r="J44" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K44" s="75" t="str"/>
       <x:c r="L44" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Adaptation to changing or partially known forward models. Basis: Complete author preprint abstract; existing journal citation retained. Sources and full-text question: screening/pilot_03.json (P043).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Known and unknown forward-model changes with reconstruction comparisons. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P043).</x:v>
       </x:c>
       <x:c r="M44" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N44" s="75" t="str">
         <x:v>Yes</x:v>
@@ -12228,18 +12236,18 @@
       <x:c r="H47" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I47" s="91" t="str">
+      <x:c r="I47" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J47" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K47" s="75"/>
+      <x:c r="J47" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K47" s="75" t="str"/>
       <x:c r="L47" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Operator-family adaptation and blind reconstruction. Basis: Complete author preprint abstract and SIAM citation. Sources and full-text question: screening/pilot_03.json (P046).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Operator-family shift and joint blind inverse reconstruction, including an explicit failure case. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P046).</x:v>
       </x:c>
       <x:c r="M47" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N47" s="75" t="str">
         <x:v>Yes</x:v>
@@ -12748,18 +12756,18 @@
       <x:c r="H60" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I60" s="91" t="str">
+      <x:c r="I60" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J60" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K60" s="75"/>
+      <x:c r="J60" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K60" s="75" t="str"/>
       <x:c r="L60" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Real blurred/sharp video acquisition and cross-dataset generalization. Basis: Complete author abstract and publisher journal metadata. Sources and full-text question: screening/pilot_03.json (P059).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Real temporally varying blur, acquisition noise and cross-dataset degradation mismatch. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P059).</x:v>
       </x:c>
       <x:c r="M60" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N60" s="75" t="str">
         <x:v>Yes</x:v>
@@ -12830,18 +12838,18 @@
       <x:c r="H62" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I62" s="91" t="str">
+      <x:c r="I62" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J62" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K62" s="75"/>
+      <x:c r="J62" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K62" s="75" t="str"/>
       <x:c r="L62" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Task-driven super-resolution across surveillance viewpoint/domain shift. Basis: Complete author preprint abstract and official repository. Sources and full-text question: screening/pilot_03.json (P061).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Explicit super-resolution training and authentic degradation failure analysis within a recognition application. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P061).</x:v>
       </x:c>
       <x:c r="M62" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N62" s="75" t="str">
         <x:v>Yes</x:v>
@@ -13099,7 +13107,7 @@
         <x:v>Targeted cornerstone search / citation chaining; mapped as P068</x:v>
       </x:c>
       <x:c r="E69" s="73" t="str">
-        <x:v>Correction Filter for Single Image Super-Resolution</x:v>
+        <x:v>Correction Filter for Single Image Super-Resolution: Robustifying Off-the-Shelf Deep Super-Resolvers</x:v>
       </x:c>
       <x:c r="F69" s="73" t="n">
         <x:v>2020</x:v>
@@ -13110,18 +13118,18 @@
       <x:c r="H69" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I69" s="91" t="str">
+      <x:c r="I69" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J69" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K69" s="75"/>
+      <x:c r="J69" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K69" s="75" t="str"/>
       <x:c r="L69" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Correction of degradation mismatch for pretrained super-resolution. Basis: Complete author preprint abstract; shorter seed conference title retained. Sources and full-text question: screening/pilot_03.json (P068).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown blur/downsampling and training-to-test kernel mismatch. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P068).</x:v>
       </x:c>
       <x:c r="M69" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N69" s="75" t="str">
         <x:v>Yes</x:v>
@@ -13230,18 +13238,18 @@
       <x:c r="H72" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I72" s="91" t="str">
+      <x:c r="I72" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J72" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K72" s="75"/>
+      <x:c r="J72" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K72" s="75" t="str"/>
       <x:c r="L72" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Title explicitly identifies restoration with unknown degradations. Basis: Specific official proceedings title located; CVF HTML/PDF access failed; complete abstract unavailable. Sources and full-text question: screening/pilot_03.json (P071).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown degradation classification, compound weather data and synthetic-to-real restoration. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P071).</x:v>
       </x:c>
       <x:c r="M72" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N72" s="75" t="str">
         <x:v>Yes</x:v>
@@ -13990,18 +13998,18 @@
       <x:c r="H91" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I91" s="91" t="str">
+      <x:c r="I91" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J91" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K91" s="75"/>
+      <x:c r="J91" s="105" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K91" s="75" t="str"/>
       <x:c r="L91" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind generative real-world video restoration and temporal fidelity. Basis: Complete author preprint abstract and official project locator. Sources and full-text question: screening/pilot_03.json (P090).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Blind compound video restoration and real-data transfer with fidelity-control ablations. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_08.json (P090).</x:v>
       </x:c>
       <x:c r="M91" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N91" s="75" t="str">
         <x:v>Yes</x:v>
@@ -14308,7 +14316,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R039dbef45afe49f4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf96550a7849344e9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14480,7 +14488,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 70 (69 include, 1 exclude), 20 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 80 (79 include, 1 exclude), 10 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14488,7 +14496,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json, full_text_06.json and full_text_07.json; current report: full_text_07_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json, full_text_06.json, full_text_07.json and full_text_08.json; current report: full_text_08_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14734,7 +14742,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6befd7af66db4c2b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7107ac29fef4b12"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record full-text checkpoint 09 (84 assessed, 6 pending)
Attempt retrieval for all ten remaining seeds and assess four accessible
full texts under protocol v0.4. Record source versions, reading extent,
criterion-level evidence and PDF hashes. Log primary retrieval routes,
access obstacles and next actions for the six unresolved papers.

Distinguish categorical degradation probabilities and clean-class
stopping from calibrated operator uncertainty and selective release.
Keep provisional VDPS evidence explicit and novelty unestablished.

Synchronize the matrix, tracker, reference exports and status documents.
Validate 84 unique assessments (83 include, 1 exclude), six pending IDs,
90 references, formula recalculation, native workbook objects and export
reimport. Preserve human/formal decisions and historic checkpoints.
No paper full texts are redistributed.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb8f08c9617304aa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R559337e820924b63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rd769c1ddf97f43ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="Rbd12f0328d8d4113"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rb31f7f4758e34983"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6c6bbef7e86a4ab6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R5805a0a486da4c53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rd23251ca970a483b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R11c845edd7414b80"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rb470cd64c9ed4950"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="24">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -287,7 +292,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="106">
+  <x:cellXfs count="107">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -522,6 +527,9 @@
     <x:xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -753,7 +761,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5c25b76948bc429b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R152de408bfb94da8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1202,7 +1210,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>80</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1219,7 +1227,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>Operator-family training, blind calibration, degradation classification and video fidelity controls have existing comparators. See screening/full_text_08_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
+        <x:v>Joint PSF estimation, compound night restoration, cross-camera video transfer and clean-class stopping have comparators. Six full texts remain pending. See screening/full_text_09_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1274,7 +1282,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 80/90 (79 include, 1 exclude); 10 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 84/90 (83 include, 1 exclude); 6 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1369,7 +1377,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47420d869d5b4af4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0257f4dd79b249b4"/>
 </x:worksheet>
 </file>
 
@@ -4351,7 +4359,7 @@
         <x:v>https://opg.optica.org/oe/abstract.cfm?uri=oe-32-17-30267</x:v>
       </x:c>
       <x:c r="AF30" s="75" t="str">
-        <x:v>Nearest robust unrolling competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Paper abstract indexed by PubMed and publisher citation. Feature codes remain provisional. Which PSF errors are held out, and does the design distinguish noise from operator error? Extract any real-system validation. Evidence: https://pubmed.ncbi.nlm.nih.gov/39573193/</x:v>
+        <x:v>Nearest robust unrolling competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Paper abstract indexed by PubMed and publisher citation. Feature codes remain provisional. Which PSF errors are held out, and does the design distinguish noise from operator error? Extract any real-system validation. Evidence: https://pubmed.ncbi.nlm.nih.gov/39573193/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P029, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="112" customHeight="1">
@@ -4449,7 +4457,7 @@
         <x:v>https://doi.org/10.1109/LSP.2024.3361806</x:v>
       </x:c>
       <x:c r="AF31" s="75" t="str">
-        <x:v>Bayesian baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional publication abstract and author list. Feature codes remain provisional. What uncertainty is lost by conditioning on an estimated representation, and what calibration or shift tests are reported? Evidence: https://www.research.ed.ac.uk/en/publications/empirical-bayesian-imaging-with-large-scale-push-forward-generati/</x:v>
+        <x:v>Bayesian baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional publication abstract and author list. Feature codes remain provisional. What uncertainty is lost by conditioning on an estimated representation, and what calibration or shift tests are reported? Evidence: https://www.research.ed.ac.uk/en/publications/empirical-bayesian-imaging-with-large-scale-push-forward-generati/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P030, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="176" customHeight="1">
@@ -4939,7 +4947,7 @@
         <x:v>https://doi.org/10.1117/12.3098133</x:v>
       </x:c>
       <x:c r="AF36" s="75" t="str">
-        <x:v>Highest-priority mismatch competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional abstract and complete proceedings metadata. Feature codes remain provisional. Can a flexible residual absorb noise or unsupported image detail? Extract identifiability constraints, optimization and held-out mismatch tests. Evidence: https://pure.kaist.ac.kr/en/publications/mitigating-forward-model-mismatch-in-inverse-problems-via-learned/</x:v>
+        <x:v>Highest-priority mismatch competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional abstract and complete proceedings metadata. Feature codes remain provisional. Can a flexible residual absorb noise or unsupported image detail? Extract identifiability constraints, optimization and held-out mismatch tests. Evidence: https://pure.kaist.ac.kr/en/publications/mitigating-forward-model-mismatch-in-inverse-problems-via-learned/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P035, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="176" customHeight="1">
@@ -5429,7 +5437,7 @@
         <x:v>https://doi.org/10.1109/TPAMI.2025.3598457</x:v>
       </x:c>
       <x:c r="AF41" s="75" t="str">
-        <x:v>Critical nearest competitor; reproduce blind Zernike experiment in pilot | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional paper abstract and official repository experiment descriptions. Feature codes remain provisional. Inspect the final paper, uncertainty treatment, changing-PSF assumptions and real-capture validation. Video plus joint time-varying operator recovery alone cannot be claimed as new. Evidence: https://pure.kaist.ac.kr/en/publications/video-diffusion-posterior-sampling-for-seeing-beyond-dynamic-scat-2/</x:v>
+        <x:v>Critical nearest competitor; reproduce blind Zernike experiment in pilot | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional paper abstract and official repository experiment descriptions. Feature codes remain provisional. Inspect the final paper, uncertainty treatment, changing-PSF assumptions and real-capture validation. Video plus joint time-varying operator recovery alone cannot be claimed as new. Evidence: https://pure.kaist.ac.kr/en/publications/video-diffusion-posterior-sampling-for-seeing-beyond-dynamic-scat-2/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P040, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="176" customHeight="1">
@@ -5788,7 +5796,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="U45" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V45" s="75" t="str">
         <x:v>No</x:v>
@@ -5803,7 +5811,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z45" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA45" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -5821,7 +5829,7 @@
         <x:v>https://doi.org/10.1109/WACV48630.2021.00045</x:v>
       </x:c>
       <x:c r="AF45" s="75" t="str">
-        <x:v>Important real-hardware joint-estimation precedent | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete institutional publication abstract and DOI metadata. Feature codes remain provisional. Are evaluated cameras or PSF families genuinely held out, and is uncertainty propagated beyond a point PSF estimate? Evidence: https://asu.elsevierpure.com/en/publications/robust-lensless-image-reconstruction-via-psf-estimation/</x:v>
+        <x:v>Important real-hardware joint-estimation precedent | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete institutional publication abstract and DOI metadata. Feature codes remain provisional. Are evaluated cameras or PSF families genuinely held out, and is uncertainty propagated beyond a point PSF estimate? Evidence: https://asu.elsevierpure.com/en/publications/robust-lensless-image-reconstruction-via-psf-estimation/ | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_09.json (P044). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="46" ht="176" customHeight="1">
@@ -6311,7 +6319,7 @@
         <x:v>https://doi.org/10.1109/TGRS.2024.3415372</x:v>
       </x:c>
       <x:c r="AF50" s="75" t="str">
-        <x:v>Occupies broad time-varying operator claim | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Publisher-indexed title and abstract excerpt; IEEE PDF retrieval failed and HAL challenged. Feature codes remain provisional. Retrieve the full text to verify the physical parameterization, motion identification, synthetic versus real evidence and any uncertainty analysis. Evidence: https://ieeexplore.ieee.org/document/10559627/</x:v>
+        <x:v>Occupies broad time-varying operator claim | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Publisher-indexed title and abstract excerpt; IEEE PDF retrieval failed and HAL challenged. Feature codes remain provisional. Retrieve the full text to verify the physical parameterization, motion identification, synthetic versus real evidence and any uncertainty analysis. Evidence: https://ieeexplore.ieee.org/document/10559627/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P049, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="176" customHeight="1">
@@ -6703,7 +6711,7 @@
         <x:v>https://doi.org/10.1007/s11263-026-02977-y</x:v>
       </x:c>
       <x:c r="AF54" s="75" t="str">
-        <x:v>Closest 2026 all-in-one video competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete publisher abstract and publication metadata. Feature codes remain provisional. Compare its study lineage and experiments with P026 AverNet before counting independent evidence. Verify temporal/compound settings and complete code/data release rather than infer release from a link. Evidence: https://link.springer.com/article/10.1007/s11263-026-02977-y</x:v>
+        <x:v>Closest 2026 all-in-one video competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete publisher abstract and publication metadata. Feature codes remain provisional. Compare its study lineage and experiments with P026 AverNet before counting independent evidence. Verify temporal/compound settings and complete code/data release rather than infer release from a link. Evidence: https://link.springer.com/article/10.1007/s11263-026-02977-y | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P053, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="176" customHeight="1">
@@ -6863,7 +6871,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T56" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U56" s="75" t="str">
         <x:v>Yes</x:v>
@@ -6881,7 +6889,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z56" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA56" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -6899,7 +6907,7 @@
         <x:v>https://doi.org/10.1007/978-3-031-20068-7_33</x:v>
       </x:c>
       <x:c r="AF56" s="75" t="str">
-        <x:v>Compound-degradation baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. How are blur, exposure, noise and processing ordered in synthesis? Determine which real examples have trustworthy references. Evidence: https://arxiv.org/abs/2202.03373</x:v>
+        <x:v>Compound-degradation baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract. Feature codes remain provisional. How are blur, exposure, noise and processing ordered in synthesis? Determine which real examples have trustworthy references. Evidence: https://arxiv.org/abs/2202.03373 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_09.json (P055). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="176" customHeight="1">
@@ -7163,7 +7171,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="V59" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>No</x:v>
       </x:c>
       <x:c r="W59" s="75" t="str">
         <x:v>No</x:v>
@@ -7175,7 +7183,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z59" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA59" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -7193,7 +7201,7 @@
         <x:v>https://doi.org/10.1109/ICCV48922.2021.00474</x:v>
       </x:c>
       <x:c r="AF59" s="75" t="str">
-        <x:v>Real paired degradation benchmark | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete institutional publication abstract and DOI metadata. Feature codes remain provisional. Quantify reference alignment and color bias, device separation and whether errors attributed to reconstruction could arise from imperfect ground truth. Evidence: https://research.polyu.edu.hk/en/publications/real-world-video-super-resolution-a-benchmark-dataset-and-a-decom/</x:v>
+        <x:v>Real paired degradation benchmark | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete institutional publication abstract and DOI metadata. Feature codes remain provisional. Quantify reference alignment and color bias, device separation and whether errors attributed to reconstruction could arise from imperfect ground truth. Evidence: https://research.polyu.edu.hk/en/publications/real-world-video-super-resolution-a-benchmark-dataset-and-a-decom/ | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, X. Evidence/version/read extent: screening/full_text_09.json (P058). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="60" ht="176" customHeight="1">
@@ -8612,13 +8620,13 @@
         <x:v>Implicit</x:v>
       </x:c>
       <x:c r="O74" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="P74" s="75" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="Q74" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="R74" s="75" t="str">
         <x:v>No</x:v>
@@ -8627,7 +8635,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="T74" s="75" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="U74" s="75" t="str">
         <x:v>Yes</x:v>
@@ -8639,13 +8647,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="X74" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="Y74" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="Z74" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA74" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -8663,7 +8671,7 @@
         <x:v>https://doi.org/10.1007/978-3-031-73661-2_19</x:v>
       </x:c>
       <x:c r="AF74" s="75" t="str">
-        <x:v>Closest automatic generative all-in-one baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and existing ECCV lineage. Feature codes remain provisional. Which unknown or combined degradations are tested independently of training, and how is structural or semantic fidelity measured? Evidence: https://arxiv.org/abs/2310.10123</x:v>
+        <x:v>Closest automatic generative all-in-one baseline | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete author preprint abstract and existing ECCV lineage. Feature codes remain provisional. Which unknown or combined degradations are tested independently of training, and how is structural or semantic fidelity measured? Evidence: https://arxiv.org/abs/2310.10123 | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_09.json (P073). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="176" customHeight="1">
@@ -10341,7 +10349,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R57e62b74796146dc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59aa96b4ce2f485e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11533,7 +11541,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="112" customHeight="1">
+    <x:row r="30" ht="144" customHeight="1">
       <x:c r="A30" s="73" t="str">
         <x:v>S029</x:v>
       </x:c>
@@ -11556,7 +11564,7 @@
       <x:c r="H30" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I30" s="81" t="str">
+      <x:c r="I30" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
       <x:c r="J30" s="75" t="str">
@@ -11564,7 +11572,7 @@
       </x:c>
       <x:c r="K30" s="75"/>
       <x:c r="L30" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Explicit model-mismatch and noise robustness. Basis: Paper abstract indexed by PubMed and publisher citation. Sources and full-text question: screening/pilot_02.json (P029).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. HTML JavaScript verification page, not PDF. Obtain the publisher PDF or an author manuscript. Complete retrieval log: screening/full_text_09.json (P029).</x:v>
       </x:c>
       <x:c r="M30" s="75" t="str">
         <x:v>No</x:v>
@@ -11573,7 +11581,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="31" ht="112" customHeight="1">
+    <x:row r="31" ht="144" customHeight="1">
       <x:c r="A31" s="73" t="str">
         <x:v>S030</x:v>
       </x:c>
@@ -11596,7 +11604,7 @@
       <x:c r="H31" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I31" s="81" t="str">
+      <x:c r="I31" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
       <x:c r="J31" s="75" t="str">
@@ -11604,7 +11612,7 @@
       </x:c>
       <x:c r="K31" s="75"/>
       <x:c r="L31" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Bayesian reconstruction uncertainty. Basis: Authors' institutional publication abstract and author list. Sources and full-text question: screening/pilot_02.json (P030).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. HTTP 403; no manuscript acquired. Obtain the accepted manuscript from the institutional record or publisher. Complete retrieval log: screening/full_text_09.json (P030).</x:v>
       </x:c>
       <x:c r="M31" s="75" t="str">
         <x:v>No</x:v>
@@ -11773,7 +11781,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="112" customHeight="1">
+    <x:row r="36" ht="144" customHeight="1">
       <x:c r="A36" s="73" t="str">
         <x:v>S035</x:v>
       </x:c>
@@ -11796,7 +11804,7 @@
       <x:c r="H36" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I36" s="81" t="str">
+      <x:c r="I36" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
       <x:c r="J36" s="75" t="str">
@@ -11804,7 +11812,7 @@
       </x:c>
       <x:c r="K36" s="75"/>
       <x:c r="L36" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Learned residual compensation for forward-model mismatch. Basis: Authors' institutional abstract and complete proceedings metadata. Sources and full-text question: screening/pilot_02.json (P035).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. Incapsula request-unsuccessful HTML; indexed snippets insufficient. Obtain the SPIE proceedings paper or an author manuscript. Complete retrieval log: screening/full_text_09.json (P035).</x:v>
       </x:c>
       <x:c r="M36" s="75" t="str">
         <x:v>No</x:v>
@@ -11973,7 +11981,7 @@
         <x:v>Yes</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="112" customHeight="1">
+    <x:row r="41" ht="144" customHeight="1">
       <x:c r="A41" s="73" t="str">
         <x:v>S040</x:v>
       </x:c>
@@ -11996,7 +12004,7 @@
       <x:c r="H41" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I41" s="81" t="str">
+      <x:c r="I41" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
       <x:c r="J41" s="75" t="str">
@@ -12004,7 +12012,7 @@
       </x:c>
       <x:c r="K41" s="75"/>
       <x:c r="L41" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Blind video reconstruction under dynamic physical degradation. Basis: Authors' institutional paper abstract and official repository experiment descriptions. Sources and full-text question: screening/pilot_02.json (P040).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. HTTP 418; no PDF acquired. Obtain the TPAMI paper; code and demonstrations do not replace eligibility assessment. Complete retrieval log: screening/full_text_09.json (P040).</x:v>
       </x:c>
       <x:c r="M41" s="75" t="str">
         <x:v>No</x:v>
@@ -12156,18 +12164,18 @@
       <x:c r="H45" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I45" s="91" t="str">
+      <x:c r="I45" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J45" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K45" s="75"/>
+      <x:c r="J45" s="106" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K45" s="75" t="str"/>
       <x:c r="L45" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint image/PSF estimation without test-time PSF access. Basis: Complete institutional publication abstract and DOI metadata. Sources and full-text question: screening/pilot_03.json (P044).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Joint PSF/image inference and added-noise robustness. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_09.json (P044).</x:v>
       </x:c>
       <x:c r="M45" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N45" s="75" t="str">
         <x:v>Yes</x:v>
@@ -12356,7 +12364,7 @@
       <x:c r="H50" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I50" s="91" t="str">
+      <x:c r="I50" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
       <x:c r="J50" s="75" t="str">
@@ -12364,7 +12372,7 @@
       </x:c>
       <x:c r="K50" s="75"/>
       <x:c r="L50" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Explicit correction of acquisition micro-vibrations in pushbroom satellite imaging. Basis: Publisher-indexed title and abstract excerpt; IEEE PDF retrieval failed and HAL challenged. Sources and full-text question: screening/pilot_03.json (P049).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. HAL verification/access-denied page. Obtain the HAL author manuscript or publisher PDF. Complete retrieval log: screening/full_text_09.json (P049).</x:v>
       </x:c>
       <x:c r="M50" s="75" t="str">
         <x:v>No</x:v>
@@ -12516,7 +12524,7 @@
       <x:c r="H54" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I54" s="91" t="str">
+      <x:c r="I54" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
       <x:c r="J54" s="75" t="str">
@@ -12524,7 +12532,7 @@
       </x:c>
       <x:c r="K54" s="75"/>
       <x:c r="L54" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Unknown and time-varying multi-degradation video restoration. Basis: Complete publisher abstract and publication metadata. Sources and full-text question: screening/pilot_03.json (P053).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. Abstract/access page, not complete methods. Obtain the full IJCV article and check its relationship to P026/AverNet. Complete retrieval log: screening/full_text_09.json (P053).</x:v>
       </x:c>
       <x:c r="M54" s="75" t="str">
         <x:v>No</x:v>
@@ -12596,18 +12604,18 @@
       <x:c r="H56" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I56" s="91" t="str">
+      <x:c r="I56" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J56" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K56" s="75"/>
+      <x:c r="J56" s="106" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K56" s="75" t="str"/>
       <x:c r="L56" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Joint low-light enhancement and deblurring. Basis: Complete author preprint abstract. Sources and full-text question: screening/pilot_03.json (P055).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Compound low-light/blur/noise restoration with synthetic-to-real evaluation. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_09.json (P055).</x:v>
       </x:c>
       <x:c r="M56" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N56" s="75" t="str">
         <x:v>Yes</x:v>
@@ -12716,18 +12724,18 @@
       <x:c r="H59" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I59" s="91" t="str">
+      <x:c r="I59" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J59" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K59" s="75"/>
+      <x:c r="J59" s="106" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K59" s="75" t="str"/>
       <x:c r="L59" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Real acquisition mismatch and cross-camera video restoration. Basis: Complete institutional publication abstract and DOI metadata. Sources and full-text question: screening/pilot_03.json (P058).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Real acquisition mismatch and cross-camera restoration tests. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_09.json (P058).</x:v>
       </x:c>
       <x:c r="M59" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N59" s="75" t="str">
         <x:v>Yes</x:v>
@@ -13318,18 +13326,18 @@
       <x:c r="H74" s="73" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="I74" s="91" t="str">
+      <x:c r="I74" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J74" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K74" s="75"/>
+      <x:c r="J74" s="106" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K74" s="75" t="str"/>
       <x:c r="L74" s="75" t="str">
-        <x:v>2026-09-16 | AI only; human pending. Automatic unknown-degradation detection and all-in-one restoration. Basis: Complete author preprint abstract and existing ECCV lineage. Sources and full-text question: screening/pilot_03.json (P073).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Unknown compound restoration with held-out acquisition tasks. PDF retrieved for assessment; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_09.json (P073).</x:v>
       </x:c>
       <x:c r="M74" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N74" s="75" t="str">
         <x:v>Yes</x:v>
@@ -14316,7 +14324,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf96550a7849344e9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7fe8e597b9c4cc8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14488,7 +14496,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 80 (79 include, 1 exclude), 10 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 84 (83 include, 1 exclude), 6 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14496,7 +14504,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json, full_text_06.json, full_text_07.json and full_text_08.json; current report: full_text_08_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json, full_text_06.json, full_text_07.json, full_text_08.json and full_text_09.json; current report: full_text_09_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14742,7 +14750,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7107ac29fef4b12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R465accd4b2394780"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record full-text checkpoint 10 (85 assessed, 5 pending)
Resolve P029 from complete publisher-supplied text and record criterion-level
eligibility, inspected extent and bounded feature codes. Distinguish mismatch
nuisance estimation from physical operator recovery and calibrated uncertainty.

Record alternate-source checks and download routes for P030, P035, P040,
P049 and P053. Preserve pending decisions when full text is unavailable.
Do not substitute abstracts, code or unverified related versions.

Synchronize the matrix, screening tracker, four reference exports and status
documents. Cumulative AI decisions: 84 include, 1 exclude, 5 pending.
Formal inclusion, human adjudication and novelty remain unresolved.

Validation: reconciled 85 unique assessed IDs across ten registers; verified
90 reference entries, formula recalculation and export/reimport. Preserved
five sheets, three tables, chart, merges, panes and validation rules.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6c6bbef7e86a4ab6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R5805a0a486da4c53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rd23251ca970a483b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R11c845edd7414b80"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="Rb470cd64c9ed4950"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R73d63f19cc2e4249"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="Rdc260367bbf64eac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="R4b67e9cee9ef46fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R328860776e464c7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R9d348ebee473436e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="24">
+  <x:fills count="25">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -292,7 +297,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="107">
+  <x:cellXfs count="108">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -530,6 +535,9 @@
     <x:xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -761,7 +769,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R152de408bfb94da8"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R056d6c583e814dca"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1210,7 +1218,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1227,7 +1235,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>Joint PSF estimation, compound night restoration, cross-camera video transfer and clean-class stopping have comparators. Six full texts remain pending. See screening/full_text_09_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
+        <x:v>P029 adds a structured mismatch-correction comparator. Calibrated operator uncertainty and selective release are not demonstrated there. Five full texts remain pending. See screening/full_text_10_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1282,7 +1290,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;" remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 84/90 (83 include, 1 exclude); 6 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 85/90 (84 include, 1 exclude); 5 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1377,7 +1385,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0257f4dd79b249b4"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d48630302c74a8a"/>
 </x:worksheet>
 </file>
 
@@ -4264,7 +4272,7 @@
         <x:v>Generative baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract with CVPR acceptance identified. Feature codes remain provisional. How do prompts and prior strength affect invented detail? Extract quantitative fidelity tests and inference costs before choosing a baseline. Evidence: https://arxiv.org/abs/2401.13627 | AI full-text 2026-09-16: include; human pending. Verified fields: O, Q, R, T, U, W, X. Evidence/version/read extent: screening/full_text_06.json (P028). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="30" ht="112" customHeight="1">
+    <x:row r="30" ht="176" customHeight="1">
       <x:c r="A30" s="85" t="str">
         <x:v>P029</x:v>
       </x:c>
@@ -4320,13 +4328,13 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="S30" s="75" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Partial</x:v>
       </x:c>
       <x:c r="T30" s="75" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="U30" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="V30" s="75" t="str">
         <x:v>No</x:v>
@@ -4341,7 +4349,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z30" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA30" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4359,7 +4367,7 @@
         <x:v>https://opg.optica.org/oe/abstract.cfm?uri=oe-32-17-30267</x:v>
       </x:c>
       <x:c r="AF30" s="75" t="str">
-        <x:v>Nearest robust unrolling competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Paper abstract indexed by PubMed and publisher citation. Feature codes remain provisional. Which PSF errors are held out, and does the design distinguish noise from operator error? Extract any real-system validation. Evidence: https://pubmed.ncbi.nlm.nih.gov/39573193/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P029, pending_access). No new feature verification.</x:v>
+        <x:v>Nearest robust unrolling competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Paper abstract indexed by PubMed and publisher citation. Feature codes remain provisional. Which PSF errors are held out, and does the design distinguish noise from operator error? Extract any real-system validation. Evidence: https://pubmed.ncbi.nlm.nih.gov/39573193/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P029, pending_access). No new feature verification. | AI full-text 2026-09-16: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_10.json (P029). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="112" customHeight="1">
@@ -4457,7 +4465,7 @@
         <x:v>https://doi.org/10.1109/LSP.2024.3361806</x:v>
       </x:c>
       <x:c r="AF31" s="75" t="str">
-        <x:v>Bayesian baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional publication abstract and author list. Feature codes remain provisional. What uncertainty is lost by conditioning on an estimated representation, and what calibration or shift tests are reported? Evidence: https://www.research.ed.ac.uk/en/publications/empirical-bayesian-imaging-with-large-scale-push-forward-generati/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P030, pending_access). No new feature verification.</x:v>
+        <x:v>Bayesian baseline | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional publication abstract and author list. Feature codes remain provisional. What uncertainty is lost by conditioning on an estimated representation, and what calibration or shift tests are reported? Evidence: https://www.research.ed.ac.uk/en/publications/empirical-bayesian-imaging-with-large-scale-push-forward-generati/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P030, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_10.json (P030, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="176" customHeight="1">
@@ -4947,7 +4955,7 @@
         <x:v>https://doi.org/10.1117/12.3098133</x:v>
       </x:c>
       <x:c r="AF36" s="75" t="str">
-        <x:v>Highest-priority mismatch competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional abstract and complete proceedings metadata. Feature codes remain provisional. Can a flexible residual absorb noise or unsupported image detail? Extract identifiability constraints, optimization and held-out mismatch tests. Evidence: https://pure.kaist.ac.kr/en/publications/mitigating-forward-model-mismatch-in-inverse-problems-via-learned/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P035, pending_access). No new feature verification.</x:v>
+        <x:v>Highest-priority mismatch competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional abstract and complete proceedings metadata. Feature codes remain provisional. Can a flexible residual absorb noise or unsupported image detail? Extract identifiability constraints, optimization and held-out mismatch tests. Evidence: https://pure.kaist.ac.kr/en/publications/mitigating-forward-model-mismatch-in-inverse-problems-via-learned/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P035, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_10.json (P035, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="176" customHeight="1">
@@ -5437,7 +5445,7 @@
         <x:v>https://doi.org/10.1109/TPAMI.2025.3598457</x:v>
       </x:c>
       <x:c r="AF41" s="75" t="str">
-        <x:v>Critical nearest competitor; reproduce blind Zernike experiment in pilot | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional paper abstract and official repository experiment descriptions. Feature codes remain provisional. Inspect the final paper, uncertainty treatment, changing-PSF assumptions and real-capture validation. Video plus joint time-varying operator recovery alone cannot be claimed as new. Evidence: https://pure.kaist.ac.kr/en/publications/video-diffusion-posterior-sampling-for-seeing-beyond-dynamic-scat-2/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P040, pending_access). No new feature verification.</x:v>
+        <x:v>Critical nearest competitor; reproduce blind Zernike experiment in pilot | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional paper abstract and official repository experiment descriptions. Feature codes remain provisional. Inspect the final paper, uncertainty treatment, changing-PSF assumptions and real-capture validation. Video plus joint time-varying operator recovery alone cannot be claimed as new. Evidence: https://pure.kaist.ac.kr/en/publications/video-diffusion-posterior-sampling-for-seeing-beyond-dynamic-scat-2/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P040, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_10.json (P040, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="176" customHeight="1">
@@ -6319,7 +6327,7 @@
         <x:v>https://doi.org/10.1109/TGRS.2024.3415372</x:v>
       </x:c>
       <x:c r="AF50" s="75" t="str">
-        <x:v>Occupies broad time-varying operator claim | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Publisher-indexed title and abstract excerpt; IEEE PDF retrieval failed and HAL challenged. Feature codes remain provisional. Retrieve the full text to verify the physical parameterization, motion identification, synthetic versus real evidence and any uncertainty analysis. Evidence: https://ieeexplore.ieee.org/document/10559627/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P049, pending_access). No new feature verification.</x:v>
+        <x:v>Occupies broad time-varying operator claim | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Publisher-indexed title and abstract excerpt; IEEE PDF retrieval failed and HAL challenged. Feature codes remain provisional. Retrieve the full text to verify the physical parameterization, motion identification, synthetic versus real evidence and any uncertainty analysis. Evidence: https://ieeexplore.ieee.org/document/10559627/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P049, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_10.json (P049, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="176" customHeight="1">
@@ -6711,7 +6719,7 @@
         <x:v>https://doi.org/10.1007/s11263-026-02977-y</x:v>
       </x:c>
       <x:c r="AF54" s="75" t="str">
-        <x:v>Closest 2026 all-in-one video competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete publisher abstract and publication metadata. Feature codes remain provisional. Compare its study lineage and experiments with P026 AverNet before counting independent evidence. Verify temporal/compound settings and complete code/data release rather than infer release from a link. Evidence: https://link.springer.com/article/10.1007/s11263-026-02977-y | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P053, pending_access). No new feature verification.</x:v>
+        <x:v>Closest 2026 all-in-one video competitor | AI pilot 2026-09-16: AI pilot: advance; human pending. Basis: Complete publisher abstract and publication metadata. Feature codes remain provisional. Compare its study lineage and experiments with P026 AverNet before counting independent evidence. Verify temporal/compound settings and complete code/data release rather than infer release from a link. Evidence: https://link.springer.com/article/10.1007/s11263-026-02977-y | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P053, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_10.json (P053, pending_access). No new feature verification.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="176" customHeight="1">
@@ -10349,7 +10357,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59aa96b4ce2f485e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re65bd4557f0f47d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11567,12 +11575,12 @@
       <x:c r="I30" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J30" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K30" s="75"/>
+      <x:c r="J30" s="107" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K30" s="75" t="str"/>
       <x:c r="L30" s="75" t="str">
-        <x:v>2026-09-16 | Full-text eligibility remains pending. HTML JavaScript verification page, not PDF. Obtain the publisher PDF or an author manuscript. Complete retrieval log: screening/full_text_09.json (P029).</x:v>
+        <x:v>2026-09-16 | AI full-text include; human pending. Explicit forward-model error and noise handling. Online full text inspected; no local PDF acquired. Version, read extent and technical extraction: screening/full_text_10.json (P029).</x:v>
       </x:c>
       <x:c r="M30" s="75" t="str">
         <x:v>No</x:v>
@@ -11612,7 +11620,7 @@
       </x:c>
       <x:c r="K31" s="75"/>
       <x:c r="L31" s="75" t="str">
-        <x:v>2026-09-16 | Full-text eligibility remains pending. HTTP 403; no manuscript acquired. Obtain the accepted manuscript from the institutional record or publisher. Complete retrieval log: screening/full_text_09.json (P030).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. Institutional record retrieved; citation metadata exposes a manuscript PDF link. Obtain the accepted manuscript from the institutional record or publisher. Complete retrieval log: screening/full_text_10.json (P030).</x:v>
       </x:c>
       <x:c r="M31" s="75" t="str">
         <x:v>No</x:v>
@@ -11812,7 +11820,7 @@
       </x:c>
       <x:c r="K36" s="75"/>
       <x:c r="L36" s="75" t="str">
-        <x:v>2026-09-16 | Full-text eligibility remains pending. Incapsula request-unsuccessful HTML; indexed snippets insufficient. Obtain the SPIE proceedings paper or an author manuscript. Complete retrieval log: screening/full_text_09.json (P035).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. Incapsula verification HTML returned instead of a PDF; full text not acquired. Obtain the SPIE proceedings paper or an author manuscript. Complete retrieval log: screening/full_text_10.json (P035).</x:v>
       </x:c>
       <x:c r="M36" s="75" t="str">
         <x:v>No</x:v>
@@ -12012,7 +12020,7 @@
       </x:c>
       <x:c r="K41" s="75"/>
       <x:c r="L41" s="75" t="str">
-        <x:v>2026-09-16 | Full-text eligibility remains pending. HTTP 418; no PDF acquired. Obtain the TPAMI paper; code and demonstrations do not replace eligibility assessment. Complete retrieval log: screening/full_text_09.json (P040).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. Abstract and request-full-text record; complete article unavailable. Obtain the TPAMI paper; code and demonstrations do not replace eligibility assessment. Complete retrieval log: screening/full_text_10.json (P040).</x:v>
       </x:c>
       <x:c r="M41" s="75" t="str">
         <x:v>No</x:v>
@@ -12372,7 +12380,7 @@
       </x:c>
       <x:c r="K50" s="75"/>
       <x:c r="L50" s="75" t="str">
-        <x:v>2026-09-16 | Full-text eligibility remains pending. HAL verification/access-denied page. Obtain the HAL author manuscript or publisher PDF. Complete retrieval log: screening/full_text_09.json (P049).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. Public OpenAlex location check and targeted author searches did not yield a new manuscript route; HAL remains the alternate locator. Obtain the HAL author manuscript or publisher PDF. Complete retrieval log: screening/full_text_10.json (P049).</x:v>
       </x:c>
       <x:c r="M50" s="75" t="str">
         <x:v>No</x:v>
@@ -12532,7 +12540,7 @@
       </x:c>
       <x:c r="K54" s="75"/>
       <x:c r="L54" s="75" t="str">
-        <x:v>2026-09-16 | Full-text eligibility remains pending. Abstract/access page, not complete methods. Obtain the full IJCV article and check its relationship to P026/AverNet. Complete retrieval log: screening/full_text_09.json (P053).</x:v>
+        <x:v>2026-09-16 | Full-text eligibility remains pending. Public OpenAlex location check and targeted author searches did not yield a new manuscript route; publisher record remains the primary locator. Obtain the full IJCV article and check its relationship to P026/AverNet. Complete retrieval log: screening/full_text_10.json (P053).</x:v>
       </x:c>
       <x:c r="M54" s="75" t="str">
         <x:v>No</x:v>
@@ -14324,7 +14332,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7fe8e597b9c4cc8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re45d785f189c4129"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14496,7 +14504,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 84 (83 include, 1 exclude), 6 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 85 (84 include, 1 exclude), 5 remain. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14504,7 +14512,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json, full_text_06.json, full_text_07.json, full_text_08.json and full_text_09.json; current report: full_text_09_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative full-text progress: screening/full_text_01.json, full_text_02.json, full_text_03.json, full_text_04.json, full_text_05.json, full_text_06.json, full_text_07.json, full_text_08.json, full_text_09.json and full_text_10.json; current report: full_text_10_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14750,7 +14758,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R465accd4b2394780"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1359f49ef87e457a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Assess final P035 full text and close the 90-record AI reading pass
Assess the user-supplied SPIE article from Professor Jang, recording identity,
source hash, criterion-level evidence, feature codes and reproduction limits.
Update the matrix, screening log and CSV/BibTeX/RIS references to 90 assessed:
89 include recommendations, one exclude, zero awaiting full text.

Document overlap in residual correction, signal absorption, valid-region
recovery and the empirical mismatch threshold. Distinguish the reference-
dependent threshold from observable calibrated selection. Retain the original
topic and require experimental benefit before claiming novelty.

Validate counts, formula recalculation, earlier decisions, native tables,
validation, panes, charts and relationship targets; inspect changed views.
Preserve historical checkpoints, formal decisions and prior experiment files.
The supplied paper and rendered pages are not redistributed.
</commit_message>
<xml_diff>
--- a/literature/evidence_matrix_2020_2026.xlsx
+++ b/literature/evidence_matrix_2020_2026.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Refcfa4fca632467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="R9a0e462952ef4815"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rf26e1b8fcdb743d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="R9b9ce02431894193"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R53a8c9c10dfd4ac5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R039e26a8fd594c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence Matrix" sheetId="2" r:id="Re686833d78b74fe1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Screening Log" sheetId="3" r:id="Rebc00e9bb39e4902"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review Protocol" sheetId="4" r:id="Rebe98aaff75c4959"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coding Dictionary" sheetId="5" r:id="R3be504c6b8fb434f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -79,7 +79,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="26">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,6 +154,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -302,7 +307,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="109">
+  <x:cellXfs count="110">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -546,6 +551,9 @@
     <x:xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -777,7 +785,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8e871800755d429a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8c010afd271142d0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1226,7 +1234,7 @@
       </x:c>
       <x:c r="E15" s="98" t="n">
         <x:f>COUNTIF('Screening Log'!J2:J101,"AI full-text: include")+COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")</x:f>
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1243,7 +1251,7 @@
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="32" t="str">
-        <x:v>VDPS confirms blind time-varying physical-parameter estimation. FaverNet follows AverNet; image sampling and variance maps do not establish calibration. Only P035 full text remains pending. See screening/full_text_11_report.md for assumptions and version-specific limits. Earlier checkpoints remain available. Novelty is unestablished.</x:v>
+        <x:v>P035 adds learned residual correction and an empirical failure threshold. Its true-model discrepancy is not a calibrated score for unknown captures. Test observable reliability scores against strong controls. See screening/full_text_12_report.md. Novelty remains unestablished.</x:v>
       </x:c>
       <x:c r="B17" s="32"/>
       <x:c r="C17" s="32"/>
@@ -1298,7 +1306,7 @@
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="35" t="str">
         <x:f>"Initial triage: 90/90. AI full-text assessed: "&amp;E15&amp;"/90 ("&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: include")&amp;" include, "&amp;COUNTIF('Screening Log'!J2:J101,"AI full-text: exclude")&amp;" exclude); "&amp;(B6-E15)&amp;IF(B6-E15=1," remains."," remain.")&amp;" Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified."</x:f>
-        <x:v>Initial triage: 90/90. AI full-text assessed: 89/90 (88 include, 1 exclude); 1 remains. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
+        <x:v>Initial triage: 90/90. AI full-text assessed: 90/90 (89 include, 1 exclude); 0 remain. Human adjudication and formal inclusion pending. Novelty unestablished. Only explicitly logged features are verified.</x:v>
       </x:c>
       <x:c r="B22" s="35"/>
       <x:c r="C22" s="35"/>
@@ -1393,7 +1401,7 @@
     <x:mergeCell ref="A27:H29"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0cbaaa64dd645a7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd51fec3a26b745f3"/>
 </x:worksheet>
 </file>
 
@@ -4868,7 +4876,7 @@
         <x:v>Failure-detection candidate | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Author preprint abstract; final conference metadata still pending. Feature codes remain provisional. Does it generalize to natural images and unseen acquisition families? Calibration-free estimation is not a coverage guarantee. Resolve the CAMSAP lineage before locking metadata. Evidence: https://arxiv.org/abs/2510.10947 | AI full-text 2026-09-16: include; human pending. Verified fields: P, Q, R, S, T, X. Evidence/version/read extent: screening/full_text_02.json (P034). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="112" customHeight="1">
+    <x:row r="36" ht="176" customHeight="1">
       <x:c r="A36" s="85" t="str">
         <x:v>P035</x:v>
       </x:c>
@@ -4876,13 +4884,13 @@
         <x:v>2026</x:v>
       </x:c>
       <x:c r="C36" s="75" t="str">
-        <x:v>Lee &amp; Jang</x:v>
+        <x:v>Lee, Chanseok; Jang, Mooseok</x:v>
       </x:c>
       <x:c r="D36" s="75" t="str">
         <x:v>Mitigating Forward Model Mismatch in Inverse Problems via Learned Residuals and Diffusion Priors</x:v>
       </x:c>
       <x:c r="E36" s="75" t="str">
-        <x:v>SPIE</x:v>
+        <x:v>Proceedings of SPIE 14016, 140160D (SPIE ABC 2025; published 2026)</x:v>
       </x:c>
       <x:c r="F36" s="75" t="str">
         <x:v>Conference</x:v>
@@ -4891,22 +4899,22 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H36" s="75" t="str">
-        <x:v>Computational imaging</x:v>
+        <x:v>Digital holographic microscopy; scattering imaging</x:v>
       </x:c>
       <x:c r="I36" s="75" t="str">
-        <x:v>Scientific imaging</x:v>
+        <x:v>Beads and tissue fields; simulated scattering</x:v>
       </x:c>
       <x:c r="J36" s="75" t="str">
-        <x:v>Approximate differentiable operator</x:v>
+        <x:v>Diffraction intensity F(x,d); memory-effect convolution</x:v>
       </x:c>
       <x:c r="K36" s="75" t="str">
         <x:v>Approximate</x:v>
       </x:c>
       <x:c r="L36" s="75" t="str">
-        <x:v>Residual model discrepancy</x:v>
+        <x:v>Propagation-distance error; violation of angular memory effect</x:v>
       </x:c>
       <x:c r="M36" s="75" t="str">
-        <x:v>Diffusion plus learned residual</x:v>
+        <x:v>Diffusion posterior sampling with learned additive residual</x:v>
       </x:c>
       <x:c r="N36" s="75" t="str">
         <x:v>Soft likelihood</x:v>
@@ -4915,37 +4923,37 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="P36" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q36" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="R36" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="S36" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="Q36" s="75" t="str">
+      <x:c r="T36" s="75" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="U36" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="V36" s="75" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="W36" s="75" t="str">
         <x:v>Partial</x:v>
       </x:c>
-      <x:c r="R36" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="S36" s="75" t="str">
-        <x:v>Yes</x:v>
-      </x:c>
-      <x:c r="T36" s="75" t="str">
+      <x:c r="X36" s="75" t="str">
         <x:v>Partial</x:v>
-      </x:c>
-      <x:c r="U36" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="V36" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="W36" s="75" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="X36" s="75" t="str">
-        <x:v>No</x:v>
       </x:c>
       <x:c r="Y36" s="75" t="str">
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="Z36" s="75" t="str">
-        <x:v>Abstract inspected; full-text pending</x:v>
+        <x:v>AI full-text eligibility assessed; selected features verified</x:v>
       </x:c>
       <x:c r="AA36" s="75" t="str">
         <x:v>Pending formal eligibility</x:v>
@@ -4954,16 +4962,16 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="AC36" s="75" t="str">
-        <x:v>Learns measurement residual mismatch during diffusion inversion</x:v>
+        <x:v>Regularised residual correction, two-stage diffusion refinement and empirical mismatch boundary</x:v>
       </x:c>
       <x:c r="AD36" s="75" t="str">
-        <x:v>No calibrated joint UQ, abstention or surveillance benchmark</x:v>
+        <x:v>No calibrated selected-region error control; threshold uses true/perturbed model evaluations. Valid-region recovery is simulated; source-disjoint validation underreported.</x:v>
       </x:c>
       <x:c r="AE36" s="75" t="str">
         <x:v>https://doi.org/10.1117/12.3098133</x:v>
       </x:c>
       <x:c r="AF36" s="75" t="str">
-        <x:v>Highest-priority mismatch competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional abstract and complete proceedings metadata. Feature codes remain provisional. Can a flexible residual absorb noise or unsupported image detail? Extract identifiability constraints, optimization and held-out mismatch tests. Evidence: https://pure.kaist.ac.kr/en/publications/mitigating-forward-model-mismatch-in-inverse-problems-via-learned/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P035, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_10.json (P035, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_11.json (P035, pending_access). No new feature verification.</x:v>
+        <x:v>Highest-priority mismatch competitor | AI pilot 2026-09-16: advance to full-text review; human pending. Basis: Authors' institutional abstract and complete proceedings metadata. Feature codes remain provisional. Can a flexible residual absorb noise or unsupported image detail? Extract identifiability constraints, optimization and held-out mismatch tests. Evidence: https://pure.kaist.ac.kr/en/publications/mitigating-forward-model-mismatch-in-inverse-problems-via-learned/ | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_09.json (P035, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_10.json (P035, pending_access). No new feature verification. | Retrieval 2026-09-16: full-text eligibility pending. Source attempts and next action: screening/full_text_11.json (P035, pending_access). No new feature verification. | AI full-text 2026-09-17: include; human pending. Verified fields: O, P, Q, R, S, T, U, V, W, X. Evidence/version/read extent: screening/full_text_12.json (P035). Unlisted feature codes remain provisional.</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="176" customHeight="1">
@@ -10365,7 +10373,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd699b298488845ed"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16712a24758c45a8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11823,15 +11831,15 @@
       <x:c r="I36" s="93" t="str">
         <x:v>AI pilot: advance</x:v>
       </x:c>
-      <x:c r="J36" s="75" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="K36" s="75"/>
+      <x:c r="J36" s="109" t="str">
+        <x:v>AI full-text: include</x:v>
+      </x:c>
+      <x:c r="K36" s="75" t="str"/>
       <x:c r="L36" s="75" t="str">
-        <x:v>2026-09-16 | Full-text eligibility remains pending. Full article route could not be retrieved; no complete text acquired. Obtain an author manuscript or a full publisher copy through library access/document delivery. Mooseok Jang can be contacted at the public address in P040, PDF p. 1: mooseok@kaist.ac.kr. No message has been sent. Complete retrieval log: screening/full_text_11.json (P035).</x:v>
+        <x:v>2026-09-17 | AI full-text include; human pending. Explicit forward-model discrepancy correction, image/residual identifiability and empirical operational-boundary analysis (sections 2.3-3.3). Uploaded PDF verified and inspected; source/version/hash in register; not committed. Version, read extent and technical extraction: screening/full_text_12.json (P035).</x:v>
       </x:c>
       <x:c r="M36" s="75" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N36" s="75" t="str">
         <x:v>Yes</x:v>
@@ -14340,7 +14348,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51ef18cb9c7f4415"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b74b42e25c8499f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14512,7 +14520,7 @@
         <x:v>Current PRISMA status</x:v>
       </x:c>
       <x:c r="B22" s="60" t="str">
-        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 89 (88 include, 1 exclude), 1 remains. All human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
+        <x:v>Initial triage 90/90 (82 advance, 8 unclear). AI full-text assessed: 90 (89 include, 1 exclude), 0 remain. Human adjudication and formal searches/inclusion pending. Formal inclusion/exclusion counts remain zero.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="62" customHeight="1">
@@ -14520,7 +14528,7 @@
         <x:v>Seed-corpus rule</x:v>
       </x:c>
       <x:c r="B23" s="78" t="str">
-        <x:v>90 seed records retained. Cumulative evidence: screening/full_text_01.json through full_text_11.json. Current report: full_text_11_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
+        <x:v>90 seed records retained. Cumulative evidence: screening/full_text_01.json through full_text_12.json. Current report: full_text_12_report.md. AI decisions require human adjudication. Only listed feature fields are verified; other codes remain provisional.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14766,7 +14774,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfa447c8b8634dfa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03f5771023194d09"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>